<commit_message>
logs: nifty precision signals 2026-06-04
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Signals" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00276221"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL1"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -662,6 +667,252 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>54300</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>54332.8</v>
+      </c>
+      <c r="H2" t="n">
+        <v>88</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>7</v>
+      </c>
+      <c r="L2" t="n">
+        <v>54248.6</v>
+      </c>
+      <c r="M2" t="n">
+        <v>54211.9</v>
+      </c>
+      <c r="N2" t="n">
+        <v>54329.3</v>
+      </c>
+      <c r="O2" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>54137.3</v>
+      </c>
+      <c r="R2" t="n">
+        <v>53837.6</v>
+      </c>
+      <c r="S2" t="n">
+        <v>54295.6</v>
+      </c>
+      <c r="T2" t="n">
+        <v>53028.4</v>
+      </c>
+      <c r="U2" t="n">
+        <v>54052</v>
+      </c>
+      <c r="V2" t="n">
+        <v>53662</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>54264</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB2" t="n">
+        <v>54212.8</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>54692.8</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>15.99</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>54300</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>54323.4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>88</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>7</v>
+      </c>
+      <c r="L3" t="n">
+        <v>54293</v>
+      </c>
+      <c r="M3" t="n">
+        <v>54259.4</v>
+      </c>
+      <c r="N3" t="n">
+        <v>54322.1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>54137.3</v>
+      </c>
+      <c r="R3" t="n">
+        <v>53837.6</v>
+      </c>
+      <c r="S3" t="n">
+        <v>54295.6</v>
+      </c>
+      <c r="T3" t="n">
+        <v>53028.4</v>
+      </c>
+      <c r="U3" t="n">
+        <v>54052</v>
+      </c>
+      <c r="V3" t="n">
+        <v>53662</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y3" t="n">
+        <v>54312.9</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
+        <v>54203.4</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>54683.4</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-05
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,10 @@
     <font>
       <b val="1"/>
       <color rgb="00276221"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +65,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL3"/>
+  <dimension ref="A1:AL9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -906,12 +911,732 @@
       <c r="AF3" t="n">
         <v>15.96</v>
       </c>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>74200</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>74174.39999999999</v>
+      </c>
+      <c r="H4" t="n">
+        <v>78</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" t="n">
+        <v>74252.39999999999</v>
+      </c>
+      <c r="M4" t="n">
+        <v>74323.39999999999</v>
+      </c>
+      <c r="N4" t="n">
+        <v>74190.60000000001</v>
+      </c>
+      <c r="O4" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>74713.10000000001</v>
+      </c>
+      <c r="R4" t="n">
+        <v>74484.3</v>
+      </c>
+      <c r="S4" t="n">
+        <v>74543.5</v>
+      </c>
+      <c r="T4" t="n">
+        <v>73809.5</v>
+      </c>
+      <c r="U4" t="n">
+        <v>74298.8</v>
+      </c>
+      <c r="V4" t="n">
+        <v>74176.5</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>74261.7</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB4" t="n">
+        <v>74374.39999999999</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>73574.39999999999</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>16.12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>23300</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>23323.2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>78</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" t="n">
+        <v>23325.1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>23348.4</v>
+      </c>
+      <c r="N5" t="n">
+        <v>23327.7</v>
+      </c>
+      <c r="O5" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>23513.7</v>
+      </c>
+      <c r="R5" t="n">
+        <v>23440.2</v>
+      </c>
+      <c r="S5" t="n">
+        <v>23465.2</v>
+      </c>
+      <c r="T5" t="n">
+        <v>23249.6</v>
+      </c>
+      <c r="U5" t="n">
+        <v>23411.1</v>
+      </c>
+      <c r="V5" t="n">
+        <v>23357.4</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>23337.3</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB5" t="n">
+        <v>23363.2</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>23203.2</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>16.08</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>54300</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>54273.9</v>
+      </c>
+      <c r="H6" t="n">
+        <v>81</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" t="n">
+        <v>54284.5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>54354.8</v>
+      </c>
+      <c r="N6" t="n">
+        <v>54286</v>
+      </c>
+      <c r="O6" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>54519.1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>54316.4</v>
+      </c>
+      <c r="S6" t="n">
+        <v>54459.6</v>
+      </c>
+      <c r="T6" t="n">
+        <v>53837.6</v>
+      </c>
+      <c r="U6" t="n">
+        <v>54270</v>
+      </c>
+      <c r="V6" t="n">
+        <v>54148.6</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>54285.5</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB6" t="n">
+        <v>54393.9</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>53913.9</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>16.08</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>74100</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>74130.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>88</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>7</v>
+      </c>
+      <c r="L7" t="n">
+        <v>74126.8</v>
+      </c>
+      <c r="M7" t="n">
+        <v>74201</v>
+      </c>
+      <c r="N7" t="n">
+        <v>74137.7</v>
+      </c>
+      <c r="O7" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>74713.10000000001</v>
+      </c>
+      <c r="R7" t="n">
+        <v>74484.3</v>
+      </c>
+      <c r="S7" t="n">
+        <v>74543.5</v>
+      </c>
+      <c r="T7" t="n">
+        <v>73809.5</v>
+      </c>
+      <c r="U7" t="n">
+        <v>74298.8</v>
+      </c>
+      <c r="V7" t="n">
+        <v>74176.5</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>74162.39999999999</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>74330.5</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>73530.5</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>16.15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>14:53</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>74100</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>74095.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>88</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" t="n">
+        <v>74128.60000000001</v>
+      </c>
+      <c r="M8" t="n">
+        <v>74164.5</v>
+      </c>
+      <c r="N8" t="n">
+        <v>74125.89999999999</v>
+      </c>
+      <c r="O8" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>74713.10000000001</v>
+      </c>
+      <c r="R8" t="n">
+        <v>74484.3</v>
+      </c>
+      <c r="S8" t="n">
+        <v>74543.5</v>
+      </c>
+      <c r="T8" t="n">
+        <v>73809.5</v>
+      </c>
+      <c r="U8" t="n">
+        <v>74298.8</v>
+      </c>
+      <c r="V8" t="n">
+        <v>74176.5</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>74162.39999999999</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>74295.5</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>73495.5</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>15.85</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15:08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>54500</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>54493</v>
+      </c>
+      <c r="H9" t="n">
+        <v>85</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" t="n">
+        <v>54432.2</v>
+      </c>
+      <c r="M9" t="n">
+        <v>54391.1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>54481.5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>54519.1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>54316.4</v>
+      </c>
+      <c r="S9" t="n">
+        <v>54459.6</v>
+      </c>
+      <c r="T9" t="n">
+        <v>53837.6</v>
+      </c>
+      <c r="U9" t="n">
+        <v>54270</v>
+      </c>
+      <c r="V9" t="n">
+        <v>54148.6</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>54525.5</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>54373</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>54853</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-08
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL9"/>
+  <dimension ref="A1:AL11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1631,12 +1631,252 @@
       <c r="AF9" t="n">
         <v>15.88</v>
       </c>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>73600</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>73618.39999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>79</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" t="n">
+        <v>73658.5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>73701.39999999999</v>
+      </c>
+      <c r="N10" t="n">
+        <v>73619.8</v>
+      </c>
+      <c r="O10" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>73564.39999999999</v>
+      </c>
+      <c r="R10" t="n">
+        <v>73328.3</v>
+      </c>
+      <c r="S10" t="n">
+        <v>74713.10000000001</v>
+      </c>
+      <c r="T10" t="n">
+        <v>73992.3</v>
+      </c>
+      <c r="U10" t="n">
+        <v>74352.7</v>
+      </c>
+      <c r="V10" t="n">
+        <v>74279.8</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>0.786</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>73513.89999999999</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>73818.39999999999</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>73018.39999999999</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>17.17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:16</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>23150</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>23125.2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>87</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" t="n">
+        <v>23145.8</v>
+      </c>
+      <c r="M11" t="n">
+        <v>23162.2</v>
+      </c>
+      <c r="N11" t="n">
+        <v>23128.7</v>
+      </c>
+      <c r="O11" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>23156.8</v>
+      </c>
+      <c r="R11" t="n">
+        <v>23071.5</v>
+      </c>
+      <c r="S11" t="n">
+        <v>23513.7</v>
+      </c>
+      <c r="T11" t="n">
+        <v>23282.8</v>
+      </c>
+      <c r="U11" t="n">
+        <v>23398.2</v>
+      </c>
+      <c r="V11" t="n">
+        <v>23378.6</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>23124.2</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>23165.2</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>23005.2</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>17.02</v>
+      </c>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-10
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL11"/>
+  <dimension ref="A1:AL16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1871,12 +1871,612 @@
       <c r="AF11" t="n">
         <v>17.02</v>
       </c>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>23400</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>23383.3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>98</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>23388</v>
+      </c>
+      <c r="M12" t="n">
+        <v>23385.3</v>
+      </c>
+      <c r="N12" t="n">
+        <v>23382.3</v>
+      </c>
+      <c r="O12" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>23349.2</v>
+      </c>
+      <c r="R12" t="n">
+        <v>23220.6</v>
+      </c>
+      <c r="S12" t="n">
+        <v>23279.3</v>
+      </c>
+      <c r="T12" t="n">
+        <v>23105.1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>23233.9</v>
+      </c>
+      <c r="V12" t="n">
+        <v>23192.2</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>23376.6</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB12" t="n">
+        <v>23343.3</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>23503.3</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>15.48</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>55500</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>55482.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>88</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>55477.2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>55459.8</v>
+      </c>
+      <c r="N13" t="n">
+        <v>55466.8</v>
+      </c>
+      <c r="O13" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>55394.7</v>
+      </c>
+      <c r="R13" t="n">
+        <v>55096</v>
+      </c>
+      <c r="S13" t="n">
+        <v>55315.9</v>
+      </c>
+      <c r="T13" t="n">
+        <v>54266.8</v>
+      </c>
+      <c r="U13" t="n">
+        <v>55096.5</v>
+      </c>
+      <c r="V13" t="n">
+        <v>54791.3</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>55446.4</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>55362.3</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>55842.3</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>15.48</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>74500</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>74464.8</v>
+      </c>
+      <c r="H14" t="n">
+        <v>83</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>7</v>
+      </c>
+      <c r="L14" t="n">
+        <v>74493.10000000001</v>
+      </c>
+      <c r="M14" t="n">
+        <v>74467.60000000001</v>
+      </c>
+      <c r="N14" t="n">
+        <v>74483.39999999999</v>
+      </c>
+      <c r="O14" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>74352.89999999999</v>
+      </c>
+      <c r="R14" t="n">
+        <v>73897.8</v>
+      </c>
+      <c r="S14" t="n">
+        <v>74032</v>
+      </c>
+      <c r="T14" t="n">
+        <v>73426.8</v>
+      </c>
+      <c r="U14" t="n">
+        <v>73855.5</v>
+      </c>
+      <c r="V14" t="n">
+        <v>73729.39999999999</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>74442.10000000001</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB14" t="n">
+        <v>74264.8</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>75064.8</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>15.48</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>74500</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>74527.89999999999</v>
+      </c>
+      <c r="H15" t="n">
+        <v>98</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" t="n">
+        <v>74497.39999999999</v>
+      </c>
+      <c r="M15" t="n">
+        <v>74471.7</v>
+      </c>
+      <c r="N15" t="n">
+        <v>74498.8</v>
+      </c>
+      <c r="O15" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>74352.89999999999</v>
+      </c>
+      <c r="R15" t="n">
+        <v>73897.8</v>
+      </c>
+      <c r="S15" t="n">
+        <v>74032</v>
+      </c>
+      <c r="T15" t="n">
+        <v>73426.8</v>
+      </c>
+      <c r="U15" t="n">
+        <v>73855.5</v>
+      </c>
+      <c r="V15" t="n">
+        <v>73729.39999999999</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>74442.10000000001</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>74327.89999999999</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>75127.89999999999</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>15.48</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>74400</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>74399.8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>83</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" t="n">
+        <v>74431.2</v>
+      </c>
+      <c r="M16" t="n">
+        <v>74446.5</v>
+      </c>
+      <c r="N16" t="n">
+        <v>74390.8</v>
+      </c>
+      <c r="O16" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>74352.89999999999</v>
+      </c>
+      <c r="R16" t="n">
+        <v>73897.8</v>
+      </c>
+      <c r="S16" t="n">
+        <v>74032</v>
+      </c>
+      <c r="T16" t="n">
+        <v>73426.8</v>
+      </c>
+      <c r="U16" t="n">
+        <v>73855.5</v>
+      </c>
+      <c r="V16" t="n">
+        <v>73729.39999999999</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y16" t="n">
+        <v>74442.10000000001</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>74199.8</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>74999.8</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>15.52</v>
+      </c>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-12
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL16"/>
+  <dimension ref="A1:AL22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2471,12 +2471,732 @@
       <c r="AF16" t="n">
         <v>15.52</v>
       </c>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
-      <c r="AL16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>56300</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>56349.5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>85</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" t="n">
+        <v>56220.6</v>
+      </c>
+      <c r="M17" t="n">
+        <v>56092.6</v>
+      </c>
+      <c r="N17" t="n">
+        <v>56344.9</v>
+      </c>
+      <c r="O17" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>56013.9</v>
+      </c>
+      <c r="R17" t="n">
+        <v>55847.6</v>
+      </c>
+      <c r="S17" t="n">
+        <v>55599.9</v>
+      </c>
+      <c r="T17" t="n">
+        <v>54770.2</v>
+      </c>
+      <c r="U17" t="n">
+        <v>55204.8</v>
+      </c>
+      <c r="V17" t="n">
+        <v>55185</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y17" t="n">
+        <v>56250.1</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>56229.5</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>56709.5</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>14.83</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>74991.60000000001</v>
+      </c>
+      <c r="H18" t="n">
+        <v>88</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>7</v>
+      </c>
+      <c r="L18" t="n">
+        <v>74792.8</v>
+      </c>
+      <c r="M18" t="n">
+        <v>74688.60000000001</v>
+      </c>
+      <c r="N18" t="n">
+        <v>74985.8</v>
+      </c>
+      <c r="O18" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>74854.89999999999</v>
+      </c>
+      <c r="R18" t="n">
+        <v>74693.89999999999</v>
+      </c>
+      <c r="S18" t="n">
+        <v>74393.10000000001</v>
+      </c>
+      <c r="T18" t="n">
+        <v>73520.2</v>
+      </c>
+      <c r="U18" t="n">
+        <v>73956.60000000001</v>
+      </c>
+      <c r="V18" t="n">
+        <v>73873.7</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>74929.8</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>74791.60000000001</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>75591.60000000001</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>14.83</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>23500</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>23509.3</v>
+      </c>
+      <c r="H19" t="n">
+        <v>88</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>7</v>
+      </c>
+      <c r="L19" t="n">
+        <v>23479.2</v>
+      </c>
+      <c r="M19" t="n">
+        <v>23432</v>
+      </c>
+      <c r="N19" t="n">
+        <v>23505.8</v>
+      </c>
+      <c r="O19" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>23455.9</v>
+      </c>
+      <c r="R19" t="n">
+        <v>23400.6</v>
+      </c>
+      <c r="S19" t="n">
+        <v>23327.2</v>
+      </c>
+      <c r="T19" t="n">
+        <v>23072.4</v>
+      </c>
+      <c r="U19" t="n">
+        <v>23199.8</v>
+      </c>
+      <c r="V19" t="n">
+        <v>23191</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y19" t="n">
+        <v>23494.3</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>23469.3</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>23629.3</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>14.79</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>56600</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>56629.9</v>
+      </c>
+      <c r="H20" t="n">
+        <v>85</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>6</v>
+      </c>
+      <c r="L20" t="n">
+        <v>56490.1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>56312.2</v>
+      </c>
+      <c r="N20" t="n">
+        <v>56616.6</v>
+      </c>
+      <c r="O20" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>56013.9</v>
+      </c>
+      <c r="R20" t="n">
+        <v>55847.6</v>
+      </c>
+      <c r="S20" t="n">
+        <v>55599.9</v>
+      </c>
+      <c r="T20" t="n">
+        <v>54770.2</v>
+      </c>
+      <c r="U20" t="n">
+        <v>55204.8</v>
+      </c>
+      <c r="V20" t="n">
+        <v>55185</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>56445.3</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>56509.9</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>56989.9</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>14.89</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>75200</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>75183.60000000001</v>
+      </c>
+      <c r="H21" t="n">
+        <v>88</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>7</v>
+      </c>
+      <c r="L21" t="n">
+        <v>75047.10000000001</v>
+      </c>
+      <c r="M21" t="n">
+        <v>74881</v>
+      </c>
+      <c r="N21" t="n">
+        <v>75181.89999999999</v>
+      </c>
+      <c r="O21" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>74854.89999999999</v>
+      </c>
+      <c r="R21" t="n">
+        <v>74693.89999999999</v>
+      </c>
+      <c r="S21" t="n">
+        <v>74393.10000000001</v>
+      </c>
+      <c r="T21" t="n">
+        <v>73520.2</v>
+      </c>
+      <c r="U21" t="n">
+        <v>73956.60000000001</v>
+      </c>
+      <c r="V21" t="n">
+        <v>73873.7</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y21" t="n">
+        <v>75079.2</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>74983.60000000001</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>75783.60000000001</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>14.89</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>23600</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>23579.9</v>
+      </c>
+      <c r="H22" t="n">
+        <v>85</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" t="n">
+        <v>23545.3</v>
+      </c>
+      <c r="M22" t="n">
+        <v>23494.2</v>
+      </c>
+      <c r="N22" t="n">
+        <v>23576.1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>23455.9</v>
+      </c>
+      <c r="R22" t="n">
+        <v>23400.6</v>
+      </c>
+      <c r="S22" t="n">
+        <v>23327.2</v>
+      </c>
+      <c r="T22" t="n">
+        <v>23072.4</v>
+      </c>
+      <c r="U22" t="n">
+        <v>23199.8</v>
+      </c>
+      <c r="V22" t="n">
+        <v>23191</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>23537.6</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>23539.9</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>23699.9</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>14.89</v>
+      </c>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-16
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL22"/>
+  <dimension ref="A1:AL25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3191,12 +3191,372 @@
       <c r="AF22" t="n">
         <v>14.89</v>
       </c>
-      <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr"/>
-      <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
-      <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>23993.9</v>
+      </c>
+      <c r="H23" t="n">
+        <v>88</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>7</v>
+      </c>
+      <c r="L23" t="n">
+        <v>23987.1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>23977.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>23988.8</v>
+      </c>
+      <c r="O23" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>23940.6</v>
+      </c>
+      <c r="R23" t="n">
+        <v>23889.2</v>
+      </c>
+      <c r="S23" t="n">
+        <v>24009.1</v>
+      </c>
+      <c r="T23" t="n">
+        <v>23818.1</v>
+      </c>
+      <c r="U23" t="n">
+        <v>23913.6</v>
+      </c>
+      <c r="V23" t="n">
+        <v>23875.1</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y23" t="n">
+        <v>23975.6</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>23953.9</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>24113.9</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>13.35</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>76800</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>76783.5</v>
+      </c>
+      <c r="H24" t="n">
+        <v>88</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L24" t="n">
+        <v>76786</v>
+      </c>
+      <c r="M24" t="n">
+        <v>76751.39999999999</v>
+      </c>
+      <c r="N24" t="n">
+        <v>76767.10000000001</v>
+      </c>
+      <c r="O24" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>76606.10000000001</v>
+      </c>
+      <c r="R24" t="n">
+        <v>76444.60000000001</v>
+      </c>
+      <c r="S24" t="n">
+        <v>76817.2</v>
+      </c>
+      <c r="T24" t="n">
+        <v>76144.10000000001</v>
+      </c>
+      <c r="U24" t="n">
+        <v>76480.60000000001</v>
+      </c>
+      <c r="V24" t="n">
+        <v>76336.7</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y24" t="n">
+        <v>76751.3</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>76583.5</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>77383.5</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>13.35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>76800</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>76830.2</v>
+      </c>
+      <c r="H25" t="n">
+        <v>98</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>8</v>
+      </c>
+      <c r="L25" t="n">
+        <v>76796.5</v>
+      </c>
+      <c r="M25" t="n">
+        <v>76764.89999999999</v>
+      </c>
+      <c r="N25" t="n">
+        <v>76809.39999999999</v>
+      </c>
+      <c r="O25" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>76606.10000000001</v>
+      </c>
+      <c r="R25" t="n">
+        <v>76444.60000000001</v>
+      </c>
+      <c r="S25" t="n">
+        <v>76817.2</v>
+      </c>
+      <c r="T25" t="n">
+        <v>76144.10000000001</v>
+      </c>
+      <c r="U25" t="n">
+        <v>76480.60000000001</v>
+      </c>
+      <c r="V25" t="n">
+        <v>76336.7</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y25" t="n">
+        <v>76751.3</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>76630.2</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>77430.2</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr"/>
+      <c r="AL25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-17
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL25"/>
+  <dimension ref="A1:AL30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3551,12 +3551,612 @@
       <c r="AF25" t="n">
         <v>13.35</v>
       </c>
-      <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
-      <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>57517.4</v>
+      </c>
+      <c r="H26" t="n">
+        <v>98</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>8</v>
+      </c>
+      <c r="L26" t="n">
+        <v>57543.9</v>
+      </c>
+      <c r="M26" t="n">
+        <v>57542.2</v>
+      </c>
+      <c r="N26" t="n">
+        <v>57509.2</v>
+      </c>
+      <c r="O26" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>57439.2</v>
+      </c>
+      <c r="R26" t="n">
+        <v>57222.4</v>
+      </c>
+      <c r="S26" t="n">
+        <v>57397.2</v>
+      </c>
+      <c r="T26" t="n">
+        <v>57076.2</v>
+      </c>
+      <c r="U26" t="n">
+        <v>57274.7</v>
+      </c>
+      <c r="V26" t="n">
+        <v>57236.8</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y26" t="n">
+        <v>57545.3</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>57397.4</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>57877.4</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>24060.6</v>
+      </c>
+      <c r="H27" t="n">
+        <v>86</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>7</v>
+      </c>
+      <c r="L27" t="n">
+        <v>24045.5</v>
+      </c>
+      <c r="M27" t="n">
+        <v>24044</v>
+      </c>
+      <c r="N27" t="n">
+        <v>24055.1</v>
+      </c>
+      <c r="O27" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>24045.4</v>
+      </c>
+      <c r="R27" t="n">
+        <v>23969.8</v>
+      </c>
+      <c r="S27" t="n">
+        <v>24002.2</v>
+      </c>
+      <c r="T27" t="n">
+        <v>23889.2</v>
+      </c>
+      <c r="U27" t="n">
+        <v>23977.9</v>
+      </c>
+      <c r="V27" t="n">
+        <v>23945.8</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y27" t="n">
+        <v>24055.1</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>24020.6</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>24180.6</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>57580.8</v>
+      </c>
+      <c r="H28" t="n">
+        <v>98</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>8</v>
+      </c>
+      <c r="L28" t="n">
+        <v>57542.7</v>
+      </c>
+      <c r="M28" t="n">
+        <v>57540.9</v>
+      </c>
+      <c r="N28" t="n">
+        <v>57565.6</v>
+      </c>
+      <c r="O28" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>57439.2</v>
+      </c>
+      <c r="R28" t="n">
+        <v>57222.4</v>
+      </c>
+      <c r="S28" t="n">
+        <v>57397.2</v>
+      </c>
+      <c r="T28" t="n">
+        <v>57076.2</v>
+      </c>
+      <c r="U28" t="n">
+        <v>57274.7</v>
+      </c>
+      <c r="V28" t="n">
+        <v>57236.8</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y28" t="n">
+        <v>57545.3</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>57460.8</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>57940.8</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>13.15</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>24100</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>24083.2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>98</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>8</v>
+      </c>
+      <c r="L29" t="n">
+        <v>24070.5</v>
+      </c>
+      <c r="M29" t="n">
+        <v>24058.3</v>
+      </c>
+      <c r="N29" t="n">
+        <v>24082.4</v>
+      </c>
+      <c r="O29" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>24045.4</v>
+      </c>
+      <c r="R29" t="n">
+        <v>23969.8</v>
+      </c>
+      <c r="S29" t="n">
+        <v>24002.2</v>
+      </c>
+      <c r="T29" t="n">
+        <v>23889.2</v>
+      </c>
+      <c r="U29" t="n">
+        <v>23977.9</v>
+      </c>
+      <c r="V29" t="n">
+        <v>23945.8</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y29" t="n">
+        <v>24075.3</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>24043.2</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>24203.2</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>13.15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>77200</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>77178.60000000001</v>
+      </c>
+      <c r="H30" t="n">
+        <v>88</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>7</v>
+      </c>
+      <c r="L30" t="n">
+        <v>77078</v>
+      </c>
+      <c r="M30" t="n">
+        <v>77051.2</v>
+      </c>
+      <c r="N30" t="n">
+        <v>77160.2</v>
+      </c>
+      <c r="O30" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>77080.10000000001</v>
+      </c>
+      <c r="R30" t="n">
+        <v>76769.2</v>
+      </c>
+      <c r="S30" t="n">
+        <v>76846</v>
+      </c>
+      <c r="T30" t="n">
+        <v>76444.60000000001</v>
+      </c>
+      <c r="U30" t="n">
+        <v>76754</v>
+      </c>
+      <c r="V30" t="n">
+        <v>76645.3</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y30" t="n">
+        <v>77112.8</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>76978.60000000001</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>77778.60000000001</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+      <c r="AL30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-18
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL30"/>
+  <dimension ref="A1:AL35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4151,12 +4151,609 @@
       <c r="AF30" t="n">
         <v>13.15</v>
       </c>
-      <c r="AG30" t="inlineStr"/>
-      <c r="AH30" t="inlineStr"/>
-      <c r="AI30" t="inlineStr"/>
-      <c r="AJ30" t="inlineStr"/>
-      <c r="AK30" t="inlineStr"/>
-      <c r="AL30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>57900</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>57868.7</v>
+      </c>
+      <c r="H31" t="n">
+        <v>83</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>7</v>
+      </c>
+      <c r="L31" t="n">
+        <v>57892.1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>57889</v>
+      </c>
+      <c r="N31" t="n">
+        <v>57875.4</v>
+      </c>
+      <c r="O31" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>57818.9</v>
+      </c>
+      <c r="R31" t="n">
+        <v>57591.9</v>
+      </c>
+      <c r="S31" t="n">
+        <v>57645.1</v>
+      </c>
+      <c r="T31" t="n">
+        <v>57222.4</v>
+      </c>
+      <c r="U31" t="n">
+        <v>57525.4</v>
+      </c>
+      <c r="V31" t="n">
+        <v>57433.7</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y31" t="n">
+        <v>57868.5</v>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>57748.7</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>58228.7</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>12.86</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>77200</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>77237.8</v>
+      </c>
+      <c r="H32" t="n">
+        <v>81</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>7</v>
+      </c>
+      <c r="L32" t="n">
+        <v>77266.2</v>
+      </c>
+      <c r="M32" t="n">
+        <v>77253.7</v>
+      </c>
+      <c r="N32" t="n">
+        <v>77236.60000000001</v>
+      </c>
+      <c r="O32" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>77281.8</v>
+      </c>
+      <c r="R32" t="n">
+        <v>77045.8</v>
+      </c>
+      <c r="S32" t="n">
+        <v>77219</v>
+      </c>
+      <c r="T32" t="n">
+        <v>76769.2</v>
+      </c>
+      <c r="U32" t="n">
+        <v>77101.8</v>
+      </c>
+      <c r="V32" t="n">
+        <v>76994.10000000001</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y32" t="n">
+        <v>77225.8</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>77037.8</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>77837.8</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>12.86</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>24147.8</v>
+      </c>
+      <c r="H33" t="n">
+        <v>88</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>7</v>
+      </c>
+      <c r="L33" t="n">
+        <v>24111</v>
+      </c>
+      <c r="M33" t="n">
+        <v>24107.5</v>
+      </c>
+      <c r="N33" t="n">
+        <v>24134.6</v>
+      </c>
+      <c r="O33" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>24129.6</v>
+      </c>
+      <c r="R33" t="n">
+        <v>24059.7</v>
+      </c>
+      <c r="S33" t="n">
+        <v>24107.8</v>
+      </c>
+      <c r="T33" t="n">
+        <v>23969.8</v>
+      </c>
+      <c r="U33" t="n">
+        <v>24066.9</v>
+      </c>
+      <c r="V33" t="n">
+        <v>24038.8</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y33" t="n">
+        <v>24127</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>24107.8</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>24267.8</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>12.86</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>57900</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>57926.9</v>
+      </c>
+      <c r="H34" t="n">
+        <v>98</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>8</v>
+      </c>
+      <c r="L34" t="n">
+        <v>57876.7</v>
+      </c>
+      <c r="M34" t="n">
+        <v>57875.6</v>
+      </c>
+      <c r="N34" t="n">
+        <v>57918.3</v>
+      </c>
+      <c r="O34" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>57818.9</v>
+      </c>
+      <c r="R34" t="n">
+        <v>57591.9</v>
+      </c>
+      <c r="S34" t="n">
+        <v>57645.1</v>
+      </c>
+      <c r="T34" t="n">
+        <v>57222.4</v>
+      </c>
+      <c r="U34" t="n">
+        <v>57525.4</v>
+      </c>
+      <c r="V34" t="n">
+        <v>57433.7</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y34" t="n">
+        <v>57868.5</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>57806.9</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>58286.9</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>12.86</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>77400</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>77353.39999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>88</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>7</v>
+      </c>
+      <c r="L35" t="n">
+        <v>77247.10000000001</v>
+      </c>
+      <c r="M35" t="n">
+        <v>77237.7</v>
+      </c>
+      <c r="N35" t="n">
+        <v>77318</v>
+      </c>
+      <c r="O35" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
+        <v>77281.8</v>
+      </c>
+      <c r="R35" t="n">
+        <v>77045.8</v>
+      </c>
+      <c r="S35" t="n">
+        <v>77219</v>
+      </c>
+      <c r="T35" t="n">
+        <v>76769.2</v>
+      </c>
+      <c r="U35" t="n">
+        <v>77101.8</v>
+      </c>
+      <c r="V35" t="n">
+        <v>76994.10000000001</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y35" t="n">
+        <v>77280.8</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>77153.39999999999</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>77953.39999999999</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
+      <c r="AL35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-19
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL35"/>
+  <dimension ref="A1:AL37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4748,12 +4748,252 @@
       <c r="AF35" t="n">
         <v>12.86</v>
       </c>
-      <c r="AG35" t="inlineStr"/>
-      <c r="AH35" t="inlineStr"/>
-      <c r="AI35" t="inlineStr"/>
-      <c r="AJ35" t="inlineStr"/>
-      <c r="AK35" t="inlineStr"/>
-      <c r="AL35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>23907.8</v>
+      </c>
+      <c r="H36" t="n">
+        <v>98</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>8</v>
+      </c>
+      <c r="L36" t="n">
+        <v>23952.4</v>
+      </c>
+      <c r="M36" t="n">
+        <v>23956.1</v>
+      </c>
+      <c r="N36" t="n">
+        <v>23915.5</v>
+      </c>
+      <c r="O36" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q36" t="n">
+        <v>23991.2</v>
+      </c>
+      <c r="R36" t="n">
+        <v>23940.4</v>
+      </c>
+      <c r="S36" t="n">
+        <v>24188.9</v>
+      </c>
+      <c r="T36" t="n">
+        <v>24037.2</v>
+      </c>
+      <c r="U36" t="n">
+        <v>24157.3</v>
+      </c>
+      <c r="V36" t="n">
+        <v>24113.1</v>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y36" t="n">
+        <v>23927.1</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>23947.8</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>23787.8</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>13.19</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>76481</v>
+      </c>
+      <c r="H37" t="n">
+        <v>98</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>8</v>
+      </c>
+      <c r="L37" t="n">
+        <v>76622.60000000001</v>
+      </c>
+      <c r="M37" t="n">
+        <v>76633.5</v>
+      </c>
+      <c r="N37" t="n">
+        <v>76508.10000000001</v>
+      </c>
+      <c r="O37" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q37" t="n">
+        <v>76844</v>
+      </c>
+      <c r="R37" t="n">
+        <v>76609.8</v>
+      </c>
+      <c r="S37" t="n">
+        <v>77486.39999999999</v>
+      </c>
+      <c r="T37" t="n">
+        <v>76953.3</v>
+      </c>
+      <c r="U37" t="n">
+        <v>77346.60000000001</v>
+      </c>
+      <c r="V37" t="n">
+        <v>77219.8</v>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y37" t="n">
+        <v>76566.7</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>76681</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>75881</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr"/>
+      <c r="AK37" t="inlineStr"/>
+      <c r="AL37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-22
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL37"/>
+  <dimension ref="A1:AL38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4988,12 +4988,132 @@
       <c r="AF37" t="n">
         <v>12.99</v>
       </c>
-      <c r="AG37" t="inlineStr"/>
-      <c r="AH37" t="inlineStr"/>
-      <c r="AI37" t="inlineStr"/>
-      <c r="AJ37" t="inlineStr"/>
-      <c r="AK37" t="inlineStr"/>
-      <c r="AL37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>57900</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>57916.7</v>
+      </c>
+      <c r="H38" t="n">
+        <v>86</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>7</v>
+      </c>
+      <c r="L38" t="n">
+        <v>57939.7</v>
+      </c>
+      <c r="M38" t="n">
+        <v>57920.2</v>
+      </c>
+      <c r="N38" t="n">
+        <v>57929.9</v>
+      </c>
+      <c r="O38" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q38" t="n">
+        <v>57914.9</v>
+      </c>
+      <c r="R38" t="n">
+        <v>57775.1</v>
+      </c>
+      <c r="S38" t="n">
+        <v>57803.6</v>
+      </c>
+      <c r="T38" t="n">
+        <v>57465.1</v>
+      </c>
+      <c r="U38" t="n">
+        <v>57688</v>
+      </c>
+      <c r="V38" t="n">
+        <v>57634.4</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y38" t="n">
+        <v>57919.3</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB38" t="n">
+        <v>57796.7</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>58276.7</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
+      <c r="AJ38" t="inlineStr"/>
+      <c r="AK38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-23
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL38"/>
+  <dimension ref="A1:AL44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5108,12 +5108,732 @@
       <c r="AF38" t="n">
         <v>12.83</v>
       </c>
-      <c r="AG38" t="inlineStr"/>
-      <c r="AH38" t="inlineStr"/>
-      <c r="AI38" t="inlineStr"/>
-      <c r="AJ38" t="inlineStr"/>
-      <c r="AK38" t="inlineStr"/>
-      <c r="AL38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>57450.1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>83</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>7</v>
+      </c>
+      <c r="L39" t="n">
+        <v>57444.9</v>
+      </c>
+      <c r="M39" t="n">
+        <v>57515.1</v>
+      </c>
+      <c r="N39" t="n">
+        <v>57450.1</v>
+      </c>
+      <c r="O39" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q39" t="n">
+        <v>57948.6</v>
+      </c>
+      <c r="R39" t="n">
+        <v>57782.1</v>
+      </c>
+      <c r="S39" t="n">
+        <v>58008.4</v>
+      </c>
+      <c r="T39" t="n">
+        <v>57720.7</v>
+      </c>
+      <c r="U39" t="n">
+        <v>57882</v>
+      </c>
+      <c r="V39" t="n">
+        <v>57864.6</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y39" t="n">
+        <v>57504.3</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB39" t="n">
+        <v>57570.1</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>57090.1</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>13.69</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>76600</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>76589.2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>83</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>7</v>
+      </c>
+      <c r="L40" t="n">
+        <v>76596.2</v>
+      </c>
+      <c r="M40" t="n">
+        <v>76696.3</v>
+      </c>
+      <c r="N40" t="n">
+        <v>76589.2</v>
+      </c>
+      <c r="O40" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
+        <v>77058.60000000001</v>
+      </c>
+      <c r="R40" t="n">
+        <v>76880.60000000001</v>
+      </c>
+      <c r="S40" t="n">
+        <v>77323.8</v>
+      </c>
+      <c r="T40" t="n">
+        <v>77015</v>
+      </c>
+      <c r="U40" t="n">
+        <v>77169.39999999999</v>
+      </c>
+      <c r="V40" t="n">
+        <v>77119.2</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y40" t="n">
+        <v>76633.3</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB40" t="n">
+        <v>76789.2</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>75989.2</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>13.69</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>23894.8</v>
+      </c>
+      <c r="H41" t="n">
+        <v>83</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>7</v>
+      </c>
+      <c r="L41" t="n">
+        <v>23892.7</v>
+      </c>
+      <c r="M41" t="n">
+        <v>23918.8</v>
+      </c>
+      <c r="N41" t="n">
+        <v>23894.8</v>
+      </c>
+      <c r="O41" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q41" t="n">
+        <v>24095.1</v>
+      </c>
+      <c r="R41" t="n">
+        <v>24040.8</v>
+      </c>
+      <c r="S41" t="n">
+        <v>24168</v>
+      </c>
+      <c r="T41" t="n">
+        <v>24073.8</v>
+      </c>
+      <c r="U41" t="n">
+        <v>24120.9</v>
+      </c>
+      <c r="V41" t="n">
+        <v>24098.2</v>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y41" t="n">
+        <v>23917.7</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB41" t="n">
+        <v>23934.8</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>23774.8</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>13.86</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>57300</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>57338.1</v>
+      </c>
+      <c r="H42" t="n">
+        <v>83</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>7</v>
+      </c>
+      <c r="L42" t="n">
+        <v>57331.2</v>
+      </c>
+      <c r="M42" t="n">
+        <v>57398.8</v>
+      </c>
+      <c r="N42" t="n">
+        <v>57338.1</v>
+      </c>
+      <c r="O42" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
+        <v>57948.6</v>
+      </c>
+      <c r="R42" t="n">
+        <v>57782.1</v>
+      </c>
+      <c r="S42" t="n">
+        <v>58008.4</v>
+      </c>
+      <c r="T42" t="n">
+        <v>57720.7</v>
+      </c>
+      <c r="U42" t="n">
+        <v>57882</v>
+      </c>
+      <c r="V42" t="n">
+        <v>57864.6</v>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y42" t="n">
+        <v>57407.7</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB42" t="n">
+        <v>57458.1</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>56978.1</v>
+      </c>
+      <c r="AE42" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF42" t="n">
+        <v>13.86</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>76466</v>
+      </c>
+      <c r="H43" t="n">
+        <v>83</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>7</v>
+      </c>
+      <c r="L43" t="n">
+        <v>76463.3</v>
+      </c>
+      <c r="M43" t="n">
+        <v>76541</v>
+      </c>
+      <c r="N43" t="n">
+        <v>76466</v>
+      </c>
+      <c r="O43" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q43" t="n">
+        <v>77058.60000000001</v>
+      </c>
+      <c r="R43" t="n">
+        <v>76880.60000000001</v>
+      </c>
+      <c r="S43" t="n">
+        <v>77323.8</v>
+      </c>
+      <c r="T43" t="n">
+        <v>77015</v>
+      </c>
+      <c r="U43" t="n">
+        <v>77169.39999999999</v>
+      </c>
+      <c r="V43" t="n">
+        <v>77119.2</v>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y43" t="n">
+        <v>76534</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB43" t="n">
+        <v>76666</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>75866</v>
+      </c>
+      <c r="AE43" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF43" t="n">
+        <v>13.84</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>76200</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>76229.10000000001</v>
+      </c>
+      <c r="H44" t="n">
+        <v>85</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>6</v>
+      </c>
+      <c r="L44" t="n">
+        <v>76386.2</v>
+      </c>
+      <c r="M44" t="n">
+        <v>76460</v>
+      </c>
+      <c r="N44" t="n">
+        <v>76256.8</v>
+      </c>
+      <c r="O44" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q44" t="n">
+        <v>77058.60000000001</v>
+      </c>
+      <c r="R44" t="n">
+        <v>76880.60000000001</v>
+      </c>
+      <c r="S44" t="n">
+        <v>77323.8</v>
+      </c>
+      <c r="T44" t="n">
+        <v>77015</v>
+      </c>
+      <c r="U44" t="n">
+        <v>77169.39999999999</v>
+      </c>
+      <c r="V44" t="n">
+        <v>77119.2</v>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y44" t="n">
+        <v>76394</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB44" t="n">
+        <v>76429.10000000001</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>75629.10000000001</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>14.03</v>
+      </c>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
+      <c r="AJ44" t="inlineStr"/>
+      <c r="AK44" t="inlineStr"/>
+      <c r="AL44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-24
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL44"/>
+  <dimension ref="A1:AL50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5828,12 +5828,732 @@
       <c r="AF44" t="n">
         <v>14.03</v>
       </c>
-      <c r="AG44" t="inlineStr"/>
-      <c r="AH44" t="inlineStr"/>
-      <c r="AI44" t="inlineStr"/>
-      <c r="AJ44" t="inlineStr"/>
-      <c r="AK44" t="inlineStr"/>
-      <c r="AL44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>58047.1</v>
+      </c>
+      <c r="H45" t="n">
+        <v>85</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>6</v>
+      </c>
+      <c r="L45" t="n">
+        <v>58045</v>
+      </c>
+      <c r="M45" t="n">
+        <v>58003.2</v>
+      </c>
+      <c r="N45" t="n">
+        <v>58040</v>
+      </c>
+      <c r="O45" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q45" t="n">
+        <v>57544.4</v>
+      </c>
+      <c r="R45" t="n">
+        <v>57074.9</v>
+      </c>
+      <c r="S45" t="n">
+        <v>57958.6</v>
+      </c>
+      <c r="T45" t="n">
+        <v>57080.2</v>
+      </c>
+      <c r="U45" t="n">
+        <v>57519.4</v>
+      </c>
+      <c r="V45" t="n">
+        <v>57241.6</v>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y45" t="n">
+        <v>57889.1</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB45" t="n">
+        <v>57927.1</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>58407.1</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>13.55</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>76900</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>76890.89999999999</v>
+      </c>
+      <c r="H46" t="n">
+        <v>78</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>6</v>
+      </c>
+      <c r="L46" t="n">
+        <v>76875.7</v>
+      </c>
+      <c r="M46" t="n">
+        <v>76847.60000000001</v>
+      </c>
+      <c r="N46" t="n">
+        <v>76885.2</v>
+      </c>
+      <c r="O46" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
+        <v>76462.8</v>
+      </c>
+      <c r="R46" t="n">
+        <v>76134.2</v>
+      </c>
+      <c r="S46" t="n">
+        <v>77194.8</v>
+      </c>
+      <c r="T46" t="n">
+        <v>76188.7</v>
+      </c>
+      <c r="U46" t="n">
+        <v>76691.8</v>
+      </c>
+      <c r="V46" t="n">
+        <v>76364.8</v>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y46" t="n">
+        <v>76777.60000000001</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB46" t="n">
+        <v>76690.89999999999</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>77490.89999999999</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>13.55</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>58200</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>58189.5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>75</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>5</v>
+      </c>
+      <c r="L47" t="n">
+        <v>58135.7</v>
+      </c>
+      <c r="M47" t="n">
+        <v>58073.6</v>
+      </c>
+      <c r="N47" t="n">
+        <v>58181.1</v>
+      </c>
+      <c r="O47" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>57544.4</v>
+      </c>
+      <c r="R47" t="n">
+        <v>57074.9</v>
+      </c>
+      <c r="S47" t="n">
+        <v>57958.6</v>
+      </c>
+      <c r="T47" t="n">
+        <v>57080.2</v>
+      </c>
+      <c r="U47" t="n">
+        <v>57519.4</v>
+      </c>
+      <c r="V47" t="n">
+        <v>57241.6</v>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y47" t="n">
+        <v>57952.3</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB47" t="n">
+        <v>58069.5</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>58549.5</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>13.47</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>24049.9</v>
+      </c>
+      <c r="H48" t="n">
+        <v>78</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>6</v>
+      </c>
+      <c r="L48" t="n">
+        <v>24050.6</v>
+      </c>
+      <c r="M48" t="n">
+        <v>24035.5</v>
+      </c>
+      <c r="N48" t="n">
+        <v>24048.9</v>
+      </c>
+      <c r="O48" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>23884.7</v>
+      </c>
+      <c r="R48" t="n">
+        <v>23790.2</v>
+      </c>
+      <c r="S48" t="n">
+        <v>24135.2</v>
+      </c>
+      <c r="T48" t="n">
+        <v>23785.2</v>
+      </c>
+      <c r="U48" t="n">
+        <v>23960.2</v>
+      </c>
+      <c r="V48" t="n">
+        <v>23850.2</v>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y48" t="n">
+        <v>24019.1</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB48" t="n">
+        <v>24009.9</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>24169.9</v>
+      </c>
+      <c r="AE48" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>13.47</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>58200</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>58176.6</v>
+      </c>
+      <c r="H49" t="n">
+        <v>85</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>6</v>
+      </c>
+      <c r="L49" t="n">
+        <v>58158.2</v>
+      </c>
+      <c r="M49" t="n">
+        <v>58119.3</v>
+      </c>
+      <c r="N49" t="n">
+        <v>58166.2</v>
+      </c>
+      <c r="O49" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>57544.4</v>
+      </c>
+      <c r="R49" t="n">
+        <v>57074.9</v>
+      </c>
+      <c r="S49" t="n">
+        <v>57958.6</v>
+      </c>
+      <c r="T49" t="n">
+        <v>57080.2</v>
+      </c>
+      <c r="U49" t="n">
+        <v>57519.4</v>
+      </c>
+      <c r="V49" t="n">
+        <v>57241.6</v>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y49" t="n">
+        <v>57959</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>0.374</v>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB49" t="n">
+        <v>58056.6</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>58536.6</v>
+      </c>
+      <c r="AE49" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>13.47</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>77100</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>77071.10000000001</v>
+      </c>
+      <c r="H50" t="n">
+        <v>75</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>5</v>
+      </c>
+      <c r="L50" t="n">
+        <v>77068.5</v>
+      </c>
+      <c r="M50" t="n">
+        <v>77018.3</v>
+      </c>
+      <c r="N50" t="n">
+        <v>77055.2</v>
+      </c>
+      <c r="O50" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q50" t="n">
+        <v>76462.8</v>
+      </c>
+      <c r="R50" t="n">
+        <v>76134.2</v>
+      </c>
+      <c r="S50" t="n">
+        <v>77194.8</v>
+      </c>
+      <c r="T50" t="n">
+        <v>76188.7</v>
+      </c>
+      <c r="U50" t="n">
+        <v>76691.8</v>
+      </c>
+      <c r="V50" t="n">
+        <v>76364.8</v>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y50" t="n">
+        <v>76940.89999999999</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB50" t="n">
+        <v>76871.10000000001</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>77671.10000000001</v>
+      </c>
+      <c r="AE50" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>13.57</v>
+      </c>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr"/>
+      <c r="AJ50" t="inlineStr"/>
+      <c r="AK50" t="inlineStr"/>
+      <c r="AL50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-25
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL50"/>
+  <dimension ref="A1:AL52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6548,12 +6548,252 @@
       <c r="AF50" t="n">
         <v>13.57</v>
       </c>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr"/>
-      <c r="AI50" t="inlineStr"/>
-      <c r="AJ50" t="inlineStr"/>
-      <c r="AK50" t="inlineStr"/>
-      <c r="AL50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>77593.5</v>
+      </c>
+      <c r="H51" t="n">
+        <v>76</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>6</v>
+      </c>
+      <c r="L51" t="n">
+        <v>77601.10000000001</v>
+      </c>
+      <c r="M51" t="n">
+        <v>77599.10000000001</v>
+      </c>
+      <c r="N51" t="n">
+        <v>77587.60000000001</v>
+      </c>
+      <c r="O51" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
+        <v>77476.10000000001</v>
+      </c>
+      <c r="R51" t="n">
+        <v>77286.3</v>
+      </c>
+      <c r="S51" t="n">
+        <v>77190.10000000001</v>
+      </c>
+      <c r="T51" t="n">
+        <v>76134.2</v>
+      </c>
+      <c r="U51" t="n">
+        <v>76881.39999999999</v>
+      </c>
+      <c r="V51" t="n">
+        <v>76662.10000000001</v>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y51" t="n">
+        <v>77605.7</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB51" t="n">
+        <v>77393.5</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>78193.5</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>12.99</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>58600</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>58561.9</v>
+      </c>
+      <c r="H52" t="n">
+        <v>76</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>6</v>
+      </c>
+      <c r="L52" t="n">
+        <v>58541.3</v>
+      </c>
+      <c r="M52" t="n">
+        <v>58538.1</v>
+      </c>
+      <c r="N52" t="n">
+        <v>58549.7</v>
+      </c>
+      <c r="O52" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>58503.6</v>
+      </c>
+      <c r="R52" t="n">
+        <v>58360.6</v>
+      </c>
+      <c r="S52" t="n">
+        <v>58256</v>
+      </c>
+      <c r="T52" t="n">
+        <v>57074.9</v>
+      </c>
+      <c r="U52" t="n">
+        <v>58003.6</v>
+      </c>
+      <c r="V52" t="n">
+        <v>57665.4</v>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y52" t="n">
+        <v>58573.7</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB52" t="n">
+        <v>58441.9</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>58921.9</v>
+      </c>
+      <c r="AE52" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF52" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
+      <c r="AJ52" t="inlineStr"/>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-29
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL52"/>
+  <dimension ref="A1:AL56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6788,12 +6788,492 @@
       <c r="AF52" t="n">
         <v>12.9</v>
       </c>
-      <c r="AG52" t="inlineStr"/>
-      <c r="AH52" t="inlineStr"/>
-      <c r="AI52" t="inlineStr"/>
-      <c r="AJ52" t="inlineStr"/>
-      <c r="AK52" t="inlineStr"/>
-      <c r="AL52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>23950</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>23947.6</v>
+      </c>
+      <c r="H53" t="n">
+        <v>88</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>7</v>
+      </c>
+      <c r="L53" t="n">
+        <v>23953.8</v>
+      </c>
+      <c r="M53" t="n">
+        <v>23959.4</v>
+      </c>
+      <c r="N53" t="n">
+        <v>23954.4</v>
+      </c>
+      <c r="O53" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
+        <v>24110.7</v>
+      </c>
+      <c r="R53" t="n">
+        <v>24033.7</v>
+      </c>
+      <c r="S53" t="n">
+        <v>24261.1</v>
+      </c>
+      <c r="T53" t="n">
+        <v>24039.3</v>
+      </c>
+      <c r="U53" t="n">
+        <v>24150.2</v>
+      </c>
+      <c r="V53" t="n">
+        <v>24085.3</v>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y53" t="n">
+        <v>23969.7</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB53" t="n">
+        <v>23987.6</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>23827.6</v>
+      </c>
+      <c r="AE53" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>13.87</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>76716.5</v>
+      </c>
+      <c r="H54" t="n">
+        <v>88</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>7</v>
+      </c>
+      <c r="L54" t="n">
+        <v>76725.60000000001</v>
+      </c>
+      <c r="M54" t="n">
+        <v>76745.8</v>
+      </c>
+      <c r="N54" t="n">
+        <v>76736.60000000001</v>
+      </c>
+      <c r="O54" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q54" t="n">
+        <v>77225.10000000001</v>
+      </c>
+      <c r="R54" t="n">
+        <v>76998.60000000001</v>
+      </c>
+      <c r="S54" t="n">
+        <v>77803</v>
+      </c>
+      <c r="T54" t="n">
+        <v>77002.5</v>
+      </c>
+      <c r="U54" t="n">
+        <v>77402.8</v>
+      </c>
+      <c r="V54" t="n">
+        <v>77201.2</v>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y54" t="n">
+        <v>76764.10000000001</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB54" t="n">
+        <v>76916.5</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>76116.5</v>
+      </c>
+      <c r="AE54" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF54" t="n">
+        <v>13.87</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>57717</v>
+      </c>
+      <c r="H55" t="n">
+        <v>88</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>7</v>
+      </c>
+      <c r="L55" t="n">
+        <v>57831.5</v>
+      </c>
+      <c r="M55" t="n">
+        <v>57841.1</v>
+      </c>
+      <c r="N55" t="n">
+        <v>57762.1</v>
+      </c>
+      <c r="O55" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
+        <v>58316.1</v>
+      </c>
+      <c r="R55" t="n">
+        <v>57995.4</v>
+      </c>
+      <c r="S55" t="n">
+        <v>58705.4</v>
+      </c>
+      <c r="T55" t="n">
+        <v>58110.9</v>
+      </c>
+      <c r="U55" t="n">
+        <v>58408.2</v>
+      </c>
+      <c r="V55" t="n">
+        <v>58260.9</v>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y55" t="n">
+        <v>57800.6</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB55" t="n">
+        <v>57837</v>
+      </c>
+      <c r="AC55" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>57357</v>
+      </c>
+      <c r="AE55" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF55" t="n">
+        <v>13.81</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>76689</v>
+      </c>
+      <c r="H56" t="n">
+        <v>88</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>7</v>
+      </c>
+      <c r="L56" t="n">
+        <v>76729.5</v>
+      </c>
+      <c r="M56" t="n">
+        <v>76739.89999999999</v>
+      </c>
+      <c r="N56" t="n">
+        <v>76712.2</v>
+      </c>
+      <c r="O56" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q56" t="n">
+        <v>77225.10000000001</v>
+      </c>
+      <c r="R56" t="n">
+        <v>76998.60000000001</v>
+      </c>
+      <c r="S56" t="n">
+        <v>77803</v>
+      </c>
+      <c r="T56" t="n">
+        <v>77002.5</v>
+      </c>
+      <c r="U56" t="n">
+        <v>77402.8</v>
+      </c>
+      <c r="V56" t="n">
+        <v>77201.2</v>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y56" t="n">
+        <v>76764.10000000001</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB56" t="n">
+        <v>76889</v>
+      </c>
+      <c r="AC56" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>76089</v>
+      </c>
+      <c r="AE56" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF56" t="n">
+        <v>13.81</v>
+      </c>
+      <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr"/>
+      <c r="AJ56" t="inlineStr"/>
+      <c r="AK56" t="inlineStr"/>
+      <c r="AL56" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-06-30
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL56"/>
+  <dimension ref="A1:AL62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7268,12 +7268,732 @@
       <c r="AF56" t="n">
         <v>13.81</v>
       </c>
-      <c r="AG56" t="inlineStr"/>
-      <c r="AH56" t="inlineStr"/>
-      <c r="AI56" t="inlineStr"/>
-      <c r="AJ56" t="inlineStr"/>
-      <c r="AK56" t="inlineStr"/>
-      <c r="AL56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>76600</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>76598.89999999999</v>
+      </c>
+      <c r="H57" t="n">
+        <v>83</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>7</v>
+      </c>
+      <c r="L57" t="n">
+        <v>76669.39999999999</v>
+      </c>
+      <c r="M57" t="n">
+        <v>76680.89999999999</v>
+      </c>
+      <c r="N57" t="n">
+        <v>76615.8</v>
+      </c>
+      <c r="O57" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q57" t="n">
+        <v>77005.8</v>
+      </c>
+      <c r="R57" t="n">
+        <v>76601</v>
+      </c>
+      <c r="S57" t="n">
+        <v>77252.7</v>
+      </c>
+      <c r="T57" t="n">
+        <v>76621.8</v>
+      </c>
+      <c r="U57" t="n">
+        <v>76937.2</v>
+      </c>
+      <c r="V57" t="n">
+        <v>76798</v>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y57" t="n">
+        <v>76587.8</v>
+      </c>
+      <c r="Z57" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB57" t="n">
+        <v>76798.89999999999</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>75998.89999999999</v>
+      </c>
+      <c r="AE57" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF57" t="n">
+        <v>13.37</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>57634.9</v>
+      </c>
+      <c r="H58" t="n">
+        <v>83</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>7</v>
+      </c>
+      <c r="L58" t="n">
+        <v>57666</v>
+      </c>
+      <c r="M58" t="n">
+        <v>57694.6</v>
+      </c>
+      <c r="N58" t="n">
+        <v>57638.1</v>
+      </c>
+      <c r="O58" t="n">
+        <v>38</v>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q58" t="n">
+        <v>58011.9</v>
+      </c>
+      <c r="R58" t="n">
+        <v>57725.1</v>
+      </c>
+      <c r="S58" t="n">
+        <v>58316.1</v>
+      </c>
+      <c r="T58" t="n">
+        <v>57641.4</v>
+      </c>
+      <c r="U58" t="n">
+        <v>57978.8</v>
+      </c>
+      <c r="V58" t="n">
+        <v>57878.3</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y58" t="n">
+        <v>57691.3</v>
+      </c>
+      <c r="Z58" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB58" t="n">
+        <v>57754.9</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>57274.9</v>
+      </c>
+      <c r="AE58" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF58" t="n">
+        <v>13.37</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>23883.2</v>
+      </c>
+      <c r="H59" t="n">
+        <v>88</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>7</v>
+      </c>
+      <c r="L59" t="n">
+        <v>23924.9</v>
+      </c>
+      <c r="M59" t="n">
+        <v>23930.5</v>
+      </c>
+      <c r="N59" t="n">
+        <v>23899.5</v>
+      </c>
+      <c r="O59" t="n">
+        <v>31</v>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q59" t="n">
+        <v>24031.6</v>
+      </c>
+      <c r="R59" t="n">
+        <v>23890.8</v>
+      </c>
+      <c r="S59" t="n">
+        <v>24120</v>
+      </c>
+      <c r="T59" t="n">
+        <v>23925.2</v>
+      </c>
+      <c r="U59" t="n">
+        <v>24022.6</v>
+      </c>
+      <c r="V59" t="n">
+        <v>23993.2</v>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y59" t="n">
+        <v>23894.5</v>
+      </c>
+      <c r="Z59" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB59" t="n">
+        <v>23923.2</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>23763.2</v>
+      </c>
+      <c r="AE59" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF59" t="n">
+        <v>13.39</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>76494</v>
+      </c>
+      <c r="H60" t="n">
+        <v>88</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>7</v>
+      </c>
+      <c r="L60" t="n">
+        <v>76627.89999999999</v>
+      </c>
+      <c r="M60" t="n">
+        <v>76656</v>
+      </c>
+      <c r="N60" t="n">
+        <v>76542.7</v>
+      </c>
+      <c r="O60" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q60" t="n">
+        <v>77005.8</v>
+      </c>
+      <c r="R60" t="n">
+        <v>76601</v>
+      </c>
+      <c r="S60" t="n">
+        <v>77252.7</v>
+      </c>
+      <c r="T60" t="n">
+        <v>76621.8</v>
+      </c>
+      <c r="U60" t="n">
+        <v>76937.2</v>
+      </c>
+      <c r="V60" t="n">
+        <v>76798</v>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y60" t="n">
+        <v>76587.8</v>
+      </c>
+      <c r="Z60" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB60" t="n">
+        <v>76694</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>75894</v>
+      </c>
+      <c r="AE60" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF60" t="n">
+        <v>13.47</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>57664.8</v>
+      </c>
+      <c r="H61" t="n">
+        <v>76</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>6</v>
+      </c>
+      <c r="L61" t="n">
+        <v>57591.6</v>
+      </c>
+      <c r="M61" t="n">
+        <v>57632.9</v>
+      </c>
+      <c r="N61" t="n">
+        <v>57613.6</v>
+      </c>
+      <c r="O61" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q61" t="n">
+        <v>58011.9</v>
+      </c>
+      <c r="R61" t="n">
+        <v>57725.1</v>
+      </c>
+      <c r="S61" t="n">
+        <v>58316.1</v>
+      </c>
+      <c r="T61" t="n">
+        <v>57641.4</v>
+      </c>
+      <c r="U61" t="n">
+        <v>57978.8</v>
+      </c>
+      <c r="V61" t="n">
+        <v>57878.3</v>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y61" t="n">
+        <v>57674.1</v>
+      </c>
+      <c r="Z61" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB61" t="n">
+        <v>57784.8</v>
+      </c>
+      <c r="AC61" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>57304.8</v>
+      </c>
+      <c r="AE61" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF61" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>23850</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>23836.1</v>
+      </c>
+      <c r="H62" t="n">
+        <v>85</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
+        <v>6</v>
+      </c>
+      <c r="L62" t="n">
+        <v>23909.8</v>
+      </c>
+      <c r="M62" t="n">
+        <v>23920</v>
+      </c>
+      <c r="N62" t="n">
+        <v>23857.9</v>
+      </c>
+      <c r="O62" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q62" t="n">
+        <v>24031.6</v>
+      </c>
+      <c r="R62" t="n">
+        <v>23890.8</v>
+      </c>
+      <c r="S62" t="n">
+        <v>24120</v>
+      </c>
+      <c r="T62" t="n">
+        <v>23925.2</v>
+      </c>
+      <c r="U62" t="n">
+        <v>24022.6</v>
+      </c>
+      <c r="V62" t="n">
+        <v>23993.2</v>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y62" t="n">
+        <v>23878.7</v>
+      </c>
+      <c r="Z62" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB62" t="n">
+        <v>23876.1</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>23716.1</v>
+      </c>
+      <c r="AE62" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF62" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr"/>
+      <c r="AJ62" t="inlineStr"/>
+      <c r="AK62" t="inlineStr"/>
+      <c r="AL62" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-01
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL62"/>
+  <dimension ref="A1:AL68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7988,12 +7988,732 @@
       <c r="AF62" t="n">
         <v>13.35</v>
       </c>
-      <c r="AG62" t="inlineStr"/>
-      <c r="AH62" t="inlineStr"/>
-      <c r="AI62" t="inlineStr"/>
-      <c r="AJ62" t="inlineStr"/>
-      <c r="AK62" t="inlineStr"/>
-      <c r="AL62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>58016.2</v>
+      </c>
+      <c r="H63" t="n">
+        <v>83</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
+        <v>7</v>
+      </c>
+      <c r="L63" t="n">
+        <v>57994.8</v>
+      </c>
+      <c r="M63" t="n">
+        <v>57965.6</v>
+      </c>
+      <c r="N63" t="n">
+        <v>58020.3</v>
+      </c>
+      <c r="O63" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q63" t="n">
+        <v>57651.8</v>
+      </c>
+      <c r="R63" t="n">
+        <v>57487.9</v>
+      </c>
+      <c r="S63" t="n">
+        <v>58011.9</v>
+      </c>
+      <c r="T63" t="n">
+        <v>57457.7</v>
+      </c>
+      <c r="U63" t="n">
+        <v>57734.8</v>
+      </c>
+      <c r="V63" t="n">
+        <v>57705.3</v>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y63" t="n">
+        <v>57932.7</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB63" t="n">
+        <v>57896.2</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>58376.2</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>13.32</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>77000</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>76975.89999999999</v>
+      </c>
+      <c r="H64" t="n">
+        <v>88</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
+        <v>7</v>
+      </c>
+      <c r="L64" t="n">
+        <v>77007.10000000001</v>
+      </c>
+      <c r="M64" t="n">
+        <v>76998.89999999999</v>
+      </c>
+      <c r="N64" t="n">
+        <v>76965.89999999999</v>
+      </c>
+      <c r="O64" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q64" t="n">
+        <v>76695.39999999999</v>
+      </c>
+      <c r="R64" t="n">
+        <v>76543.3</v>
+      </c>
+      <c r="S64" t="n">
+        <v>77005.8</v>
+      </c>
+      <c r="T64" t="n">
+        <v>76331.2</v>
+      </c>
+      <c r="U64" t="n">
+        <v>76668.5</v>
+      </c>
+      <c r="V64" t="n">
+        <v>76541.8</v>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y64" t="n">
+        <v>76972.8</v>
+      </c>
+      <c r="Z64" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB64" t="n">
+        <v>76775.89999999999</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>77575.89999999999</v>
+      </c>
+      <c r="AE64" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF64" t="n">
+        <v>13.32</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>77100</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>77058.89999999999</v>
+      </c>
+      <c r="H65" t="n">
+        <v>98</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>8</v>
+      </c>
+      <c r="L65" t="n">
+        <v>77017.39999999999</v>
+      </c>
+      <c r="M65" t="n">
+        <v>77004.39999999999</v>
+      </c>
+      <c r="N65" t="n">
+        <v>77034.3</v>
+      </c>
+      <c r="O65" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q65" t="n">
+        <v>76695.39999999999</v>
+      </c>
+      <c r="R65" t="n">
+        <v>76543.3</v>
+      </c>
+      <c r="S65" t="n">
+        <v>77005.8</v>
+      </c>
+      <c r="T65" t="n">
+        <v>76331.2</v>
+      </c>
+      <c r="U65" t="n">
+        <v>76668.5</v>
+      </c>
+      <c r="V65" t="n">
+        <v>76541.8</v>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y65" t="n">
+        <v>76972.8</v>
+      </c>
+      <c r="Z65" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB65" t="n">
+        <v>76858.89999999999</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>77658.89999999999</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>13.32</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>24033.6</v>
+      </c>
+      <c r="H66" t="n">
+        <v>83</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>7</v>
+      </c>
+      <c r="L66" t="n">
+        <v>24027.4</v>
+      </c>
+      <c r="M66" t="n">
+        <v>24023.3</v>
+      </c>
+      <c r="N66" t="n">
+        <v>24033.6</v>
+      </c>
+      <c r="O66" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q66" t="n">
+        <v>23934.4</v>
+      </c>
+      <c r="R66" t="n">
+        <v>23896</v>
+      </c>
+      <c r="S66" t="n">
+        <v>24031.6</v>
+      </c>
+      <c r="T66" t="n">
+        <v>23830.2</v>
+      </c>
+      <c r="U66" t="n">
+        <v>23930.9</v>
+      </c>
+      <c r="V66" t="n">
+        <v>23922.1</v>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y66" t="n">
+        <v>24013.4</v>
+      </c>
+      <c r="Z66" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB66" t="n">
+        <v>23993.6</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>24153.6</v>
+      </c>
+      <c r="AE66" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF66" t="n">
+        <v>13.32</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>58017.6</v>
+      </c>
+      <c r="H67" t="n">
+        <v>83</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
+        <v>7</v>
+      </c>
+      <c r="L67" t="n">
+        <v>57997</v>
+      </c>
+      <c r="M67" t="n">
+        <v>57978.6</v>
+      </c>
+      <c r="N67" t="n">
+        <v>58017.6</v>
+      </c>
+      <c r="O67" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q67" t="n">
+        <v>57651.8</v>
+      </c>
+      <c r="R67" t="n">
+        <v>57487.9</v>
+      </c>
+      <c r="S67" t="n">
+        <v>58011.9</v>
+      </c>
+      <c r="T67" t="n">
+        <v>57457.7</v>
+      </c>
+      <c r="U67" t="n">
+        <v>57734.8</v>
+      </c>
+      <c r="V67" t="n">
+        <v>57705.3</v>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y67" t="n">
+        <v>57932.7</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB67" t="n">
+        <v>57897.6</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>58377.6</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>13.32</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>77000</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>77029.5</v>
+      </c>
+      <c r="H68" t="n">
+        <v>83</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>7</v>
+      </c>
+      <c r="L68" t="n">
+        <v>77018.39999999999</v>
+      </c>
+      <c r="M68" t="n">
+        <v>77010</v>
+      </c>
+      <c r="N68" t="n">
+        <v>77029.5</v>
+      </c>
+      <c r="O68" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q68" t="n">
+        <v>76695.39999999999</v>
+      </c>
+      <c r="R68" t="n">
+        <v>76543.3</v>
+      </c>
+      <c r="S68" t="n">
+        <v>77005.8</v>
+      </c>
+      <c r="T68" t="n">
+        <v>76331.2</v>
+      </c>
+      <c r="U68" t="n">
+        <v>76668.5</v>
+      </c>
+      <c r="V68" t="n">
+        <v>76541.8</v>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y68" t="n">
+        <v>76972.8</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB68" t="n">
+        <v>76829.5</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD68" t="n">
+        <v>77629.5</v>
+      </c>
+      <c r="AE68" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF68" t="n">
+        <v>13.32</v>
+      </c>
+      <c r="AG68" t="inlineStr"/>
+      <c r="AH68" t="inlineStr"/>
+      <c r="AI68" t="inlineStr"/>
+      <c r="AJ68" t="inlineStr"/>
+      <c r="AK68" t="inlineStr"/>
+      <c r="AL68" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-02
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL68"/>
+  <dimension ref="A1:AL74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8708,12 +8708,732 @@
       <c r="AF68" t="n">
         <v>13.32</v>
       </c>
-      <c r="AG68" t="inlineStr"/>
-      <c r="AH68" t="inlineStr"/>
-      <c r="AI68" t="inlineStr"/>
-      <c r="AJ68" t="inlineStr"/>
-      <c r="AK68" t="inlineStr"/>
-      <c r="AL68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>24127.2</v>
+      </c>
+      <c r="H69" t="n">
+        <v>89</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>7</v>
+      </c>
+      <c r="L69" t="n">
+        <v>24122.7</v>
+      </c>
+      <c r="M69" t="n">
+        <v>24115.7</v>
+      </c>
+      <c r="N69" t="n">
+        <v>24126</v>
+      </c>
+      <c r="O69" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q69" t="n">
+        <v>24127.2</v>
+      </c>
+      <c r="R69" t="n">
+        <v>24062.2</v>
+      </c>
+      <c r="S69" t="n">
+        <v>24049.6</v>
+      </c>
+      <c r="T69" t="n">
+        <v>23896</v>
+      </c>
+      <c r="U69" t="n">
+        <v>23983</v>
+      </c>
+      <c r="V69" t="n">
+        <v>23972.8</v>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y69" t="n">
+        <v>24122.1</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB69" t="n">
+        <v>24087.2</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>24247.2</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF69" t="n">
+        <v>12.57</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>77300</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>77327.10000000001</v>
+      </c>
+      <c r="H70" t="n">
+        <v>79</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>6</v>
+      </c>
+      <c r="L70" t="n">
+        <v>77309</v>
+      </c>
+      <c r="M70" t="n">
+        <v>77279.2</v>
+      </c>
+      <c r="N70" t="n">
+        <v>77324.7</v>
+      </c>
+      <c r="O70" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q70" t="n">
+        <v>77348.8</v>
+      </c>
+      <c r="R70" t="n">
+        <v>77083</v>
+      </c>
+      <c r="S70" t="n">
+        <v>77105.5</v>
+      </c>
+      <c r="T70" t="n">
+        <v>76543.3</v>
+      </c>
+      <c r="U70" t="n">
+        <v>76890.10000000001</v>
+      </c>
+      <c r="V70" t="n">
+        <v>76824.39999999999</v>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y70" t="n">
+        <v>77308</v>
+      </c>
+      <c r="Z70" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB70" t="n">
+        <v>77127.10000000001</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD70" t="n">
+        <v>77927.10000000001</v>
+      </c>
+      <c r="AE70" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF70" t="n">
+        <v>12.57</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>24143.8</v>
+      </c>
+      <c r="H71" t="n">
+        <v>98</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
+        <v>8</v>
+      </c>
+      <c r="L71" t="n">
+        <v>24140</v>
+      </c>
+      <c r="M71" t="n">
+        <v>24129.2</v>
+      </c>
+      <c r="N71" t="n">
+        <v>24142.4</v>
+      </c>
+      <c r="O71" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q71" t="n">
+        <v>24127.2</v>
+      </c>
+      <c r="R71" t="n">
+        <v>24062.2</v>
+      </c>
+      <c r="S71" t="n">
+        <v>24049.6</v>
+      </c>
+      <c r="T71" t="n">
+        <v>23896</v>
+      </c>
+      <c r="U71" t="n">
+        <v>23983</v>
+      </c>
+      <c r="V71" t="n">
+        <v>23972.8</v>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y71" t="n">
+        <v>24136.3</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB71" t="n">
+        <v>24103.8</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>24263.8</v>
+      </c>
+      <c r="AE71" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF71" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>77400</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>77381.10000000001</v>
+      </c>
+      <c r="H72" t="n">
+        <v>83</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
+        <v>7</v>
+      </c>
+      <c r="L72" t="n">
+        <v>77358.5</v>
+      </c>
+      <c r="M72" t="n">
+        <v>77321.3</v>
+      </c>
+      <c r="N72" t="n">
+        <v>77384.89999999999</v>
+      </c>
+      <c r="O72" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q72" t="n">
+        <v>77348.8</v>
+      </c>
+      <c r="R72" t="n">
+        <v>77083</v>
+      </c>
+      <c r="S72" t="n">
+        <v>77105.5</v>
+      </c>
+      <c r="T72" t="n">
+        <v>76543.3</v>
+      </c>
+      <c r="U72" t="n">
+        <v>76890.10000000001</v>
+      </c>
+      <c r="V72" t="n">
+        <v>76824.39999999999</v>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y72" t="n">
+        <v>77361.2</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB72" t="n">
+        <v>77181.10000000001</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>77981.10000000001</v>
+      </c>
+      <c r="AE72" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF72" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>77400</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>77372.7</v>
+      </c>
+      <c r="H73" t="n">
+        <v>98</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K73" t="n">
+        <v>8</v>
+      </c>
+      <c r="L73" t="n">
+        <v>77369.5</v>
+      </c>
+      <c r="M73" t="n">
+        <v>77333.5</v>
+      </c>
+      <c r="N73" t="n">
+        <v>77369</v>
+      </c>
+      <c r="O73" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q73" t="n">
+        <v>77348.8</v>
+      </c>
+      <c r="R73" t="n">
+        <v>77083</v>
+      </c>
+      <c r="S73" t="n">
+        <v>77105.5</v>
+      </c>
+      <c r="T73" t="n">
+        <v>76543.3</v>
+      </c>
+      <c r="U73" t="n">
+        <v>76890.10000000001</v>
+      </c>
+      <c r="V73" t="n">
+        <v>76824.39999999999</v>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y73" t="n">
+        <v>77361.2</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB73" t="n">
+        <v>77172.7</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD73" t="n">
+        <v>77972.7</v>
+      </c>
+      <c r="AE73" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF73" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>24137.8</v>
+      </c>
+      <c r="H74" t="n">
+        <v>98</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K74" t="n">
+        <v>8</v>
+      </c>
+      <c r="L74" t="n">
+        <v>24136.2</v>
+      </c>
+      <c r="M74" t="n">
+        <v>24131.7</v>
+      </c>
+      <c r="N74" t="n">
+        <v>24136.1</v>
+      </c>
+      <c r="O74" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q74" t="n">
+        <v>24127.2</v>
+      </c>
+      <c r="R74" t="n">
+        <v>24062.2</v>
+      </c>
+      <c r="S74" t="n">
+        <v>24049.6</v>
+      </c>
+      <c r="T74" t="n">
+        <v>23896</v>
+      </c>
+      <c r="U74" t="n">
+        <v>23983</v>
+      </c>
+      <c r="V74" t="n">
+        <v>23972.8</v>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y74" t="n">
+        <v>24136.3</v>
+      </c>
+      <c r="Z74" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB74" t="n">
+        <v>24097.8</v>
+      </c>
+      <c r="AC74" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD74" t="n">
+        <v>24257.8</v>
+      </c>
+      <c r="AE74" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF74" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="AG74" t="inlineStr"/>
+      <c r="AH74" t="inlineStr"/>
+      <c r="AI74" t="inlineStr"/>
+      <c r="AJ74" t="inlineStr"/>
+      <c r="AK74" t="inlineStr"/>
+      <c r="AL74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-03
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL74"/>
+  <dimension ref="A1:AL80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9428,12 +9428,732 @@
       <c r="AF74" t="n">
         <v>12.51</v>
       </c>
-      <c r="AG74" t="inlineStr"/>
-      <c r="AH74" t="inlineStr"/>
-      <c r="AI74" t="inlineStr"/>
-      <c r="AJ74" t="inlineStr"/>
-      <c r="AK74" t="inlineStr"/>
-      <c r="AL74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>57900</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>57933.1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>78</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K75" t="n">
+        <v>6</v>
+      </c>
+      <c r="L75" t="n">
+        <v>57969.2</v>
+      </c>
+      <c r="M75" t="n">
+        <v>57994.6</v>
+      </c>
+      <c r="N75" t="n">
+        <v>57942.7</v>
+      </c>
+      <c r="O75" t="n">
+        <v>41</v>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q75" t="n">
+        <v>58313.5</v>
+      </c>
+      <c r="R75" t="n">
+        <v>57979.1</v>
+      </c>
+      <c r="S75" t="n">
+        <v>58395.7</v>
+      </c>
+      <c r="T75" t="n">
+        <v>57885.4</v>
+      </c>
+      <c r="U75" t="n">
+        <v>58140.6</v>
+      </c>
+      <c r="V75" t="n">
+        <v>58025.4</v>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y75" t="n">
+        <v>58010.3</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB75" t="n">
+        <v>58053.1</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD75" t="n">
+        <v>57573.1</v>
+      </c>
+      <c r="AE75" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF75" t="n">
+        <v>11.81</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>78000</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>78025.3</v>
+      </c>
+      <c r="H76" t="n">
+        <v>86</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K76" t="n">
+        <v>7</v>
+      </c>
+      <c r="L76" t="n">
+        <v>78045</v>
+      </c>
+      <c r="M76" t="n">
+        <v>78034.7</v>
+      </c>
+      <c r="N76" t="n">
+        <v>78024</v>
+      </c>
+      <c r="O76" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q76" t="n">
+        <v>78139.39999999999</v>
+      </c>
+      <c r="R76" t="n">
+        <v>77855.3</v>
+      </c>
+      <c r="S76" t="n">
+        <v>77577.39999999999</v>
+      </c>
+      <c r="T76" t="n">
+        <v>77083</v>
+      </c>
+      <c r="U76" t="n">
+        <v>77444.89999999999</v>
+      </c>
+      <c r="V76" t="n">
+        <v>77330.2</v>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y76" t="n">
+        <v>78030.8</v>
+      </c>
+      <c r="Z76" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB76" t="n">
+        <v>77825.3</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD76" t="n">
+        <v>78625.3</v>
+      </c>
+      <c r="AE76" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF76" t="n">
+        <v>11.81</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>57800</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>57849</v>
+      </c>
+      <c r="H77" t="n">
+        <v>90</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>6</v>
+      </c>
+      <c r="L77" t="n">
+        <v>57938.9</v>
+      </c>
+      <c r="M77" t="n">
+        <v>57978.1</v>
+      </c>
+      <c r="N77" t="n">
+        <v>57864.7</v>
+      </c>
+      <c r="O77" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q77" t="n">
+        <v>58313.5</v>
+      </c>
+      <c r="R77" t="n">
+        <v>57979.1</v>
+      </c>
+      <c r="S77" t="n">
+        <v>58395.7</v>
+      </c>
+      <c r="T77" t="n">
+        <v>57885.4</v>
+      </c>
+      <c r="U77" t="n">
+        <v>58140.6</v>
+      </c>
+      <c r="V77" t="n">
+        <v>58025.4</v>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y77" t="n">
+        <v>57958.6</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB77" t="n">
+        <v>57969</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD77" t="n">
+        <v>57489</v>
+      </c>
+      <c r="AE77" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF77" t="n">
+        <v>11.89</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>24305.1</v>
+      </c>
+      <c r="H78" t="n">
+        <v>75</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
+        <v>5</v>
+      </c>
+      <c r="L78" t="n">
+        <v>24325.2</v>
+      </c>
+      <c r="M78" t="n">
+        <v>24335.5</v>
+      </c>
+      <c r="N78" t="n">
+        <v>24307.6</v>
+      </c>
+      <c r="O78" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q78" t="n">
+        <v>24375.7</v>
+      </c>
+      <c r="R78" t="n">
+        <v>24295.4</v>
+      </c>
+      <c r="S78" t="n">
+        <v>24194.6</v>
+      </c>
+      <c r="T78" t="n">
+        <v>24062.2</v>
+      </c>
+      <c r="U78" t="n">
+        <v>24154.8</v>
+      </c>
+      <c r="V78" t="n">
+        <v>24128.4</v>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y78" t="n">
+        <v>24314.4</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB78" t="n">
+        <v>24345.1</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>24185.1</v>
+      </c>
+      <c r="AE78" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF78" t="n">
+        <v>11.89</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>57800</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>57811.9</v>
+      </c>
+      <c r="H79" t="n">
+        <v>90</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K79" t="n">
+        <v>6</v>
+      </c>
+      <c r="L79" t="n">
+        <v>57876.3</v>
+      </c>
+      <c r="M79" t="n">
+        <v>57927</v>
+      </c>
+      <c r="N79" t="n">
+        <v>57820.2</v>
+      </c>
+      <c r="O79" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q79" t="n">
+        <v>58313.5</v>
+      </c>
+      <c r="R79" t="n">
+        <v>57979.1</v>
+      </c>
+      <c r="S79" t="n">
+        <v>58395.7</v>
+      </c>
+      <c r="T79" t="n">
+        <v>57885.4</v>
+      </c>
+      <c r="U79" t="n">
+        <v>58140.6</v>
+      </c>
+      <c r="V79" t="n">
+        <v>58025.4</v>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y79" t="n">
+        <v>57928.6</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB79" t="n">
+        <v>57931.9</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD79" t="n">
+        <v>57451.9</v>
+      </c>
+      <c r="AE79" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF79" t="n">
+        <v>11.95</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>77900</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>77880.8</v>
+      </c>
+      <c r="H80" t="n">
+        <v>75</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
+        <v>5</v>
+      </c>
+      <c r="L80" t="n">
+        <v>77949.89999999999</v>
+      </c>
+      <c r="M80" t="n">
+        <v>77987.2</v>
+      </c>
+      <c r="N80" t="n">
+        <v>77887.5</v>
+      </c>
+      <c r="O80" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q80" t="n">
+        <v>78139.39999999999</v>
+      </c>
+      <c r="R80" t="n">
+        <v>77855.3</v>
+      </c>
+      <c r="S80" t="n">
+        <v>77577.39999999999</v>
+      </c>
+      <c r="T80" t="n">
+        <v>77083</v>
+      </c>
+      <c r="U80" t="n">
+        <v>77444.89999999999</v>
+      </c>
+      <c r="V80" t="n">
+        <v>77330.2</v>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y80" t="n">
+        <v>77922.3</v>
+      </c>
+      <c r="Z80" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB80" t="n">
+        <v>78080.8</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>77280.8</v>
+      </c>
+      <c r="AE80" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF80" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="AG80" t="inlineStr"/>
+      <c r="AH80" t="inlineStr"/>
+      <c r="AI80" t="inlineStr"/>
+      <c r="AJ80" t="inlineStr"/>
+      <c r="AK80" t="inlineStr"/>
+      <c r="AL80" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-06
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL80"/>
+  <dimension ref="A1:AL86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10148,12 +10148,732 @@
       <c r="AF80" t="n">
         <v>11.95</v>
       </c>
-      <c r="AG80" t="inlineStr"/>
-      <c r="AH80" t="inlineStr"/>
-      <c r="AI80" t="inlineStr"/>
-      <c r="AJ80" t="inlineStr"/>
-      <c r="AK80" t="inlineStr"/>
-      <c r="AL80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>24450</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>24429.3</v>
+      </c>
+      <c r="H81" t="n">
+        <v>88</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K81" t="n">
+        <v>7</v>
+      </c>
+      <c r="L81" t="n">
+        <v>24438</v>
+      </c>
+      <c r="M81" t="n">
+        <v>24436.3</v>
+      </c>
+      <c r="N81" t="n">
+        <v>24430.8</v>
+      </c>
+      <c r="O81" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q81" t="n">
+        <v>24359.1</v>
+      </c>
+      <c r="R81" t="n">
+        <v>24290.1</v>
+      </c>
+      <c r="S81" t="n">
+        <v>24375.7</v>
+      </c>
+      <c r="T81" t="n">
+        <v>24252.8</v>
+      </c>
+      <c r="U81" t="n">
+        <v>24314.2</v>
+      </c>
+      <c r="V81" t="n">
+        <v>24285.8</v>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y81" t="n">
+        <v>24418.6</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB81" t="n">
+        <v>24389.3</v>
+      </c>
+      <c r="AC81" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>24549.3</v>
+      </c>
+      <c r="AE81" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF81" t="n">
+        <v>11.92</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>58400</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>58395.9</v>
+      </c>
+      <c r="H82" t="n">
+        <v>88</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
+        <v>7</v>
+      </c>
+      <c r="L82" t="n">
+        <v>58406.6</v>
+      </c>
+      <c r="M82" t="n">
+        <v>58396.4</v>
+      </c>
+      <c r="N82" t="n">
+        <v>58397.2</v>
+      </c>
+      <c r="O82" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q82" t="n">
+        <v>58348.9</v>
+      </c>
+      <c r="R82" t="n">
+        <v>57943</v>
+      </c>
+      <c r="S82" t="n">
+        <v>58313.5</v>
+      </c>
+      <c r="T82" t="n">
+        <v>57799.1</v>
+      </c>
+      <c r="U82" t="n">
+        <v>58056.3</v>
+      </c>
+      <c r="V82" t="n">
+        <v>58000.9</v>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y82" t="n">
+        <v>58350.6</v>
+      </c>
+      <c r="Z82" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB82" t="n">
+        <v>58275.9</v>
+      </c>
+      <c r="AC82" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD82" t="n">
+        <v>58755.9</v>
+      </c>
+      <c r="AE82" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF82" t="n">
+        <v>11.92</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>78400</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>78357.10000000001</v>
+      </c>
+      <c r="H83" t="n">
+        <v>100</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>8</v>
+      </c>
+      <c r="L83" t="n">
+        <v>78345.2</v>
+      </c>
+      <c r="M83" t="n">
+        <v>78324.8</v>
+      </c>
+      <c r="N83" t="n">
+        <v>78348.7</v>
+      </c>
+      <c r="O83" t="n">
+        <v>57</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q83" t="n">
+        <v>78087.2</v>
+      </c>
+      <c r="R83" t="n">
+        <v>77882.60000000001</v>
+      </c>
+      <c r="S83" t="n">
+        <v>78139.39999999999</v>
+      </c>
+      <c r="T83" t="n">
+        <v>77710</v>
+      </c>
+      <c r="U83" t="n">
+        <v>77924.7</v>
+      </c>
+      <c r="V83" t="n">
+        <v>77817.5</v>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y83" t="n">
+        <v>78268.5</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB83" t="n">
+        <v>78157.10000000001</v>
+      </c>
+      <c r="AC83" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>78957.10000000001</v>
+      </c>
+      <c r="AE83" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF83" t="n">
+        <v>11.92</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>58400</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>58367.8</v>
+      </c>
+      <c r="H84" t="n">
+        <v>100</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>8</v>
+      </c>
+      <c r="L84" t="n">
+        <v>58396.5</v>
+      </c>
+      <c r="M84" t="n">
+        <v>58392.5</v>
+      </c>
+      <c r="N84" t="n">
+        <v>58366.8</v>
+      </c>
+      <c r="O84" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q84" t="n">
+        <v>58348.9</v>
+      </c>
+      <c r="R84" t="n">
+        <v>57943</v>
+      </c>
+      <c r="S84" t="n">
+        <v>58313.5</v>
+      </c>
+      <c r="T84" t="n">
+        <v>57799.1</v>
+      </c>
+      <c r="U84" t="n">
+        <v>58056.3</v>
+      </c>
+      <c r="V84" t="n">
+        <v>58000.9</v>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y84" t="n">
+        <v>58350.6</v>
+      </c>
+      <c r="Z84" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB84" t="n">
+        <v>58247.8</v>
+      </c>
+      <c r="AC84" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>58727.8</v>
+      </c>
+      <c r="AE84" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF84" t="n">
+        <v>11.92</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>58400</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>58351.6</v>
+      </c>
+      <c r="H85" t="n">
+        <v>88</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>7</v>
+      </c>
+      <c r="L85" t="n">
+        <v>58358.4</v>
+      </c>
+      <c r="M85" t="n">
+        <v>58372.1</v>
+      </c>
+      <c r="N85" t="n">
+        <v>58343.1</v>
+      </c>
+      <c r="O85" t="n">
+        <v>44</v>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q85" t="n">
+        <v>58348.9</v>
+      </c>
+      <c r="R85" t="n">
+        <v>57943</v>
+      </c>
+      <c r="S85" t="n">
+        <v>58313.5</v>
+      </c>
+      <c r="T85" t="n">
+        <v>57799.1</v>
+      </c>
+      <c r="U85" t="n">
+        <v>58056.3</v>
+      </c>
+      <c r="V85" t="n">
+        <v>58000.9</v>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y85" t="n">
+        <v>58350.6</v>
+      </c>
+      <c r="Z85" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB85" t="n">
+        <v>58231.6</v>
+      </c>
+      <c r="AC85" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD85" t="n">
+        <v>58711.6</v>
+      </c>
+      <c r="AE85" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF85" t="n">
+        <v>11.92</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>24450</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>24440.3</v>
+      </c>
+      <c r="H86" t="n">
+        <v>100</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>8</v>
+      </c>
+      <c r="L86" t="n">
+        <v>24421</v>
+      </c>
+      <c r="M86" t="n">
+        <v>24419.1</v>
+      </c>
+      <c r="N86" t="n">
+        <v>24440.3</v>
+      </c>
+      <c r="O86" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q86" t="n">
+        <v>24359.1</v>
+      </c>
+      <c r="R86" t="n">
+        <v>24290.1</v>
+      </c>
+      <c r="S86" t="n">
+        <v>24375.7</v>
+      </c>
+      <c r="T86" t="n">
+        <v>24252.8</v>
+      </c>
+      <c r="U86" t="n">
+        <v>24314.2</v>
+      </c>
+      <c r="V86" t="n">
+        <v>24285.8</v>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y86" t="n">
+        <v>24418.6</v>
+      </c>
+      <c r="Z86" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB86" t="n">
+        <v>24400.3</v>
+      </c>
+      <c r="AC86" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>24560.3</v>
+      </c>
+      <c r="AE86" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF86" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="AG86" t="inlineStr"/>
+      <c r="AH86" t="inlineStr"/>
+      <c r="AI86" t="inlineStr"/>
+      <c r="AJ86" t="inlineStr"/>
+      <c r="AK86" t="inlineStr"/>
+      <c r="AL86" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-07
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL86"/>
+  <dimension ref="A1:AL93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10868,12 +10868,852 @@
       <c r="AF86" t="n">
         <v>11.78</v>
       </c>
-      <c r="AG86" t="inlineStr"/>
-      <c r="AH86" t="inlineStr"/>
-      <c r="AI86" t="inlineStr"/>
-      <c r="AJ86" t="inlineStr"/>
-      <c r="AK86" t="inlineStr"/>
-      <c r="AL86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>13:09</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>58300</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>58280.9</v>
+      </c>
+      <c r="H87" t="n">
+        <v>87</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>6</v>
+      </c>
+      <c r="L87" t="n">
+        <v>58332.9</v>
+      </c>
+      <c r="M87" t="n">
+        <v>58366.8</v>
+      </c>
+      <c r="N87" t="n">
+        <v>58297.1</v>
+      </c>
+      <c r="O87" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q87" t="n">
+        <v>58554.2</v>
+      </c>
+      <c r="R87" t="n">
+        <v>58342.4</v>
+      </c>
+      <c r="S87" t="n">
+        <v>58476.6</v>
+      </c>
+      <c r="T87" t="n">
+        <v>57943</v>
+      </c>
+      <c r="U87" t="n">
+        <v>58245.3</v>
+      </c>
+      <c r="V87" t="n">
+        <v>58209.8</v>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y87" t="n">
+        <v>58344.2</v>
+      </c>
+      <c r="Z87" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB87" t="n">
+        <v>58400.9</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>57920.9</v>
+      </c>
+      <c r="AE87" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF87" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>13:09</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>78400</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>78402</v>
+      </c>
+      <c r="H88" t="n">
+        <v>76</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>5</v>
+      </c>
+      <c r="L88" t="n">
+        <v>78473</v>
+      </c>
+      <c r="M88" t="n">
+        <v>78505.7</v>
+      </c>
+      <c r="N88" t="n">
+        <v>78422.89999999999</v>
+      </c>
+      <c r="O88" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q88" t="n">
+        <v>78485.89999999999</v>
+      </c>
+      <c r="R88" t="n">
+        <v>78273.8</v>
+      </c>
+      <c r="S88" t="n">
+        <v>78397.89999999999</v>
+      </c>
+      <c r="T88" t="n">
+        <v>77882.60000000001</v>
+      </c>
+      <c r="U88" t="n">
+        <v>78236.8</v>
+      </c>
+      <c r="V88" t="n">
+        <v>78140.3</v>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y88" t="n">
+        <v>78396.89999999999</v>
+      </c>
+      <c r="Z88" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB88" t="n">
+        <v>78602</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD88" t="n">
+        <v>77802</v>
+      </c>
+      <c r="AE88" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF88" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>24400</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>24421.2</v>
+      </c>
+      <c r="H89" t="n">
+        <v>77</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>5</v>
+      </c>
+      <c r="L89" t="n">
+        <v>24454.2</v>
+      </c>
+      <c r="M89" t="n">
+        <v>24472.2</v>
+      </c>
+      <c r="N89" t="n">
+        <v>24427.1</v>
+      </c>
+      <c r="O89" t="n">
+        <v>25</v>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q89" t="n">
+        <v>24482.1</v>
+      </c>
+      <c r="R89" t="n">
+        <v>24428.5</v>
+      </c>
+      <c r="S89" t="n">
+        <v>24458.2</v>
+      </c>
+      <c r="T89" t="n">
+        <v>24290.1</v>
+      </c>
+      <c r="U89" t="n">
+        <v>24407.2</v>
+      </c>
+      <c r="V89" t="n">
+        <v>24374.2</v>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y89" t="n">
+        <v>24435.5</v>
+      </c>
+      <c r="Z89" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB89" t="n">
+        <v>24461.2</v>
+      </c>
+      <c r="AC89" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD89" t="n">
+        <v>24301.2</v>
+      </c>
+      <c r="AE89" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF89" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>58200</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>58239.6</v>
+      </c>
+      <c r="H90" t="n">
+        <v>87</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>6</v>
+      </c>
+      <c r="L90" t="n">
+        <v>58274.1</v>
+      </c>
+      <c r="M90" t="n">
+        <v>58317.2</v>
+      </c>
+      <c r="N90" t="n">
+        <v>58249.1</v>
+      </c>
+      <c r="O90" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q90" t="n">
+        <v>58554.2</v>
+      </c>
+      <c r="R90" t="n">
+        <v>58342.4</v>
+      </c>
+      <c r="S90" t="n">
+        <v>58476.6</v>
+      </c>
+      <c r="T90" t="n">
+        <v>57943</v>
+      </c>
+      <c r="U90" t="n">
+        <v>58245.3</v>
+      </c>
+      <c r="V90" t="n">
+        <v>58209.8</v>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y90" t="n">
+        <v>58294.9</v>
+      </c>
+      <c r="Z90" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB90" t="n">
+        <v>58359.6</v>
+      </c>
+      <c r="AC90" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD90" t="n">
+        <v>57879.6</v>
+      </c>
+      <c r="AE90" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF90" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>78300</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>78266.7</v>
+      </c>
+      <c r="H91" t="n">
+        <v>77</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>5</v>
+      </c>
+      <c r="L91" t="n">
+        <v>78329.2</v>
+      </c>
+      <c r="M91" t="n">
+        <v>78398.10000000001</v>
+      </c>
+      <c r="N91" t="n">
+        <v>78283.2</v>
+      </c>
+      <c r="O91" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q91" t="n">
+        <v>78485.89999999999</v>
+      </c>
+      <c r="R91" t="n">
+        <v>78273.8</v>
+      </c>
+      <c r="S91" t="n">
+        <v>78397.89999999999</v>
+      </c>
+      <c r="T91" t="n">
+        <v>77882.60000000001</v>
+      </c>
+      <c r="U91" t="n">
+        <v>78236.8</v>
+      </c>
+      <c r="V91" t="n">
+        <v>78140.3</v>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y91" t="n">
+        <v>78307.8</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB91" t="n">
+        <v>78466.7</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>77666.7</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>24450</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>24461.8</v>
+      </c>
+      <c r="H92" t="n">
+        <v>76</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>5</v>
+      </c>
+      <c r="L92" t="n">
+        <v>24450.5</v>
+      </c>
+      <c r="M92" t="n">
+        <v>24455.2</v>
+      </c>
+      <c r="N92" t="n">
+        <v>24462.4</v>
+      </c>
+      <c r="O92" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q92" t="n">
+        <v>24482.1</v>
+      </c>
+      <c r="R92" t="n">
+        <v>24428.5</v>
+      </c>
+      <c r="S92" t="n">
+        <v>24458.2</v>
+      </c>
+      <c r="T92" t="n">
+        <v>24290.1</v>
+      </c>
+      <c r="U92" t="n">
+        <v>24407.2</v>
+      </c>
+      <c r="V92" t="n">
+        <v>24374.2</v>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y92" t="n">
+        <v>24458.2</v>
+      </c>
+      <c r="Z92" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB92" t="n">
+        <v>24501.8</v>
+      </c>
+      <c r="AC92" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD92" t="n">
+        <v>24341.8</v>
+      </c>
+      <c r="AE92" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF92" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>58300</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>58296.3</v>
+      </c>
+      <c r="H93" t="n">
+        <v>87</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>6</v>
+      </c>
+      <c r="L93" t="n">
+        <v>58282.3</v>
+      </c>
+      <c r="M93" t="n">
+        <v>58300</v>
+      </c>
+      <c r="N93" t="n">
+        <v>58303.8</v>
+      </c>
+      <c r="O93" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q93" t="n">
+        <v>58554.2</v>
+      </c>
+      <c r="R93" t="n">
+        <v>58342.4</v>
+      </c>
+      <c r="S93" t="n">
+        <v>58476.6</v>
+      </c>
+      <c r="T93" t="n">
+        <v>57943</v>
+      </c>
+      <c r="U93" t="n">
+        <v>58245.3</v>
+      </c>
+      <c r="V93" t="n">
+        <v>58209.8</v>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y93" t="n">
+        <v>58294.9</v>
+      </c>
+      <c r="Z93" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB93" t="n">
+        <v>58416.3</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD93" t="n">
+        <v>57936.3</v>
+      </c>
+      <c r="AE93" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF93" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="AG93" t="inlineStr"/>
+      <c r="AH93" t="inlineStr"/>
+      <c r="AI93" t="inlineStr"/>
+      <c r="AJ93" t="inlineStr"/>
+      <c r="AK93" t="inlineStr"/>
+      <c r="AL93" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-08
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL93"/>
+  <dimension ref="A1:AL99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11708,12 +11708,732 @@
       <c r="AF93" t="n">
         <v>11.68</v>
       </c>
-      <c r="AG93" t="inlineStr"/>
-      <c r="AH93" t="inlineStr"/>
-      <c r="AI93" t="inlineStr"/>
-      <c r="AJ93" t="inlineStr"/>
-      <c r="AK93" t="inlineStr"/>
-      <c r="AL93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>24218.8</v>
+      </c>
+      <c r="H94" t="n">
+        <v>78</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>6</v>
+      </c>
+      <c r="L94" t="n">
+        <v>24237.6</v>
+      </c>
+      <c r="M94" t="n">
+        <v>24251.1</v>
+      </c>
+      <c r="N94" t="n">
+        <v>24224</v>
+      </c>
+      <c r="O94" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q94" t="n">
+        <v>24294.2</v>
+      </c>
+      <c r="R94" t="n">
+        <v>24232.1</v>
+      </c>
+      <c r="S94" t="n">
+        <v>24530.2</v>
+      </c>
+      <c r="T94" t="n">
+        <v>24349.5</v>
+      </c>
+      <c r="U94" t="n">
+        <v>24439.8</v>
+      </c>
+      <c r="V94" t="n">
+        <v>24383.3</v>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y94" t="n">
+        <v>24227.8</v>
+      </c>
+      <c r="Z94" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB94" t="n">
+        <v>24258.8</v>
+      </c>
+      <c r="AC94" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD94" t="n">
+        <v>24098.8</v>
+      </c>
+      <c r="AE94" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF94" t="n">
+        <v>12.21</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>57749.6</v>
+      </c>
+      <c r="H95" t="n">
+        <v>78</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>6</v>
+      </c>
+      <c r="L95" t="n">
+        <v>57807.7</v>
+      </c>
+      <c r="M95" t="n">
+        <v>57855.9</v>
+      </c>
+      <c r="N95" t="n">
+        <v>57750.6</v>
+      </c>
+      <c r="O95" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q95" t="n">
+        <v>58001.3</v>
+      </c>
+      <c r="R95" t="n">
+        <v>57816.1</v>
+      </c>
+      <c r="S95" t="n">
+        <v>58554.2</v>
+      </c>
+      <c r="T95" t="n">
+        <v>58110.2</v>
+      </c>
+      <c r="U95" t="n">
+        <v>58332.2</v>
+      </c>
+      <c r="V95" t="n">
+        <v>58200.4</v>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y95" t="n">
+        <v>57776.7</v>
+      </c>
+      <c r="Z95" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB95" t="n">
+        <v>57869.6</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>57389.6</v>
+      </c>
+      <c r="AE95" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF95" t="n">
+        <v>12.21</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>77594.39999999999</v>
+      </c>
+      <c r="H96" t="n">
+        <v>78</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>6</v>
+      </c>
+      <c r="L96" t="n">
+        <v>77650</v>
+      </c>
+      <c r="M96" t="n">
+        <v>77696.3</v>
+      </c>
+      <c r="N96" t="n">
+        <v>77607.2</v>
+      </c>
+      <c r="O96" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q96" t="n">
+        <v>77841.8</v>
+      </c>
+      <c r="R96" t="n">
+        <v>77620.39999999999</v>
+      </c>
+      <c r="S96" t="n">
+        <v>78664.3</v>
+      </c>
+      <c r="T96" t="n">
+        <v>78170.39999999999</v>
+      </c>
+      <c r="U96" t="n">
+        <v>78417.39999999999</v>
+      </c>
+      <c r="V96" t="n">
+        <v>78259.8</v>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y96" t="n">
+        <v>77619.8</v>
+      </c>
+      <c r="Z96" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB96" t="n">
+        <v>77794.39999999999</v>
+      </c>
+      <c r="AC96" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD96" t="n">
+        <v>76994.39999999999</v>
+      </c>
+      <c r="AE96" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF96" t="n">
+        <v>12.21</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>24211.1</v>
+      </c>
+      <c r="H97" t="n">
+        <v>78</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>6</v>
+      </c>
+      <c r="L97" t="n">
+        <v>24212</v>
+      </c>
+      <c r="M97" t="n">
+        <v>24229.5</v>
+      </c>
+      <c r="N97" t="n">
+        <v>24211.4</v>
+      </c>
+      <c r="O97" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q97" t="n">
+        <v>24294.2</v>
+      </c>
+      <c r="R97" t="n">
+        <v>24232.1</v>
+      </c>
+      <c r="S97" t="n">
+        <v>24530.2</v>
+      </c>
+      <c r="T97" t="n">
+        <v>24349.5</v>
+      </c>
+      <c r="U97" t="n">
+        <v>24439.8</v>
+      </c>
+      <c r="V97" t="n">
+        <v>24383.3</v>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y97" t="n">
+        <v>24210.5</v>
+      </c>
+      <c r="Z97" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB97" t="n">
+        <v>24251.1</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD97" t="n">
+        <v>24091.1</v>
+      </c>
+      <c r="AE97" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF97" t="n">
+        <v>12.21</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>57800</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>57808.9</v>
+      </c>
+      <c r="H98" t="n">
+        <v>91</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>7</v>
+      </c>
+      <c r="L98" t="n">
+        <v>57793.2</v>
+      </c>
+      <c r="M98" t="n">
+        <v>57827.8</v>
+      </c>
+      <c r="N98" t="n">
+        <v>57814.8</v>
+      </c>
+      <c r="O98" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q98" t="n">
+        <v>58001.3</v>
+      </c>
+      <c r="R98" t="n">
+        <v>57816.1</v>
+      </c>
+      <c r="S98" t="n">
+        <v>58554.2</v>
+      </c>
+      <c r="T98" t="n">
+        <v>58110.2</v>
+      </c>
+      <c r="U98" t="n">
+        <v>58332.2</v>
+      </c>
+      <c r="V98" t="n">
+        <v>58200.4</v>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y98" t="n">
+        <v>57819.6</v>
+      </c>
+      <c r="Z98" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB98" t="n">
+        <v>57928.9</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>57448.9</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF98" t="n">
+        <v>12.19</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>24224.6</v>
+      </c>
+      <c r="H99" t="n">
+        <v>91</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>7</v>
+      </c>
+      <c r="L99" t="n">
+        <v>24218</v>
+      </c>
+      <c r="M99" t="n">
+        <v>24228.2</v>
+      </c>
+      <c r="N99" t="n">
+        <v>24228.1</v>
+      </c>
+      <c r="O99" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q99" t="n">
+        <v>24294.2</v>
+      </c>
+      <c r="R99" t="n">
+        <v>24232.1</v>
+      </c>
+      <c r="S99" t="n">
+        <v>24530.2</v>
+      </c>
+      <c r="T99" t="n">
+        <v>24349.5</v>
+      </c>
+      <c r="U99" t="n">
+        <v>24439.8</v>
+      </c>
+      <c r="V99" t="n">
+        <v>24383.3</v>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y99" t="n">
+        <v>24226.5</v>
+      </c>
+      <c r="Z99" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB99" t="n">
+        <v>24264.6</v>
+      </c>
+      <c r="AC99" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD99" t="n">
+        <v>24104.6</v>
+      </c>
+      <c r="AE99" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF99" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="AG99" t="inlineStr"/>
+      <c r="AH99" t="inlineStr"/>
+      <c r="AI99" t="inlineStr"/>
+      <c r="AJ99" t="inlineStr"/>
+      <c r="AK99" t="inlineStr"/>
+      <c r="AL99" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-10
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL99"/>
+  <dimension ref="A1:AL105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12428,12 +12428,732 @@
       <c r="AF99" t="n">
         <v>12.19</v>
       </c>
-      <c r="AG99" t="inlineStr"/>
-      <c r="AH99" t="inlineStr"/>
-      <c r="AI99" t="inlineStr"/>
-      <c r="AJ99" t="inlineStr"/>
-      <c r="AK99" t="inlineStr"/>
-      <c r="AL99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>24196</v>
+      </c>
+      <c r="H100" t="n">
+        <v>98</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>8</v>
+      </c>
+      <c r="L100" t="n">
+        <v>24187.6</v>
+      </c>
+      <c r="M100" t="n">
+        <v>24183.4</v>
+      </c>
+      <c r="N100" t="n">
+        <v>24194.9</v>
+      </c>
+      <c r="O100" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q100" t="n">
+        <v>24187.3</v>
+      </c>
+      <c r="R100" t="n">
+        <v>24125.1</v>
+      </c>
+      <c r="S100" t="n">
+        <v>24133.3</v>
+      </c>
+      <c r="T100" t="n">
+        <v>23926.6</v>
+      </c>
+      <c r="U100" t="n">
+        <v>24030</v>
+      </c>
+      <c r="V100" t="n">
+        <v>23997.9</v>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y100" t="n">
+        <v>24202</v>
+      </c>
+      <c r="Z100" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB100" t="n">
+        <v>24156</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD100" t="n">
+        <v>24316</v>
+      </c>
+      <c r="AE100" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF100" t="n">
+        <v>12.37</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>58100</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>58141.9</v>
+      </c>
+      <c r="H101" t="n">
+        <v>85</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>6</v>
+      </c>
+      <c r="L101" t="n">
+        <v>58027.4</v>
+      </c>
+      <c r="M101" t="n">
+        <v>57964.4</v>
+      </c>
+      <c r="N101" t="n">
+        <v>58127</v>
+      </c>
+      <c r="O101" t="n">
+        <v>82</v>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q101" t="n">
+        <v>57882.4</v>
+      </c>
+      <c r="R101" t="n">
+        <v>57592.5</v>
+      </c>
+      <c r="S101" t="n">
+        <v>57464.2</v>
+      </c>
+      <c r="T101" t="n">
+        <v>56867.3</v>
+      </c>
+      <c r="U101" t="n">
+        <v>57270.4</v>
+      </c>
+      <c r="V101" t="n">
+        <v>57165.8</v>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y101" t="n">
+        <v>58013.7</v>
+      </c>
+      <c r="Z101" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB101" t="n">
+        <v>58021.9</v>
+      </c>
+      <c r="AC101" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD101" t="n">
+        <v>58501.9</v>
+      </c>
+      <c r="AE101" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF101" t="n">
+        <v>12.37</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>77511.5</v>
+      </c>
+      <c r="H102" t="n">
+        <v>89</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>7</v>
+      </c>
+      <c r="L102" t="n">
+        <v>77477.5</v>
+      </c>
+      <c r="M102" t="n">
+        <v>77464.39999999999</v>
+      </c>
+      <c r="N102" t="n">
+        <v>77505.8</v>
+      </c>
+      <c r="O102" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q102" t="n">
+        <v>77523.39999999999</v>
+      </c>
+      <c r="R102" t="n">
+        <v>77340.5</v>
+      </c>
+      <c r="S102" t="n">
+        <v>77322.10000000001</v>
+      </c>
+      <c r="T102" t="n">
+        <v>76576.10000000001</v>
+      </c>
+      <c r="U102" t="n">
+        <v>76949.10000000001</v>
+      </c>
+      <c r="V102" t="n">
+        <v>76810.89999999999</v>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y102" t="n">
+        <v>77493.5</v>
+      </c>
+      <c r="Z102" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB102" t="n">
+        <v>77311.5</v>
+      </c>
+      <c r="AC102" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD102" t="n">
+        <v>78111.5</v>
+      </c>
+      <c r="AE102" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF102" t="n">
+        <v>12.37</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>58003.7</v>
+      </c>
+      <c r="H103" t="n">
+        <v>100</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>8</v>
+      </c>
+      <c r="L103" t="n">
+        <v>58025.1</v>
+      </c>
+      <c r="M103" t="n">
+        <v>57984.6</v>
+      </c>
+      <c r="N103" t="n">
+        <v>58000</v>
+      </c>
+      <c r="O103" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q103" t="n">
+        <v>57882.4</v>
+      </c>
+      <c r="R103" t="n">
+        <v>57592.5</v>
+      </c>
+      <c r="S103" t="n">
+        <v>57464.2</v>
+      </c>
+      <c r="T103" t="n">
+        <v>56867.3</v>
+      </c>
+      <c r="U103" t="n">
+        <v>57270.4</v>
+      </c>
+      <c r="V103" t="n">
+        <v>57165.8</v>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y103" t="n">
+        <v>58000</v>
+      </c>
+      <c r="Z103" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB103" t="n">
+        <v>57883.7</v>
+      </c>
+      <c r="AC103" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD103" t="n">
+        <v>58363.7</v>
+      </c>
+      <c r="AE103" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF103" t="n">
+        <v>12.35</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>24190.5</v>
+      </c>
+      <c r="H104" t="n">
+        <v>100</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>8</v>
+      </c>
+      <c r="L104" t="n">
+        <v>24181.9</v>
+      </c>
+      <c r="M104" t="n">
+        <v>24181.1</v>
+      </c>
+      <c r="N104" t="n">
+        <v>24188.5</v>
+      </c>
+      <c r="O104" t="n">
+        <v>56</v>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q104" t="n">
+        <v>24187.3</v>
+      </c>
+      <c r="R104" t="n">
+        <v>24125.1</v>
+      </c>
+      <c r="S104" t="n">
+        <v>24133.3</v>
+      </c>
+      <c r="T104" t="n">
+        <v>23926.6</v>
+      </c>
+      <c r="U104" t="n">
+        <v>24030</v>
+      </c>
+      <c r="V104" t="n">
+        <v>23997.9</v>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y104" t="n">
+        <v>24187.3</v>
+      </c>
+      <c r="Z104" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB104" t="n">
+        <v>24150.5</v>
+      </c>
+      <c r="AC104" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD104" t="n">
+        <v>24310.5</v>
+      </c>
+      <c r="AE104" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF104" t="n">
+        <v>12.34</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>77455.8</v>
+      </c>
+      <c r="H105" t="n">
+        <v>83</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>7</v>
+      </c>
+      <c r="L105" t="n">
+        <v>77479.7</v>
+      </c>
+      <c r="M105" t="n">
+        <v>77473.10000000001</v>
+      </c>
+      <c r="N105" t="n">
+        <v>77452.39999999999</v>
+      </c>
+      <c r="O105" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q105" t="n">
+        <v>77523.39999999999</v>
+      </c>
+      <c r="R105" t="n">
+        <v>77340.5</v>
+      </c>
+      <c r="S105" t="n">
+        <v>77322.10000000001</v>
+      </c>
+      <c r="T105" t="n">
+        <v>76576.10000000001</v>
+      </c>
+      <c r="U105" t="n">
+        <v>76949.10000000001</v>
+      </c>
+      <c r="V105" t="n">
+        <v>76810.89999999999</v>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Y105" t="n">
+        <v>77464.3</v>
+      </c>
+      <c r="Z105" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB105" t="n">
+        <v>77255.8</v>
+      </c>
+      <c r="AC105" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD105" t="n">
+        <v>78055.8</v>
+      </c>
+      <c r="AE105" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF105" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="AG105" t="inlineStr"/>
+      <c r="AH105" t="inlineStr"/>
+      <c r="AI105" t="inlineStr"/>
+      <c r="AJ105" t="inlineStr"/>
+      <c r="AK105" t="inlineStr"/>
+      <c r="AL105" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-13
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL105"/>
+  <dimension ref="A1:AL111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13148,12 +13148,732 @@
       <c r="AF105" t="n">
         <v>12.34</v>
       </c>
-      <c r="AG105" t="inlineStr"/>
-      <c r="AH105" t="inlineStr"/>
-      <c r="AI105" t="inlineStr"/>
-      <c r="AJ105" t="inlineStr"/>
-      <c r="AK105" t="inlineStr"/>
-      <c r="AL105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>77400</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>77439.8</v>
+      </c>
+      <c r="H106" t="n">
+        <v>79</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>5</v>
+      </c>
+      <c r="L106" t="n">
+        <v>77393.7</v>
+      </c>
+      <c r="M106" t="n">
+        <v>77352.2</v>
+      </c>
+      <c r="N106" t="n">
+        <v>77432.39999999999</v>
+      </c>
+      <c r="O106" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q106" t="n">
+        <v>77001.2</v>
+      </c>
+      <c r="R106" t="n">
+        <v>76881.3</v>
+      </c>
+      <c r="S106" t="n">
+        <v>77640.8</v>
+      </c>
+      <c r="T106" t="n">
+        <v>77340.5</v>
+      </c>
+      <c r="U106" t="n">
+        <v>77543.2</v>
+      </c>
+      <c r="V106" t="n">
+        <v>77490.7</v>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y106" t="n">
+        <v>77311.60000000001</v>
+      </c>
+      <c r="Z106" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB106" t="n">
+        <v>77239.8</v>
+      </c>
+      <c r="AC106" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD106" t="n">
+        <v>78039.8</v>
+      </c>
+      <c r="AE106" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF106" t="n">
+        <v>13.36</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>57958.6</v>
+      </c>
+      <c r="H107" t="n">
+        <v>82</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>6</v>
+      </c>
+      <c r="L107" t="n">
+        <v>57898.4</v>
+      </c>
+      <c r="M107" t="n">
+        <v>57885</v>
+      </c>
+      <c r="N107" t="n">
+        <v>57940.2</v>
+      </c>
+      <c r="O107" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q107" t="n">
+        <v>57650.8</v>
+      </c>
+      <c r="R107" t="n">
+        <v>57493.8</v>
+      </c>
+      <c r="S107" t="n">
+        <v>58251.9</v>
+      </c>
+      <c r="T107" t="n">
+        <v>57592.5</v>
+      </c>
+      <c r="U107" t="n">
+        <v>58008.1</v>
+      </c>
+      <c r="V107" t="n">
+        <v>57922.2</v>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y107" t="n">
+        <v>57933.9</v>
+      </c>
+      <c r="Z107" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB107" t="n">
+        <v>57838.6</v>
+      </c>
+      <c r="AC107" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD107" t="n">
+        <v>58318.6</v>
+      </c>
+      <c r="AE107" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF107" t="n">
+        <v>13.36</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>24202.7</v>
+      </c>
+      <c r="H108" t="n">
+        <v>75</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>5</v>
+      </c>
+      <c r="L108" t="n">
+        <v>24180.8</v>
+      </c>
+      <c r="M108" t="n">
+        <v>24159.5</v>
+      </c>
+      <c r="N108" t="n">
+        <v>24201.4</v>
+      </c>
+      <c r="O108" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q108" t="n">
+        <v>24044</v>
+      </c>
+      <c r="R108" t="n">
+        <v>24000.8</v>
+      </c>
+      <c r="S108" t="n">
+        <v>24228.2</v>
+      </c>
+      <c r="T108" t="n">
+        <v>24125.1</v>
+      </c>
+      <c r="U108" t="n">
+        <v>24200</v>
+      </c>
+      <c r="V108" t="n">
+        <v>24176.6</v>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y108" t="n">
+        <v>24158.9</v>
+      </c>
+      <c r="Z108" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB108" t="n">
+        <v>24162.7</v>
+      </c>
+      <c r="AC108" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD108" t="n">
+        <v>24322.7</v>
+      </c>
+      <c r="AE108" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF108" t="n">
+        <v>13.39</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>24240.4</v>
+      </c>
+      <c r="H109" t="n">
+        <v>85</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>6</v>
+      </c>
+      <c r="L109" t="n">
+        <v>24203.7</v>
+      </c>
+      <c r="M109" t="n">
+        <v>24176.4</v>
+      </c>
+      <c r="N109" t="n">
+        <v>24237.4</v>
+      </c>
+      <c r="O109" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q109" t="n">
+        <v>24044</v>
+      </c>
+      <c r="R109" t="n">
+        <v>24000.8</v>
+      </c>
+      <c r="S109" t="n">
+        <v>24228.2</v>
+      </c>
+      <c r="T109" t="n">
+        <v>24125.1</v>
+      </c>
+      <c r="U109" t="n">
+        <v>24200</v>
+      </c>
+      <c r="V109" t="n">
+        <v>24176.6</v>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y109" t="n">
+        <v>24198.6</v>
+      </c>
+      <c r="Z109" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="AA109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB109" t="n">
+        <v>24200.4</v>
+      </c>
+      <c r="AC109" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD109" t="n">
+        <v>24360.4</v>
+      </c>
+      <c r="AE109" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF109" t="n">
+        <v>13.37</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>57970.7</v>
+      </c>
+      <c r="H110" t="n">
+        <v>82</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>6</v>
+      </c>
+      <c r="L110" t="n">
+        <v>57969.7</v>
+      </c>
+      <c r="M110" t="n">
+        <v>57935.6</v>
+      </c>
+      <c r="N110" t="n">
+        <v>57965.8</v>
+      </c>
+      <c r="O110" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q110" t="n">
+        <v>57650.8</v>
+      </c>
+      <c r="R110" t="n">
+        <v>57493.8</v>
+      </c>
+      <c r="S110" t="n">
+        <v>58251.9</v>
+      </c>
+      <c r="T110" t="n">
+        <v>57592.5</v>
+      </c>
+      <c r="U110" t="n">
+        <v>58008.1</v>
+      </c>
+      <c r="V110" t="n">
+        <v>57922.2</v>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y110" t="n">
+        <v>57959.5</v>
+      </c>
+      <c r="Z110" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB110" t="n">
+        <v>57850.7</v>
+      </c>
+      <c r="AC110" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD110" t="n">
+        <v>58330.7</v>
+      </c>
+      <c r="AE110" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF110" t="n">
+        <v>13.37</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>77700</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>77725.89999999999</v>
+      </c>
+      <c r="H111" t="n">
+        <v>85</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>6</v>
+      </c>
+      <c r="L111" t="n">
+        <v>77601</v>
+      </c>
+      <c r="M111" t="n">
+        <v>77503.10000000001</v>
+      </c>
+      <c r="N111" t="n">
+        <v>77718.5</v>
+      </c>
+      <c r="O111" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q111" t="n">
+        <v>77001.2</v>
+      </c>
+      <c r="R111" t="n">
+        <v>76881.3</v>
+      </c>
+      <c r="S111" t="n">
+        <v>77640.8</v>
+      </c>
+      <c r="T111" t="n">
+        <v>77340.5</v>
+      </c>
+      <c r="U111" t="n">
+        <v>77543.2</v>
+      </c>
+      <c r="V111" t="n">
+        <v>77490.7</v>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y111" t="n">
+        <v>77573.10000000001</v>
+      </c>
+      <c r="Z111" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB111" t="n">
+        <v>77525.89999999999</v>
+      </c>
+      <c r="AC111" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD111" t="n">
+        <v>78325.89999999999</v>
+      </c>
+      <c r="AE111" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF111" t="n">
+        <v>13.45</v>
+      </c>
+      <c r="AG111" t="inlineStr"/>
+      <c r="AH111" t="inlineStr"/>
+      <c r="AI111" t="inlineStr"/>
+      <c r="AJ111" t="inlineStr"/>
+      <c r="AK111" t="inlineStr"/>
+      <c r="AL111" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-14
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL111"/>
+  <dimension ref="A1:AL116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13868,12 +13868,612 @@
       <c r="AF111" t="n">
         <v>13.45</v>
       </c>
-      <c r="AG111" t="inlineStr"/>
-      <c r="AH111" t="inlineStr"/>
-      <c r="AI111" t="inlineStr"/>
-      <c r="AJ111" t="inlineStr"/>
-      <c r="AK111" t="inlineStr"/>
-      <c r="AL111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>12:47</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>57432.8</v>
+      </c>
+      <c r="H112" t="n">
+        <v>88</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>7</v>
+      </c>
+      <c r="L112" t="n">
+        <v>57453.5</v>
+      </c>
+      <c r="M112" t="n">
+        <v>57495.1</v>
+      </c>
+      <c r="N112" t="n">
+        <v>57433.8</v>
+      </c>
+      <c r="O112" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q112" t="n">
+        <v>57838.9</v>
+      </c>
+      <c r="R112" t="n">
+        <v>57644.7</v>
+      </c>
+      <c r="S112" t="n">
+        <v>58219.9</v>
+      </c>
+      <c r="T112" t="n">
+        <v>57493.8</v>
+      </c>
+      <c r="U112" t="n">
+        <v>58030.7</v>
+      </c>
+      <c r="V112" t="n">
+        <v>57856.8</v>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y112" t="n">
+        <v>57488.3</v>
+      </c>
+      <c r="Z112" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="AA112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB112" t="n">
+        <v>57552.8</v>
+      </c>
+      <c r="AC112" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD112" t="n">
+        <v>57072.8</v>
+      </c>
+      <c r="AE112" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF112" t="n">
+        <v>13.57</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>57432.8</v>
+      </c>
+      <c r="H113" t="n">
+        <v>88</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>7</v>
+      </c>
+      <c r="L113" t="n">
+        <v>57456.4</v>
+      </c>
+      <c r="M113" t="n">
+        <v>57480.3</v>
+      </c>
+      <c r="N113" t="n">
+        <v>57438.6</v>
+      </c>
+      <c r="O113" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q113" t="n">
+        <v>57838.9</v>
+      </c>
+      <c r="R113" t="n">
+        <v>57644.7</v>
+      </c>
+      <c r="S113" t="n">
+        <v>58219.9</v>
+      </c>
+      <c r="T113" t="n">
+        <v>57493.8</v>
+      </c>
+      <c r="U113" t="n">
+        <v>58030.7</v>
+      </c>
+      <c r="V113" t="n">
+        <v>57856.8</v>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y113" t="n">
+        <v>57488.3</v>
+      </c>
+      <c r="Z113" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB113" t="n">
+        <v>57552.8</v>
+      </c>
+      <c r="AC113" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD113" t="n">
+        <v>57072.8</v>
+      </c>
+      <c r="AE113" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF113" t="n">
+        <v>13.59</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>24048.2</v>
+      </c>
+      <c r="H114" t="n">
+        <v>78</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>6</v>
+      </c>
+      <c r="L114" t="n">
+        <v>24071.1</v>
+      </c>
+      <c r="M114" t="n">
+        <v>24081</v>
+      </c>
+      <c r="N114" t="n">
+        <v>24048.7</v>
+      </c>
+      <c r="O114" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q114" t="n">
+        <v>24156.4</v>
+      </c>
+      <c r="R114" t="n">
+        <v>24050.6</v>
+      </c>
+      <c r="S114" t="n">
+        <v>24259.7</v>
+      </c>
+      <c r="T114" t="n">
+        <v>24000.8</v>
+      </c>
+      <c r="U114" t="n">
+        <v>24182.5</v>
+      </c>
+      <c r="V114" t="n">
+        <v>24130.2</v>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y114" t="n">
+        <v>24066.4</v>
+      </c>
+      <c r="Z114" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB114" t="n">
+        <v>24088.2</v>
+      </c>
+      <c r="AC114" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD114" t="n">
+        <v>23928.2</v>
+      </c>
+      <c r="AE114" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF114" t="n">
+        <v>13.65</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>57430.3</v>
+      </c>
+      <c r="H115" t="n">
+        <v>88</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>7</v>
+      </c>
+      <c r="L115" t="n">
+        <v>57415.5</v>
+      </c>
+      <c r="M115" t="n">
+        <v>57439.6</v>
+      </c>
+      <c r="N115" t="n">
+        <v>57432</v>
+      </c>
+      <c r="O115" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q115" t="n">
+        <v>57838.9</v>
+      </c>
+      <c r="R115" t="n">
+        <v>57644.7</v>
+      </c>
+      <c r="S115" t="n">
+        <v>58219.9</v>
+      </c>
+      <c r="T115" t="n">
+        <v>57493.8</v>
+      </c>
+      <c r="U115" t="n">
+        <v>58030.7</v>
+      </c>
+      <c r="V115" t="n">
+        <v>57856.8</v>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y115" t="n">
+        <v>57417.7</v>
+      </c>
+      <c r="Z115" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB115" t="n">
+        <v>57550.3</v>
+      </c>
+      <c r="AC115" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD115" t="n">
+        <v>57070.3</v>
+      </c>
+      <c r="AE115" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF115" t="n">
+        <v>13.69</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>14:37</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>57403.9</v>
+      </c>
+      <c r="H116" t="n">
+        <v>88</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>7</v>
+      </c>
+      <c r="L116" t="n">
+        <v>57417.1</v>
+      </c>
+      <c r="M116" t="n">
+        <v>57429.9</v>
+      </c>
+      <c r="N116" t="n">
+        <v>57421.2</v>
+      </c>
+      <c r="O116" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q116" t="n">
+        <v>57838.9</v>
+      </c>
+      <c r="R116" t="n">
+        <v>57644.7</v>
+      </c>
+      <c r="S116" t="n">
+        <v>58219.9</v>
+      </c>
+      <c r="T116" t="n">
+        <v>57493.8</v>
+      </c>
+      <c r="U116" t="n">
+        <v>58030.7</v>
+      </c>
+      <c r="V116" t="n">
+        <v>57856.8</v>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y116" t="n">
+        <v>57417.7</v>
+      </c>
+      <c r="Z116" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AA116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB116" t="n">
+        <v>57523.9</v>
+      </c>
+      <c r="AC116" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD116" t="n">
+        <v>57043.9</v>
+      </c>
+      <c r="AE116" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF116" t="n">
+        <v>13.69</v>
+      </c>
+      <c r="AG116" t="inlineStr"/>
+      <c r="AH116" t="inlineStr"/>
+      <c r="AI116" t="inlineStr"/>
+      <c r="AJ116" t="inlineStr"/>
+      <c r="AK116" t="inlineStr"/>
+      <c r="AL116" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-15
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL116"/>
+  <dimension ref="A1:AL118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14468,12 +14468,252 @@
       <c r="AF116" t="n">
         <v>13.69</v>
       </c>
-      <c r="AG116" t="inlineStr"/>
-      <c r="AH116" t="inlineStr"/>
-      <c r="AI116" t="inlineStr"/>
-      <c r="AJ116" t="inlineStr"/>
-      <c r="AK116" t="inlineStr"/>
-      <c r="AL116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>58100</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>58107.2</v>
+      </c>
+      <c r="H117" t="n">
+        <v>83</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>7</v>
+      </c>
+      <c r="L117" t="n">
+        <v>58019.6</v>
+      </c>
+      <c r="M117" t="n">
+        <v>58018.6</v>
+      </c>
+      <c r="N117" t="n">
+        <v>58107.2</v>
+      </c>
+      <c r="O117" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q117" t="n">
+        <v>58059.2</v>
+      </c>
+      <c r="R117" t="n">
+        <v>57622.6</v>
+      </c>
+      <c r="S117" t="n">
+        <v>57838.9</v>
+      </c>
+      <c r="T117" t="n">
+        <v>57287.6</v>
+      </c>
+      <c r="U117" t="n">
+        <v>57563.2</v>
+      </c>
+      <c r="V117" t="n">
+        <v>57486.8</v>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y117" t="n">
+        <v>58023.5</v>
+      </c>
+      <c r="Z117" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="AA117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB117" t="n">
+        <v>57987.2</v>
+      </c>
+      <c r="AC117" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD117" t="n">
+        <v>58467.2</v>
+      </c>
+      <c r="AE117" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF117" t="n">
+        <v>13.12</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>24073.4</v>
+      </c>
+      <c r="H118" t="n">
+        <v>85</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>6</v>
+      </c>
+      <c r="L118" t="n">
+        <v>24078.8</v>
+      </c>
+      <c r="M118" t="n">
+        <v>24083</v>
+      </c>
+      <c r="N118" t="n">
+        <v>24078.5</v>
+      </c>
+      <c r="O118" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q118" t="n">
+        <v>24211.7</v>
+      </c>
+      <c r="R118" t="n">
+        <v>24074.7</v>
+      </c>
+      <c r="S118" t="n">
+        <v>24156.4</v>
+      </c>
+      <c r="T118" t="n">
+        <v>24023.9</v>
+      </c>
+      <c r="U118" t="n">
+        <v>24090.2</v>
+      </c>
+      <c r="V118" t="n">
+        <v>24053.5</v>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y118" t="n">
+        <v>24087.6</v>
+      </c>
+      <c r="Z118" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB118" t="n">
+        <v>24113.4</v>
+      </c>
+      <c r="AC118" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD118" t="n">
+        <v>23953.4</v>
+      </c>
+      <c r="AE118" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF118" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="AG118" t="inlineStr"/>
+      <c r="AH118" t="inlineStr"/>
+      <c r="AI118" t="inlineStr"/>
+      <c r="AJ118" t="inlineStr"/>
+      <c r="AK118" t="inlineStr"/>
+      <c r="AL118" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-16
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL118"/>
+  <dimension ref="A1:AL124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14708,12 +14708,732 @@
       <c r="AF118" t="n">
         <v>13.25</v>
       </c>
-      <c r="AG118" t="inlineStr"/>
-      <c r="AH118" t="inlineStr"/>
-      <c r="AI118" t="inlineStr"/>
-      <c r="AJ118" t="inlineStr"/>
-      <c r="AK118" t="inlineStr"/>
-      <c r="AL118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>77511.3</v>
+      </c>
+      <c r="H119" t="n">
+        <v>76</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>6</v>
+      </c>
+      <c r="L119" t="n">
+        <v>77471.3</v>
+      </c>
+      <c r="M119" t="n">
+        <v>77447.7</v>
+      </c>
+      <c r="N119" t="n">
+        <v>77488.60000000001</v>
+      </c>
+      <c r="O119" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q119" t="n">
+        <v>77513.10000000001</v>
+      </c>
+      <c r="R119" t="n">
+        <v>77277.2</v>
+      </c>
+      <c r="S119" t="n">
+        <v>77646.3</v>
+      </c>
+      <c r="T119" t="n">
+        <v>76984.3</v>
+      </c>
+      <c r="U119" t="n">
+        <v>77315.3</v>
+      </c>
+      <c r="V119" t="n">
+        <v>77228.7</v>
+      </c>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y119" t="n">
+        <v>77507.5</v>
+      </c>
+      <c r="Z119" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB119" t="n">
+        <v>77311.3</v>
+      </c>
+      <c r="AC119" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD119" t="n">
+        <v>78111.3</v>
+      </c>
+      <c r="AE119" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF119" t="n">
+        <v>12.85</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>57580.4</v>
+      </c>
+      <c r="H120" t="n">
+        <v>78</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>6</v>
+      </c>
+      <c r="L120" t="n">
+        <v>57642.6</v>
+      </c>
+      <c r="M120" t="n">
+        <v>57665.8</v>
+      </c>
+      <c r="N120" t="n">
+        <v>57598.4</v>
+      </c>
+      <c r="O120" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q120" t="n">
+        <v>57895</v>
+      </c>
+      <c r="R120" t="n">
+        <v>57645.6</v>
+      </c>
+      <c r="S120" t="n">
+        <v>58147.3</v>
+      </c>
+      <c r="T120" t="n">
+        <v>57545.2</v>
+      </c>
+      <c r="U120" t="n">
+        <v>57846.2</v>
+      </c>
+      <c r="V120" t="n">
+        <v>57761.5</v>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y120" t="n">
+        <v>57642.3</v>
+      </c>
+      <c r="Z120" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB120" t="n">
+        <v>57700.4</v>
+      </c>
+      <c r="AC120" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD120" t="n">
+        <v>57220.4</v>
+      </c>
+      <c r="AE120" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF120" t="n">
+        <v>12.82</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>57641.7</v>
+      </c>
+      <c r="H121" t="n">
+        <v>88</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>7</v>
+      </c>
+      <c r="L121" t="n">
+        <v>57640.5</v>
+      </c>
+      <c r="M121" t="n">
+        <v>57652.7</v>
+      </c>
+      <c r="N121" t="n">
+        <v>57659.3</v>
+      </c>
+      <c r="O121" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q121" t="n">
+        <v>57895</v>
+      </c>
+      <c r="R121" t="n">
+        <v>57645.6</v>
+      </c>
+      <c r="S121" t="n">
+        <v>58147.3</v>
+      </c>
+      <c r="T121" t="n">
+        <v>57545.2</v>
+      </c>
+      <c r="U121" t="n">
+        <v>57846.2</v>
+      </c>
+      <c r="V121" t="n">
+        <v>57761.5</v>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y121" t="n">
+        <v>57642.3</v>
+      </c>
+      <c r="Z121" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB121" t="n">
+        <v>57761.7</v>
+      </c>
+      <c r="AC121" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD121" t="n">
+        <v>57281.7</v>
+      </c>
+      <c r="AE121" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF121" t="n">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>77494.39999999999</v>
+      </c>
+      <c r="H122" t="n">
+        <v>76</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>6</v>
+      </c>
+      <c r="L122" t="n">
+        <v>77450.3</v>
+      </c>
+      <c r="M122" t="n">
+        <v>77447.3</v>
+      </c>
+      <c r="N122" t="n">
+        <v>77474</v>
+      </c>
+      <c r="O122" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q122" t="n">
+        <v>77513.10000000001</v>
+      </c>
+      <c r="R122" t="n">
+        <v>77277.2</v>
+      </c>
+      <c r="S122" t="n">
+        <v>77646.3</v>
+      </c>
+      <c r="T122" t="n">
+        <v>76984.3</v>
+      </c>
+      <c r="U122" t="n">
+        <v>77315.3</v>
+      </c>
+      <c r="V122" t="n">
+        <v>77228.7</v>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y122" t="n">
+        <v>77507.5</v>
+      </c>
+      <c r="Z122" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB122" t="n">
+        <v>77294.39999999999</v>
+      </c>
+      <c r="AC122" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD122" t="n">
+        <v>78094.39999999999</v>
+      </c>
+      <c r="AE122" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF122" t="n">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>57584.6</v>
+      </c>
+      <c r="H123" t="n">
+        <v>88</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>7</v>
+      </c>
+      <c r="L123" t="n">
+        <v>57601.5</v>
+      </c>
+      <c r="M123" t="n">
+        <v>57622.6</v>
+      </c>
+      <c r="N123" t="n">
+        <v>57585.3</v>
+      </c>
+      <c r="O123" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q123" t="n">
+        <v>57895</v>
+      </c>
+      <c r="R123" t="n">
+        <v>57645.6</v>
+      </c>
+      <c r="S123" t="n">
+        <v>58147.3</v>
+      </c>
+      <c r="T123" t="n">
+        <v>57545.2</v>
+      </c>
+      <c r="U123" t="n">
+        <v>57846.2</v>
+      </c>
+      <c r="V123" t="n">
+        <v>57761.5</v>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y123" t="n">
+        <v>57641.8</v>
+      </c>
+      <c r="Z123" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB123" t="n">
+        <v>57704.6</v>
+      </c>
+      <c r="AC123" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD123" t="n">
+        <v>57224.6</v>
+      </c>
+      <c r="AE123" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF123" t="n">
+        <v>12.86</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>13:34</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>24100</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>24086.3</v>
+      </c>
+      <c r="H124" t="n">
+        <v>78</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>6</v>
+      </c>
+      <c r="L124" t="n">
+        <v>24113.5</v>
+      </c>
+      <c r="M124" t="n">
+        <v>24125.8</v>
+      </c>
+      <c r="N124" t="n">
+        <v>24091.2</v>
+      </c>
+      <c r="O124" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q124" t="n">
+        <v>24166.8</v>
+      </c>
+      <c r="R124" t="n">
+        <v>24118.7</v>
+      </c>
+      <c r="S124" t="n">
+        <v>24220.1</v>
+      </c>
+      <c r="T124" t="n">
+        <v>24010.9</v>
+      </c>
+      <c r="U124" t="n">
+        <v>24115.5</v>
+      </c>
+      <c r="V124" t="n">
+        <v>24087.5</v>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y124" t="n">
+        <v>24100.4</v>
+      </c>
+      <c r="Z124" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB124" t="n">
+        <v>24126.3</v>
+      </c>
+      <c r="AC124" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD124" t="n">
+        <v>23966.3</v>
+      </c>
+      <c r="AE124" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF124" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="AG124" t="inlineStr"/>
+      <c r="AH124" t="inlineStr"/>
+      <c r="AI124" t="inlineStr"/>
+      <c r="AJ124" t="inlineStr"/>
+      <c r="AK124" t="inlineStr"/>
+      <c r="AL124" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-17
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL124"/>
+  <dimension ref="A1:AL131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15428,12 +15428,852 @@
       <c r="AF124" t="n">
         <v>13.01</v>
       </c>
-      <c r="AG124" t="inlineStr"/>
-      <c r="AH124" t="inlineStr"/>
-      <c r="AI124" t="inlineStr"/>
-      <c r="AJ124" t="inlineStr"/>
-      <c r="AK124" t="inlineStr"/>
-      <c r="AL124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G125" t="n">
+        <v>24268.6</v>
+      </c>
+      <c r="H125" t="n">
+        <v>83</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>7</v>
+      </c>
+      <c r="L125" t="n">
+        <v>24256.4</v>
+      </c>
+      <c r="M125" t="n">
+        <v>24248.9</v>
+      </c>
+      <c r="N125" t="n">
+        <v>24269.2</v>
+      </c>
+      <c r="O125" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q125" t="n">
+        <v>24211.4</v>
+      </c>
+      <c r="R125" t="n">
+        <v>24100.9</v>
+      </c>
+      <c r="S125" t="n">
+        <v>24186</v>
+      </c>
+      <c r="T125" t="n">
+        <v>24050.4</v>
+      </c>
+      <c r="U125" t="n">
+        <v>24118.2</v>
+      </c>
+      <c r="V125" t="n">
+        <v>24093.5</v>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y125" t="n">
+        <v>24244.1</v>
+      </c>
+      <c r="Z125" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB125" t="n">
+        <v>24228.6</v>
+      </c>
+      <c r="AC125" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD125" t="n">
+        <v>24388.6</v>
+      </c>
+      <c r="AE125" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF125" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>58100</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>58076.9</v>
+      </c>
+      <c r="H126" t="n">
+        <v>83</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>7</v>
+      </c>
+      <c r="L126" t="n">
+        <v>58071</v>
+      </c>
+      <c r="M126" t="n">
+        <v>58044</v>
+      </c>
+      <c r="N126" t="n">
+        <v>58078</v>
+      </c>
+      <c r="O126" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q126" t="n">
+        <v>57831.1</v>
+      </c>
+      <c r="R126" t="n">
+        <v>57548.8</v>
+      </c>
+      <c r="S126" t="n">
+        <v>57895</v>
+      </c>
+      <c r="T126" t="n">
+        <v>57420.1</v>
+      </c>
+      <c r="U126" t="n">
+        <v>57657.6</v>
+      </c>
+      <c r="V126" t="n">
+        <v>57620.5</v>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y126" t="n">
+        <v>58034.6</v>
+      </c>
+      <c r="Z126" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB126" t="n">
+        <v>57956.9</v>
+      </c>
+      <c r="AC126" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD126" t="n">
+        <v>58436.9</v>
+      </c>
+      <c r="AE126" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF126" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>77900</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>77882.39999999999</v>
+      </c>
+      <c r="H127" t="n">
+        <v>98</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>8</v>
+      </c>
+      <c r="L127" t="n">
+        <v>77875.5</v>
+      </c>
+      <c r="M127" t="n">
+        <v>77847.7</v>
+      </c>
+      <c r="N127" t="n">
+        <v>77881.8</v>
+      </c>
+      <c r="O127" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q127" t="n">
+        <v>77698.7</v>
+      </c>
+      <c r="R127" t="n">
+        <v>77322.3</v>
+      </c>
+      <c r="S127" t="n">
+        <v>77578.60000000001</v>
+      </c>
+      <c r="T127" t="n">
+        <v>77153</v>
+      </c>
+      <c r="U127" t="n">
+        <v>77365.8</v>
+      </c>
+      <c r="V127" t="n">
+        <v>77246.5</v>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y127" t="n">
+        <v>77830.39999999999</v>
+      </c>
+      <c r="Z127" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB127" t="n">
+        <v>77682.39999999999</v>
+      </c>
+      <c r="AC127" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD127" t="n">
+        <v>78482.39999999999</v>
+      </c>
+      <c r="AE127" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF127" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>58100</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>58109</v>
+      </c>
+      <c r="H128" t="n">
+        <v>98</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>8</v>
+      </c>
+      <c r="L128" t="n">
+        <v>58081.5</v>
+      </c>
+      <c r="M128" t="n">
+        <v>58051.5</v>
+      </c>
+      <c r="N128" t="n">
+        <v>58104.2</v>
+      </c>
+      <c r="O128" t="n">
+        <v>64</v>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q128" t="n">
+        <v>57831.1</v>
+      </c>
+      <c r="R128" t="n">
+        <v>57548.8</v>
+      </c>
+      <c r="S128" t="n">
+        <v>57895</v>
+      </c>
+      <c r="T128" t="n">
+        <v>57420.1</v>
+      </c>
+      <c r="U128" t="n">
+        <v>57657.6</v>
+      </c>
+      <c r="V128" t="n">
+        <v>57620.5</v>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y128" t="n">
+        <v>58034.6</v>
+      </c>
+      <c r="Z128" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB128" t="n">
+        <v>57989</v>
+      </c>
+      <c r="AC128" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD128" t="n">
+        <v>58469</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF128" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>12:17</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>24274.7</v>
+      </c>
+      <c r="H129" t="n">
+        <v>83</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>7</v>
+      </c>
+      <c r="L129" t="n">
+        <v>24270.6</v>
+      </c>
+      <c r="M129" t="n">
+        <v>24260.6</v>
+      </c>
+      <c r="N129" t="n">
+        <v>24277.1</v>
+      </c>
+      <c r="O129" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q129" t="n">
+        <v>24211.4</v>
+      </c>
+      <c r="R129" t="n">
+        <v>24100.9</v>
+      </c>
+      <c r="S129" t="n">
+        <v>24186</v>
+      </c>
+      <c r="T129" t="n">
+        <v>24050.4</v>
+      </c>
+      <c r="U129" t="n">
+        <v>24118.2</v>
+      </c>
+      <c r="V129" t="n">
+        <v>24093.5</v>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y129" t="n">
+        <v>24244.1</v>
+      </c>
+      <c r="Z129" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB129" t="n">
+        <v>24234.7</v>
+      </c>
+      <c r="AC129" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD129" t="n">
+        <v>24394.7</v>
+      </c>
+      <c r="AE129" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF129" t="n">
+        <v>13.27</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>12:22</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>58100</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>58098.1</v>
+      </c>
+      <c r="H130" t="n">
+        <v>83</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>7</v>
+      </c>
+      <c r="L130" t="n">
+        <v>58094.1</v>
+      </c>
+      <c r="M130" t="n">
+        <v>58072.1</v>
+      </c>
+      <c r="N130" t="n">
+        <v>58105.6</v>
+      </c>
+      <c r="O130" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q130" t="n">
+        <v>57831.1</v>
+      </c>
+      <c r="R130" t="n">
+        <v>57548.8</v>
+      </c>
+      <c r="S130" t="n">
+        <v>57895</v>
+      </c>
+      <c r="T130" t="n">
+        <v>57420.1</v>
+      </c>
+      <c r="U130" t="n">
+        <v>57657.6</v>
+      </c>
+      <c r="V130" t="n">
+        <v>57620.5</v>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y130" t="n">
+        <v>58034.6</v>
+      </c>
+      <c r="Z130" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB130" t="n">
+        <v>57978.1</v>
+      </c>
+      <c r="AC130" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD130" t="n">
+        <v>58458.1</v>
+      </c>
+      <c r="AE130" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF130" t="n">
+        <v>13.27</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>12:22</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>77900</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>77949.7</v>
+      </c>
+      <c r="H131" t="n">
+        <v>83</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K131" t="n">
+        <v>7</v>
+      </c>
+      <c r="L131" t="n">
+        <v>77951.89999999999</v>
+      </c>
+      <c r="M131" t="n">
+        <v>77907.8</v>
+      </c>
+      <c r="N131" t="n">
+        <v>77961.89999999999</v>
+      </c>
+      <c r="O131" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q131" t="n">
+        <v>77698.7</v>
+      </c>
+      <c r="R131" t="n">
+        <v>77322.3</v>
+      </c>
+      <c r="S131" t="n">
+        <v>77578.60000000001</v>
+      </c>
+      <c r="T131" t="n">
+        <v>77153</v>
+      </c>
+      <c r="U131" t="n">
+        <v>77365.8</v>
+      </c>
+      <c r="V131" t="n">
+        <v>77246.5</v>
+      </c>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X131" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y131" t="n">
+        <v>77849.89999999999</v>
+      </c>
+      <c r="Z131" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB131" t="n">
+        <v>77749.7</v>
+      </c>
+      <c r="AC131" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD131" t="n">
+        <v>78549.7</v>
+      </c>
+      <c r="AE131" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF131" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="AG131" t="inlineStr"/>
+      <c r="AH131" t="inlineStr"/>
+      <c r="AI131" t="inlineStr"/>
+      <c r="AJ131" t="inlineStr"/>
+      <c r="AK131" t="inlineStr"/>
+      <c r="AL131" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-20
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL131"/>
+  <dimension ref="A1:AL132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16268,12 +16268,132 @@
       <c r="AF131" t="n">
         <v>13.27</v>
       </c>
-      <c r="AG131" t="inlineStr"/>
-      <c r="AH131" t="inlineStr"/>
-      <c r="AI131" t="inlineStr"/>
-      <c r="AJ131" t="inlineStr"/>
-      <c r="AK131" t="inlineStr"/>
-      <c r="AL131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>77533.7</v>
+      </c>
+      <c r="H132" t="n">
+        <v>81</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>6</v>
+      </c>
+      <c r="L132" t="n">
+        <v>77506.60000000001</v>
+      </c>
+      <c r="M132" t="n">
+        <v>77539</v>
+      </c>
+      <c r="N132" t="n">
+        <v>77538.3</v>
+      </c>
+      <c r="O132" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q132" t="n">
+        <v>77852.3</v>
+      </c>
+      <c r="R132" t="n">
+        <v>77545.60000000001</v>
+      </c>
+      <c r="S132" t="n">
+        <v>78277.39999999999</v>
+      </c>
+      <c r="T132" t="n">
+        <v>77322.3</v>
+      </c>
+      <c r="U132" t="n">
+        <v>78033.89999999999</v>
+      </c>
+      <c r="V132" t="n">
+        <v>77799.89999999999</v>
+      </c>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X132" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y132" t="n">
+        <v>77554.39999999999</v>
+      </c>
+      <c r="Z132" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB132" t="n">
+        <v>77733.7</v>
+      </c>
+      <c r="AC132" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD132" t="n">
+        <v>76933.7</v>
+      </c>
+      <c r="AE132" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF132" t="n">
+        <v>13.23</v>
+      </c>
+      <c r="AG132" t="inlineStr"/>
+      <c r="AH132" t="inlineStr"/>
+      <c r="AI132" t="inlineStr"/>
+      <c r="AJ132" t="inlineStr"/>
+      <c r="AK132" t="inlineStr"/>
+      <c r="AL132" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-21
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL132"/>
+  <dimension ref="A1:AL138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16388,12 +16388,732 @@
       <c r="AF132" t="n">
         <v>13.23</v>
       </c>
-      <c r="AG132" t="inlineStr"/>
-      <c r="AH132" t="inlineStr"/>
-      <c r="AI132" t="inlineStr"/>
-      <c r="AJ132" t="inlineStr"/>
-      <c r="AK132" t="inlineStr"/>
-      <c r="AL132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>57980.8</v>
+      </c>
+      <c r="H133" t="n">
+        <v>77</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>6</v>
+      </c>
+      <c r="L133" t="n">
+        <v>57924</v>
+      </c>
+      <c r="M133" t="n">
+        <v>57921.5</v>
+      </c>
+      <c r="N133" t="n">
+        <v>57967.7</v>
+      </c>
+      <c r="O133" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q133" t="n">
+        <v>58226.6</v>
+      </c>
+      <c r="R133" t="n">
+        <v>57836.2</v>
+      </c>
+      <c r="S133" t="n">
+        <v>58107.6</v>
+      </c>
+      <c r="T133" t="n">
+        <v>57533.1</v>
+      </c>
+      <c r="U133" t="n">
+        <v>57923.7</v>
+      </c>
+      <c r="V133" t="n">
+        <v>57820.3</v>
+      </c>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X133" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y133" t="n">
+        <v>57985.3</v>
+      </c>
+      <c r="Z133" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB133" t="n">
+        <v>57860.8</v>
+      </c>
+      <c r="AC133" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD133" t="n">
+        <v>58340.8</v>
+      </c>
+      <c r="AE133" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF133" t="n">
+        <v>12.74</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>24145.4</v>
+      </c>
+      <c r="H134" t="n">
+        <v>78</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K134" t="n">
+        <v>6</v>
+      </c>
+      <c r="L134" t="n">
+        <v>24160.2</v>
+      </c>
+      <c r="M134" t="n">
+        <v>24169.9</v>
+      </c>
+      <c r="N134" t="n">
+        <v>24145.5</v>
+      </c>
+      <c r="O134" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q134" t="n">
+        <v>24262.2</v>
+      </c>
+      <c r="R134" t="n">
+        <v>24206.8</v>
+      </c>
+      <c r="S134" t="n">
+        <v>24265.6</v>
+      </c>
+      <c r="T134" t="n">
+        <v>24136.2</v>
+      </c>
+      <c r="U134" t="n">
+        <v>24226.6</v>
+      </c>
+      <c r="V134" t="n">
+        <v>24200.9</v>
+      </c>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X134" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y134" t="n">
+        <v>24165.7</v>
+      </c>
+      <c r="Z134" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB134" t="n">
+        <v>24185.4</v>
+      </c>
+      <c r="AC134" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD134" t="n">
+        <v>24025.4</v>
+      </c>
+      <c r="AE134" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF134" t="n">
+        <v>12.72</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>77400</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>77353.2</v>
+      </c>
+      <c r="H135" t="n">
+        <v>88</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K135" t="n">
+        <v>7</v>
+      </c>
+      <c r="L135" t="n">
+        <v>77404.89999999999</v>
+      </c>
+      <c r="M135" t="n">
+        <v>77438.7</v>
+      </c>
+      <c r="N135" t="n">
+        <v>77358.5</v>
+      </c>
+      <c r="O135" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q135" t="n">
+        <v>77750.5</v>
+      </c>
+      <c r="R135" t="n">
+        <v>77550.60000000001</v>
+      </c>
+      <c r="S135" t="n">
+        <v>77852.3</v>
+      </c>
+      <c r="T135" t="n">
+        <v>77370.3</v>
+      </c>
+      <c r="U135" t="n">
+        <v>77676.10000000001</v>
+      </c>
+      <c r="V135" t="n">
+        <v>77611.3</v>
+      </c>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y135" t="n">
+        <v>77435.7</v>
+      </c>
+      <c r="Z135" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="AA135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB135" t="n">
+        <v>77553.2</v>
+      </c>
+      <c r="AC135" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD135" t="n">
+        <v>76753.2</v>
+      </c>
+      <c r="AE135" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF135" t="n">
+        <v>12.72</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>77494.10000000001</v>
+      </c>
+      <c r="H136" t="n">
+        <v>76</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>6</v>
+      </c>
+      <c r="L136" t="n">
+        <v>77431.5</v>
+      </c>
+      <c r="M136" t="n">
+        <v>77436</v>
+      </c>
+      <c r="N136" t="n">
+        <v>77480.39999999999</v>
+      </c>
+      <c r="O136" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q136" t="n">
+        <v>77750.5</v>
+      </c>
+      <c r="R136" t="n">
+        <v>77550.60000000001</v>
+      </c>
+      <c r="S136" t="n">
+        <v>77852.3</v>
+      </c>
+      <c r="T136" t="n">
+        <v>77370.3</v>
+      </c>
+      <c r="U136" t="n">
+        <v>77676.10000000001</v>
+      </c>
+      <c r="V136" t="n">
+        <v>77611.3</v>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y136" t="n">
+        <v>77495.89999999999</v>
+      </c>
+      <c r="Z136" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB136" t="n">
+        <v>77694.10000000001</v>
+      </c>
+      <c r="AC136" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD136" t="n">
+        <v>76894.10000000001</v>
+      </c>
+      <c r="AE136" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF136" t="n">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>77462.2</v>
+      </c>
+      <c r="H137" t="n">
+        <v>88</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K137" t="n">
+        <v>7</v>
+      </c>
+      <c r="L137" t="n">
+        <v>77437.3</v>
+      </c>
+      <c r="M137" t="n">
+        <v>77438.2</v>
+      </c>
+      <c r="N137" t="n">
+        <v>77469.5</v>
+      </c>
+      <c r="O137" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q137" t="n">
+        <v>77750.5</v>
+      </c>
+      <c r="R137" t="n">
+        <v>77550.60000000001</v>
+      </c>
+      <c r="S137" t="n">
+        <v>77852.3</v>
+      </c>
+      <c r="T137" t="n">
+        <v>77370.3</v>
+      </c>
+      <c r="U137" t="n">
+        <v>77676.10000000001</v>
+      </c>
+      <c r="V137" t="n">
+        <v>77611.3</v>
+      </c>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y137" t="n">
+        <v>77435.7</v>
+      </c>
+      <c r="Z137" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB137" t="n">
+        <v>77662.2</v>
+      </c>
+      <c r="AC137" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD137" t="n">
+        <v>76862.2</v>
+      </c>
+      <c r="AE137" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF137" t="n">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>77400</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>77421.89999999999</v>
+      </c>
+      <c r="H138" t="n">
+        <v>88</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K138" t="n">
+        <v>7</v>
+      </c>
+      <c r="L138" t="n">
+        <v>77426.7</v>
+      </c>
+      <c r="M138" t="n">
+        <v>77431.7</v>
+      </c>
+      <c r="N138" t="n">
+        <v>77425.60000000001</v>
+      </c>
+      <c r="O138" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q138" t="n">
+        <v>77750.5</v>
+      </c>
+      <c r="R138" t="n">
+        <v>77550.60000000001</v>
+      </c>
+      <c r="S138" t="n">
+        <v>77852.3</v>
+      </c>
+      <c r="T138" t="n">
+        <v>77370.3</v>
+      </c>
+      <c r="U138" t="n">
+        <v>77676.10000000001</v>
+      </c>
+      <c r="V138" t="n">
+        <v>77611.3</v>
+      </c>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y138" t="n">
+        <v>77435.7</v>
+      </c>
+      <c r="Z138" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB138" t="n">
+        <v>77621.89999999999</v>
+      </c>
+      <c r="AC138" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD138" t="n">
+        <v>76821.89999999999</v>
+      </c>
+      <c r="AE138" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF138" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="AG138" t="inlineStr"/>
+      <c r="AH138" t="inlineStr"/>
+      <c r="AI138" t="inlineStr"/>
+      <c r="AJ138" t="inlineStr"/>
+      <c r="AK138" t="inlineStr"/>
+      <c r="AL138" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-22
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL138"/>
+  <dimension ref="A1:AL145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17108,12 +17108,852 @@
       <c r="AF138" t="n">
         <v>12.63</v>
       </c>
-      <c r="AG138" t="inlineStr"/>
-      <c r="AH138" t="inlineStr"/>
-      <c r="AI138" t="inlineStr"/>
-      <c r="AJ138" t="inlineStr"/>
-      <c r="AK138" t="inlineStr"/>
-      <c r="AL138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
+        <v>24005.8</v>
+      </c>
+      <c r="H139" t="n">
+        <v>83</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K139" t="n">
+        <v>7</v>
+      </c>
+      <c r="L139" t="n">
+        <v>24027</v>
+      </c>
+      <c r="M139" t="n">
+        <v>24029.3</v>
+      </c>
+      <c r="N139" t="n">
+        <v>24009.6</v>
+      </c>
+      <c r="O139" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q139" t="n">
+        <v>24164.7</v>
+      </c>
+      <c r="R139" t="n">
+        <v>24047.2</v>
+      </c>
+      <c r="S139" t="n">
+        <v>24262.2</v>
+      </c>
+      <c r="T139" t="n">
+        <v>24135.9</v>
+      </c>
+      <c r="U139" t="n">
+        <v>24199</v>
+      </c>
+      <c r="V139" t="n">
+        <v>24195.6</v>
+      </c>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y139" t="n">
+        <v>24018.9</v>
+      </c>
+      <c r="Z139" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="AA139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB139" t="n">
+        <v>24045.8</v>
+      </c>
+      <c r="AC139" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD139" t="n">
+        <v>23885.8</v>
+      </c>
+      <c r="AE139" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF139" t="n">
+        <v>12.97</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>76900</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
+        <v>76905.8</v>
+      </c>
+      <c r="H140" t="n">
+        <v>83</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K140" t="n">
+        <v>7</v>
+      </c>
+      <c r="L140" t="n">
+        <v>76900.8</v>
+      </c>
+      <c r="M140" t="n">
+        <v>76901.10000000001</v>
+      </c>
+      <c r="N140" t="n">
+        <v>76906.2</v>
+      </c>
+      <c r="O140" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q140" t="n">
+        <v>77363.60000000001</v>
+      </c>
+      <c r="R140" t="n">
+        <v>76963.60000000001</v>
+      </c>
+      <c r="S140" t="n">
+        <v>77750.5</v>
+      </c>
+      <c r="T140" t="n">
+        <v>77338.5</v>
+      </c>
+      <c r="U140" t="n">
+        <v>77544.5</v>
+      </c>
+      <c r="V140" t="n">
+        <v>77494.89999999999</v>
+      </c>
+      <c r="W140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y140" t="n">
+        <v>76873.60000000001</v>
+      </c>
+      <c r="Z140" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AA140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB140" t="n">
+        <v>77105.8</v>
+      </c>
+      <c r="AC140" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD140" t="n">
+        <v>76305.8</v>
+      </c>
+      <c r="AE140" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF140" t="n">
+        <v>12.97</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>57104.4</v>
+      </c>
+      <c r="H141" t="n">
+        <v>75</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K141" t="n">
+        <v>5</v>
+      </c>
+      <c r="L141" t="n">
+        <v>57182.7</v>
+      </c>
+      <c r="M141" t="n">
+        <v>57233.6</v>
+      </c>
+      <c r="N141" t="n">
+        <v>57111.4</v>
+      </c>
+      <c r="O141" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q141" t="n">
+        <v>57784.4</v>
+      </c>
+      <c r="R141" t="n">
+        <v>57333.1</v>
+      </c>
+      <c r="S141" t="n">
+        <v>58226.6</v>
+      </c>
+      <c r="T141" t="n">
+        <v>57804.9</v>
+      </c>
+      <c r="U141" t="n">
+        <v>58015.8</v>
+      </c>
+      <c r="V141" t="n">
+        <v>57883.7</v>
+      </c>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y141" t="n">
+        <v>57260.1</v>
+      </c>
+      <c r="Z141" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB141" t="n">
+        <v>57224.4</v>
+      </c>
+      <c r="AC141" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD141" t="n">
+        <v>56744.4</v>
+      </c>
+      <c r="AE141" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF141" t="n">
+        <v>13.03</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G142" t="n">
+        <v>23986.4</v>
+      </c>
+      <c r="H142" t="n">
+        <v>98</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K142" t="n">
+        <v>8</v>
+      </c>
+      <c r="L142" t="n">
+        <v>24001.4</v>
+      </c>
+      <c r="M142" t="n">
+        <v>24014.4</v>
+      </c>
+      <c r="N142" t="n">
+        <v>23988.6</v>
+      </c>
+      <c r="O142" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q142" t="n">
+        <v>24164.7</v>
+      </c>
+      <c r="R142" t="n">
+        <v>24047.2</v>
+      </c>
+      <c r="S142" t="n">
+        <v>24262.2</v>
+      </c>
+      <c r="T142" t="n">
+        <v>24135.9</v>
+      </c>
+      <c r="U142" t="n">
+        <v>24199</v>
+      </c>
+      <c r="V142" t="n">
+        <v>24195.6</v>
+      </c>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y142" t="n">
+        <v>24014.9</v>
+      </c>
+      <c r="Z142" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB142" t="n">
+        <v>24026.4</v>
+      </c>
+      <c r="AC142" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD142" t="n">
+        <v>23866.4</v>
+      </c>
+      <c r="AE142" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF142" t="n">
+        <v>13.13</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G143" t="n">
+        <v>76721.7</v>
+      </c>
+      <c r="H143" t="n">
+        <v>88</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>7</v>
+      </c>
+      <c r="L143" t="n">
+        <v>76786.7</v>
+      </c>
+      <c r="M143" t="n">
+        <v>76834.89999999999</v>
+      </c>
+      <c r="N143" t="n">
+        <v>76736.10000000001</v>
+      </c>
+      <c r="O143" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q143" t="n">
+        <v>77363.60000000001</v>
+      </c>
+      <c r="R143" t="n">
+        <v>76963.60000000001</v>
+      </c>
+      <c r="S143" t="n">
+        <v>77750.5</v>
+      </c>
+      <c r="T143" t="n">
+        <v>77338.5</v>
+      </c>
+      <c r="U143" t="n">
+        <v>77544.5</v>
+      </c>
+      <c r="V143" t="n">
+        <v>77494.89999999999</v>
+      </c>
+      <c r="W143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y143" t="n">
+        <v>76834.60000000001</v>
+      </c>
+      <c r="Z143" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="AA143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB143" t="n">
+        <v>76921.7</v>
+      </c>
+      <c r="AC143" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD143" t="n">
+        <v>76121.7</v>
+      </c>
+      <c r="AE143" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF143" t="n">
+        <v>13.14</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G144" t="n">
+        <v>24007.5</v>
+      </c>
+      <c r="H144" t="n">
+        <v>83</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K144" t="n">
+        <v>7</v>
+      </c>
+      <c r="L144" t="n">
+        <v>23996.8</v>
+      </c>
+      <c r="M144" t="n">
+        <v>24004.6</v>
+      </c>
+      <c r="N144" t="n">
+        <v>24007.4</v>
+      </c>
+      <c r="O144" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q144" t="n">
+        <v>24164.7</v>
+      </c>
+      <c r="R144" t="n">
+        <v>24047.2</v>
+      </c>
+      <c r="S144" t="n">
+        <v>24262.2</v>
+      </c>
+      <c r="T144" t="n">
+        <v>24135.9</v>
+      </c>
+      <c r="U144" t="n">
+        <v>24199</v>
+      </c>
+      <c r="V144" t="n">
+        <v>24195.6</v>
+      </c>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y144" t="n">
+        <v>24009.5</v>
+      </c>
+      <c r="Z144" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AA144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB144" t="n">
+        <v>24047.5</v>
+      </c>
+      <c r="AC144" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD144" t="n">
+        <v>23887.5</v>
+      </c>
+      <c r="AE144" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF144" t="n">
+        <v>13.01</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G145" t="n">
+        <v>57116.6</v>
+      </c>
+      <c r="H145" t="n">
+        <v>88</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K145" t="n">
+        <v>7</v>
+      </c>
+      <c r="L145" t="n">
+        <v>57101.1</v>
+      </c>
+      <c r="M145" t="n">
+        <v>57145.1</v>
+      </c>
+      <c r="N145" t="n">
+        <v>57120.7</v>
+      </c>
+      <c r="O145" t="n">
+        <v>43</v>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q145" t="n">
+        <v>57784.4</v>
+      </c>
+      <c r="R145" t="n">
+        <v>57333.1</v>
+      </c>
+      <c r="S145" t="n">
+        <v>58226.6</v>
+      </c>
+      <c r="T145" t="n">
+        <v>57804.9</v>
+      </c>
+      <c r="U145" t="n">
+        <v>58015.8</v>
+      </c>
+      <c r="V145" t="n">
+        <v>57883.7</v>
+      </c>
+      <c r="W145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X145" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y145" t="n">
+        <v>57163.7</v>
+      </c>
+      <c r="Z145" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="AA145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB145" t="n">
+        <v>57236.6</v>
+      </c>
+      <c r="AC145" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD145" t="n">
+        <v>56756.6</v>
+      </c>
+      <c r="AE145" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF145" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="AG145" t="inlineStr"/>
+      <c r="AH145" t="inlineStr"/>
+      <c r="AI145" t="inlineStr"/>
+      <c r="AJ145" t="inlineStr"/>
+      <c r="AK145" t="inlineStr"/>
+      <c r="AL145" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-23
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL145"/>
+  <dimension ref="A1:AL151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17948,12 +17948,732 @@
       <c r="AF145" t="n">
         <v>13.01</v>
       </c>
-      <c r="AG145" t="inlineStr"/>
-      <c r="AH145" t="inlineStr"/>
-      <c r="AI145" t="inlineStr"/>
-      <c r="AJ145" t="inlineStr"/>
-      <c r="AK145" t="inlineStr"/>
-      <c r="AL145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>23850</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G146" t="n">
+        <v>23843.5</v>
+      </c>
+      <c r="H146" t="n">
+        <v>83</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>7</v>
+      </c>
+      <c r="L146" t="n">
+        <v>23849</v>
+      </c>
+      <c r="M146" t="n">
+        <v>23878.2</v>
+      </c>
+      <c r="N146" t="n">
+        <v>23843.5</v>
+      </c>
+      <c r="O146" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q146" t="n">
+        <v>23951.5</v>
+      </c>
+      <c r="R146" t="n">
+        <v>23876.8</v>
+      </c>
+      <c r="S146" t="n">
+        <v>24164.7</v>
+      </c>
+      <c r="T146" t="n">
+        <v>23961.6</v>
+      </c>
+      <c r="U146" t="n">
+        <v>24063.1</v>
+      </c>
+      <c r="V146" t="n">
+        <v>24015.1</v>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y146" t="n">
+        <v>23844.9</v>
+      </c>
+      <c r="Z146" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB146" t="n">
+        <v>23883.5</v>
+      </c>
+      <c r="AC146" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD146" t="n">
+        <v>23723.5</v>
+      </c>
+      <c r="AE146" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF146" t="n">
+        <v>13.42</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>56400</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G147" t="n">
+        <v>56424.8</v>
+      </c>
+      <c r="H147" t="n">
+        <v>88</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>7</v>
+      </c>
+      <c r="L147" t="n">
+        <v>56438.2</v>
+      </c>
+      <c r="M147" t="n">
+        <v>56501.3</v>
+      </c>
+      <c r="N147" t="n">
+        <v>56432.5</v>
+      </c>
+      <c r="O147" t="n">
+        <v>41</v>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q147" t="n">
+        <v>56925.4</v>
+      </c>
+      <c r="R147" t="n">
+        <v>56648.9</v>
+      </c>
+      <c r="S147" t="n">
+        <v>57784.4</v>
+      </c>
+      <c r="T147" t="n">
+        <v>56971.9</v>
+      </c>
+      <c r="U147" t="n">
+        <v>57378.2</v>
+      </c>
+      <c r="V147" t="n">
+        <v>57207.5</v>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y147" t="n">
+        <v>56504.8</v>
+      </c>
+      <c r="Z147" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB147" t="n">
+        <v>56544.8</v>
+      </c>
+      <c r="AC147" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD147" t="n">
+        <v>56064.8</v>
+      </c>
+      <c r="AE147" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF147" t="n">
+        <v>13.42</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>76200</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G148" t="n">
+        <v>76234.60000000001</v>
+      </c>
+      <c r="H148" t="n">
+        <v>78</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>6</v>
+      </c>
+      <c r="L148" t="n">
+        <v>76303.39999999999</v>
+      </c>
+      <c r="M148" t="n">
+        <v>76402.3</v>
+      </c>
+      <c r="N148" t="n">
+        <v>76239.2</v>
+      </c>
+      <c r="O148" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q148" t="n">
+        <v>76566.60000000001</v>
+      </c>
+      <c r="R148" t="n">
+        <v>76348</v>
+      </c>
+      <c r="S148" t="n">
+        <v>77363.60000000001</v>
+      </c>
+      <c r="T148" t="n">
+        <v>76642.60000000001</v>
+      </c>
+      <c r="U148" t="n">
+        <v>77003.10000000001</v>
+      </c>
+      <c r="V148" t="n">
+        <v>76837.7</v>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y148" t="n">
+        <v>76296.7</v>
+      </c>
+      <c r="Z148" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB148" t="n">
+        <v>76434.60000000001</v>
+      </c>
+      <c r="AC148" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD148" t="n">
+        <v>75634.60000000001</v>
+      </c>
+      <c r="AE148" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF148" t="n">
+        <v>13.42</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>76300</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G149" t="n">
+        <v>76285</v>
+      </c>
+      <c r="H149" t="n">
+        <v>88</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K149" t="n">
+        <v>7</v>
+      </c>
+      <c r="L149" t="n">
+        <v>76296.10000000001</v>
+      </c>
+      <c r="M149" t="n">
+        <v>76381.60000000001</v>
+      </c>
+      <c r="N149" t="n">
+        <v>76295.60000000001</v>
+      </c>
+      <c r="O149" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q149" t="n">
+        <v>76566.60000000001</v>
+      </c>
+      <c r="R149" t="n">
+        <v>76348</v>
+      </c>
+      <c r="S149" t="n">
+        <v>77363.60000000001</v>
+      </c>
+      <c r="T149" t="n">
+        <v>76642.60000000001</v>
+      </c>
+      <c r="U149" t="n">
+        <v>77003.10000000001</v>
+      </c>
+      <c r="V149" t="n">
+        <v>76837.7</v>
+      </c>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X149" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y149" t="n">
+        <v>76280.89999999999</v>
+      </c>
+      <c r="Z149" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AA149" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB149" t="n">
+        <v>76485</v>
+      </c>
+      <c r="AC149" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD149" t="n">
+        <v>75685</v>
+      </c>
+      <c r="AE149" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF149" t="n">
+        <v>13.42</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>23850</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G150" t="n">
+        <v>23854.8</v>
+      </c>
+      <c r="H150" t="n">
+        <v>98</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>8</v>
+      </c>
+      <c r="L150" t="n">
+        <v>23852.4</v>
+      </c>
+      <c r="M150" t="n">
+        <v>23866.9</v>
+      </c>
+      <c r="N150" t="n">
+        <v>23856.7</v>
+      </c>
+      <c r="O150" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q150" t="n">
+        <v>23951.5</v>
+      </c>
+      <c r="R150" t="n">
+        <v>23876.8</v>
+      </c>
+      <c r="S150" t="n">
+        <v>24164.7</v>
+      </c>
+      <c r="T150" t="n">
+        <v>23961.6</v>
+      </c>
+      <c r="U150" t="n">
+        <v>24063.1</v>
+      </c>
+      <c r="V150" t="n">
+        <v>24015.1</v>
+      </c>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y150" t="n">
+        <v>23844.9</v>
+      </c>
+      <c r="Z150" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="AA150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB150" t="n">
+        <v>23894.8</v>
+      </c>
+      <c r="AC150" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD150" t="n">
+        <v>23734.8</v>
+      </c>
+      <c r="AE150" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF150" t="n">
+        <v>13.55</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>56500</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G151" t="n">
+        <v>56529.2</v>
+      </c>
+      <c r="H151" t="n">
+        <v>88</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K151" t="n">
+        <v>7</v>
+      </c>
+      <c r="L151" t="n">
+        <v>56496.4</v>
+      </c>
+      <c r="M151" t="n">
+        <v>56506.9</v>
+      </c>
+      <c r="N151" t="n">
+        <v>56530.4</v>
+      </c>
+      <c r="O151" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q151" t="n">
+        <v>56925.4</v>
+      </c>
+      <c r="R151" t="n">
+        <v>56648.9</v>
+      </c>
+      <c r="S151" t="n">
+        <v>57784.4</v>
+      </c>
+      <c r="T151" t="n">
+        <v>56971.9</v>
+      </c>
+      <c r="U151" t="n">
+        <v>57378.2</v>
+      </c>
+      <c r="V151" t="n">
+        <v>57207.5</v>
+      </c>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y151" t="n">
+        <v>56504.8</v>
+      </c>
+      <c r="Z151" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="AA151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB151" t="n">
+        <v>56649.2</v>
+      </c>
+      <c r="AC151" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD151" t="n">
+        <v>56169.2</v>
+      </c>
+      <c r="AE151" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF151" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="AG151" t="inlineStr"/>
+      <c r="AH151" t="inlineStr"/>
+      <c r="AI151" t="inlineStr"/>
+      <c r="AJ151" t="inlineStr"/>
+      <c r="AK151" t="inlineStr"/>
+      <c r="AL151" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-24
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL151"/>
+  <dimension ref="A1:AL157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18668,12 +18668,732 @@
       <c r="AF151" t="n">
         <v>13.56</v>
       </c>
-      <c r="AG151" t="inlineStr"/>
-      <c r="AH151" t="inlineStr"/>
-      <c r="AI151" t="inlineStr"/>
-      <c r="AJ151" t="inlineStr"/>
-      <c r="AK151" t="inlineStr"/>
-      <c r="AL151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>56400</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G152" t="n">
+        <v>56384.9</v>
+      </c>
+      <c r="H152" t="n">
+        <v>82</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K152" t="n">
+        <v>6</v>
+      </c>
+      <c r="L152" t="n">
+        <v>56281.3</v>
+      </c>
+      <c r="M152" t="n">
+        <v>56228.1</v>
+      </c>
+      <c r="N152" t="n">
+        <v>56383.4</v>
+      </c>
+      <c r="O152" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q152" t="n">
+        <v>56341.9</v>
+      </c>
+      <c r="R152" t="n">
+        <v>56096.9</v>
+      </c>
+      <c r="S152" t="n">
+        <v>56925.4</v>
+      </c>
+      <c r="T152" t="n">
+        <v>56374.9</v>
+      </c>
+      <c r="U152" t="n">
+        <v>56650.1</v>
+      </c>
+      <c r="V152" t="n">
+        <v>56592.3</v>
+      </c>
+      <c r="W152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X152" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y152" t="n">
+        <v>56324.7</v>
+      </c>
+      <c r="Z152" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="AA152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB152" t="n">
+        <v>56264.9</v>
+      </c>
+      <c r="AC152" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD152" t="n">
+        <v>56744.9</v>
+      </c>
+      <c r="AE152" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF152" t="n">
+        <v>14.23</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>56700</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G153" t="n">
+        <v>56701.2</v>
+      </c>
+      <c r="H153" t="n">
+        <v>75</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K153" t="n">
+        <v>5</v>
+      </c>
+      <c r="L153" t="n">
+        <v>56552.7</v>
+      </c>
+      <c r="M153" t="n">
+        <v>56413.9</v>
+      </c>
+      <c r="N153" t="n">
+        <v>56693.2</v>
+      </c>
+      <c r="O153" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q153" t="n">
+        <v>56341.9</v>
+      </c>
+      <c r="R153" t="n">
+        <v>56096.9</v>
+      </c>
+      <c r="S153" t="n">
+        <v>56925.4</v>
+      </c>
+      <c r="T153" t="n">
+        <v>56374.9</v>
+      </c>
+      <c r="U153" t="n">
+        <v>56650.1</v>
+      </c>
+      <c r="V153" t="n">
+        <v>56592.3</v>
+      </c>
+      <c r="W153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y153" t="n">
+        <v>56581.7</v>
+      </c>
+      <c r="Z153" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="AA153" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB153" t="n">
+        <v>56581.2</v>
+      </c>
+      <c r="AC153" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD153" t="n">
+        <v>57061.2</v>
+      </c>
+      <c r="AE153" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF153" t="n">
+        <v>14.23</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>23800</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G154" t="n">
+        <v>23792</v>
+      </c>
+      <c r="H154" t="n">
+        <v>82</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K154" t="n">
+        <v>6</v>
+      </c>
+      <c r="L154" t="n">
+        <v>23780.6</v>
+      </c>
+      <c r="M154" t="n">
+        <v>23753.6</v>
+      </c>
+      <c r="N154" t="n">
+        <v>23789.9</v>
+      </c>
+      <c r="O154" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q154" t="n">
+        <v>23762.8</v>
+      </c>
+      <c r="R154" t="n">
+        <v>23650.3</v>
+      </c>
+      <c r="S154" t="n">
+        <v>23990.7</v>
+      </c>
+      <c r="T154" t="n">
+        <v>23807.3</v>
+      </c>
+      <c r="U154" t="n">
+        <v>23899</v>
+      </c>
+      <c r="V154" t="n">
+        <v>23881.1</v>
+      </c>
+      <c r="W154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X154" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y154" t="n">
+        <v>23771.2</v>
+      </c>
+      <c r="Z154" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="AA154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB154" t="n">
+        <v>23752</v>
+      </c>
+      <c r="AC154" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD154" t="n">
+        <v>23912</v>
+      </c>
+      <c r="AE154" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF154" t="n">
+        <v>14.06</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>56700</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G155" t="n">
+        <v>56745.6</v>
+      </c>
+      <c r="H155" t="n">
+        <v>75</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K155" t="n">
+        <v>5</v>
+      </c>
+      <c r="L155" t="n">
+        <v>56681</v>
+      </c>
+      <c r="M155" t="n">
+        <v>56568.3</v>
+      </c>
+      <c r="N155" t="n">
+        <v>56732.9</v>
+      </c>
+      <c r="O155" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q155" t="n">
+        <v>56341.9</v>
+      </c>
+      <c r="R155" t="n">
+        <v>56096.9</v>
+      </c>
+      <c r="S155" t="n">
+        <v>56925.4</v>
+      </c>
+      <c r="T155" t="n">
+        <v>56374.9</v>
+      </c>
+      <c r="U155" t="n">
+        <v>56650.1</v>
+      </c>
+      <c r="V155" t="n">
+        <v>56592.3</v>
+      </c>
+      <c r="W155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y155" t="n">
+        <v>56613.1</v>
+      </c>
+      <c r="Z155" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="AA155" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB155" t="n">
+        <v>56625.6</v>
+      </c>
+      <c r="AC155" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD155" t="n">
+        <v>57105.6</v>
+      </c>
+      <c r="AE155" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF155" t="n">
+        <v>14.06</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>76100</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G156" t="n">
+        <v>76090.89999999999</v>
+      </c>
+      <c r="H156" t="n">
+        <v>82</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K156" t="n">
+        <v>6</v>
+      </c>
+      <c r="L156" t="n">
+        <v>76064.5</v>
+      </c>
+      <c r="M156" t="n">
+        <v>75968.3</v>
+      </c>
+      <c r="N156" t="n">
+        <v>76090</v>
+      </c>
+      <c r="O156" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q156" t="n">
+        <v>75995.7</v>
+      </c>
+      <c r="R156" t="n">
+        <v>75670.5</v>
+      </c>
+      <c r="S156" t="n">
+        <v>76726.60000000001</v>
+      </c>
+      <c r="T156" t="n">
+        <v>76152.89999999999</v>
+      </c>
+      <c r="U156" t="n">
+        <v>76439.8</v>
+      </c>
+      <c r="V156" t="n">
+        <v>76407.5</v>
+      </c>
+      <c r="W156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y156" t="n">
+        <v>76046.5</v>
+      </c>
+      <c r="Z156" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="AA156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB156" t="n">
+        <v>75890.89999999999</v>
+      </c>
+      <c r="AC156" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD156" t="n">
+        <v>76690.89999999999</v>
+      </c>
+      <c r="AE156" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF156" t="n">
+        <v>14.06</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>56700</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G157" t="n">
+        <v>56668.9</v>
+      </c>
+      <c r="H157" t="n">
+        <v>88</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K157" t="n">
+        <v>7</v>
+      </c>
+      <c r="L157" t="n">
+        <v>56677.6</v>
+      </c>
+      <c r="M157" t="n">
+        <v>56586.2</v>
+      </c>
+      <c r="N157" t="n">
+        <v>56667.9</v>
+      </c>
+      <c r="O157" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q157" t="n">
+        <v>56341.9</v>
+      </c>
+      <c r="R157" t="n">
+        <v>56096.9</v>
+      </c>
+      <c r="S157" t="n">
+        <v>56925.4</v>
+      </c>
+      <c r="T157" t="n">
+        <v>56374.9</v>
+      </c>
+      <c r="U157" t="n">
+        <v>56650.1</v>
+      </c>
+      <c r="V157" t="n">
+        <v>56592.3</v>
+      </c>
+      <c r="W157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X157" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y157" t="n">
+        <v>56613.1</v>
+      </c>
+      <c r="Z157" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="AA157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB157" t="n">
+        <v>56548.9</v>
+      </c>
+      <c r="AC157" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD157" t="n">
+        <v>57028.9</v>
+      </c>
+      <c r="AE157" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF157" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="AG157" t="inlineStr"/>
+      <c r="AH157" t="inlineStr"/>
+      <c r="AI157" t="inlineStr"/>
+      <c r="AJ157" t="inlineStr"/>
+      <c r="AK157" t="inlineStr"/>
+      <c r="AL157" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-27
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL157"/>
+  <dimension ref="A1:AL163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19388,12 +19388,732 @@
       <c r="AF157" t="n">
         <v>14.06</v>
       </c>
-      <c r="AG157" t="inlineStr"/>
-      <c r="AH157" t="inlineStr"/>
-      <c r="AI157" t="inlineStr"/>
-      <c r="AJ157" t="inlineStr"/>
-      <c r="AK157" t="inlineStr"/>
-      <c r="AL157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>23950</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G158" t="n">
+        <v>23960.8</v>
+      </c>
+      <c r="H158" t="n">
+        <v>76</v>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K158" t="n">
+        <v>6</v>
+      </c>
+      <c r="L158" t="n">
+        <v>23954.6</v>
+      </c>
+      <c r="M158" t="n">
+        <v>23951.4</v>
+      </c>
+      <c r="N158" t="n">
+        <v>23957.2</v>
+      </c>
+      <c r="O158" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q158" t="n">
+        <v>23963.2</v>
+      </c>
+      <c r="R158" t="n">
+        <v>23897.2</v>
+      </c>
+      <c r="S158" t="n">
+        <v>23823.6</v>
+      </c>
+      <c r="T158" t="n">
+        <v>23606.4</v>
+      </c>
+      <c r="U158" t="n">
+        <v>23763</v>
+      </c>
+      <c r="V158" t="n">
+        <v>23715</v>
+      </c>
+      <c r="W158" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y158" t="n">
+        <v>23955</v>
+      </c>
+      <c r="Z158" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB158" t="n">
+        <v>23920.8</v>
+      </c>
+      <c r="AC158" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD158" t="n">
+        <v>24080.8</v>
+      </c>
+      <c r="AE158" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF158" t="n">
+        <v>13.09</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G159" t="n">
+        <v>76703.7</v>
+      </c>
+      <c r="H159" t="n">
+        <v>98</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K159" t="n">
+        <v>8</v>
+      </c>
+      <c r="L159" t="n">
+        <v>76709.39999999999</v>
+      </c>
+      <c r="M159" t="n">
+        <v>76699.8</v>
+      </c>
+      <c r="N159" t="n">
+        <v>76700.60000000001</v>
+      </c>
+      <c r="O159" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q159" t="n">
+        <v>76690.39999999999</v>
+      </c>
+      <c r="R159" t="n">
+        <v>76531.39999999999</v>
+      </c>
+      <c r="S159" t="n">
+        <v>76209.89999999999</v>
+      </c>
+      <c r="T159" t="n">
+        <v>75477.3</v>
+      </c>
+      <c r="U159" t="n">
+        <v>75987.39999999999</v>
+      </c>
+      <c r="V159" t="n">
+        <v>75843.60000000001</v>
+      </c>
+      <c r="W159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X159" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y159" t="n">
+        <v>76712.10000000001</v>
+      </c>
+      <c r="Z159" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AA159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB159" t="n">
+        <v>76503.7</v>
+      </c>
+      <c r="AC159" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD159" t="n">
+        <v>77303.7</v>
+      </c>
+      <c r="AE159" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF159" t="n">
+        <v>13.09</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>23950</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G160" t="n">
+        <v>23963.9</v>
+      </c>
+      <c r="H160" t="n">
+        <v>88</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K160" t="n">
+        <v>7</v>
+      </c>
+      <c r="L160" t="n">
+        <v>23957.9</v>
+      </c>
+      <c r="M160" t="n">
+        <v>23953.6</v>
+      </c>
+      <c r="N160" t="n">
+        <v>23963.6</v>
+      </c>
+      <c r="O160" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q160" t="n">
+        <v>23963.2</v>
+      </c>
+      <c r="R160" t="n">
+        <v>23897.2</v>
+      </c>
+      <c r="S160" t="n">
+        <v>23823.6</v>
+      </c>
+      <c r="T160" t="n">
+        <v>23606.4</v>
+      </c>
+      <c r="U160" t="n">
+        <v>23763</v>
+      </c>
+      <c r="V160" t="n">
+        <v>23715</v>
+      </c>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y160" t="n">
+        <v>23955</v>
+      </c>
+      <c r="Z160" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AA160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB160" t="n">
+        <v>23923.9</v>
+      </c>
+      <c r="AC160" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD160" t="n">
+        <v>24083.9</v>
+      </c>
+      <c r="AE160" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF160" t="n">
+        <v>13.09</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>76800</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G161" t="n">
+        <v>76775.10000000001</v>
+      </c>
+      <c r="H161" t="n">
+        <v>88</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K161" t="n">
+        <v>7</v>
+      </c>
+      <c r="L161" t="n">
+        <v>76734.8</v>
+      </c>
+      <c r="M161" t="n">
+        <v>76716.5</v>
+      </c>
+      <c r="N161" t="n">
+        <v>76769.5</v>
+      </c>
+      <c r="O161" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q161" t="n">
+        <v>76690.39999999999</v>
+      </c>
+      <c r="R161" t="n">
+        <v>76531.39999999999</v>
+      </c>
+      <c r="S161" t="n">
+        <v>76209.89999999999</v>
+      </c>
+      <c r="T161" t="n">
+        <v>75477.3</v>
+      </c>
+      <c r="U161" t="n">
+        <v>75987.39999999999</v>
+      </c>
+      <c r="V161" t="n">
+        <v>75843.60000000001</v>
+      </c>
+      <c r="W161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X161" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y161" t="n">
+        <v>76724.89999999999</v>
+      </c>
+      <c r="Z161" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AA161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB161" t="n">
+        <v>76575.10000000001</v>
+      </c>
+      <c r="AC161" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD161" t="n">
+        <v>77375.10000000001</v>
+      </c>
+      <c r="AE161" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF161" t="n">
+        <v>13.06</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>23950</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G162" t="n">
+        <v>23957.7</v>
+      </c>
+      <c r="H162" t="n">
+        <v>76</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K162" t="n">
+        <v>6</v>
+      </c>
+      <c r="L162" t="n">
+        <v>23957.3</v>
+      </c>
+      <c r="M162" t="n">
+        <v>23955.9</v>
+      </c>
+      <c r="N162" t="n">
+        <v>23956.4</v>
+      </c>
+      <c r="O162" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q162" t="n">
+        <v>23963.2</v>
+      </c>
+      <c r="R162" t="n">
+        <v>23897.2</v>
+      </c>
+      <c r="S162" t="n">
+        <v>23823.6</v>
+      </c>
+      <c r="T162" t="n">
+        <v>23606.4</v>
+      </c>
+      <c r="U162" t="n">
+        <v>23763</v>
+      </c>
+      <c r="V162" t="n">
+        <v>23715</v>
+      </c>
+      <c r="W162" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y162" t="n">
+        <v>23959.8</v>
+      </c>
+      <c r="Z162" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="AA162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB162" t="n">
+        <v>23917.7</v>
+      </c>
+      <c r="AC162" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD162" t="n">
+        <v>24077.7</v>
+      </c>
+      <c r="AE162" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF162" t="n">
+        <v>13.06</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G163" t="n">
+        <v>76704.39999999999</v>
+      </c>
+      <c r="H163" t="n">
+        <v>100</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K163" t="n">
+        <v>8</v>
+      </c>
+      <c r="L163" t="n">
+        <v>76719.10000000001</v>
+      </c>
+      <c r="M163" t="n">
+        <v>76714.8</v>
+      </c>
+      <c r="N163" t="n">
+        <v>76686.89999999999</v>
+      </c>
+      <c r="O163" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q163" t="n">
+        <v>76690.39999999999</v>
+      </c>
+      <c r="R163" t="n">
+        <v>76531.39999999999</v>
+      </c>
+      <c r="S163" t="n">
+        <v>76209.89999999999</v>
+      </c>
+      <c r="T163" t="n">
+        <v>75477.3</v>
+      </c>
+      <c r="U163" t="n">
+        <v>75987.39999999999</v>
+      </c>
+      <c r="V163" t="n">
+        <v>75843.60000000001</v>
+      </c>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y163" t="n">
+        <v>76692.39999999999</v>
+      </c>
+      <c r="Z163" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="AA163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB163" t="n">
+        <v>76504.39999999999</v>
+      </c>
+      <c r="AC163" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD163" t="n">
+        <v>77304.39999999999</v>
+      </c>
+      <c r="AE163" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF163" t="n">
+        <v>13.06</v>
+      </c>
+      <c r="AG163" t="inlineStr"/>
+      <c r="AH163" t="inlineStr"/>
+      <c r="AI163" t="inlineStr"/>
+      <c r="AJ163" t="inlineStr"/>
+      <c r="AK163" t="inlineStr"/>
+      <c r="AL163" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-28
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL163"/>
+  <dimension ref="A1:AL169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20108,12 +20108,732 @@
       <c r="AF163" t="n">
         <v>13.06</v>
       </c>
-      <c r="AG163" t="inlineStr"/>
-      <c r="AH163" t="inlineStr"/>
-      <c r="AI163" t="inlineStr"/>
-      <c r="AJ163" t="inlineStr"/>
-      <c r="AK163" t="inlineStr"/>
-      <c r="AL163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>76900</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G164" t="n">
+        <v>76927</v>
+      </c>
+      <c r="H164" t="n">
+        <v>78</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K164" t="n">
+        <v>7</v>
+      </c>
+      <c r="L164" t="n">
+        <v>76897</v>
+      </c>
+      <c r="M164" t="n">
+        <v>76890.60000000001</v>
+      </c>
+      <c r="N164" t="n">
+        <v>76917.60000000001</v>
+      </c>
+      <c r="O164" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q164" t="n">
+        <v>76986.8</v>
+      </c>
+      <c r="R164" t="n">
+        <v>76741.7</v>
+      </c>
+      <c r="S164" t="n">
+        <v>76901.5</v>
+      </c>
+      <c r="T164" t="n">
+        <v>76520.60000000001</v>
+      </c>
+      <c r="U164" t="n">
+        <v>76794.2</v>
+      </c>
+      <c r="V164" t="n">
+        <v>76711</v>
+      </c>
+      <c r="W164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X164" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y164" t="n">
+        <v>76928.89999999999</v>
+      </c>
+      <c r="Z164" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AA164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB164" t="n">
+        <v>76727</v>
+      </c>
+      <c r="AC164" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD164" t="n">
+        <v>77527</v>
+      </c>
+      <c r="AE164" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF164" t="n">
+        <v>12.56</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G165" t="n">
+        <v>24021.1</v>
+      </c>
+      <c r="H165" t="n">
+        <v>78</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K165" t="n">
+        <v>7</v>
+      </c>
+      <c r="L165" t="n">
+        <v>24016.9</v>
+      </c>
+      <c r="M165" t="n">
+        <v>24015.9</v>
+      </c>
+      <c r="N165" t="n">
+        <v>24021</v>
+      </c>
+      <c r="O165" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q165" t="n">
+        <v>24039.8</v>
+      </c>
+      <c r="R165" t="n">
+        <v>23969.2</v>
+      </c>
+      <c r="S165" t="n">
+        <v>24011.1</v>
+      </c>
+      <c r="T165" t="n">
+        <v>23891.7</v>
+      </c>
+      <c r="U165" t="n">
+        <v>23986.2</v>
+      </c>
+      <c r="V165" t="n">
+        <v>23951.4</v>
+      </c>
+      <c r="W165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y165" t="n">
+        <v>24024.1</v>
+      </c>
+      <c r="Z165" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AA165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB165" t="n">
+        <v>23981.1</v>
+      </c>
+      <c r="AC165" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD165" t="n">
+        <v>24141.1</v>
+      </c>
+      <c r="AE165" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF165" t="n">
+        <v>12.51</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G166" t="n">
+        <v>24021.9</v>
+      </c>
+      <c r="H166" t="n">
+        <v>78</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K166" t="n">
+        <v>7</v>
+      </c>
+      <c r="L166" t="n">
+        <v>24019.4</v>
+      </c>
+      <c r="M166" t="n">
+        <v>24017.9</v>
+      </c>
+      <c r="N166" t="n">
+        <v>24020.2</v>
+      </c>
+      <c r="O166" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q166" t="n">
+        <v>24039.8</v>
+      </c>
+      <c r="R166" t="n">
+        <v>23969.2</v>
+      </c>
+      <c r="S166" t="n">
+        <v>24011.1</v>
+      </c>
+      <c r="T166" t="n">
+        <v>23891.7</v>
+      </c>
+      <c r="U166" t="n">
+        <v>23986.2</v>
+      </c>
+      <c r="V166" t="n">
+        <v>23951.4</v>
+      </c>
+      <c r="W166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X166" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y166" t="n">
+        <v>24024.1</v>
+      </c>
+      <c r="Z166" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="AA166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB166" t="n">
+        <v>23981.9</v>
+      </c>
+      <c r="AC166" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD166" t="n">
+        <v>24141.9</v>
+      </c>
+      <c r="AE166" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF166" t="n">
+        <v>12.56</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>12:47</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>77000</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G167" t="n">
+        <v>76953.3</v>
+      </c>
+      <c r="H167" t="n">
+        <v>86</v>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K167" t="n">
+        <v>7</v>
+      </c>
+      <c r="L167" t="n">
+        <v>76934.60000000001</v>
+      </c>
+      <c r="M167" t="n">
+        <v>76916.89999999999</v>
+      </c>
+      <c r="N167" t="n">
+        <v>76950.10000000001</v>
+      </c>
+      <c r="O167" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q167" t="n">
+        <v>76986.8</v>
+      </c>
+      <c r="R167" t="n">
+        <v>76741.7</v>
+      </c>
+      <c r="S167" t="n">
+        <v>76901.5</v>
+      </c>
+      <c r="T167" t="n">
+        <v>76520.60000000001</v>
+      </c>
+      <c r="U167" t="n">
+        <v>76794.2</v>
+      </c>
+      <c r="V167" t="n">
+        <v>76711</v>
+      </c>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y167" t="n">
+        <v>76928.89999999999</v>
+      </c>
+      <c r="Z167" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB167" t="n">
+        <v>76753.3</v>
+      </c>
+      <c r="AC167" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD167" t="n">
+        <v>77553.3</v>
+      </c>
+      <c r="AE167" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF167" t="n">
+        <v>12.56</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>56900</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G168" t="n">
+        <v>56866.9</v>
+      </c>
+      <c r="H168" t="n">
+        <v>88</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K168" t="n">
+        <v>7</v>
+      </c>
+      <c r="L168" t="n">
+        <v>56911.4</v>
+      </c>
+      <c r="M168" t="n">
+        <v>56938.6</v>
+      </c>
+      <c r="N168" t="n">
+        <v>56867.7</v>
+      </c>
+      <c r="O168" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q168" t="n">
+        <v>57051.7</v>
+      </c>
+      <c r="R168" t="n">
+        <v>56889.8</v>
+      </c>
+      <c r="S168" t="n">
+        <v>57329.3</v>
+      </c>
+      <c r="T168" t="n">
+        <v>56929.1</v>
+      </c>
+      <c r="U168" t="n">
+        <v>57129.2</v>
+      </c>
+      <c r="V168" t="n">
+        <v>57120.4</v>
+      </c>
+      <c r="W168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y168" t="n">
+        <v>56852.6</v>
+      </c>
+      <c r="Z168" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB168" t="n">
+        <v>56986.9</v>
+      </c>
+      <c r="AC168" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD168" t="n">
+        <v>56506.9</v>
+      </c>
+      <c r="AE168" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF168" t="n">
+        <v>12.58</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>56800</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G169" t="n">
+        <v>56818.5</v>
+      </c>
+      <c r="H169" t="n">
+        <v>88</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K169" t="n">
+        <v>7</v>
+      </c>
+      <c r="L169" t="n">
+        <v>56849.1</v>
+      </c>
+      <c r="M169" t="n">
+        <v>56890.9</v>
+      </c>
+      <c r="N169" t="n">
+        <v>56820.1</v>
+      </c>
+      <c r="O169" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q169" t="n">
+        <v>57051.7</v>
+      </c>
+      <c r="R169" t="n">
+        <v>56889.8</v>
+      </c>
+      <c r="S169" t="n">
+        <v>57329.3</v>
+      </c>
+      <c r="T169" t="n">
+        <v>56929.1</v>
+      </c>
+      <c r="U169" t="n">
+        <v>57129.2</v>
+      </c>
+      <c r="V169" t="n">
+        <v>57120.4</v>
+      </c>
+      <c r="W169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y169" t="n">
+        <v>56847.4</v>
+      </c>
+      <c r="Z169" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="AA169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB169" t="n">
+        <v>56938.5</v>
+      </c>
+      <c r="AC169" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD169" t="n">
+        <v>56458.5</v>
+      </c>
+      <c r="AE169" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF169" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="AG169" t="inlineStr"/>
+      <c r="AH169" t="inlineStr"/>
+      <c r="AI169" t="inlineStr"/>
+      <c r="AJ169" t="inlineStr"/>
+      <c r="AK169" t="inlineStr"/>
+      <c r="AL169" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-29
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL169"/>
+  <dimension ref="A1:AL175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20828,12 +20828,732 @@
       <c r="AF169" t="n">
         <v>12.69</v>
       </c>
-      <c r="AG169" t="inlineStr"/>
-      <c r="AH169" t="inlineStr"/>
-      <c r="AI169" t="inlineStr"/>
-      <c r="AJ169" t="inlineStr"/>
-      <c r="AK169" t="inlineStr"/>
-      <c r="AL169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G170" t="n">
+        <v>24226.5</v>
+      </c>
+      <c r="H170" t="n">
+        <v>83</v>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K170" t="n">
+        <v>7</v>
+      </c>
+      <c r="L170" t="n">
+        <v>24228.4</v>
+      </c>
+      <c r="M170" t="n">
+        <v>24225.3</v>
+      </c>
+      <c r="N170" t="n">
+        <v>24226.9</v>
+      </c>
+      <c r="O170" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q170" t="n">
+        <v>24196.2</v>
+      </c>
+      <c r="R170" t="n">
+        <v>24141.8</v>
+      </c>
+      <c r="S170" t="n">
+        <v>24041</v>
+      </c>
+      <c r="T170" t="n">
+        <v>23954.7</v>
+      </c>
+      <c r="U170" t="n">
+        <v>23997.8</v>
+      </c>
+      <c r="V170" t="n">
+        <v>23988.6</v>
+      </c>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X170" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y170" t="n">
+        <v>24219.8</v>
+      </c>
+      <c r="Z170" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AA170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB170" t="n">
+        <v>24186.5</v>
+      </c>
+      <c r="AC170" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD170" t="n">
+        <v>24346.5</v>
+      </c>
+      <c r="AE170" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF170" t="n">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>57200</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G171" t="n">
+        <v>57180.6</v>
+      </c>
+      <c r="H171" t="n">
+        <v>83</v>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K171" t="n">
+        <v>7</v>
+      </c>
+      <c r="L171" t="n">
+        <v>57163.4</v>
+      </c>
+      <c r="M171" t="n">
+        <v>57140.7</v>
+      </c>
+      <c r="N171" t="n">
+        <v>57180.9</v>
+      </c>
+      <c r="O171" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q171" t="n">
+        <v>57142.3</v>
+      </c>
+      <c r="R171" t="n">
+        <v>56965.1</v>
+      </c>
+      <c r="S171" t="n">
+        <v>57051.7</v>
+      </c>
+      <c r="T171" t="n">
+        <v>56672.5</v>
+      </c>
+      <c r="U171" t="n">
+        <v>56862.1</v>
+      </c>
+      <c r="V171" t="n">
+        <v>56766.5</v>
+      </c>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X171" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y171" t="n">
+        <v>57138.6</v>
+      </c>
+      <c r="Z171" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB171" t="n">
+        <v>57060.6</v>
+      </c>
+      <c r="AC171" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD171" t="n">
+        <v>57540.6</v>
+      </c>
+      <c r="AE171" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF171" t="n">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G172" t="n">
+        <v>77609.10000000001</v>
+      </c>
+      <c r="H172" t="n">
+        <v>98</v>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K172" t="n">
+        <v>8</v>
+      </c>
+      <c r="L172" t="n">
+        <v>77606.5</v>
+      </c>
+      <c r="M172" t="n">
+        <v>77591.3</v>
+      </c>
+      <c r="N172" t="n">
+        <v>77607.60000000001</v>
+      </c>
+      <c r="O172" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q172" t="n">
+        <v>77552.10000000001</v>
+      </c>
+      <c r="R172" t="n">
+        <v>77354.89999999999</v>
+      </c>
+      <c r="S172" t="n">
+        <v>76986.8</v>
+      </c>
+      <c r="T172" t="n">
+        <v>76672.8</v>
+      </c>
+      <c r="U172" t="n">
+        <v>76829.8</v>
+      </c>
+      <c r="V172" t="n">
+        <v>76787.2</v>
+      </c>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y172" t="n">
+        <v>77576.8</v>
+      </c>
+      <c r="Z172" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AA172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB172" t="n">
+        <v>77409.10000000001</v>
+      </c>
+      <c r="AC172" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD172" t="n">
+        <v>78209.10000000001</v>
+      </c>
+      <c r="AE172" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF172" t="n">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>57200</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G173" t="n">
+        <v>57200.7</v>
+      </c>
+      <c r="H173" t="n">
+        <v>98</v>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K173" t="n">
+        <v>8</v>
+      </c>
+      <c r="L173" t="n">
+        <v>57172.4</v>
+      </c>
+      <c r="M173" t="n">
+        <v>57147</v>
+      </c>
+      <c r="N173" t="n">
+        <v>57197</v>
+      </c>
+      <c r="O173" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q173" t="n">
+        <v>57142.3</v>
+      </c>
+      <c r="R173" t="n">
+        <v>56965.1</v>
+      </c>
+      <c r="S173" t="n">
+        <v>57051.7</v>
+      </c>
+      <c r="T173" t="n">
+        <v>56672.5</v>
+      </c>
+      <c r="U173" t="n">
+        <v>56862.1</v>
+      </c>
+      <c r="V173" t="n">
+        <v>56766.5</v>
+      </c>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X173" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y173" t="n">
+        <v>57150.4</v>
+      </c>
+      <c r="Z173" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="AA173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB173" t="n">
+        <v>57080.7</v>
+      </c>
+      <c r="AC173" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD173" t="n">
+        <v>57560.7</v>
+      </c>
+      <c r="AE173" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF173" t="n">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G174" t="n">
+        <v>24231.7</v>
+      </c>
+      <c r="H174" t="n">
+        <v>98</v>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K174" t="n">
+        <v>8</v>
+      </c>
+      <c r="L174" t="n">
+        <v>24232.3</v>
+      </c>
+      <c r="M174" t="n">
+        <v>24228.6</v>
+      </c>
+      <c r="N174" t="n">
+        <v>24231.1</v>
+      </c>
+      <c r="O174" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q174" t="n">
+        <v>24196.2</v>
+      </c>
+      <c r="R174" t="n">
+        <v>24141.8</v>
+      </c>
+      <c r="S174" t="n">
+        <v>24041</v>
+      </c>
+      <c r="T174" t="n">
+        <v>23954.7</v>
+      </c>
+      <c r="U174" t="n">
+        <v>23997.8</v>
+      </c>
+      <c r="V174" t="n">
+        <v>23988.6</v>
+      </c>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X174" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y174" t="n">
+        <v>24222.5</v>
+      </c>
+      <c r="Z174" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AA174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB174" t="n">
+        <v>24191.7</v>
+      </c>
+      <c r="AC174" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD174" t="n">
+        <v>24351.7</v>
+      </c>
+      <c r="AE174" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF174" t="n">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G175" t="n">
+        <v>77615.89999999999</v>
+      </c>
+      <c r="H175" t="n">
+        <v>83</v>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>7</v>
+      </c>
+      <c r="L175" t="n">
+        <v>77614.5</v>
+      </c>
+      <c r="M175" t="n">
+        <v>77601.3</v>
+      </c>
+      <c r="N175" t="n">
+        <v>77621.89999999999</v>
+      </c>
+      <c r="O175" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q175" t="n">
+        <v>77552.10000000001</v>
+      </c>
+      <c r="R175" t="n">
+        <v>77354.89999999999</v>
+      </c>
+      <c r="S175" t="n">
+        <v>76986.8</v>
+      </c>
+      <c r="T175" t="n">
+        <v>76672.8</v>
+      </c>
+      <c r="U175" t="n">
+        <v>76829.8</v>
+      </c>
+      <c r="V175" t="n">
+        <v>76787.2</v>
+      </c>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y175" t="n">
+        <v>77582</v>
+      </c>
+      <c r="Z175" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB175" t="n">
+        <v>77415.89999999999</v>
+      </c>
+      <c r="AC175" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD175" t="n">
+        <v>78215.89999999999</v>
+      </c>
+      <c r="AE175" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF175" t="n">
+        <v>12.13</v>
+      </c>
+      <c r="AG175" t="inlineStr"/>
+      <c r="AH175" t="inlineStr"/>
+      <c r="AI175" t="inlineStr"/>
+      <c r="AJ175" t="inlineStr"/>
+      <c r="AK175" t="inlineStr"/>
+      <c r="AL175" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-30
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL175"/>
+  <dimension ref="A1:AL181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21548,12 +21548,732 @@
       <c r="AF175" t="n">
         <v>12.13</v>
       </c>
-      <c r="AG175" t="inlineStr"/>
-      <c r="AH175" t="inlineStr"/>
-      <c r="AI175" t="inlineStr"/>
-      <c r="AJ175" t="inlineStr"/>
-      <c r="AK175" t="inlineStr"/>
-      <c r="AL175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>56800</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G176" t="n">
+        <v>56832.7</v>
+      </c>
+      <c r="H176" t="n">
+        <v>83</v>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K176" t="n">
+        <v>7</v>
+      </c>
+      <c r="L176" t="n">
+        <v>56868.8</v>
+      </c>
+      <c r="M176" t="n">
+        <v>56878</v>
+      </c>
+      <c r="N176" t="n">
+        <v>56840.5</v>
+      </c>
+      <c r="O176" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q176" t="n">
+        <v>57118.4</v>
+      </c>
+      <c r="R176" t="n">
+        <v>56870.1</v>
+      </c>
+      <c r="S176" t="n">
+        <v>57315.4</v>
+      </c>
+      <c r="T176" t="n">
+        <v>56939.7</v>
+      </c>
+      <c r="U176" t="n">
+        <v>57171.6</v>
+      </c>
+      <c r="V176" t="n">
+        <v>57127.5</v>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X176" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y176" t="n">
+        <v>56851.4</v>
+      </c>
+      <c r="Z176" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AA176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB176" t="n">
+        <v>56952.7</v>
+      </c>
+      <c r="AC176" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD176" t="n">
+        <v>56472.7</v>
+      </c>
+      <c r="AE176" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF176" t="n">
+        <v>12.14</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>77700</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G177" t="n">
+        <v>77697.3</v>
+      </c>
+      <c r="H177" t="n">
+        <v>76</v>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K177" t="n">
+        <v>6</v>
+      </c>
+      <c r="L177" t="n">
+        <v>77681.39999999999</v>
+      </c>
+      <c r="M177" t="n">
+        <v>77672.7</v>
+      </c>
+      <c r="N177" t="n">
+        <v>77682.10000000001</v>
+      </c>
+      <c r="O177" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q177" t="n">
+        <v>77734.2</v>
+      </c>
+      <c r="R177" t="n">
+        <v>77458.8</v>
+      </c>
+      <c r="S177" t="n">
+        <v>77765.39999999999</v>
+      </c>
+      <c r="T177" t="n">
+        <v>77354.89999999999</v>
+      </c>
+      <c r="U177" t="n">
+        <v>77623.39999999999</v>
+      </c>
+      <c r="V177" t="n">
+        <v>77560.2</v>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X177" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y177" t="n">
+        <v>77681.10000000001</v>
+      </c>
+      <c r="Z177" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AA177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB177" t="n">
+        <v>77497.3</v>
+      </c>
+      <c r="AC177" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD177" t="n">
+        <v>78297.3</v>
+      </c>
+      <c r="AE177" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF177" t="n">
+        <v>12.15</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G178" t="n">
+        <v>24304.8</v>
+      </c>
+      <c r="H178" t="n">
+        <v>88</v>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>7</v>
+      </c>
+      <c r="L178" t="n">
+        <v>24269.3</v>
+      </c>
+      <c r="M178" t="n">
+        <v>24264.9</v>
+      </c>
+      <c r="N178" t="n">
+        <v>24290.5</v>
+      </c>
+      <c r="O178" t="n">
+        <v>72</v>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q178" t="n">
+        <v>24280.2</v>
+      </c>
+      <c r="R178" t="n">
+        <v>24190</v>
+      </c>
+      <c r="S178" t="n">
+        <v>24283</v>
+      </c>
+      <c r="T178" t="n">
+        <v>24141.8</v>
+      </c>
+      <c r="U178" t="n">
+        <v>24232.1</v>
+      </c>
+      <c r="V178" t="n">
+        <v>24212.4</v>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X178" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y178" t="n">
+        <v>24277.7</v>
+      </c>
+      <c r="Z178" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="AA178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB178" t="n">
+        <v>24264.8</v>
+      </c>
+      <c r="AC178" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD178" t="n">
+        <v>24424.8</v>
+      </c>
+      <c r="AE178" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF178" t="n">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>77800</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G179" t="n">
+        <v>77828.3</v>
+      </c>
+      <c r="H179" t="n">
+        <v>88</v>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K179" t="n">
+        <v>7</v>
+      </c>
+      <c r="L179" t="n">
+        <v>77707.2</v>
+      </c>
+      <c r="M179" t="n">
+        <v>77686.10000000001</v>
+      </c>
+      <c r="N179" t="n">
+        <v>77780.89999999999</v>
+      </c>
+      <c r="O179" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q179" t="n">
+        <v>77734.2</v>
+      </c>
+      <c r="R179" t="n">
+        <v>77458.8</v>
+      </c>
+      <c r="S179" t="n">
+        <v>77765.39999999999</v>
+      </c>
+      <c r="T179" t="n">
+        <v>77354.89999999999</v>
+      </c>
+      <c r="U179" t="n">
+        <v>77623.39999999999</v>
+      </c>
+      <c r="V179" t="n">
+        <v>77560.2</v>
+      </c>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X179" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y179" t="n">
+        <v>77741.10000000001</v>
+      </c>
+      <c r="Z179" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="AA179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB179" t="n">
+        <v>77628.3</v>
+      </c>
+      <c r="AC179" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD179" t="n">
+        <v>78428.3</v>
+      </c>
+      <c r="AE179" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF179" t="n">
+        <v>12.09</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G180" t="n">
+        <v>24287.1</v>
+      </c>
+      <c r="H180" t="n">
+        <v>86</v>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K180" t="n">
+        <v>7</v>
+      </c>
+      <c r="L180" t="n">
+        <v>24289.5</v>
+      </c>
+      <c r="M180" t="n">
+        <v>24279.4</v>
+      </c>
+      <c r="N180" t="n">
+        <v>24287.5</v>
+      </c>
+      <c r="O180" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q180" t="n">
+        <v>24280.2</v>
+      </c>
+      <c r="R180" t="n">
+        <v>24190</v>
+      </c>
+      <c r="S180" t="n">
+        <v>24283</v>
+      </c>
+      <c r="T180" t="n">
+        <v>24141.8</v>
+      </c>
+      <c r="U180" t="n">
+        <v>24232.1</v>
+      </c>
+      <c r="V180" t="n">
+        <v>24212.4</v>
+      </c>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X180" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y180" t="n">
+        <v>24277.2</v>
+      </c>
+      <c r="Z180" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="AA180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB180" t="n">
+        <v>24247.1</v>
+      </c>
+      <c r="AC180" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD180" t="n">
+        <v>24407.1</v>
+      </c>
+      <c r="AE180" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF180" t="n">
+        <v>12.18</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>77800</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G181" t="n">
+        <v>77815.2</v>
+      </c>
+      <c r="H181" t="n">
+        <v>98</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K181" t="n">
+        <v>8</v>
+      </c>
+      <c r="L181" t="n">
+        <v>77778.39999999999</v>
+      </c>
+      <c r="M181" t="n">
+        <v>77731.7</v>
+      </c>
+      <c r="N181" t="n">
+        <v>77811.5</v>
+      </c>
+      <c r="O181" t="n">
+        <v>64</v>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q181" t="n">
+        <v>77734.2</v>
+      </c>
+      <c r="R181" t="n">
+        <v>77458.8</v>
+      </c>
+      <c r="S181" t="n">
+        <v>77765.39999999999</v>
+      </c>
+      <c r="T181" t="n">
+        <v>77354.89999999999</v>
+      </c>
+      <c r="U181" t="n">
+        <v>77623.39999999999</v>
+      </c>
+      <c r="V181" t="n">
+        <v>77560.2</v>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y181" t="n">
+        <v>77795.39999999999</v>
+      </c>
+      <c r="Z181" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB181" t="n">
+        <v>77615.2</v>
+      </c>
+      <c r="AC181" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD181" t="n">
+        <v>78415.2</v>
+      </c>
+      <c r="AE181" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF181" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="AG181" t="inlineStr"/>
+      <c r="AH181" t="inlineStr"/>
+      <c r="AI181" t="inlineStr"/>
+      <c r="AJ181" t="inlineStr"/>
+      <c r="AK181" t="inlineStr"/>
+      <c r="AL181" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-07-31
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL181"/>
+  <dimension ref="A1:AL187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22268,12 +22268,732 @@
       <c r="AF181" t="n">
         <v>12.18</v>
       </c>
-      <c r="AG181" t="inlineStr"/>
-      <c r="AH181" t="inlineStr"/>
-      <c r="AI181" t="inlineStr"/>
-      <c r="AJ181" t="inlineStr"/>
-      <c r="AK181" t="inlineStr"/>
-      <c r="AL181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>24350</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G182" t="n">
+        <v>24373.2</v>
+      </c>
+      <c r="H182" t="n">
+        <v>91</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K182" t="n">
+        <v>7</v>
+      </c>
+      <c r="L182" t="n">
+        <v>24365.7</v>
+      </c>
+      <c r="M182" t="n">
+        <v>24360.7</v>
+      </c>
+      <c r="N182" t="n">
+        <v>24370.9</v>
+      </c>
+      <c r="O182" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q182" t="n">
+        <v>24377.6</v>
+      </c>
+      <c r="R182" t="n">
+        <v>24328.2</v>
+      </c>
+      <c r="S182" t="n">
+        <v>24342.9</v>
+      </c>
+      <c r="T182" t="n">
+        <v>24190</v>
+      </c>
+      <c r="U182" t="n">
+        <v>24286.6</v>
+      </c>
+      <c r="V182" t="n">
+        <v>24266.5</v>
+      </c>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y182" t="n">
+        <v>24365.9</v>
+      </c>
+      <c r="Z182" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB182" t="n">
+        <v>24333.2</v>
+      </c>
+      <c r="AC182" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD182" t="n">
+        <v>24493.2</v>
+      </c>
+      <c r="AE182" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF182" t="n">
+        <v>11.85</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>78000</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G183" t="n">
+        <v>78043.5</v>
+      </c>
+      <c r="H183" t="n">
+        <v>100</v>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K183" t="n">
+        <v>8</v>
+      </c>
+      <c r="L183" t="n">
+        <v>78025.8</v>
+      </c>
+      <c r="M183" t="n">
+        <v>78007.60000000001</v>
+      </c>
+      <c r="N183" t="n">
+        <v>78040.3</v>
+      </c>
+      <c r="O183" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q183" t="n">
+        <v>78041.89999999999</v>
+      </c>
+      <c r="R183" t="n">
+        <v>77897.10000000001</v>
+      </c>
+      <c r="S183" t="n">
+        <v>77960.10000000001</v>
+      </c>
+      <c r="T183" t="n">
+        <v>77458.8</v>
+      </c>
+      <c r="U183" t="n">
+        <v>77855.2</v>
+      </c>
+      <c r="V183" t="n">
+        <v>77709.39999999999</v>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y183" t="n">
+        <v>78031.60000000001</v>
+      </c>
+      <c r="Z183" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB183" t="n">
+        <v>77843.5</v>
+      </c>
+      <c r="AC183" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD183" t="n">
+        <v>78643.5</v>
+      </c>
+      <c r="AE183" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF183" t="n">
+        <v>11.85</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>57300</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G184" t="n">
+        <v>57250.9</v>
+      </c>
+      <c r="H184" t="n">
+        <v>84</v>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K184" t="n">
+        <v>7</v>
+      </c>
+      <c r="L184" t="n">
+        <v>57208.6</v>
+      </c>
+      <c r="M184" t="n">
+        <v>57204.6</v>
+      </c>
+      <c r="N184" t="n">
+        <v>57235.8</v>
+      </c>
+      <c r="O184" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q184" t="n">
+        <v>57409.9</v>
+      </c>
+      <c r="R184" t="n">
+        <v>57225.9</v>
+      </c>
+      <c r="S184" t="n">
+        <v>57236.6</v>
+      </c>
+      <c r="T184" t="n">
+        <v>56768.9</v>
+      </c>
+      <c r="U184" t="n">
+        <v>57069.5</v>
+      </c>
+      <c r="V184" t="n">
+        <v>57002.8</v>
+      </c>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>0.786</t>
+        </is>
+      </c>
+      <c r="Y184" t="n">
+        <v>57265.3</v>
+      </c>
+      <c r="Z184" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA184" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB184" t="n">
+        <v>57130.9</v>
+      </c>
+      <c r="AC184" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD184" t="n">
+        <v>57610.9</v>
+      </c>
+      <c r="AE184" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF184" t="n">
+        <v>11.93</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>24400</v>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G185" t="n">
+        <v>24398.7</v>
+      </c>
+      <c r="H185" t="n">
+        <v>93</v>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K185" t="n">
+        <v>7</v>
+      </c>
+      <c r="L185" t="n">
+        <v>24384.8</v>
+      </c>
+      <c r="M185" t="n">
+        <v>24373.6</v>
+      </c>
+      <c r="N185" t="n">
+        <v>24398.1</v>
+      </c>
+      <c r="O185" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q185" t="n">
+        <v>24377.6</v>
+      </c>
+      <c r="R185" t="n">
+        <v>24328.2</v>
+      </c>
+      <c r="S185" t="n">
+        <v>24342.9</v>
+      </c>
+      <c r="T185" t="n">
+        <v>24190</v>
+      </c>
+      <c r="U185" t="n">
+        <v>24286.6</v>
+      </c>
+      <c r="V185" t="n">
+        <v>24266.5</v>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X185" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y185" t="n">
+        <v>24383.9</v>
+      </c>
+      <c r="Z185" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB185" t="n">
+        <v>24358.7</v>
+      </c>
+      <c r="AC185" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD185" t="n">
+        <v>24518.7</v>
+      </c>
+      <c r="AE185" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF185" t="n">
+        <v>11.91</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>78100</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G186" t="n">
+        <v>78133.60000000001</v>
+      </c>
+      <c r="H186" t="n">
+        <v>93</v>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K186" t="n">
+        <v>7</v>
+      </c>
+      <c r="L186" t="n">
+        <v>78073.5</v>
+      </c>
+      <c r="M186" t="n">
+        <v>78040.7</v>
+      </c>
+      <c r="N186" t="n">
+        <v>78120.60000000001</v>
+      </c>
+      <c r="O186" t="n">
+        <v>73</v>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q186" t="n">
+        <v>78041.89999999999</v>
+      </c>
+      <c r="R186" t="n">
+        <v>77897.10000000001</v>
+      </c>
+      <c r="S186" t="n">
+        <v>77960.10000000001</v>
+      </c>
+      <c r="T186" t="n">
+        <v>77458.8</v>
+      </c>
+      <c r="U186" t="n">
+        <v>77855.2</v>
+      </c>
+      <c r="V186" t="n">
+        <v>77709.39999999999</v>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X186" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y186" t="n">
+        <v>78079.7</v>
+      </c>
+      <c r="Z186" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB186" t="n">
+        <v>77933.60000000001</v>
+      </c>
+      <c r="AC186" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD186" t="n">
+        <v>78733.60000000001</v>
+      </c>
+      <c r="AE186" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF186" t="n">
+        <v>11.91</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>57200</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G187" t="n">
+        <v>57246.4</v>
+      </c>
+      <c r="H187" t="n">
+        <v>84</v>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K187" t="n">
+        <v>7</v>
+      </c>
+      <c r="L187" t="n">
+        <v>57230</v>
+      </c>
+      <c r="M187" t="n">
+        <v>57218.8</v>
+      </c>
+      <c r="N187" t="n">
+        <v>57239.9</v>
+      </c>
+      <c r="O187" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q187" t="n">
+        <v>57409.9</v>
+      </c>
+      <c r="R187" t="n">
+        <v>57225.9</v>
+      </c>
+      <c r="S187" t="n">
+        <v>57236.6</v>
+      </c>
+      <c r="T187" t="n">
+        <v>56768.9</v>
+      </c>
+      <c r="U187" t="n">
+        <v>57069.5</v>
+      </c>
+      <c r="V187" t="n">
+        <v>57002.8</v>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr">
+        <is>
+          <t>0.786</t>
+        </is>
+      </c>
+      <c r="Y187" t="n">
+        <v>57265.3</v>
+      </c>
+      <c r="Z187" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB187" t="n">
+        <v>57126.4</v>
+      </c>
+      <c r="AC187" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD187" t="n">
+        <v>57606.4</v>
+      </c>
+      <c r="AE187" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF187" t="n">
+        <v>11.94</v>
+      </c>
+      <c r="AG187" t="inlineStr"/>
+      <c r="AH187" t="inlineStr"/>
+      <c r="AI187" t="inlineStr"/>
+      <c r="AJ187" t="inlineStr"/>
+      <c r="AK187" t="inlineStr"/>
+      <c r="AL187" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-03
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL187"/>
+  <dimension ref="A1:AL193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22988,12 +22988,732 @@
       <c r="AF187" t="n">
         <v>11.94</v>
       </c>
-      <c r="AG187" t="inlineStr"/>
-      <c r="AH187" t="inlineStr"/>
-      <c r="AI187" t="inlineStr"/>
-      <c r="AJ187" t="inlineStr"/>
-      <c r="AK187" t="inlineStr"/>
-      <c r="AL187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>78700</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G188" t="n">
+        <v>78736.8</v>
+      </c>
+      <c r="H188" t="n">
+        <v>83</v>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K188" t="n">
+        <v>7</v>
+      </c>
+      <c r="L188" t="n">
+        <v>78743.60000000001</v>
+      </c>
+      <c r="M188" t="n">
+        <v>78736.5</v>
+      </c>
+      <c r="N188" t="n">
+        <v>78726.5</v>
+      </c>
+      <c r="O188" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q188" t="n">
+        <v>78809.8</v>
+      </c>
+      <c r="R188" t="n">
+        <v>78505.60000000001</v>
+      </c>
+      <c r="S188" t="n">
+        <v>78270.7</v>
+      </c>
+      <c r="T188" t="n">
+        <v>77811.3</v>
+      </c>
+      <c r="U188" t="n">
+        <v>78076.8</v>
+      </c>
+      <c r="V188" t="n">
+        <v>78041</v>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y188" t="n">
+        <v>78738</v>
+      </c>
+      <c r="Z188" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB188" t="n">
+        <v>78536.8</v>
+      </c>
+      <c r="AC188" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD188" t="n">
+        <v>79336.8</v>
+      </c>
+      <c r="AE188" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF188" t="n">
+        <v>11.97</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>24600</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G189" t="n">
+        <v>24579.1</v>
+      </c>
+      <c r="H189" t="n">
+        <v>76</v>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K189" t="n">
+        <v>6</v>
+      </c>
+      <c r="L189" t="n">
+        <v>24588.3</v>
+      </c>
+      <c r="M189" t="n">
+        <v>24589.6</v>
+      </c>
+      <c r="N189" t="n">
+        <v>24580.6</v>
+      </c>
+      <c r="O189" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q189" t="n">
+        <v>24568</v>
+      </c>
+      <c r="R189" t="n">
+        <v>24515.5</v>
+      </c>
+      <c r="S189" t="n">
+        <v>24429.4</v>
+      </c>
+      <c r="T189" t="n">
+        <v>24299.7</v>
+      </c>
+      <c r="U189" t="n">
+        <v>24366</v>
+      </c>
+      <c r="V189" t="n">
+        <v>24364.5</v>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y189" t="n">
+        <v>24573.6</v>
+      </c>
+      <c r="Z189" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB189" t="n">
+        <v>24539.1</v>
+      </c>
+      <c r="AC189" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD189" t="n">
+        <v>24699.1</v>
+      </c>
+      <c r="AE189" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF189" t="n">
+        <v>11.97</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>24600</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G190" t="n">
+        <v>24583.6</v>
+      </c>
+      <c r="H190" t="n">
+        <v>88</v>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K190" t="n">
+        <v>7</v>
+      </c>
+      <c r="L190" t="n">
+        <v>24584.9</v>
+      </c>
+      <c r="M190" t="n">
+        <v>24587.5</v>
+      </c>
+      <c r="N190" t="n">
+        <v>24581.7</v>
+      </c>
+      <c r="O190" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q190" t="n">
+        <v>24568</v>
+      </c>
+      <c r="R190" t="n">
+        <v>24515.5</v>
+      </c>
+      <c r="S190" t="n">
+        <v>24429.4</v>
+      </c>
+      <c r="T190" t="n">
+        <v>24299.7</v>
+      </c>
+      <c r="U190" t="n">
+        <v>24366</v>
+      </c>
+      <c r="V190" t="n">
+        <v>24364.5</v>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y190" t="n">
+        <v>24587.3</v>
+      </c>
+      <c r="Z190" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB190" t="n">
+        <v>24543.6</v>
+      </c>
+      <c r="AC190" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD190" t="n">
+        <v>24703.6</v>
+      </c>
+      <c r="AE190" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF190" t="n">
+        <v>11.97</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G191" t="n">
+        <v>57697.6</v>
+      </c>
+      <c r="H191" t="n">
+        <v>76</v>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K191" t="n">
+        <v>6</v>
+      </c>
+      <c r="L191" t="n">
+        <v>57701.6</v>
+      </c>
+      <c r="M191" t="n">
+        <v>57728.2</v>
+      </c>
+      <c r="N191" t="n">
+        <v>57693.6</v>
+      </c>
+      <c r="O191" t="n">
+        <v>43</v>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q191" t="n">
+        <v>57619.9</v>
+      </c>
+      <c r="R191" t="n">
+        <v>57470.4</v>
+      </c>
+      <c r="S191" t="n">
+        <v>57409.9</v>
+      </c>
+      <c r="T191" t="n">
+        <v>57142</v>
+      </c>
+      <c r="U191" t="n">
+        <v>57275.9</v>
+      </c>
+      <c r="V191" t="n">
+        <v>57234.7</v>
+      </c>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y191" t="n">
+        <v>57707.1</v>
+      </c>
+      <c r="Z191" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB191" t="n">
+        <v>57577.6</v>
+      </c>
+      <c r="AC191" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD191" t="n">
+        <v>58057.6</v>
+      </c>
+      <c r="AE191" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF191" t="n">
+        <v>11.97</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>24600</v>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G192" t="n">
+        <v>24600.3</v>
+      </c>
+      <c r="H192" t="n">
+        <v>100</v>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K192" t="n">
+        <v>8</v>
+      </c>
+      <c r="L192" t="n">
+        <v>24590.9</v>
+      </c>
+      <c r="M192" t="n">
+        <v>24589.7</v>
+      </c>
+      <c r="N192" t="n">
+        <v>24600.2</v>
+      </c>
+      <c r="O192" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q192" t="n">
+        <v>24568</v>
+      </c>
+      <c r="R192" t="n">
+        <v>24515.5</v>
+      </c>
+      <c r="S192" t="n">
+        <v>24429.4</v>
+      </c>
+      <c r="T192" t="n">
+        <v>24299.7</v>
+      </c>
+      <c r="U192" t="n">
+        <v>24366</v>
+      </c>
+      <c r="V192" t="n">
+        <v>24364.5</v>
+      </c>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X192" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y192" t="n">
+        <v>24587.3</v>
+      </c>
+      <c r="Z192" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB192" t="n">
+        <v>24560.3</v>
+      </c>
+      <c r="AC192" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD192" t="n">
+        <v>24720.3</v>
+      </c>
+      <c r="AE192" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF192" t="n">
+        <v>11.93</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G193" t="n">
+        <v>57715.1</v>
+      </c>
+      <c r="H193" t="n">
+        <v>76</v>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K193" t="n">
+        <v>6</v>
+      </c>
+      <c r="L193" t="n">
+        <v>57711.1</v>
+      </c>
+      <c r="M193" t="n">
+        <v>57720.2</v>
+      </c>
+      <c r="N193" t="n">
+        <v>57714.4</v>
+      </c>
+      <c r="O193" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q193" t="n">
+        <v>57619.9</v>
+      </c>
+      <c r="R193" t="n">
+        <v>57470.4</v>
+      </c>
+      <c r="S193" t="n">
+        <v>57409.9</v>
+      </c>
+      <c r="T193" t="n">
+        <v>57142</v>
+      </c>
+      <c r="U193" t="n">
+        <v>57275.9</v>
+      </c>
+      <c r="V193" t="n">
+        <v>57234.7</v>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y193" t="n">
+        <v>57707.1</v>
+      </c>
+      <c r="Z193" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB193" t="n">
+        <v>57595.1</v>
+      </c>
+      <c r="AC193" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD193" t="n">
+        <v>58075.1</v>
+      </c>
+      <c r="AE193" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF193" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="AG193" t="inlineStr"/>
+      <c r="AH193" t="inlineStr"/>
+      <c r="AI193" t="inlineStr"/>
+      <c r="AJ193" t="inlineStr"/>
+      <c r="AK193" t="inlineStr"/>
+      <c r="AL193" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-04
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL193"/>
+  <dimension ref="A1:AL199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23708,12 +23708,732 @@
       <c r="AF193" t="n">
         <v>11.95</v>
       </c>
-      <c r="AG193" t="inlineStr"/>
-      <c r="AH193" t="inlineStr"/>
-      <c r="AI193" t="inlineStr"/>
-      <c r="AJ193" t="inlineStr"/>
-      <c r="AK193" t="inlineStr"/>
-      <c r="AL193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>24550</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G194" t="n">
+        <v>24529.1</v>
+      </c>
+      <c r="H194" t="n">
+        <v>78</v>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K194" t="n">
+        <v>6</v>
+      </c>
+      <c r="L194" t="n">
+        <v>24553.9</v>
+      </c>
+      <c r="M194" t="n">
+        <v>24572.1</v>
+      </c>
+      <c r="N194" t="n">
+        <v>24530.4</v>
+      </c>
+      <c r="O194" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q194" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="R194" t="n">
+        <v>24591.3</v>
+      </c>
+      <c r="S194" t="n">
+        <v>24774.3</v>
+      </c>
+      <c r="T194" t="n">
+        <v>24515.5</v>
+      </c>
+      <c r="U194" t="n">
+        <v>24731.2</v>
+      </c>
+      <c r="V194" t="n">
+        <v>24644.9</v>
+      </c>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X194" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y194" t="n">
+        <v>24559.4</v>
+      </c>
+      <c r="Z194" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB194" t="n">
+        <v>24569.1</v>
+      </c>
+      <c r="AC194" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD194" t="n">
+        <v>24409.1</v>
+      </c>
+      <c r="AE194" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF194" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>78500</v>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G195" t="n">
+        <v>78479.89999999999</v>
+      </c>
+      <c r="H195" t="n">
+        <v>83</v>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K195" t="n">
+        <v>7</v>
+      </c>
+      <c r="L195" t="n">
+        <v>78556.8</v>
+      </c>
+      <c r="M195" t="n">
+        <v>78623.89999999999</v>
+      </c>
+      <c r="N195" t="n">
+        <v>78466.39999999999</v>
+      </c>
+      <c r="O195" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q195" t="n">
+        <v>79133</v>
+      </c>
+      <c r="R195" t="n">
+        <v>78730.39999999999</v>
+      </c>
+      <c r="S195" t="n">
+        <v>78809.8</v>
+      </c>
+      <c r="T195" t="n">
+        <v>78505.60000000001</v>
+      </c>
+      <c r="U195" t="n">
+        <v>78657.7</v>
+      </c>
+      <c r="V195" t="n">
+        <v>78645.3</v>
+      </c>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X195" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y195" t="n">
+        <v>78595.2</v>
+      </c>
+      <c r="Z195" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB195" t="n">
+        <v>78679.89999999999</v>
+      </c>
+      <c r="AC195" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD195" t="n">
+        <v>77879.89999999999</v>
+      </c>
+      <c r="AE195" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF195" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D196" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G196" t="n">
+        <v>24516.4</v>
+      </c>
+      <c r="H196" t="n">
+        <v>78</v>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K196" t="n">
+        <v>6</v>
+      </c>
+      <c r="L196" t="n">
+        <v>24525.9</v>
+      </c>
+      <c r="M196" t="n">
+        <v>24547.4</v>
+      </c>
+      <c r="N196" t="n">
+        <v>24516.6</v>
+      </c>
+      <c r="O196" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q196" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="R196" t="n">
+        <v>24591.3</v>
+      </c>
+      <c r="S196" t="n">
+        <v>24774.3</v>
+      </c>
+      <c r="T196" t="n">
+        <v>24515.5</v>
+      </c>
+      <c r="U196" t="n">
+        <v>24731.2</v>
+      </c>
+      <c r="V196" t="n">
+        <v>24644.9</v>
+      </c>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X196" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y196" t="n">
+        <v>24537</v>
+      </c>
+      <c r="Z196" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB196" t="n">
+        <v>24556.4</v>
+      </c>
+      <c r="AC196" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD196" t="n">
+        <v>24396.4</v>
+      </c>
+      <c r="AE196" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF196" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>57465.2</v>
+      </c>
+      <c r="H197" t="n">
+        <v>75</v>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K197" t="n">
+        <v>5</v>
+      </c>
+      <c r="L197" t="n">
+        <v>57533.9</v>
+      </c>
+      <c r="M197" t="n">
+        <v>57586.5</v>
+      </c>
+      <c r="N197" t="n">
+        <v>57484</v>
+      </c>
+      <c r="O197" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q197" t="n">
+        <v>58038.6</v>
+      </c>
+      <c r="R197" t="n">
+        <v>57655.6</v>
+      </c>
+      <c r="S197" t="n">
+        <v>58247.9</v>
+      </c>
+      <c r="T197" t="n">
+        <v>57470.4</v>
+      </c>
+      <c r="U197" t="n">
+        <v>58118.4</v>
+      </c>
+      <c r="V197" t="n">
+        <v>57859.2</v>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y197" t="n">
+        <v>57600.6</v>
+      </c>
+      <c r="Z197" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB197" t="n">
+        <v>57585.2</v>
+      </c>
+      <c r="AC197" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD197" t="n">
+        <v>57105.2</v>
+      </c>
+      <c r="AE197" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF197" t="n">
+        <v>12.31</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>78500</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>78469.10000000001</v>
+      </c>
+      <c r="H198" t="n">
+        <v>98</v>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K198" t="n">
+        <v>8</v>
+      </c>
+      <c r="L198" t="n">
+        <v>78497.89999999999</v>
+      </c>
+      <c r="M198" t="n">
+        <v>78564.5</v>
+      </c>
+      <c r="N198" t="n">
+        <v>78469.60000000001</v>
+      </c>
+      <c r="O198" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q198" t="n">
+        <v>79133</v>
+      </c>
+      <c r="R198" t="n">
+        <v>78730.39999999999</v>
+      </c>
+      <c r="S198" t="n">
+        <v>78809.8</v>
+      </c>
+      <c r="T198" t="n">
+        <v>78505.60000000001</v>
+      </c>
+      <c r="U198" t="n">
+        <v>78657.7</v>
+      </c>
+      <c r="V198" t="n">
+        <v>78645.3</v>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y198" t="n">
+        <v>78574.10000000001</v>
+      </c>
+      <c r="Z198" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB198" t="n">
+        <v>78669.10000000001</v>
+      </c>
+      <c r="AC198" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD198" t="n">
+        <v>77869.10000000001</v>
+      </c>
+      <c r="AE198" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF198" t="n">
+        <v>12.31</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>24502.1</v>
+      </c>
+      <c r="H199" t="n">
+        <v>88</v>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K199" t="n">
+        <v>7</v>
+      </c>
+      <c r="L199" t="n">
+        <v>24509.5</v>
+      </c>
+      <c r="M199" t="n">
+        <v>24530.1</v>
+      </c>
+      <c r="N199" t="n">
+        <v>24504.1</v>
+      </c>
+      <c r="O199" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q199" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="R199" t="n">
+        <v>24591.3</v>
+      </c>
+      <c r="S199" t="n">
+        <v>24774.3</v>
+      </c>
+      <c r="T199" t="n">
+        <v>24515.5</v>
+      </c>
+      <c r="U199" t="n">
+        <v>24731.2</v>
+      </c>
+      <c r="V199" t="n">
+        <v>24644.9</v>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y199" t="n">
+        <v>24530.3</v>
+      </c>
+      <c r="Z199" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB199" t="n">
+        <v>24542.1</v>
+      </c>
+      <c r="AC199" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD199" t="n">
+        <v>24382.1</v>
+      </c>
+      <c r="AE199" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF199" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="AG199" t="inlineStr"/>
+      <c r="AH199" t="inlineStr"/>
+      <c r="AI199" t="inlineStr"/>
+      <c r="AJ199" t="inlineStr"/>
+      <c r="AK199" t="inlineStr"/>
+      <c r="AL199" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-05
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL199"/>
+  <dimension ref="A1:AL207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24428,12 +24428,972 @@
       <c r="AF199" t="n">
         <v>12.31</v>
       </c>
-      <c r="AG199" t="inlineStr"/>
-      <c r="AH199" t="inlineStr"/>
-      <c r="AI199" t="inlineStr"/>
-      <c r="AJ199" t="inlineStr"/>
-      <c r="AK199" t="inlineStr"/>
-      <c r="AL199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>24550</v>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G200" t="n">
+        <v>24547.2</v>
+      </c>
+      <c r="H200" t="n">
+        <v>78</v>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K200" t="n">
+        <v>6</v>
+      </c>
+      <c r="L200" t="n">
+        <v>24570.5</v>
+      </c>
+      <c r="M200" t="n">
+        <v>24585.5</v>
+      </c>
+      <c r="N200" t="n">
+        <v>24553.3</v>
+      </c>
+      <c r="O200" t="n">
+        <v>28</v>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q200" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="R200" t="n">
+        <v>24611.4</v>
+      </c>
+      <c r="S200" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="T200" t="n">
+        <v>24428.2</v>
+      </c>
+      <c r="U200" t="n">
+        <v>24592.4</v>
+      </c>
+      <c r="V200" t="n">
+        <v>24547.4</v>
+      </c>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X200" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y200" t="n">
+        <v>24573.9</v>
+      </c>
+      <c r="Z200" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB200" t="n">
+        <v>24587.2</v>
+      </c>
+      <c r="AC200" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD200" t="n">
+        <v>24427.2</v>
+      </c>
+      <c r="AE200" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF200" t="n">
+        <v>12.28</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>24521.3</v>
+      </c>
+      <c r="H201" t="n">
+        <v>78</v>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K201" t="n">
+        <v>6</v>
+      </c>
+      <c r="L201" t="n">
+        <v>24534.1</v>
+      </c>
+      <c r="M201" t="n">
+        <v>24554.3</v>
+      </c>
+      <c r="N201" t="n">
+        <v>24527.6</v>
+      </c>
+      <c r="O201" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q201" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="R201" t="n">
+        <v>24611.4</v>
+      </c>
+      <c r="S201" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="T201" t="n">
+        <v>24428.2</v>
+      </c>
+      <c r="U201" t="n">
+        <v>24592.4</v>
+      </c>
+      <c r="V201" t="n">
+        <v>24547.4</v>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y201" t="n">
+        <v>24546.4</v>
+      </c>
+      <c r="Z201" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="AA201" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB201" t="n">
+        <v>24561.3</v>
+      </c>
+      <c r="AC201" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD201" t="n">
+        <v>24401.3</v>
+      </c>
+      <c r="AE201" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF201" t="n">
+        <v>12.52</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G202" t="n">
+        <v>24507.9</v>
+      </c>
+      <c r="H202" t="n">
+        <v>75</v>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>5</v>
+      </c>
+      <c r="L202" t="n">
+        <v>24525.3</v>
+      </c>
+      <c r="M202" t="n">
+        <v>24541.5</v>
+      </c>
+      <c r="N202" t="n">
+        <v>24512.4</v>
+      </c>
+      <c r="O202" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q202" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="R202" t="n">
+        <v>24611.4</v>
+      </c>
+      <c r="S202" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="T202" t="n">
+        <v>24428.2</v>
+      </c>
+      <c r="U202" t="n">
+        <v>24592.4</v>
+      </c>
+      <c r="V202" t="n">
+        <v>24547.4</v>
+      </c>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y202" t="n">
+        <v>24546</v>
+      </c>
+      <c r="Z202" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="AA202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB202" t="n">
+        <v>24547.9</v>
+      </c>
+      <c r="AC202" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD202" t="n">
+        <v>24387.9</v>
+      </c>
+      <c r="AE202" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF202" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G203" t="n">
+        <v>24511.9</v>
+      </c>
+      <c r="H203" t="n">
+        <v>88</v>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K203" t="n">
+        <v>7</v>
+      </c>
+      <c r="L203" t="n">
+        <v>24522.4</v>
+      </c>
+      <c r="M203" t="n">
+        <v>24537.3</v>
+      </c>
+      <c r="N203" t="n">
+        <v>24517.4</v>
+      </c>
+      <c r="O203" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q203" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="R203" t="n">
+        <v>24611.4</v>
+      </c>
+      <c r="S203" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="T203" t="n">
+        <v>24428.2</v>
+      </c>
+      <c r="U203" t="n">
+        <v>24592.4</v>
+      </c>
+      <c r="V203" t="n">
+        <v>24547.4</v>
+      </c>
+      <c r="W203" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X203" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y203" t="n">
+        <v>24538.9</v>
+      </c>
+      <c r="Z203" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AA203" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB203" t="n">
+        <v>24551.9</v>
+      </c>
+      <c r="AC203" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD203" t="n">
+        <v>24391.9</v>
+      </c>
+      <c r="AE203" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF203" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>57517.9</v>
+      </c>
+      <c r="H204" t="n">
+        <v>78</v>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K204" t="n">
+        <v>6</v>
+      </c>
+      <c r="L204" t="n">
+        <v>57534.5</v>
+      </c>
+      <c r="M204" t="n">
+        <v>57575.5</v>
+      </c>
+      <c r="N204" t="n">
+        <v>57538.6</v>
+      </c>
+      <c r="O204" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q204" t="n">
+        <v>57925.8</v>
+      </c>
+      <c r="R204" t="n">
+        <v>57654.7</v>
+      </c>
+      <c r="S204" t="n">
+        <v>58038.6</v>
+      </c>
+      <c r="T204" t="n">
+        <v>57352.6</v>
+      </c>
+      <c r="U204" t="n">
+        <v>57836.7</v>
+      </c>
+      <c r="V204" t="n">
+        <v>57695.6</v>
+      </c>
+      <c r="W204" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X204" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y204" t="n">
+        <v>57567.7</v>
+      </c>
+      <c r="Z204" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="AA204" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB204" t="n">
+        <v>57637.9</v>
+      </c>
+      <c r="AC204" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD204" t="n">
+        <v>57157.9</v>
+      </c>
+      <c r="AE204" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF204" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>24506.7</v>
+      </c>
+      <c r="H205" t="n">
+        <v>88</v>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K205" t="n">
+        <v>7</v>
+      </c>
+      <c r="L205" t="n">
+        <v>24515.8</v>
+      </c>
+      <c r="M205" t="n">
+        <v>24527.6</v>
+      </c>
+      <c r="N205" t="n">
+        <v>24509.5</v>
+      </c>
+      <c r="O205" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q205" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="R205" t="n">
+        <v>24611.4</v>
+      </c>
+      <c r="S205" t="n">
+        <v>24666.7</v>
+      </c>
+      <c r="T205" t="n">
+        <v>24428.2</v>
+      </c>
+      <c r="U205" t="n">
+        <v>24592.4</v>
+      </c>
+      <c r="V205" t="n">
+        <v>24547.4</v>
+      </c>
+      <c r="W205" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X205" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y205" t="n">
+        <v>24538.6</v>
+      </c>
+      <c r="Z205" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AA205" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB205" t="n">
+        <v>24546.7</v>
+      </c>
+      <c r="AC205" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD205" t="n">
+        <v>24386.7</v>
+      </c>
+      <c r="AE205" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF205" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>57531.9</v>
+      </c>
+      <c r="H206" t="n">
+        <v>78</v>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K206" t="n">
+        <v>6</v>
+      </c>
+      <c r="L206" t="n">
+        <v>57544.3</v>
+      </c>
+      <c r="M206" t="n">
+        <v>57564.5</v>
+      </c>
+      <c r="N206" t="n">
+        <v>57538.7</v>
+      </c>
+      <c r="O206" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q206" t="n">
+        <v>57925.8</v>
+      </c>
+      <c r="R206" t="n">
+        <v>57654.7</v>
+      </c>
+      <c r="S206" t="n">
+        <v>58038.6</v>
+      </c>
+      <c r="T206" t="n">
+        <v>57352.6</v>
+      </c>
+      <c r="U206" t="n">
+        <v>57836.7</v>
+      </c>
+      <c r="V206" t="n">
+        <v>57695.6</v>
+      </c>
+      <c r="W206" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y206" t="n">
+        <v>57567.7</v>
+      </c>
+      <c r="Z206" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="AA206" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB206" t="n">
+        <v>57651.9</v>
+      </c>
+      <c r="AC206" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD206" t="n">
+        <v>57171.9</v>
+      </c>
+      <c r="AE206" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF206" t="n">
+        <v>12.54</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>78400</v>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G207" t="n">
+        <v>78392.8</v>
+      </c>
+      <c r="H207" t="n">
+        <v>78</v>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K207" t="n">
+        <v>6</v>
+      </c>
+      <c r="L207" t="n">
+        <v>78388.39999999999</v>
+      </c>
+      <c r="M207" t="n">
+        <v>78435.89999999999</v>
+      </c>
+      <c r="N207" t="n">
+        <v>78394.60000000001</v>
+      </c>
+      <c r="O207" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q207" t="n">
+        <v>79000.7</v>
+      </c>
+      <c r="R207" t="n">
+        <v>78791.7</v>
+      </c>
+      <c r="S207" t="n">
+        <v>79133</v>
+      </c>
+      <c r="T207" t="n">
+        <v>78212.60000000001</v>
+      </c>
+      <c r="U207" t="n">
+        <v>78672.8</v>
+      </c>
+      <c r="V207" t="n">
+        <v>78510.2</v>
+      </c>
+      <c r="W207" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X207" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y207" t="n">
+        <v>78475.3</v>
+      </c>
+      <c r="Z207" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AA207" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB207" t="n">
+        <v>78592.8</v>
+      </c>
+      <c r="AC207" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD207" t="n">
+        <v>77792.8</v>
+      </c>
+      <c r="AE207" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF207" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="AG207" t="inlineStr"/>
+      <c r="AH207" t="inlineStr"/>
+      <c r="AI207" t="inlineStr"/>
+      <c r="AJ207" t="inlineStr"/>
+      <c r="AK207" t="inlineStr"/>
+      <c r="AL207" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-06
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL207"/>
+  <dimension ref="A1:AL214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25388,12 +25388,852 @@
       <c r="AF207" t="n">
         <v>12.54</v>
       </c>
-      <c r="AG207" t="inlineStr"/>
-      <c r="AH207" t="inlineStr"/>
-      <c r="AI207" t="inlineStr"/>
-      <c r="AJ207" t="inlineStr"/>
-      <c r="AK207" t="inlineStr"/>
-      <c r="AL207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>24650</v>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>24648.8</v>
+      </c>
+      <c r="H208" t="n">
+        <v>76</v>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K208" t="n">
+        <v>6</v>
+      </c>
+      <c r="L208" t="n">
+        <v>24650.2</v>
+      </c>
+      <c r="M208" t="n">
+        <v>24646.6</v>
+      </c>
+      <c r="N208" t="n">
+        <v>24648.8</v>
+      </c>
+      <c r="O208" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q208" t="n">
+        <v>24646.9</v>
+      </c>
+      <c r="R208" t="n">
+        <v>24607.8</v>
+      </c>
+      <c r="S208" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="T208" t="n">
+        <v>24498.2</v>
+      </c>
+      <c r="U208" t="n">
+        <v>24611</v>
+      </c>
+      <c r="V208" t="n">
+        <v>24583.7</v>
+      </c>
+      <c r="W208" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X208" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y208" t="n">
+        <v>24650.4</v>
+      </c>
+      <c r="Z208" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AA208" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB208" t="n">
+        <v>24608.8</v>
+      </c>
+      <c r="AC208" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD208" t="n">
+        <v>24768.8</v>
+      </c>
+      <c r="AE208" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF208" t="n">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>78800</v>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>78804.5</v>
+      </c>
+      <c r="H209" t="n">
+        <v>76</v>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>6</v>
+      </c>
+      <c r="L209" t="n">
+        <v>78792.5</v>
+      </c>
+      <c r="M209" t="n">
+        <v>78776.39999999999</v>
+      </c>
+      <c r="N209" t="n">
+        <v>78804.5</v>
+      </c>
+      <c r="O209" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q209" t="n">
+        <v>78786.89999999999</v>
+      </c>
+      <c r="R209" t="n">
+        <v>78647.60000000001</v>
+      </c>
+      <c r="S209" t="n">
+        <v>79000.7</v>
+      </c>
+      <c r="T209" t="n">
+        <v>78286.5</v>
+      </c>
+      <c r="U209" t="n">
+        <v>78643.60000000001</v>
+      </c>
+      <c r="V209" t="n">
+        <v>78601.89999999999</v>
+      </c>
+      <c r="W209" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X209" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y209" t="n">
+        <v>78806</v>
+      </c>
+      <c r="Z209" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA209" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB209" t="n">
+        <v>78604.5</v>
+      </c>
+      <c r="AC209" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD209" t="n">
+        <v>79404.5</v>
+      </c>
+      <c r="AE209" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF209" t="n">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>57957.1</v>
+      </c>
+      <c r="H210" t="n">
+        <v>88</v>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K210" t="n">
+        <v>7</v>
+      </c>
+      <c r="L210" t="n">
+        <v>57940.5</v>
+      </c>
+      <c r="M210" t="n">
+        <v>57913.9</v>
+      </c>
+      <c r="N210" t="n">
+        <v>57956</v>
+      </c>
+      <c r="O210" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q210" t="n">
+        <v>57858.1</v>
+      </c>
+      <c r="R210" t="n">
+        <v>57716.9</v>
+      </c>
+      <c r="S210" t="n">
+        <v>57929.7</v>
+      </c>
+      <c r="T210" t="n">
+        <v>57457.1</v>
+      </c>
+      <c r="U210" t="n">
+        <v>57724.4</v>
+      </c>
+      <c r="V210" t="n">
+        <v>57693.4</v>
+      </c>
+      <c r="W210" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X210" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y210" t="n">
+        <v>57921.8</v>
+      </c>
+      <c r="Z210" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="AA210" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB210" t="n">
+        <v>57837.1</v>
+      </c>
+      <c r="AC210" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD210" t="n">
+        <v>58317.1</v>
+      </c>
+      <c r="AE210" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF210" t="n">
+        <v>12.24</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>78800</v>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>78805.10000000001</v>
+      </c>
+      <c r="H211" t="n">
+        <v>91</v>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K211" t="n">
+        <v>7</v>
+      </c>
+      <c r="L211" t="n">
+        <v>78811.3</v>
+      </c>
+      <c r="M211" t="n">
+        <v>78793</v>
+      </c>
+      <c r="N211" t="n">
+        <v>78805</v>
+      </c>
+      <c r="O211" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q211" t="n">
+        <v>78786.89999999999</v>
+      </c>
+      <c r="R211" t="n">
+        <v>78647.60000000001</v>
+      </c>
+      <c r="S211" t="n">
+        <v>79000.7</v>
+      </c>
+      <c r="T211" t="n">
+        <v>78286.5</v>
+      </c>
+      <c r="U211" t="n">
+        <v>78643.60000000001</v>
+      </c>
+      <c r="V211" t="n">
+        <v>78601.89999999999</v>
+      </c>
+      <c r="W211" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X211" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y211" t="n">
+        <v>78806</v>
+      </c>
+      <c r="Z211" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AA211" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB211" t="n">
+        <v>78605.10000000001</v>
+      </c>
+      <c r="AC211" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD211" t="n">
+        <v>79405.10000000001</v>
+      </c>
+      <c r="AE211" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF211" t="n">
+        <v>12.24</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>24650</v>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>24647.4</v>
+      </c>
+      <c r="H212" t="n">
+        <v>91</v>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K212" t="n">
+        <v>7</v>
+      </c>
+      <c r="L212" t="n">
+        <v>24645</v>
+      </c>
+      <c r="M212" t="n">
+        <v>24644.8</v>
+      </c>
+      <c r="N212" t="n">
+        <v>24647.1</v>
+      </c>
+      <c r="O212" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q212" t="n">
+        <v>24646.9</v>
+      </c>
+      <c r="R212" t="n">
+        <v>24607.8</v>
+      </c>
+      <c r="S212" t="n">
+        <v>24669.2</v>
+      </c>
+      <c r="T212" t="n">
+        <v>24498.2</v>
+      </c>
+      <c r="U212" t="n">
+        <v>24611</v>
+      </c>
+      <c r="V212" t="n">
+        <v>24583.7</v>
+      </c>
+      <c r="W212" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X212" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y212" t="n">
+        <v>24650.4</v>
+      </c>
+      <c r="Z212" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA212" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB212" t="n">
+        <v>24607.4</v>
+      </c>
+      <c r="AC212" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD212" t="n">
+        <v>24767.4</v>
+      </c>
+      <c r="AE212" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF212" t="n">
+        <v>12.24</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>57900</v>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>57938.1</v>
+      </c>
+      <c r="H213" t="n">
+        <v>83</v>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K213" t="n">
+        <v>7</v>
+      </c>
+      <c r="L213" t="n">
+        <v>57932.6</v>
+      </c>
+      <c r="M213" t="n">
+        <v>57921</v>
+      </c>
+      <c r="N213" t="n">
+        <v>57940</v>
+      </c>
+      <c r="O213" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q213" t="n">
+        <v>57858.1</v>
+      </c>
+      <c r="R213" t="n">
+        <v>57716.9</v>
+      </c>
+      <c r="S213" t="n">
+        <v>57929.7</v>
+      </c>
+      <c r="T213" t="n">
+        <v>57457.1</v>
+      </c>
+      <c r="U213" t="n">
+        <v>57724.4</v>
+      </c>
+      <c r="V213" t="n">
+        <v>57693.4</v>
+      </c>
+      <c r="W213" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X213" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y213" t="n">
+        <v>57921.8</v>
+      </c>
+      <c r="Z213" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AA213" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB213" t="n">
+        <v>57818.1</v>
+      </c>
+      <c r="AC213" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD213" t="n">
+        <v>58298.1</v>
+      </c>
+      <c r="AE213" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF213" t="n">
+        <v>12.24</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>78800</v>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>78822.39999999999</v>
+      </c>
+      <c r="H214" t="n">
+        <v>91</v>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K214" t="n">
+        <v>7</v>
+      </c>
+      <c r="L214" t="n">
+        <v>78811.60000000001</v>
+      </c>
+      <c r="M214" t="n">
+        <v>78800.3</v>
+      </c>
+      <c r="N214" t="n">
+        <v>78820.5</v>
+      </c>
+      <c r="O214" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q214" t="n">
+        <v>78786.89999999999</v>
+      </c>
+      <c r="R214" t="n">
+        <v>78647.60000000001</v>
+      </c>
+      <c r="S214" t="n">
+        <v>79000.7</v>
+      </c>
+      <c r="T214" t="n">
+        <v>78286.5</v>
+      </c>
+      <c r="U214" t="n">
+        <v>78643.60000000001</v>
+      </c>
+      <c r="V214" t="n">
+        <v>78601.89999999999</v>
+      </c>
+      <c r="W214" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X214" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y214" t="n">
+        <v>78806</v>
+      </c>
+      <c r="Z214" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AA214" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB214" t="n">
+        <v>78622.39999999999</v>
+      </c>
+      <c r="AC214" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD214" t="n">
+        <v>79422.39999999999</v>
+      </c>
+      <c r="AE214" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF214" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="AG214" t="inlineStr"/>
+      <c r="AH214" t="inlineStr"/>
+      <c r="AI214" t="inlineStr"/>
+      <c r="AJ214" t="inlineStr"/>
+      <c r="AK214" t="inlineStr"/>
+      <c r="AL214" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-07
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL214"/>
+  <dimension ref="A1:AL217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26228,12 +26228,372 @@
       <c r="AF214" t="n">
         <v>12.24</v>
       </c>
-      <c r="AG214" t="inlineStr"/>
-      <c r="AH214" t="inlineStr"/>
-      <c r="AI214" t="inlineStr"/>
-      <c r="AJ214" t="inlineStr"/>
-      <c r="AK214" t="inlineStr"/>
-      <c r="AL214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>24550</v>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G215" t="n">
+        <v>24526.3</v>
+      </c>
+      <c r="H215" t="n">
+        <v>83</v>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K215" t="n">
+        <v>7</v>
+      </c>
+      <c r="L215" t="n">
+        <v>24544.8</v>
+      </c>
+      <c r="M215" t="n">
+        <v>24551.9</v>
+      </c>
+      <c r="N215" t="n">
+        <v>24526.3</v>
+      </c>
+      <c r="O215" t="n">
+        <v>38</v>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q215" t="n">
+        <v>24620</v>
+      </c>
+      <c r="R215" t="n">
+        <v>24535.1</v>
+      </c>
+      <c r="S215" t="n">
+        <v>24676.8</v>
+      </c>
+      <c r="T215" t="n">
+        <v>24605.9</v>
+      </c>
+      <c r="U215" t="n">
+        <v>24641.4</v>
+      </c>
+      <c r="V215" t="n">
+        <v>24637.8</v>
+      </c>
+      <c r="W215" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X215" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y215" t="n">
+        <v>24545.8</v>
+      </c>
+      <c r="Z215" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="AA215" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB215" t="n">
+        <v>24566.3</v>
+      </c>
+      <c r="AC215" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD215" t="n">
+        <v>24406.3</v>
+      </c>
+      <c r="AE215" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF215" t="n">
+        <v>12.39</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G216" t="n">
+        <v>57746.4</v>
+      </c>
+      <c r="H216" t="n">
+        <v>88</v>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K216" t="n">
+        <v>7</v>
+      </c>
+      <c r="L216" t="n">
+        <v>57787.4</v>
+      </c>
+      <c r="M216" t="n">
+        <v>57797</v>
+      </c>
+      <c r="N216" t="n">
+        <v>57764.7</v>
+      </c>
+      <c r="O216" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q216" t="n">
+        <v>57936.4</v>
+      </c>
+      <c r="R216" t="n">
+        <v>57795.1</v>
+      </c>
+      <c r="S216" t="n">
+        <v>58076.6</v>
+      </c>
+      <c r="T216" t="n">
+        <v>57716.9</v>
+      </c>
+      <c r="U216" t="n">
+        <v>58008</v>
+      </c>
+      <c r="V216" t="n">
+        <v>57896.8</v>
+      </c>
+      <c r="W216" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X216" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y216" t="n">
+        <v>57746.9</v>
+      </c>
+      <c r="Z216" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AA216" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB216" t="n">
+        <v>57866.4</v>
+      </c>
+      <c r="AC216" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD216" t="n">
+        <v>57386.4</v>
+      </c>
+      <c r="AE216" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF216" t="n">
+        <v>12.15</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>78500</v>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G217" t="n">
+        <v>78491.89999999999</v>
+      </c>
+      <c r="H217" t="n">
+        <v>86</v>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K217" t="n">
+        <v>7</v>
+      </c>
+      <c r="L217" t="n">
+        <v>78457.10000000001</v>
+      </c>
+      <c r="M217" t="n">
+        <v>78467.60000000001</v>
+      </c>
+      <c r="N217" t="n">
+        <v>78492.10000000001</v>
+      </c>
+      <c r="O217" t="n">
+        <v>53</v>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q217" t="n">
+        <v>78757.39999999999</v>
+      </c>
+      <c r="R217" t="n">
+        <v>78487.7</v>
+      </c>
+      <c r="S217" t="n">
+        <v>79486.60000000001</v>
+      </c>
+      <c r="T217" t="n">
+        <v>78597.3</v>
+      </c>
+      <c r="U217" t="n">
+        <v>79042</v>
+      </c>
+      <c r="V217" t="n">
+        <v>78983.8</v>
+      </c>
+      <c r="W217" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X217" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y217" t="n">
+        <v>78467.2</v>
+      </c>
+      <c r="Z217" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="AA217" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB217" t="n">
+        <v>78691.89999999999</v>
+      </c>
+      <c r="AC217" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD217" t="n">
+        <v>77891.89999999999</v>
+      </c>
+      <c r="AE217" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF217" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="AG217" t="inlineStr"/>
+      <c r="AH217" t="inlineStr"/>
+      <c r="AI217" t="inlineStr"/>
+      <c r="AJ217" t="inlineStr"/>
+      <c r="AK217" t="inlineStr"/>
+      <c r="AL217" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-10
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL217"/>
+  <dimension ref="A1:AL223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26588,12 +26588,732 @@
       <c r="AF217" t="n">
         <v>12.15</v>
       </c>
-      <c r="AG217" t="inlineStr"/>
-      <c r="AH217" t="inlineStr"/>
-      <c r="AI217" t="inlineStr"/>
-      <c r="AJ217" t="inlineStr"/>
-      <c r="AK217" t="inlineStr"/>
-      <c r="AL217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>78700</v>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G218" t="n">
+        <v>78650.3</v>
+      </c>
+      <c r="H218" t="n">
+        <v>76</v>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K218" t="n">
+        <v>6</v>
+      </c>
+      <c r="L218" t="n">
+        <v>78566.89999999999</v>
+      </c>
+      <c r="M218" t="n">
+        <v>78537.60000000001</v>
+      </c>
+      <c r="N218" t="n">
+        <v>78638.5</v>
+      </c>
+      <c r="O218" t="n">
+        <v>44</v>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q218" t="n">
+        <v>78672.10000000001</v>
+      </c>
+      <c r="R218" t="n">
+        <v>78439.39999999999</v>
+      </c>
+      <c r="S218" t="n">
+        <v>78757.39999999999</v>
+      </c>
+      <c r="T218" t="n">
+        <v>78377.60000000001</v>
+      </c>
+      <c r="U218" t="n">
+        <v>78567.5</v>
+      </c>
+      <c r="V218" t="n">
+        <v>78521.89999999999</v>
+      </c>
+      <c r="W218" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X218" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y218" t="n">
+        <v>78617.2</v>
+      </c>
+      <c r="Z218" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AA218" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB218" t="n">
+        <v>78450.3</v>
+      </c>
+      <c r="AC218" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD218" t="n">
+        <v>79250.3</v>
+      </c>
+      <c r="AE218" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF218" t="n">
+        <v>12.62</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>12:17</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>24600</v>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G219" t="n">
+        <v>24617.4</v>
+      </c>
+      <c r="H219" t="n">
+        <v>76</v>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K219" t="n">
+        <v>6</v>
+      </c>
+      <c r="L219" t="n">
+        <v>24599.3</v>
+      </c>
+      <c r="M219" t="n">
+        <v>24593.3</v>
+      </c>
+      <c r="N219" t="n">
+        <v>24613.4</v>
+      </c>
+      <c r="O219" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q219" t="n">
+        <v>24620.6</v>
+      </c>
+      <c r="R219" t="n">
+        <v>24555.2</v>
+      </c>
+      <c r="S219" t="n">
+        <v>24629.8</v>
+      </c>
+      <c r="T219" t="n">
+        <v>24522.9</v>
+      </c>
+      <c r="U219" t="n">
+        <v>24576.4</v>
+      </c>
+      <c r="V219" t="n">
+        <v>24572.6</v>
+      </c>
+      <c r="W219" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X219" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y219" t="n">
+        <v>24605.1</v>
+      </c>
+      <c r="Z219" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AA219" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB219" t="n">
+        <v>24577.4</v>
+      </c>
+      <c r="AC219" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD219" t="n">
+        <v>24737.4</v>
+      </c>
+      <c r="AE219" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF219" t="n">
+        <v>12.62</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>78700</v>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G220" t="n">
+        <v>78663.8</v>
+      </c>
+      <c r="H220" t="n">
+        <v>76</v>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K220" t="n">
+        <v>6</v>
+      </c>
+      <c r="L220" t="n">
+        <v>78601</v>
+      </c>
+      <c r="M220" t="n">
+        <v>78584</v>
+      </c>
+      <c r="N220" t="n">
+        <v>78647.89999999999</v>
+      </c>
+      <c r="O220" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q220" t="n">
+        <v>78672.10000000001</v>
+      </c>
+      <c r="R220" t="n">
+        <v>78439.39999999999</v>
+      </c>
+      <c r="S220" t="n">
+        <v>78757.39999999999</v>
+      </c>
+      <c r="T220" t="n">
+        <v>78377.60000000001</v>
+      </c>
+      <c r="U220" t="n">
+        <v>78567.5</v>
+      </c>
+      <c r="V220" t="n">
+        <v>78521.89999999999</v>
+      </c>
+      <c r="W220" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X220" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y220" t="n">
+        <v>78617.2</v>
+      </c>
+      <c r="Z220" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AA220" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB220" t="n">
+        <v>78463.8</v>
+      </c>
+      <c r="AC220" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD220" t="n">
+        <v>79263.8</v>
+      </c>
+      <c r="AE220" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF220" t="n">
+        <v>12.62</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G221" t="n">
+        <v>57640.6</v>
+      </c>
+      <c r="H221" t="n">
+        <v>83</v>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K221" t="n">
+        <v>7</v>
+      </c>
+      <c r="L221" t="n">
+        <v>57663.5</v>
+      </c>
+      <c r="M221" t="n">
+        <v>57670.9</v>
+      </c>
+      <c r="N221" t="n">
+        <v>57643.1</v>
+      </c>
+      <c r="O221" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q221" t="n">
+        <v>58012.6</v>
+      </c>
+      <c r="R221" t="n">
+        <v>57714.4</v>
+      </c>
+      <c r="S221" t="n">
+        <v>57993.8</v>
+      </c>
+      <c r="T221" t="n">
+        <v>57688.3</v>
+      </c>
+      <c r="U221" t="n">
+        <v>57841</v>
+      </c>
+      <c r="V221" t="n">
+        <v>57778</v>
+      </c>
+      <c r="W221" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X221" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y221" t="n">
+        <v>57642.2</v>
+      </c>
+      <c r="Z221" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AA221" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB221" t="n">
+        <v>57760.6</v>
+      </c>
+      <c r="AC221" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD221" t="n">
+        <v>57280.6</v>
+      </c>
+      <c r="AE221" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF221" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G222" t="n">
+        <v>57601.8</v>
+      </c>
+      <c r="H222" t="n">
+        <v>83</v>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K222" t="n">
+        <v>7</v>
+      </c>
+      <c r="L222" t="n">
+        <v>57618</v>
+      </c>
+      <c r="M222" t="n">
+        <v>57641.3</v>
+      </c>
+      <c r="N222" t="n">
+        <v>57605</v>
+      </c>
+      <c r="O222" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q222" t="n">
+        <v>58012.6</v>
+      </c>
+      <c r="R222" t="n">
+        <v>57714.4</v>
+      </c>
+      <c r="S222" t="n">
+        <v>57993.8</v>
+      </c>
+      <c r="T222" t="n">
+        <v>57688.3</v>
+      </c>
+      <c r="U222" t="n">
+        <v>57841</v>
+      </c>
+      <c r="V222" t="n">
+        <v>57778</v>
+      </c>
+      <c r="W222" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X222" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y222" t="n">
+        <v>57642.2</v>
+      </c>
+      <c r="Z222" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="AA222" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB222" t="n">
+        <v>57721.8</v>
+      </c>
+      <c r="AC222" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD222" t="n">
+        <v>57241.8</v>
+      </c>
+      <c r="AE222" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF222" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G223" t="n">
+        <v>57612.8</v>
+      </c>
+      <c r="H223" t="n">
+        <v>83</v>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K223" t="n">
+        <v>7</v>
+      </c>
+      <c r="L223" t="n">
+        <v>57623</v>
+      </c>
+      <c r="M223" t="n">
+        <v>57632.9</v>
+      </c>
+      <c r="N223" t="n">
+        <v>57617.3</v>
+      </c>
+      <c r="O223" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q223" t="n">
+        <v>58012.6</v>
+      </c>
+      <c r="R223" t="n">
+        <v>57714.4</v>
+      </c>
+      <c r="S223" t="n">
+        <v>57993.8</v>
+      </c>
+      <c r="T223" t="n">
+        <v>57688.3</v>
+      </c>
+      <c r="U223" t="n">
+        <v>57841</v>
+      </c>
+      <c r="V223" t="n">
+        <v>57778</v>
+      </c>
+      <c r="W223" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y223" t="n">
+        <v>57642.2</v>
+      </c>
+      <c r="Z223" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="AA223" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB223" t="n">
+        <v>57732.8</v>
+      </c>
+      <c r="AC223" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD223" t="n">
+        <v>57252.8</v>
+      </c>
+      <c r="AE223" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF223" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="AG223" t="inlineStr"/>
+      <c r="AH223" t="inlineStr"/>
+      <c r="AI223" t="inlineStr"/>
+      <c r="AJ223" t="inlineStr"/>
+      <c r="AK223" t="inlineStr"/>
+      <c r="AL223" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-11
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL223"/>
+  <dimension ref="A1:AL229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27308,12 +27308,732 @@
       <c r="AF223" t="n">
         <v>12.45</v>
       </c>
-      <c r="AG223" t="inlineStr"/>
-      <c r="AH223" t="inlineStr"/>
-      <c r="AI223" t="inlineStr"/>
-      <c r="AJ223" t="inlineStr"/>
-      <c r="AK223" t="inlineStr"/>
-      <c r="AL223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>57200</v>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G224" t="n">
+        <v>57242.6</v>
+      </c>
+      <c r="H224" t="n">
+        <v>83</v>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K224" t="n">
+        <v>7</v>
+      </c>
+      <c r="L224" t="n">
+        <v>57245.2</v>
+      </c>
+      <c r="M224" t="n">
+        <v>57254.9</v>
+      </c>
+      <c r="N224" t="n">
+        <v>57253</v>
+      </c>
+      <c r="O224" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q224" t="n">
+        <v>57605.4</v>
+      </c>
+      <c r="R224" t="n">
+        <v>57284.9</v>
+      </c>
+      <c r="S224" t="n">
+        <v>58012.6</v>
+      </c>
+      <c r="T224" t="n">
+        <v>57527.8</v>
+      </c>
+      <c r="U224" t="n">
+        <v>57770.2</v>
+      </c>
+      <c r="V224" t="n">
+        <v>57714.7</v>
+      </c>
+      <c r="W224" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y224" t="n">
+        <v>57264.1</v>
+      </c>
+      <c r="Z224" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AA224" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB224" t="n">
+        <v>57362.6</v>
+      </c>
+      <c r="AC224" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD224" t="n">
+        <v>56882.6</v>
+      </c>
+      <c r="AE224" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF224" t="n">
+        <v>12.18</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>78200</v>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G225" t="n">
+        <v>78173.10000000001</v>
+      </c>
+      <c r="H225" t="n">
+        <v>83</v>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K225" t="n">
+        <v>7</v>
+      </c>
+      <c r="L225" t="n">
+        <v>78175.10000000001</v>
+      </c>
+      <c r="M225" t="n">
+        <v>78185.5</v>
+      </c>
+      <c r="N225" t="n">
+        <v>78181.39999999999</v>
+      </c>
+      <c r="O225" t="n">
+        <v>41</v>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q225" t="n">
+        <v>78488.60000000001</v>
+      </c>
+      <c r="R225" t="n">
+        <v>78196.7</v>
+      </c>
+      <c r="S225" t="n">
+        <v>78672.10000000001</v>
+      </c>
+      <c r="T225" t="n">
+        <v>78305.89999999999</v>
+      </c>
+      <c r="U225" t="n">
+        <v>78524.60000000001</v>
+      </c>
+      <c r="V225" t="n">
+        <v>78489</v>
+      </c>
+      <c r="W225" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X225" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y225" t="n">
+        <v>78203.39999999999</v>
+      </c>
+      <c r="Z225" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="AA225" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB225" t="n">
+        <v>78373.10000000001</v>
+      </c>
+      <c r="AC225" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD225" t="n">
+        <v>77573.10000000001</v>
+      </c>
+      <c r="AE225" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF225" t="n">
+        <v>12.28</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>78100</v>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G226" t="n">
+        <v>78107.7</v>
+      </c>
+      <c r="H226" t="n">
+        <v>83</v>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K226" t="n">
+        <v>7</v>
+      </c>
+      <c r="L226" t="n">
+        <v>78114</v>
+      </c>
+      <c r="M226" t="n">
+        <v>78133.8</v>
+      </c>
+      <c r="N226" t="n">
+        <v>78115.8</v>
+      </c>
+      <c r="O226" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q226" t="n">
+        <v>78488.60000000001</v>
+      </c>
+      <c r="R226" t="n">
+        <v>78196.7</v>
+      </c>
+      <c r="S226" t="n">
+        <v>78672.10000000001</v>
+      </c>
+      <c r="T226" t="n">
+        <v>78305.89999999999</v>
+      </c>
+      <c r="U226" t="n">
+        <v>78524.60000000001</v>
+      </c>
+      <c r="V226" t="n">
+        <v>78489</v>
+      </c>
+      <c r="W226" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X226" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y226" t="n">
+        <v>78168.60000000001</v>
+      </c>
+      <c r="Z226" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="AA226" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB226" t="n">
+        <v>78307.7</v>
+      </c>
+      <c r="AC226" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD226" t="n">
+        <v>77507.7</v>
+      </c>
+      <c r="AE226" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF226" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>24450</v>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>24441.6</v>
+      </c>
+      <c r="H227" t="n">
+        <v>83</v>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K227" t="n">
+        <v>7</v>
+      </c>
+      <c r="L227" t="n">
+        <v>24441.1</v>
+      </c>
+      <c r="M227" t="n">
+        <v>24447.6</v>
+      </c>
+      <c r="N227" t="n">
+        <v>24442.5</v>
+      </c>
+      <c r="O227" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q227" t="n">
+        <v>24575.5</v>
+      </c>
+      <c r="R227" t="n">
+        <v>24487.4</v>
+      </c>
+      <c r="S227" t="n">
+        <v>24620.6</v>
+      </c>
+      <c r="T227" t="n">
+        <v>24511.3</v>
+      </c>
+      <c r="U227" t="n">
+        <v>24577.8</v>
+      </c>
+      <c r="V227" t="n">
+        <v>24565.9</v>
+      </c>
+      <c r="W227" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X227" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y227" t="n">
+        <v>24463.8</v>
+      </c>
+      <c r="Z227" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="AA227" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB227" t="n">
+        <v>24481.6</v>
+      </c>
+      <c r="AC227" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD227" t="n">
+        <v>24321.6</v>
+      </c>
+      <c r="AE227" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF227" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>78100</v>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>78091.10000000001</v>
+      </c>
+      <c r="H228" t="n">
+        <v>83</v>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>7</v>
+      </c>
+      <c r="L228" t="n">
+        <v>78093.39999999999</v>
+      </c>
+      <c r="M228" t="n">
+        <v>78107.2</v>
+      </c>
+      <c r="N228" t="n">
+        <v>78096.39999999999</v>
+      </c>
+      <c r="O228" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q228" t="n">
+        <v>78488.60000000001</v>
+      </c>
+      <c r="R228" t="n">
+        <v>78196.7</v>
+      </c>
+      <c r="S228" t="n">
+        <v>78672.10000000001</v>
+      </c>
+      <c r="T228" t="n">
+        <v>78305.89999999999</v>
+      </c>
+      <c r="U228" t="n">
+        <v>78524.60000000001</v>
+      </c>
+      <c r="V228" t="n">
+        <v>78489</v>
+      </c>
+      <c r="W228" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X228" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y228" t="n">
+        <v>78152.2</v>
+      </c>
+      <c r="Z228" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="AA228" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB228" t="n">
+        <v>78291.10000000001</v>
+      </c>
+      <c r="AC228" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD228" t="n">
+        <v>77491.10000000001</v>
+      </c>
+      <c r="AE228" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF228" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>57381.1</v>
+      </c>
+      <c r="H229" t="n">
+        <v>76</v>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K229" t="n">
+        <v>5</v>
+      </c>
+      <c r="L229" t="n">
+        <v>57375.5</v>
+      </c>
+      <c r="M229" t="n">
+        <v>57350.9</v>
+      </c>
+      <c r="N229" t="n">
+        <v>57380.5</v>
+      </c>
+      <c r="O229" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q229" t="n">
+        <v>57605.4</v>
+      </c>
+      <c r="R229" t="n">
+        <v>57284.9</v>
+      </c>
+      <c r="S229" t="n">
+        <v>58012.6</v>
+      </c>
+      <c r="T229" t="n">
+        <v>57527.8</v>
+      </c>
+      <c r="U229" t="n">
+        <v>57770.2</v>
+      </c>
+      <c r="V229" t="n">
+        <v>57714.7</v>
+      </c>
+      <c r="W229" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X229" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y229" t="n">
+        <v>57407.4</v>
+      </c>
+      <c r="Z229" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="AA229" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB229" t="n">
+        <v>57261.1</v>
+      </c>
+      <c r="AC229" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD229" t="n">
+        <v>57741.1</v>
+      </c>
+      <c r="AE229" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF229" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="AG229" t="inlineStr"/>
+      <c r="AH229" t="inlineStr"/>
+      <c r="AI229" t="inlineStr"/>
+      <c r="AJ229" t="inlineStr"/>
+      <c r="AK229" t="inlineStr"/>
+      <c r="AL229" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-12
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL229"/>
+  <dimension ref="A1:AL235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28028,12 +28028,732 @@
       <c r="AF229" t="n">
         <v>11.95</v>
       </c>
-      <c r="AG229" t="inlineStr"/>
-      <c r="AH229" t="inlineStr"/>
-      <c r="AI229" t="inlineStr"/>
-      <c r="AJ229" t="inlineStr"/>
-      <c r="AK229" t="inlineStr"/>
-      <c r="AL229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>11:12</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>24304.8</v>
+      </c>
+      <c r="H230" t="n">
+        <v>83</v>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K230" t="n">
+        <v>7</v>
+      </c>
+      <c r="L230" t="n">
+        <v>24334</v>
+      </c>
+      <c r="M230" t="n">
+        <v>24360.8</v>
+      </c>
+      <c r="N230" t="n">
+        <v>24308.5</v>
+      </c>
+      <c r="O230" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q230" t="n">
+        <v>24472.4</v>
+      </c>
+      <c r="R230" t="n">
+        <v>24390.9</v>
+      </c>
+      <c r="S230" t="n">
+        <v>24575.5</v>
+      </c>
+      <c r="T230" t="n">
+        <v>24429.2</v>
+      </c>
+      <c r="U230" t="n">
+        <v>24502.4</v>
+      </c>
+      <c r="V230" t="n">
+        <v>24481.9</v>
+      </c>
+      <c r="W230" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X230" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y230" t="n">
+        <v>24335.9</v>
+      </c>
+      <c r="Z230" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="AA230" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB230" t="n">
+        <v>24344.8</v>
+      </c>
+      <c r="AC230" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD230" t="n">
+        <v>24184.8</v>
+      </c>
+      <c r="AE230" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF230" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>77616.2</v>
+      </c>
+      <c r="H231" t="n">
+        <v>80</v>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K231" t="n">
+        <v>6</v>
+      </c>
+      <c r="L231" t="n">
+        <v>77765.3</v>
+      </c>
+      <c r="M231" t="n">
+        <v>77836.3</v>
+      </c>
+      <c r="N231" t="n">
+        <v>77630.89999999999</v>
+      </c>
+      <c r="O231" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q231" t="n">
+        <v>78244.89999999999</v>
+      </c>
+      <c r="R231" t="n">
+        <v>77883.5</v>
+      </c>
+      <c r="S231" t="n">
+        <v>78488.60000000001</v>
+      </c>
+      <c r="T231" t="n">
+        <v>78048.3</v>
+      </c>
+      <c r="U231" t="n">
+        <v>78268.39999999999</v>
+      </c>
+      <c r="V231" t="n">
+        <v>78192.3</v>
+      </c>
+      <c r="W231" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X231" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y231" t="n">
+        <v>77764.60000000001</v>
+      </c>
+      <c r="Z231" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="AA231" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB231" t="n">
+        <v>77816.2</v>
+      </c>
+      <c r="AC231" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD231" t="n">
+        <v>77016.2</v>
+      </c>
+      <c r="AE231" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF231" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>24295</v>
+      </c>
+      <c r="H232" t="n">
+        <v>100</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K232" t="n">
+        <v>8</v>
+      </c>
+      <c r="L232" t="n">
+        <v>24310.8</v>
+      </c>
+      <c r="M232" t="n">
+        <v>24337.8</v>
+      </c>
+      <c r="N232" t="n">
+        <v>24297.2</v>
+      </c>
+      <c r="O232" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q232" t="n">
+        <v>24472.4</v>
+      </c>
+      <c r="R232" t="n">
+        <v>24390.9</v>
+      </c>
+      <c r="S232" t="n">
+        <v>24575.5</v>
+      </c>
+      <c r="T232" t="n">
+        <v>24429.2</v>
+      </c>
+      <c r="U232" t="n">
+        <v>24502.4</v>
+      </c>
+      <c r="V232" t="n">
+        <v>24481.9</v>
+      </c>
+      <c r="W232" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X232" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y232" t="n">
+        <v>24330.2</v>
+      </c>
+      <c r="Z232" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB232" t="n">
+        <v>24335</v>
+      </c>
+      <c r="AC232" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD232" t="n">
+        <v>24175</v>
+      </c>
+      <c r="AE232" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF232" t="n">
+        <v>11.94</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>11:47</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>77589.7</v>
+      </c>
+      <c r="H233" t="n">
+        <v>85</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K233" t="n">
+        <v>6</v>
+      </c>
+      <c r="L233" t="n">
+        <v>77655.3</v>
+      </c>
+      <c r="M233" t="n">
+        <v>77741</v>
+      </c>
+      <c r="N233" t="n">
+        <v>77597.10000000001</v>
+      </c>
+      <c r="O233" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q233" t="n">
+        <v>78244.89999999999</v>
+      </c>
+      <c r="R233" t="n">
+        <v>77883.5</v>
+      </c>
+      <c r="S233" t="n">
+        <v>78488.60000000001</v>
+      </c>
+      <c r="T233" t="n">
+        <v>78048.3</v>
+      </c>
+      <c r="U233" t="n">
+        <v>78268.39999999999</v>
+      </c>
+      <c r="V233" t="n">
+        <v>78192.3</v>
+      </c>
+      <c r="W233" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X233" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y233" t="n">
+        <v>77732.8</v>
+      </c>
+      <c r="Z233" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="AA233" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB233" t="n">
+        <v>77789.7</v>
+      </c>
+      <c r="AC233" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD233" t="n">
+        <v>76989.7</v>
+      </c>
+      <c r="AE233" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF233" t="n">
+        <v>11.94</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>24277.1</v>
+      </c>
+      <c r="H234" t="n">
+        <v>85</v>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K234" t="n">
+        <v>6</v>
+      </c>
+      <c r="L234" t="n">
+        <v>24287.8</v>
+      </c>
+      <c r="M234" t="n">
+        <v>24312.8</v>
+      </c>
+      <c r="N234" t="n">
+        <v>24276.5</v>
+      </c>
+      <c r="O234" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q234" t="n">
+        <v>24472.4</v>
+      </c>
+      <c r="R234" t="n">
+        <v>24390.9</v>
+      </c>
+      <c r="S234" t="n">
+        <v>24575.5</v>
+      </c>
+      <c r="T234" t="n">
+        <v>24429.2</v>
+      </c>
+      <c r="U234" t="n">
+        <v>24502.4</v>
+      </c>
+      <c r="V234" t="n">
+        <v>24481.9</v>
+      </c>
+      <c r="W234" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X234" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y234" t="n">
+        <v>24318.3</v>
+      </c>
+      <c r="Z234" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AA234" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB234" t="n">
+        <v>24317.1</v>
+      </c>
+      <c r="AC234" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD234" t="n">
+        <v>24157.1</v>
+      </c>
+      <c r="AE234" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF234" t="n">
+        <v>11.94</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>77543</v>
+      </c>
+      <c r="H235" t="n">
+        <v>85</v>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K235" t="n">
+        <v>6</v>
+      </c>
+      <c r="L235" t="n">
+        <v>77589.10000000001</v>
+      </c>
+      <c r="M235" t="n">
+        <v>77667.39999999999</v>
+      </c>
+      <c r="N235" t="n">
+        <v>77544.7</v>
+      </c>
+      <c r="O235" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q235" t="n">
+        <v>78244.89999999999</v>
+      </c>
+      <c r="R235" t="n">
+        <v>77883.5</v>
+      </c>
+      <c r="S235" t="n">
+        <v>78488.60000000001</v>
+      </c>
+      <c r="T235" t="n">
+        <v>78048.3</v>
+      </c>
+      <c r="U235" t="n">
+        <v>78268.39999999999</v>
+      </c>
+      <c r="V235" t="n">
+        <v>78192.3</v>
+      </c>
+      <c r="W235" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X235" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y235" t="n">
+        <v>77696.60000000001</v>
+      </c>
+      <c r="Z235" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="AA235" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB235" t="n">
+        <v>77743</v>
+      </c>
+      <c r="AC235" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD235" t="n">
+        <v>76943</v>
+      </c>
+      <c r="AE235" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF235" t="n">
+        <v>11.94</v>
+      </c>
+      <c r="AG235" t="inlineStr"/>
+      <c r="AH235" t="inlineStr"/>
+      <c r="AI235" t="inlineStr"/>
+      <c r="AJ235" t="inlineStr"/>
+      <c r="AK235" t="inlineStr"/>
+      <c r="AL235" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-13
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL235"/>
+  <dimension ref="A1:AL240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28748,12 +28748,612 @@
       <c r="AF235" t="n">
         <v>11.94</v>
       </c>
-      <c r="AG235" t="inlineStr"/>
-      <c r="AH235" t="inlineStr"/>
-      <c r="AI235" t="inlineStr"/>
-      <c r="AJ235" t="inlineStr"/>
-      <c r="AK235" t="inlineStr"/>
-      <c r="AL235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>24350</v>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G236" t="n">
+        <v>24370.8</v>
+      </c>
+      <c r="H236" t="n">
+        <v>76</v>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K236" t="n">
+        <v>5</v>
+      </c>
+      <c r="L236" t="n">
+        <v>24373.8</v>
+      </c>
+      <c r="M236" t="n">
+        <v>24371.7</v>
+      </c>
+      <c r="N236" t="n">
+        <v>24369.4</v>
+      </c>
+      <c r="O236" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q236" t="n">
+        <v>24428.9</v>
+      </c>
+      <c r="R236" t="n">
+        <v>24326.8</v>
+      </c>
+      <c r="S236" t="n">
+        <v>24472.4</v>
+      </c>
+      <c r="T236" t="n">
+        <v>24265.9</v>
+      </c>
+      <c r="U236" t="n">
+        <v>24413.7</v>
+      </c>
+      <c r="V236" t="n">
+        <v>24369.2</v>
+      </c>
+      <c r="W236" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X236" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y236" t="n">
+        <v>24365.8</v>
+      </c>
+      <c r="Z236" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AA236" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB236" t="n">
+        <v>24330.8</v>
+      </c>
+      <c r="AC236" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD236" t="n">
+        <v>24490.8</v>
+      </c>
+      <c r="AE236" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF236" t="n">
+        <v>11.48</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>13:16</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>77900</v>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G237" t="n">
+        <v>77894.7</v>
+      </c>
+      <c r="H237" t="n">
+        <v>76</v>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K237" t="n">
+        <v>5</v>
+      </c>
+      <c r="L237" t="n">
+        <v>77921.60000000001</v>
+      </c>
+      <c r="M237" t="n">
+        <v>77900.7</v>
+      </c>
+      <c r="N237" t="n">
+        <v>77894.2</v>
+      </c>
+      <c r="O237" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q237" t="n">
+        <v>78111.89999999999</v>
+      </c>
+      <c r="R237" t="n">
+        <v>77745</v>
+      </c>
+      <c r="S237" t="n">
+        <v>78244.89999999999</v>
+      </c>
+      <c r="T237" t="n">
+        <v>77498.3</v>
+      </c>
+      <c r="U237" t="n">
+        <v>77934.8</v>
+      </c>
+      <c r="V237" t="n">
+        <v>77871.60000000001</v>
+      </c>
+      <c r="W237" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X237" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y237" t="n">
+        <v>77885.2</v>
+      </c>
+      <c r="Z237" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA237" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB237" t="n">
+        <v>77694.7</v>
+      </c>
+      <c r="AC237" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD237" t="n">
+        <v>78494.7</v>
+      </c>
+      <c r="AE237" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF237" t="n">
+        <v>11.48</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>24350</v>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G238" t="n">
+        <v>24352.1</v>
+      </c>
+      <c r="H238" t="n">
+        <v>76</v>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K238" t="n">
+        <v>6</v>
+      </c>
+      <c r="L238" t="n">
+        <v>24363.4</v>
+      </c>
+      <c r="M238" t="n">
+        <v>24366.8</v>
+      </c>
+      <c r="N238" t="n">
+        <v>24352.7</v>
+      </c>
+      <c r="O238" t="n">
+        <v>43</v>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q238" t="n">
+        <v>24428.9</v>
+      </c>
+      <c r="R238" t="n">
+        <v>24326.8</v>
+      </c>
+      <c r="S238" t="n">
+        <v>24472.4</v>
+      </c>
+      <c r="T238" t="n">
+        <v>24265.9</v>
+      </c>
+      <c r="U238" t="n">
+        <v>24413.7</v>
+      </c>
+      <c r="V238" t="n">
+        <v>24369.2</v>
+      </c>
+      <c r="W238" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X238" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y238" t="n">
+        <v>24356.3</v>
+      </c>
+      <c r="Z238" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AA238" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB238" t="n">
+        <v>24392.1</v>
+      </c>
+      <c r="AC238" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD238" t="n">
+        <v>24232.1</v>
+      </c>
+      <c r="AE238" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF238" t="n">
+        <v>11.48</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>77800</v>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>77805.2</v>
+      </c>
+      <c r="H239" t="n">
+        <v>76</v>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K239" t="n">
+        <v>6</v>
+      </c>
+      <c r="L239" t="n">
+        <v>77866.89999999999</v>
+      </c>
+      <c r="M239" t="n">
+        <v>77878.60000000001</v>
+      </c>
+      <c r="N239" t="n">
+        <v>77821.8</v>
+      </c>
+      <c r="O239" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q239" t="n">
+        <v>78111.89999999999</v>
+      </c>
+      <c r="R239" t="n">
+        <v>77745</v>
+      </c>
+      <c r="S239" t="n">
+        <v>78244.89999999999</v>
+      </c>
+      <c r="T239" t="n">
+        <v>77498.3</v>
+      </c>
+      <c r="U239" t="n">
+        <v>77934.8</v>
+      </c>
+      <c r="V239" t="n">
+        <v>77871.60000000001</v>
+      </c>
+      <c r="W239" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X239" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y239" t="n">
+        <v>77837.39999999999</v>
+      </c>
+      <c r="Z239" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="AA239" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB239" t="n">
+        <v>78005.2</v>
+      </c>
+      <c r="AC239" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD239" t="n">
+        <v>77205.2</v>
+      </c>
+      <c r="AE239" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF239" t="n">
+        <v>11.43</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>78000</v>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G240" t="n">
+        <v>77952.89999999999</v>
+      </c>
+      <c r="H240" t="n">
+        <v>76</v>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>6</v>
+      </c>
+      <c r="L240" t="n">
+        <v>77895.10000000001</v>
+      </c>
+      <c r="M240" t="n">
+        <v>77888.8</v>
+      </c>
+      <c r="N240" t="n">
+        <v>77945.7</v>
+      </c>
+      <c r="O240" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q240" t="n">
+        <v>78111.89999999999</v>
+      </c>
+      <c r="R240" t="n">
+        <v>77745</v>
+      </c>
+      <c r="S240" t="n">
+        <v>78244.89999999999</v>
+      </c>
+      <c r="T240" t="n">
+        <v>77498.3</v>
+      </c>
+      <c r="U240" t="n">
+        <v>77934.8</v>
+      </c>
+      <c r="V240" t="n">
+        <v>77871.60000000001</v>
+      </c>
+      <c r="W240" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X240" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y240" t="n">
+        <v>77971.8</v>
+      </c>
+      <c r="Z240" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AA240" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB240" t="n">
+        <v>77752.89999999999</v>
+      </c>
+      <c r="AC240" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD240" t="n">
+        <v>78552.89999999999</v>
+      </c>
+      <c r="AE240" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF240" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="AG240" t="inlineStr"/>
+      <c r="AH240" t="inlineStr"/>
+      <c r="AI240" t="inlineStr"/>
+      <c r="AJ240" t="inlineStr"/>
+      <c r="AK240" t="inlineStr"/>
+      <c r="AL240" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-14
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Signals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL240"/>
+  <dimension ref="A1:AL246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29348,12 +29348,732 @@
       <c r="AF240" t="n">
         <v>11.43</v>
       </c>
-      <c r="AG240" t="inlineStr"/>
-      <c r="AH240" t="inlineStr"/>
-      <c r="AI240" t="inlineStr"/>
-      <c r="AJ240" t="inlineStr"/>
-      <c r="AK240" t="inlineStr"/>
-      <c r="AL240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G241" t="n">
+        <v>57462.9</v>
+      </c>
+      <c r="H241" t="n">
+        <v>78</v>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K241" t="n">
+        <v>6</v>
+      </c>
+      <c r="L241" t="n">
+        <v>57497.1</v>
+      </c>
+      <c r="M241" t="n">
+        <v>57521.5</v>
+      </c>
+      <c r="N241" t="n">
+        <v>57467.6</v>
+      </c>
+      <c r="O241" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q241" t="n">
+        <v>57600.2</v>
+      </c>
+      <c r="R241" t="n">
+        <v>57482.8</v>
+      </c>
+      <c r="S241" t="n">
+        <v>57782.9</v>
+      </c>
+      <c r="T241" t="n">
+        <v>57548.6</v>
+      </c>
+      <c r="U241" t="n">
+        <v>57665.7</v>
+      </c>
+      <c r="V241" t="n">
+        <v>57645.4</v>
+      </c>
+      <c r="W241" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X241" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y241" t="n">
+        <v>57479.6</v>
+      </c>
+      <c r="Z241" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="AA241" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB241" t="n">
+        <v>57582.9</v>
+      </c>
+      <c r="AC241" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD241" t="n">
+        <v>57102.9</v>
+      </c>
+      <c r="AE241" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF241" t="n">
+        <v>11.41</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G242" t="n">
+        <v>57409.9</v>
+      </c>
+      <c r="H242" t="n">
+        <v>93</v>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K242" t="n">
+        <v>7</v>
+      </c>
+      <c r="L242" t="n">
+        <v>57447.9</v>
+      </c>
+      <c r="M242" t="n">
+        <v>57483.5</v>
+      </c>
+      <c r="N242" t="n">
+        <v>57416.6</v>
+      </c>
+      <c r="O242" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q242" t="n">
+        <v>57600.2</v>
+      </c>
+      <c r="R242" t="n">
+        <v>57482.8</v>
+      </c>
+      <c r="S242" t="n">
+        <v>57782.9</v>
+      </c>
+      <c r="T242" t="n">
+        <v>57548.6</v>
+      </c>
+      <c r="U242" t="n">
+        <v>57665.7</v>
+      </c>
+      <c r="V242" t="n">
+        <v>57645.4</v>
+      </c>
+      <c r="W242" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X242" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y242" t="n">
+        <v>57432.5</v>
+      </c>
+      <c r="Z242" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="AA242" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB242" t="n">
+        <v>57529.9</v>
+      </c>
+      <c r="AC242" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD242" t="n">
+        <v>57049.9</v>
+      </c>
+      <c r="AE242" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF242" t="n">
+        <v>11.41</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G243" t="n">
+        <v>57412.4</v>
+      </c>
+      <c r="H243" t="n">
+        <v>78</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>6</v>
+      </c>
+      <c r="L243" t="n">
+        <v>57425.9</v>
+      </c>
+      <c r="M243" t="n">
+        <v>57456.9</v>
+      </c>
+      <c r="N243" t="n">
+        <v>57409.5</v>
+      </c>
+      <c r="O243" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q243" t="n">
+        <v>57600.2</v>
+      </c>
+      <c r="R243" t="n">
+        <v>57482.8</v>
+      </c>
+      <c r="S243" t="n">
+        <v>57782.9</v>
+      </c>
+      <c r="T243" t="n">
+        <v>57548.6</v>
+      </c>
+      <c r="U243" t="n">
+        <v>57665.7</v>
+      </c>
+      <c r="V243" t="n">
+        <v>57645.4</v>
+      </c>
+      <c r="W243" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X243" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y243" t="n">
+        <v>57432.5</v>
+      </c>
+      <c r="Z243" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB243" t="n">
+        <v>57532.4</v>
+      </c>
+      <c r="AC243" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD243" t="n">
+        <v>57052.4</v>
+      </c>
+      <c r="AE243" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF243" t="n">
+        <v>11.41</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>77800</v>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G244" t="n">
+        <v>77813.8</v>
+      </c>
+      <c r="H244" t="n">
+        <v>76</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K244" t="n">
+        <v>5</v>
+      </c>
+      <c r="L244" t="n">
+        <v>77785.7</v>
+      </c>
+      <c r="M244" t="n">
+        <v>77784.60000000001</v>
+      </c>
+      <c r="N244" t="n">
+        <v>77804</v>
+      </c>
+      <c r="O244" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q244" t="n">
+        <v>77833.39999999999</v>
+      </c>
+      <c r="R244" t="n">
+        <v>77733</v>
+      </c>
+      <c r="S244" t="n">
+        <v>78193</v>
+      </c>
+      <c r="T244" t="n">
+        <v>77399.2</v>
+      </c>
+      <c r="U244" t="n">
+        <v>77985.39999999999</v>
+      </c>
+      <c r="V244" t="n">
+        <v>77796.10000000001</v>
+      </c>
+      <c r="W244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X244" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Y244" t="n">
+        <v>77815.3</v>
+      </c>
+      <c r="Z244" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA244" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB244" t="n">
+        <v>77613.8</v>
+      </c>
+      <c r="AC244" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD244" t="n">
+        <v>78413.8</v>
+      </c>
+      <c r="AE244" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF244" t="n">
+        <v>11.41</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>57400</v>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G245" t="n">
+        <v>57449.8</v>
+      </c>
+      <c r="H245" t="n">
+        <v>91</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K245" t="n">
+        <v>7</v>
+      </c>
+      <c r="L245" t="n">
+        <v>57430.8</v>
+      </c>
+      <c r="M245" t="n">
+        <v>57456.3</v>
+      </c>
+      <c r="N245" t="n">
+        <v>57438.1</v>
+      </c>
+      <c r="O245" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q245" t="n">
+        <v>57600.2</v>
+      </c>
+      <c r="R245" t="n">
+        <v>57482.8</v>
+      </c>
+      <c r="S245" t="n">
+        <v>57782.9</v>
+      </c>
+      <c r="T245" t="n">
+        <v>57548.6</v>
+      </c>
+      <c r="U245" t="n">
+        <v>57665.7</v>
+      </c>
+      <c r="V245" t="n">
+        <v>57645.4</v>
+      </c>
+      <c r="W245" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X245" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y245" t="n">
+        <v>57464.5</v>
+      </c>
+      <c r="Z245" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AA245" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB245" t="n">
+        <v>57569.8</v>
+      </c>
+      <c r="AC245" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD245" t="n">
+        <v>57089.8</v>
+      </c>
+      <c r="AE245" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF245" t="n">
+        <v>11.41</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>77900</v>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G246" t="n">
+        <v>77858.39999999999</v>
+      </c>
+      <c r="H246" t="n">
+        <v>83</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K246" t="n">
+        <v>6</v>
+      </c>
+      <c r="L246" t="n">
+        <v>77818.7</v>
+      </c>
+      <c r="M246" t="n">
+        <v>77801.60000000001</v>
+      </c>
+      <c r="N246" t="n">
+        <v>77856.89999999999</v>
+      </c>
+      <c r="O246" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q246" t="n">
+        <v>77833.39999999999</v>
+      </c>
+      <c r="R246" t="n">
+        <v>77733</v>
+      </c>
+      <c r="S246" t="n">
+        <v>78193</v>
+      </c>
+      <c r="T246" t="n">
+        <v>77399.2</v>
+      </c>
+      <c r="U246" t="n">
+        <v>77985.39999999999</v>
+      </c>
+      <c r="V246" t="n">
+        <v>77796.10000000001</v>
+      </c>
+      <c r="W246" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X246" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y246" t="n">
+        <v>77858.8</v>
+      </c>
+      <c r="Z246" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AA246" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB246" t="n">
+        <v>77658.39999999999</v>
+      </c>
+      <c r="AC246" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD246" t="n">
+        <v>78458.39999999999</v>
+      </c>
+      <c r="AE246" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF246" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="AG246" t="inlineStr"/>
+      <c r="AH246" t="inlineStr"/>
+      <c r="AI246" t="inlineStr"/>
+      <c r="AJ246" t="inlineStr"/>
+      <c r="AK246" t="inlineStr"/>
+      <c r="AL246" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-17
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL246"/>
+  <dimension ref="A1:AL253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30068,12 +30068,852 @@
       <c r="AF246" t="n">
         <v>11.37</v>
       </c>
-      <c r="AG246" t="inlineStr"/>
-      <c r="AH246" t="inlineStr"/>
-      <c r="AI246" t="inlineStr"/>
-      <c r="AJ246" t="inlineStr"/>
-      <c r="AK246" t="inlineStr"/>
-      <c r="AL246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>77700</v>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G247" t="n">
+        <v>77692.39999999999</v>
+      </c>
+      <c r="H247" t="n">
+        <v>81</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K247" t="n">
+        <v>6</v>
+      </c>
+      <c r="L247" t="n">
+        <v>77700.89999999999</v>
+      </c>
+      <c r="M247" t="n">
+        <v>77707.8</v>
+      </c>
+      <c r="N247" t="n">
+        <v>77696.3</v>
+      </c>
+      <c r="O247" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q247" t="n">
+        <v>77912.89999999999</v>
+      </c>
+      <c r="R247" t="n">
+        <v>77657.5</v>
+      </c>
+      <c r="S247" t="n">
+        <v>78205.8</v>
+      </c>
+      <c r="T247" t="n">
+        <v>77685.3</v>
+      </c>
+      <c r="U247" t="n">
+        <v>77988</v>
+      </c>
+      <c r="V247" t="n">
+        <v>77945.60000000001</v>
+      </c>
+      <c r="W247" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X247" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y247" t="n">
+        <v>77705.3</v>
+      </c>
+      <c r="Z247" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="AA247" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB247" t="n">
+        <v>77892.39999999999</v>
+      </c>
+      <c r="AC247" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD247" t="n">
+        <v>77092.39999999999</v>
+      </c>
+      <c r="AE247" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF247" t="n">
+        <v>11.57</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G248" t="n">
+        <v>77638.8</v>
+      </c>
+      <c r="H248" t="n">
+        <v>93</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K248" t="n">
+        <v>7</v>
+      </c>
+      <c r="L248" t="n">
+        <v>77680.2</v>
+      </c>
+      <c r="M248" t="n">
+        <v>77697.3</v>
+      </c>
+      <c r="N248" t="n">
+        <v>77641</v>
+      </c>
+      <c r="O248" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q248" t="n">
+        <v>77912.89999999999</v>
+      </c>
+      <c r="R248" t="n">
+        <v>77657.5</v>
+      </c>
+      <c r="S248" t="n">
+        <v>78205.8</v>
+      </c>
+      <c r="T248" t="n">
+        <v>77685.3</v>
+      </c>
+      <c r="U248" t="n">
+        <v>77988</v>
+      </c>
+      <c r="V248" t="n">
+        <v>77945.60000000001</v>
+      </c>
+      <c r="W248" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X248" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y248" t="n">
+        <v>77699.8</v>
+      </c>
+      <c r="Z248" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="AA248" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB248" t="n">
+        <v>77838.8</v>
+      </c>
+      <c r="AC248" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD248" t="n">
+        <v>77038.8</v>
+      </c>
+      <c r="AE248" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF248" t="n">
+        <v>11.57</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G249" t="n">
+        <v>24260.2</v>
+      </c>
+      <c r="H249" t="n">
+        <v>78</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K249" t="n">
+        <v>6</v>
+      </c>
+      <c r="L249" t="n">
+        <v>24281.4</v>
+      </c>
+      <c r="M249" t="n">
+        <v>24291.7</v>
+      </c>
+      <c r="N249" t="n">
+        <v>24261.7</v>
+      </c>
+      <c r="O249" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q249" t="n">
+        <v>24357.6</v>
+      </c>
+      <c r="R249" t="n">
+        <v>24283.1</v>
+      </c>
+      <c r="S249" t="n">
+        <v>24405.2</v>
+      </c>
+      <c r="T249" t="n">
+        <v>24298.3</v>
+      </c>
+      <c r="U249" t="n">
+        <v>24361.3</v>
+      </c>
+      <c r="V249" t="n">
+        <v>24351.8</v>
+      </c>
+      <c r="W249" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X249" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y249" t="n">
+        <v>24282.7</v>
+      </c>
+      <c r="Z249" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="AA249" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB249" t="n">
+        <v>24300.2</v>
+      </c>
+      <c r="AC249" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD249" t="n">
+        <v>24140.2</v>
+      </c>
+      <c r="AE249" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF249" t="n">
+        <v>11.57</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D250" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G250" t="n">
+        <v>57149.9</v>
+      </c>
+      <c r="H250" t="n">
+        <v>78</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>6</v>
+      </c>
+      <c r="L250" t="n">
+        <v>57209</v>
+      </c>
+      <c r="M250" t="n">
+        <v>57246.5</v>
+      </c>
+      <c r="N250" t="n">
+        <v>57154.5</v>
+      </c>
+      <c r="O250" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q250" t="n">
+        <v>57472.1</v>
+      </c>
+      <c r="R250" t="n">
+        <v>57166.1</v>
+      </c>
+      <c r="S250" t="n">
+        <v>57679.8</v>
+      </c>
+      <c r="T250" t="n">
+        <v>57380.6</v>
+      </c>
+      <c r="U250" t="n">
+        <v>57530.2</v>
+      </c>
+      <c r="V250" t="n">
+        <v>57504.1</v>
+      </c>
+      <c r="W250" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X250" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y250" t="n">
+        <v>57203.1</v>
+      </c>
+      <c r="Z250" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB250" t="n">
+        <v>57269.9</v>
+      </c>
+      <c r="AC250" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD250" t="n">
+        <v>56789.9</v>
+      </c>
+      <c r="AE250" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF250" t="n">
+        <v>11.57</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>10:46</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>77567.8</v>
+      </c>
+      <c r="H251" t="n">
+        <v>78</v>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K251" t="n">
+        <v>6</v>
+      </c>
+      <c r="L251" t="n">
+        <v>77612.60000000001</v>
+      </c>
+      <c r="M251" t="n">
+        <v>77653</v>
+      </c>
+      <c r="N251" t="n">
+        <v>77573.10000000001</v>
+      </c>
+      <c r="O251" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q251" t="n">
+        <v>77912.89999999999</v>
+      </c>
+      <c r="R251" t="n">
+        <v>77657.5</v>
+      </c>
+      <c r="S251" t="n">
+        <v>78205.8</v>
+      </c>
+      <c r="T251" t="n">
+        <v>77685.3</v>
+      </c>
+      <c r="U251" t="n">
+        <v>77988</v>
+      </c>
+      <c r="V251" t="n">
+        <v>77945.60000000001</v>
+      </c>
+      <c r="W251" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X251" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y251" t="n">
+        <v>77633.2</v>
+      </c>
+      <c r="Z251" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB251" t="n">
+        <v>77767.8</v>
+      </c>
+      <c r="AC251" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD251" t="n">
+        <v>76967.8</v>
+      </c>
+      <c r="AE251" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF251" t="n">
+        <v>11.57</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G252" t="n">
+        <v>24234.6</v>
+      </c>
+      <c r="H252" t="n">
+        <v>78</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K252" t="n">
+        <v>6</v>
+      </c>
+      <c r="L252" t="n">
+        <v>24246.2</v>
+      </c>
+      <c r="M252" t="n">
+        <v>24263.4</v>
+      </c>
+      <c r="N252" t="n">
+        <v>24236.8</v>
+      </c>
+      <c r="O252" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q252" t="n">
+        <v>24357.6</v>
+      </c>
+      <c r="R252" t="n">
+        <v>24283.1</v>
+      </c>
+      <c r="S252" t="n">
+        <v>24405.2</v>
+      </c>
+      <c r="T252" t="n">
+        <v>24298.3</v>
+      </c>
+      <c r="U252" t="n">
+        <v>24361.3</v>
+      </c>
+      <c r="V252" t="n">
+        <v>24351.8</v>
+      </c>
+      <c r="W252" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y252" t="n">
+        <v>24258.9</v>
+      </c>
+      <c r="Z252" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB252" t="n">
+        <v>24274.6</v>
+      </c>
+      <c r="AC252" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD252" t="n">
+        <v>24114.6</v>
+      </c>
+      <c r="AE252" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF252" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>57200</v>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G253" t="n">
+        <v>57151.3</v>
+      </c>
+      <c r="H253" t="n">
+        <v>78</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K253" t="n">
+        <v>6</v>
+      </c>
+      <c r="L253" t="n">
+        <v>57176.9</v>
+      </c>
+      <c r="M253" t="n">
+        <v>57208.4</v>
+      </c>
+      <c r="N253" t="n">
+        <v>57158.4</v>
+      </c>
+      <c r="O253" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q253" t="n">
+        <v>57472.1</v>
+      </c>
+      <c r="R253" t="n">
+        <v>57166.1</v>
+      </c>
+      <c r="S253" t="n">
+        <v>57679.8</v>
+      </c>
+      <c r="T253" t="n">
+        <v>57380.6</v>
+      </c>
+      <c r="U253" t="n">
+        <v>57530.2</v>
+      </c>
+      <c r="V253" t="n">
+        <v>57504.1</v>
+      </c>
+      <c r="W253" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y253" t="n">
+        <v>57203.1</v>
+      </c>
+      <c r="Z253" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB253" t="n">
+        <v>57271.3</v>
+      </c>
+      <c r="AC253" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD253" t="n">
+        <v>56791.3</v>
+      </c>
+      <c r="AE253" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF253" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="AG253" t="inlineStr"/>
+      <c r="AH253" t="inlineStr"/>
+      <c r="AI253" t="inlineStr"/>
+      <c r="AJ253" t="inlineStr"/>
+      <c r="AK253" t="inlineStr"/>
+      <c r="AL253" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-18
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL253"/>
+  <dimension ref="A1:AL257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30908,12 +30908,492 @@
       <c r="AF253" t="n">
         <v>11.68</v>
       </c>
-      <c r="AG253" t="inlineStr"/>
-      <c r="AH253" t="inlineStr"/>
-      <c r="AI253" t="inlineStr"/>
-      <c r="AJ253" t="inlineStr"/>
-      <c r="AK253" t="inlineStr"/>
-      <c r="AL253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G254" t="n">
+        <v>24208.8</v>
+      </c>
+      <c r="H254" t="n">
+        <v>76</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>6</v>
+      </c>
+      <c r="L254" t="n">
+        <v>24200.4</v>
+      </c>
+      <c r="M254" t="n">
+        <v>24206.6</v>
+      </c>
+      <c r="N254" t="n">
+        <v>24208.8</v>
+      </c>
+      <c r="O254" t="n">
+        <v>54</v>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q254" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="R254" t="n">
+        <v>24214.6</v>
+      </c>
+      <c r="S254" t="n">
+        <v>24359.9</v>
+      </c>
+      <c r="T254" t="n">
+        <v>24226.9</v>
+      </c>
+      <c r="U254" t="n">
+        <v>24293.4</v>
+      </c>
+      <c r="V254" t="n">
+        <v>24289.6</v>
+      </c>
+      <c r="W254" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y254" t="n">
+        <v>24210.8</v>
+      </c>
+      <c r="Z254" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB254" t="n">
+        <v>24248.8</v>
+      </c>
+      <c r="AC254" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD254" t="n">
+        <v>24088.8</v>
+      </c>
+      <c r="AE254" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF254" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G255" t="n">
+        <v>24210.3</v>
+      </c>
+      <c r="H255" t="n">
+        <v>76</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K255" t="n">
+        <v>6</v>
+      </c>
+      <c r="L255" t="n">
+        <v>24207.9</v>
+      </c>
+      <c r="M255" t="n">
+        <v>24208.2</v>
+      </c>
+      <c r="N255" t="n">
+        <v>24210.3</v>
+      </c>
+      <c r="O255" t="n">
+        <v>54</v>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q255" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="R255" t="n">
+        <v>24214.6</v>
+      </c>
+      <c r="S255" t="n">
+        <v>24359.9</v>
+      </c>
+      <c r="T255" t="n">
+        <v>24226.9</v>
+      </c>
+      <c r="U255" t="n">
+        <v>24293.4</v>
+      </c>
+      <c r="V255" t="n">
+        <v>24289.6</v>
+      </c>
+      <c r="W255" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X255" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y255" t="n">
+        <v>24210.8</v>
+      </c>
+      <c r="Z255" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA255" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB255" t="n">
+        <v>24250.3</v>
+      </c>
+      <c r="AC255" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD255" t="n">
+        <v>24090.3</v>
+      </c>
+      <c r="AE255" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF255" t="n">
+        <v>11.63</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G256" t="n">
+        <v>24209.7</v>
+      </c>
+      <c r="H256" t="n">
+        <v>76</v>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>6</v>
+      </c>
+      <c r="L256" t="n">
+        <v>24207.3</v>
+      </c>
+      <c r="M256" t="n">
+        <v>24207.8</v>
+      </c>
+      <c r="N256" t="n">
+        <v>24209.7</v>
+      </c>
+      <c r="O256" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q256" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="R256" t="n">
+        <v>24214.6</v>
+      </c>
+      <c r="S256" t="n">
+        <v>24359.9</v>
+      </c>
+      <c r="T256" t="n">
+        <v>24226.9</v>
+      </c>
+      <c r="U256" t="n">
+        <v>24293.4</v>
+      </c>
+      <c r="V256" t="n">
+        <v>24289.6</v>
+      </c>
+      <c r="W256" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X256" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y256" t="n">
+        <v>24210.8</v>
+      </c>
+      <c r="Z256" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AA256" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB256" t="n">
+        <v>24249.7</v>
+      </c>
+      <c r="AC256" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD256" t="n">
+        <v>24089.7</v>
+      </c>
+      <c r="AE256" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF256" t="n">
+        <v>11.66</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G257" t="n">
+        <v>24204.2</v>
+      </c>
+      <c r="H257" t="n">
+        <v>76</v>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K257" t="n">
+        <v>6</v>
+      </c>
+      <c r="L257" t="n">
+        <v>24203.3</v>
+      </c>
+      <c r="M257" t="n">
+        <v>24204.9</v>
+      </c>
+      <c r="N257" t="n">
+        <v>24204.2</v>
+      </c>
+      <c r="O257" t="n">
+        <v>50</v>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q257" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="R257" t="n">
+        <v>24214.6</v>
+      </c>
+      <c r="S257" t="n">
+        <v>24359.9</v>
+      </c>
+      <c r="T257" t="n">
+        <v>24226.9</v>
+      </c>
+      <c r="U257" t="n">
+        <v>24293.4</v>
+      </c>
+      <c r="V257" t="n">
+        <v>24289.6</v>
+      </c>
+      <c r="W257" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X257" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y257" t="n">
+        <v>24210.8</v>
+      </c>
+      <c r="Z257" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AA257" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB257" t="n">
+        <v>24244.2</v>
+      </c>
+      <c r="AC257" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD257" t="n">
+        <v>24084.2</v>
+      </c>
+      <c r="AE257" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF257" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="AG257" t="inlineStr"/>
+      <c r="AH257" t="inlineStr"/>
+      <c r="AI257" t="inlineStr"/>
+      <c r="AJ257" t="inlineStr"/>
+      <c r="AK257" t="inlineStr"/>
+      <c r="AL257" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-19
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL257"/>
+  <dimension ref="A1:AL264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31388,12 +31388,852 @@
       <c r="AF257" t="n">
         <v>11.6</v>
       </c>
-      <c r="AG257" t="inlineStr"/>
-      <c r="AH257" t="inlineStr"/>
-      <c r="AI257" t="inlineStr"/>
-      <c r="AJ257" t="inlineStr"/>
-      <c r="AK257" t="inlineStr"/>
-      <c r="AL257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>24100</v>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>24095.9</v>
+      </c>
+      <c r="H258" t="n">
+        <v>81</v>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>6</v>
+      </c>
+      <c r="L258" t="n">
+        <v>24097.2</v>
+      </c>
+      <c r="M258" t="n">
+        <v>24103.2</v>
+      </c>
+      <c r="N258" t="n">
+        <v>24097.4</v>
+      </c>
+      <c r="O258" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q258" t="n">
+        <v>24166.9</v>
+      </c>
+      <c r="R258" t="n">
+        <v>24093.2</v>
+      </c>
+      <c r="S258" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="T258" t="n">
+        <v>24154.9</v>
+      </c>
+      <c r="U258" t="n">
+        <v>24212.2</v>
+      </c>
+      <c r="V258" t="n">
+        <v>24174</v>
+      </c>
+      <c r="W258" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y258" t="n">
+        <v>24089.4</v>
+      </c>
+      <c r="Z258" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AA258" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB258" t="n">
+        <v>24135.9</v>
+      </c>
+      <c r="AC258" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD258" t="n">
+        <v>23975.9</v>
+      </c>
+      <c r="AE258" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF258" t="n">
+        <v>11.49</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>77100</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>77059.5</v>
+      </c>
+      <c r="H259" t="n">
+        <v>81</v>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K259" t="n">
+        <v>6</v>
+      </c>
+      <c r="L259" t="n">
+        <v>77065.89999999999</v>
+      </c>
+      <c r="M259" t="n">
+        <v>77089.89999999999</v>
+      </c>
+      <c r="N259" t="n">
+        <v>77060.60000000001</v>
+      </c>
+      <c r="O259" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="P259" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q259" t="n">
+        <v>77270.39999999999</v>
+      </c>
+      <c r="R259" t="n">
+        <v>77049.5</v>
+      </c>
+      <c r="S259" t="n">
+        <v>77574</v>
+      </c>
+      <c r="T259" t="n">
+        <v>77180.8</v>
+      </c>
+      <c r="U259" t="n">
+        <v>77377.39999999999</v>
+      </c>
+      <c r="V259" t="n">
+        <v>77282.8</v>
+      </c>
+      <c r="W259" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X259" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y259" t="n">
+        <v>77042.10000000001</v>
+      </c>
+      <c r="Z259" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA259" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB259" t="n">
+        <v>77259.5</v>
+      </c>
+      <c r="AC259" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD259" t="n">
+        <v>76459.5</v>
+      </c>
+      <c r="AE259" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF259" t="n">
+        <v>11.49</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>10:37</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>24058.2</v>
+      </c>
+      <c r="H260" t="n">
+        <v>78</v>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K260" t="n">
+        <v>6</v>
+      </c>
+      <c r="L260" t="n">
+        <v>24077.1</v>
+      </c>
+      <c r="M260" t="n">
+        <v>24090.2</v>
+      </c>
+      <c r="N260" t="n">
+        <v>24060.9</v>
+      </c>
+      <c r="O260" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q260" t="n">
+        <v>24166.9</v>
+      </c>
+      <c r="R260" t="n">
+        <v>24093.2</v>
+      </c>
+      <c r="S260" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="T260" t="n">
+        <v>24154.9</v>
+      </c>
+      <c r="U260" t="n">
+        <v>24212.2</v>
+      </c>
+      <c r="V260" t="n">
+        <v>24174</v>
+      </c>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y260" t="n">
+        <v>24083.7</v>
+      </c>
+      <c r="Z260" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="AA260" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB260" t="n">
+        <v>24098.2</v>
+      </c>
+      <c r="AC260" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD260" t="n">
+        <v>23938.2</v>
+      </c>
+      <c r="AE260" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF260" t="n">
+        <v>11.52</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>10:37</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>57096.1</v>
+      </c>
+      <c r="H261" t="n">
+        <v>78</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K261" t="n">
+        <v>6</v>
+      </c>
+      <c r="L261" t="n">
+        <v>57133.6</v>
+      </c>
+      <c r="M261" t="n">
+        <v>57139.7</v>
+      </c>
+      <c r="N261" t="n">
+        <v>57098.5</v>
+      </c>
+      <c r="O261" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q261" t="n">
+        <v>57323.4</v>
+      </c>
+      <c r="R261" t="n">
+        <v>57096.2</v>
+      </c>
+      <c r="S261" t="n">
+        <v>57584.7</v>
+      </c>
+      <c r="T261" t="n">
+        <v>57218.8</v>
+      </c>
+      <c r="U261" t="n">
+        <v>57401.7</v>
+      </c>
+      <c r="V261" t="n">
+        <v>57308.8</v>
+      </c>
+      <c r="W261" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X261" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y261" t="n">
+        <v>57077.6</v>
+      </c>
+      <c r="Z261" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AA261" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB261" t="n">
+        <v>57216.1</v>
+      </c>
+      <c r="AC261" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD261" t="n">
+        <v>56736.1</v>
+      </c>
+      <c r="AE261" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF261" t="n">
+        <v>11.52</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>76900</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>76929.10000000001</v>
+      </c>
+      <c r="H262" t="n">
+        <v>78</v>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K262" t="n">
+        <v>6</v>
+      </c>
+      <c r="L262" t="n">
+        <v>76997.60000000001</v>
+      </c>
+      <c r="M262" t="n">
+        <v>77043.3</v>
+      </c>
+      <c r="N262" t="n">
+        <v>76933.10000000001</v>
+      </c>
+      <c r="O262" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q262" t="n">
+        <v>77270.39999999999</v>
+      </c>
+      <c r="R262" t="n">
+        <v>77049.5</v>
+      </c>
+      <c r="S262" t="n">
+        <v>77574</v>
+      </c>
+      <c r="T262" t="n">
+        <v>77180.8</v>
+      </c>
+      <c r="U262" t="n">
+        <v>77377.39999999999</v>
+      </c>
+      <c r="V262" t="n">
+        <v>77282.8</v>
+      </c>
+      <c r="W262" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y262" t="n">
+        <v>77006.5</v>
+      </c>
+      <c r="Z262" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="AA262" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB262" t="n">
+        <v>77129.10000000001</v>
+      </c>
+      <c r="AC262" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD262" t="n">
+        <v>76329.10000000001</v>
+      </c>
+      <c r="AE262" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF262" t="n">
+        <v>11.52</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>24050</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>24042</v>
+      </c>
+      <c r="H263" t="n">
+        <v>78</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K263" t="n">
+        <v>6</v>
+      </c>
+      <c r="L263" t="n">
+        <v>24056.5</v>
+      </c>
+      <c r="M263" t="n">
+        <v>24071.7</v>
+      </c>
+      <c r="N263" t="n">
+        <v>24044.7</v>
+      </c>
+      <c r="O263" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q263" t="n">
+        <v>24166.9</v>
+      </c>
+      <c r="R263" t="n">
+        <v>24093.2</v>
+      </c>
+      <c r="S263" t="n">
+        <v>24269.5</v>
+      </c>
+      <c r="T263" t="n">
+        <v>24154.9</v>
+      </c>
+      <c r="U263" t="n">
+        <v>24212.2</v>
+      </c>
+      <c r="V263" t="n">
+        <v>24174</v>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y263" t="n">
+        <v>24071.5</v>
+      </c>
+      <c r="Z263" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="AA263" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB263" t="n">
+        <v>24082</v>
+      </c>
+      <c r="AC263" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD263" t="n">
+        <v>23922</v>
+      </c>
+      <c r="AE263" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF263" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>57055.8</v>
+      </c>
+      <c r="H264" t="n">
+        <v>78</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K264" t="n">
+        <v>6</v>
+      </c>
+      <c r="L264" t="n">
+        <v>57083.6</v>
+      </c>
+      <c r="M264" t="n">
+        <v>57106.9</v>
+      </c>
+      <c r="N264" t="n">
+        <v>57064.6</v>
+      </c>
+      <c r="O264" t="n">
+        <v>27</v>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q264" t="n">
+        <v>57323.4</v>
+      </c>
+      <c r="R264" t="n">
+        <v>57096.2</v>
+      </c>
+      <c r="S264" t="n">
+        <v>57584.7</v>
+      </c>
+      <c r="T264" t="n">
+        <v>57218.8</v>
+      </c>
+      <c r="U264" t="n">
+        <v>57401.7</v>
+      </c>
+      <c r="V264" t="n">
+        <v>57308.8</v>
+      </c>
+      <c r="W264" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y264" t="n">
+        <v>57077.6</v>
+      </c>
+      <c r="Z264" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AA264" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB264" t="n">
+        <v>57175.8</v>
+      </c>
+      <c r="AC264" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD264" t="n">
+        <v>56695.8</v>
+      </c>
+      <c r="AE264" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF264" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="AG264" t="inlineStr"/>
+      <c r="AH264" t="inlineStr"/>
+      <c r="AI264" t="inlineStr"/>
+      <c r="AJ264" t="inlineStr"/>
+      <c r="AK264" t="inlineStr"/>
+      <c r="AL264" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-20
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL264"/>
+  <dimension ref="A1:AL271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32228,12 +32228,852 @@
       <c r="AF264" t="n">
         <v>11.5</v>
       </c>
-      <c r="AG264" t="inlineStr"/>
-      <c r="AH264" t="inlineStr"/>
-      <c r="AI264" t="inlineStr"/>
-      <c r="AJ264" t="inlineStr"/>
-      <c r="AK264" t="inlineStr"/>
-      <c r="AL264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>24209.3</v>
+      </c>
+      <c r="H265" t="n">
+        <v>76</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K265" t="n">
+        <v>6</v>
+      </c>
+      <c r="L265" t="n">
+        <v>24203</v>
+      </c>
+      <c r="M265" t="n">
+        <v>24198.8</v>
+      </c>
+      <c r="N265" t="n">
+        <v>24207.6</v>
+      </c>
+      <c r="O265" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q265" t="n">
+        <v>24225.2</v>
+      </c>
+      <c r="R265" t="n">
+        <v>24185.1</v>
+      </c>
+      <c r="S265" t="n">
+        <v>24166.9</v>
+      </c>
+      <c r="T265" t="n">
+        <v>24026.1</v>
+      </c>
+      <c r="U265" t="n">
+        <v>24096.5</v>
+      </c>
+      <c r="V265" t="n">
+        <v>24084.4</v>
+      </c>
+      <c r="W265" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y265" t="n">
+        <v>24209.9</v>
+      </c>
+      <c r="Z265" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA265" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB265" t="n">
+        <v>24169.3</v>
+      </c>
+      <c r="AC265" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD265" t="n">
+        <v>24329.3</v>
+      </c>
+      <c r="AE265" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF265" t="n">
+        <v>10.78</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>57644.2</v>
+      </c>
+      <c r="H266" t="n">
+        <v>78</v>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K266" t="n">
+        <v>6</v>
+      </c>
+      <c r="L266" t="n">
+        <v>57622.2</v>
+      </c>
+      <c r="M266" t="n">
+        <v>57589.1</v>
+      </c>
+      <c r="N266" t="n">
+        <v>57645.2</v>
+      </c>
+      <c r="O266" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q266" t="n">
+        <v>57600</v>
+      </c>
+      <c r="R266" t="n">
+        <v>57496.4</v>
+      </c>
+      <c r="S266" t="n">
+        <v>57323.4</v>
+      </c>
+      <c r="T266" t="n">
+        <v>57001.8</v>
+      </c>
+      <c r="U266" t="n">
+        <v>57214</v>
+      </c>
+      <c r="V266" t="n">
+        <v>57162.6</v>
+      </c>
+      <c r="W266" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y266" t="n">
+        <v>57640.9</v>
+      </c>
+      <c r="Z266" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AA266" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB266" t="n">
+        <v>57524.2</v>
+      </c>
+      <c r="AC266" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD266" t="n">
+        <v>58004.2</v>
+      </c>
+      <c r="AE266" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF266" t="n">
+        <v>10.78</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>57661.8</v>
+      </c>
+      <c r="H267" t="n">
+        <v>93</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K267" t="n">
+        <v>7</v>
+      </c>
+      <c r="L267" t="n">
+        <v>57630.7</v>
+      </c>
+      <c r="M267" t="n">
+        <v>57595.9</v>
+      </c>
+      <c r="N267" t="n">
+        <v>57659.8</v>
+      </c>
+      <c r="O267" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q267" t="n">
+        <v>57600</v>
+      </c>
+      <c r="R267" t="n">
+        <v>57496.4</v>
+      </c>
+      <c r="S267" t="n">
+        <v>57323.4</v>
+      </c>
+      <c r="T267" t="n">
+        <v>57001.8</v>
+      </c>
+      <c r="U267" t="n">
+        <v>57214</v>
+      </c>
+      <c r="V267" t="n">
+        <v>57162.6</v>
+      </c>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y267" t="n">
+        <v>57640.9</v>
+      </c>
+      <c r="Z267" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AA267" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB267" t="n">
+        <v>57541.8</v>
+      </c>
+      <c r="AC267" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD267" t="n">
+        <v>58021.8</v>
+      </c>
+      <c r="AE267" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF267" t="n">
+        <v>10.78</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G268" t="n">
+        <v>77466.10000000001</v>
+      </c>
+      <c r="H268" t="n">
+        <v>91</v>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K268" t="n">
+        <v>7</v>
+      </c>
+      <c r="L268" t="n">
+        <v>77444.8</v>
+      </c>
+      <c r="M268" t="n">
+        <v>77425.3</v>
+      </c>
+      <c r="N268" t="n">
+        <v>77462.7</v>
+      </c>
+      <c r="O268" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q268" t="n">
+        <v>77492.89999999999</v>
+      </c>
+      <c r="R268" t="n">
+        <v>77382</v>
+      </c>
+      <c r="S268" t="n">
+        <v>77270.39999999999</v>
+      </c>
+      <c r="T268" t="n">
+        <v>76702.5</v>
+      </c>
+      <c r="U268" t="n">
+        <v>76986.39999999999</v>
+      </c>
+      <c r="V268" t="n">
+        <v>76935.3</v>
+      </c>
+      <c r="W268" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y268" t="n">
+        <v>77473.39999999999</v>
+      </c>
+      <c r="Z268" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="AA268" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB268" t="n">
+        <v>77266.10000000001</v>
+      </c>
+      <c r="AC268" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD268" t="n">
+        <v>78066.10000000001</v>
+      </c>
+      <c r="AE268" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF268" t="n">
+        <v>10.78</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G269" t="n">
+        <v>24209</v>
+      </c>
+      <c r="H269" t="n">
+        <v>76</v>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K269" t="n">
+        <v>6</v>
+      </c>
+      <c r="L269" t="n">
+        <v>24209.6</v>
+      </c>
+      <c r="M269" t="n">
+        <v>24205.5</v>
+      </c>
+      <c r="N269" t="n">
+        <v>24207.8</v>
+      </c>
+      <c r="O269" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q269" t="n">
+        <v>24225.2</v>
+      </c>
+      <c r="R269" t="n">
+        <v>24185.1</v>
+      </c>
+      <c r="S269" t="n">
+        <v>24166.9</v>
+      </c>
+      <c r="T269" t="n">
+        <v>24026.1</v>
+      </c>
+      <c r="U269" t="n">
+        <v>24096.5</v>
+      </c>
+      <c r="V269" t="n">
+        <v>24084.4</v>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y269" t="n">
+        <v>24210.8</v>
+      </c>
+      <c r="Z269" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AA269" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB269" t="n">
+        <v>24169</v>
+      </c>
+      <c r="AC269" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD269" t="n">
+        <v>24329</v>
+      </c>
+      <c r="AE269" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF269" t="n">
+        <v>10.74</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G270" t="n">
+        <v>57633.1</v>
+      </c>
+      <c r="H270" t="n">
+        <v>81</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K270" t="n">
+        <v>6</v>
+      </c>
+      <c r="L270" t="n">
+        <v>57638.1</v>
+      </c>
+      <c r="M270" t="n">
+        <v>57616.8</v>
+      </c>
+      <c r="N270" t="n">
+        <v>57633.8</v>
+      </c>
+      <c r="O270" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q270" t="n">
+        <v>57600</v>
+      </c>
+      <c r="R270" t="n">
+        <v>57496.4</v>
+      </c>
+      <c r="S270" t="n">
+        <v>57323.4</v>
+      </c>
+      <c r="T270" t="n">
+        <v>57001.8</v>
+      </c>
+      <c r="U270" t="n">
+        <v>57214</v>
+      </c>
+      <c r="V270" t="n">
+        <v>57162.6</v>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y270" t="n">
+        <v>57621.5</v>
+      </c>
+      <c r="Z270" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB270" t="n">
+        <v>57513.1</v>
+      </c>
+      <c r="AC270" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD270" t="n">
+        <v>57993.1</v>
+      </c>
+      <c r="AE270" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF270" t="n">
+        <v>10.74</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G271" t="n">
+        <v>77484.60000000001</v>
+      </c>
+      <c r="H271" t="n">
+        <v>91</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K271" t="n">
+        <v>7</v>
+      </c>
+      <c r="L271" t="n">
+        <v>77473.89999999999</v>
+      </c>
+      <c r="M271" t="n">
+        <v>77450</v>
+      </c>
+      <c r="N271" t="n">
+        <v>77478.60000000001</v>
+      </c>
+      <c r="O271" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q271" t="n">
+        <v>77492.89999999999</v>
+      </c>
+      <c r="R271" t="n">
+        <v>77382</v>
+      </c>
+      <c r="S271" t="n">
+        <v>77270.39999999999</v>
+      </c>
+      <c r="T271" t="n">
+        <v>76702.5</v>
+      </c>
+      <c r="U271" t="n">
+        <v>76986.39999999999</v>
+      </c>
+      <c r="V271" t="n">
+        <v>76935.3</v>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y271" t="n">
+        <v>77481.7</v>
+      </c>
+      <c r="Z271" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AA271" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB271" t="n">
+        <v>77284.60000000001</v>
+      </c>
+      <c r="AC271" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD271" t="n">
+        <v>78084.60000000001</v>
+      </c>
+      <c r="AE271" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF271" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="AG271" t="inlineStr"/>
+      <c r="AH271" t="inlineStr"/>
+      <c r="AI271" t="inlineStr"/>
+      <c r="AJ271" t="inlineStr"/>
+      <c r="AK271" t="inlineStr"/>
+      <c r="AL271" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-21
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL271"/>
+  <dimension ref="A1:AL277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33068,12 +33068,732 @@
       <c r="AF271" t="n">
         <v>10.74</v>
       </c>
-      <c r="AG271" t="inlineStr"/>
-      <c r="AH271" t="inlineStr"/>
-      <c r="AI271" t="inlineStr"/>
-      <c r="AJ271" t="inlineStr"/>
-      <c r="AK271" t="inlineStr"/>
-      <c r="AL271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G272" t="n">
+        <v>57654.9</v>
+      </c>
+      <c r="H272" t="n">
+        <v>86</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K272" t="n">
+        <v>6</v>
+      </c>
+      <c r="L272" t="n">
+        <v>57654.6</v>
+      </c>
+      <c r="M272" t="n">
+        <v>57624.4</v>
+      </c>
+      <c r="N272" t="n">
+        <v>57646.5</v>
+      </c>
+      <c r="O272" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q272" t="n">
+        <v>57619.7</v>
+      </c>
+      <c r="R272" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="S272" t="n">
+        <v>57698.9</v>
+      </c>
+      <c r="T272" t="n">
+        <v>57435.3</v>
+      </c>
+      <c r="U272" t="n">
+        <v>57567.1</v>
+      </c>
+      <c r="V272" t="n">
+        <v>57519.6</v>
+      </c>
+      <c r="W272" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X272" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y272" t="n">
+        <v>57661.5</v>
+      </c>
+      <c r="Z272" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AA272" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB272" t="n">
+        <v>57534.9</v>
+      </c>
+      <c r="AC272" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD272" t="n">
+        <v>58014.9</v>
+      </c>
+      <c r="AE272" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF272" t="n">
+        <v>11.14</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G273" t="n">
+        <v>57723</v>
+      </c>
+      <c r="H273" t="n">
+        <v>93</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K273" t="n">
+        <v>7</v>
+      </c>
+      <c r="L273" t="n">
+        <v>57683.6</v>
+      </c>
+      <c r="M273" t="n">
+        <v>57652.5</v>
+      </c>
+      <c r="N273" t="n">
+        <v>57716.2</v>
+      </c>
+      <c r="O273" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q273" t="n">
+        <v>57619.7</v>
+      </c>
+      <c r="R273" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="S273" t="n">
+        <v>57698.9</v>
+      </c>
+      <c r="T273" t="n">
+        <v>57435.3</v>
+      </c>
+      <c r="U273" t="n">
+        <v>57567.1</v>
+      </c>
+      <c r="V273" t="n">
+        <v>57519.6</v>
+      </c>
+      <c r="W273" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X273" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y273" t="n">
+        <v>57703.8</v>
+      </c>
+      <c r="Z273" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB273" t="n">
+        <v>57603</v>
+      </c>
+      <c r="AC273" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD273" t="n">
+        <v>58083</v>
+      </c>
+      <c r="AE273" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF273" t="n">
+        <v>11.16</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>77615.8</v>
+      </c>
+      <c r="H274" t="n">
+        <v>76</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K274" t="n">
+        <v>6</v>
+      </c>
+      <c r="L274" t="n">
+        <v>77590.39999999999</v>
+      </c>
+      <c r="M274" t="n">
+        <v>77568.89999999999</v>
+      </c>
+      <c r="N274" t="n">
+        <v>77611.89999999999</v>
+      </c>
+      <c r="O274" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q274" t="n">
+        <v>77701.10000000001</v>
+      </c>
+      <c r="R274" t="n">
+        <v>77448.8</v>
+      </c>
+      <c r="S274" t="n">
+        <v>77610.5</v>
+      </c>
+      <c r="T274" t="n">
+        <v>77372.2</v>
+      </c>
+      <c r="U274" t="n">
+        <v>77522.3</v>
+      </c>
+      <c r="V274" t="n">
+        <v>77491.39999999999</v>
+      </c>
+      <c r="W274" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X274" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y274" t="n">
+        <v>77604.7</v>
+      </c>
+      <c r="Z274" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AA274" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB274" t="n">
+        <v>77415.8</v>
+      </c>
+      <c r="AC274" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD274" t="n">
+        <v>78215.8</v>
+      </c>
+      <c r="AE274" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF274" t="n">
+        <v>11.03</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G275" t="n">
+        <v>57710.6</v>
+      </c>
+      <c r="H275" t="n">
+        <v>93</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K275" t="n">
+        <v>7</v>
+      </c>
+      <c r="L275" t="n">
+        <v>57707.9</v>
+      </c>
+      <c r="M275" t="n">
+        <v>57681.3</v>
+      </c>
+      <c r="N275" t="n">
+        <v>57704.5</v>
+      </c>
+      <c r="O275" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q275" t="n">
+        <v>57619.7</v>
+      </c>
+      <c r="R275" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="S275" t="n">
+        <v>57698.9</v>
+      </c>
+      <c r="T275" t="n">
+        <v>57435.3</v>
+      </c>
+      <c r="U275" t="n">
+        <v>57567.1</v>
+      </c>
+      <c r="V275" t="n">
+        <v>57519.6</v>
+      </c>
+      <c r="W275" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y275" t="n">
+        <v>57703.8</v>
+      </c>
+      <c r="Z275" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA275" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB275" t="n">
+        <v>57590.6</v>
+      </c>
+      <c r="AC275" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD275" t="n">
+        <v>58070.6</v>
+      </c>
+      <c r="AE275" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF275" t="n">
+        <v>11.11</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>11:48</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>57701.4</v>
+      </c>
+      <c r="H276" t="n">
+        <v>78</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K276" t="n">
+        <v>6</v>
+      </c>
+      <c r="L276" t="n">
+        <v>57706.6</v>
+      </c>
+      <c r="M276" t="n">
+        <v>57693.6</v>
+      </c>
+      <c r="N276" t="n">
+        <v>57705.7</v>
+      </c>
+      <c r="O276" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q276" t="n">
+        <v>57619.7</v>
+      </c>
+      <c r="R276" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="S276" t="n">
+        <v>57698.9</v>
+      </c>
+      <c r="T276" t="n">
+        <v>57435.3</v>
+      </c>
+      <c r="U276" t="n">
+        <v>57567.1</v>
+      </c>
+      <c r="V276" t="n">
+        <v>57519.6</v>
+      </c>
+      <c r="W276" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y276" t="n">
+        <v>57703.8</v>
+      </c>
+      <c r="Z276" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AA276" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB276" t="n">
+        <v>57581.4</v>
+      </c>
+      <c r="AC276" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD276" t="n">
+        <v>58061.4</v>
+      </c>
+      <c r="AE276" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF276" t="n">
+        <v>11.06</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>57700</v>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G277" t="n">
+        <v>57676.6</v>
+      </c>
+      <c r="H277" t="n">
+        <v>81</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K277" t="n">
+        <v>6</v>
+      </c>
+      <c r="L277" t="n">
+        <v>57671.1</v>
+      </c>
+      <c r="M277" t="n">
+        <v>57676</v>
+      </c>
+      <c r="N277" t="n">
+        <v>57670.7</v>
+      </c>
+      <c r="O277" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q277" t="n">
+        <v>57619.7</v>
+      </c>
+      <c r="R277" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="S277" t="n">
+        <v>57698.9</v>
+      </c>
+      <c r="T277" t="n">
+        <v>57435.3</v>
+      </c>
+      <c r="U277" t="n">
+        <v>57567.1</v>
+      </c>
+      <c r="V277" t="n">
+        <v>57519.6</v>
+      </c>
+      <c r="W277" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y277" t="n">
+        <v>57661.5</v>
+      </c>
+      <c r="Z277" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB277" t="n">
+        <v>57556.6</v>
+      </c>
+      <c r="AC277" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD277" t="n">
+        <v>58036.6</v>
+      </c>
+      <c r="AE277" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF277" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="AG277" t="inlineStr"/>
+      <c r="AH277" t="inlineStr"/>
+      <c r="AI277" t="inlineStr"/>
+      <c r="AJ277" t="inlineStr"/>
+      <c r="AK277" t="inlineStr"/>
+      <c r="AL277" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-24
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL277"/>
+  <dimension ref="A1:AL283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33788,12 +33788,732 @@
       <c r="AF277" t="n">
         <v>11.31</v>
       </c>
-      <c r="AG277" t="inlineStr"/>
-      <c r="AH277" t="inlineStr"/>
-      <c r="AI277" t="inlineStr"/>
-      <c r="AJ277" t="inlineStr"/>
-      <c r="AK277" t="inlineStr"/>
-      <c r="AL277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G278" t="n">
+        <v>77613.2</v>
+      </c>
+      <c r="H278" t="n">
+        <v>77</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K278" t="n">
+        <v>5</v>
+      </c>
+      <c r="L278" t="n">
+        <v>77666.7</v>
+      </c>
+      <c r="M278" t="n">
+        <v>77699.8</v>
+      </c>
+      <c r="N278" t="n">
+        <v>77622.8</v>
+      </c>
+      <c r="O278" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q278" t="n">
+        <v>77785.5</v>
+      </c>
+      <c r="R278" t="n">
+        <v>77644.10000000001</v>
+      </c>
+      <c r="S278" t="n">
+        <v>77701.10000000001</v>
+      </c>
+      <c r="T278" t="n">
+        <v>77386.3</v>
+      </c>
+      <c r="U278" t="n">
+        <v>77543.7</v>
+      </c>
+      <c r="V278" t="n">
+        <v>77541.8</v>
+      </c>
+      <c r="W278" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y278" t="n">
+        <v>77649.60000000001</v>
+      </c>
+      <c r="Z278" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AA278" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB278" t="n">
+        <v>77813.2</v>
+      </c>
+      <c r="AC278" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD278" t="n">
+        <v>77013.2</v>
+      </c>
+      <c r="AE278" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF278" t="n">
+        <v>11.29</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G279" t="n">
+        <v>24230.4</v>
+      </c>
+      <c r="H279" t="n">
+        <v>83</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K279" t="n">
+        <v>6</v>
+      </c>
+      <c r="L279" t="n">
+        <v>24261.1</v>
+      </c>
+      <c r="M279" t="n">
+        <v>24272.9</v>
+      </c>
+      <c r="N279" t="n">
+        <v>24237.6</v>
+      </c>
+      <c r="O279" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q279" t="n">
+        <v>24312.8</v>
+      </c>
+      <c r="R279" t="n">
+        <v>24276.8</v>
+      </c>
+      <c r="S279" t="n">
+        <v>24282</v>
+      </c>
+      <c r="T279" t="n">
+        <v>24206.9</v>
+      </c>
+      <c r="U279" t="n">
+        <v>24249.5</v>
+      </c>
+      <c r="V279" t="n">
+        <v>24244.5</v>
+      </c>
+      <c r="W279" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y279" t="n">
+        <v>24247.6</v>
+      </c>
+      <c r="Z279" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="AA279" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB279" t="n">
+        <v>24270.4</v>
+      </c>
+      <c r="AC279" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD279" t="n">
+        <v>24110.4</v>
+      </c>
+      <c r="AE279" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF279" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G280" t="n">
+        <v>57513</v>
+      </c>
+      <c r="H280" t="n">
+        <v>83</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K280" t="n">
+        <v>6</v>
+      </c>
+      <c r="L280" t="n">
+        <v>57607.6</v>
+      </c>
+      <c r="M280" t="n">
+        <v>57667</v>
+      </c>
+      <c r="N280" t="n">
+        <v>57530.5</v>
+      </c>
+      <c r="O280" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q280" t="n">
+        <v>57873.8</v>
+      </c>
+      <c r="R280" t="n">
+        <v>57778.3</v>
+      </c>
+      <c r="S280" t="n">
+        <v>57772.2</v>
+      </c>
+      <c r="T280" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="U280" t="n">
+        <v>57717</v>
+      </c>
+      <c r="V280" t="n">
+        <v>57627.2</v>
+      </c>
+      <c r="W280" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y280" t="n">
+        <v>57593.9</v>
+      </c>
+      <c r="Z280" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="AA280" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB280" t="n">
+        <v>57633</v>
+      </c>
+      <c r="AC280" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD280" t="n">
+        <v>57153</v>
+      </c>
+      <c r="AE280" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF280" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>77500</v>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G281" t="n">
+        <v>77471.2</v>
+      </c>
+      <c r="H281" t="n">
+        <v>83</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K281" t="n">
+        <v>6</v>
+      </c>
+      <c r="L281" t="n">
+        <v>77579.39999999999</v>
+      </c>
+      <c r="M281" t="n">
+        <v>77624.60000000001</v>
+      </c>
+      <c r="N281" t="n">
+        <v>77495</v>
+      </c>
+      <c r="O281" t="n">
+        <v>14</v>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q281" t="n">
+        <v>77785.5</v>
+      </c>
+      <c r="R281" t="n">
+        <v>77644.10000000001</v>
+      </c>
+      <c r="S281" t="n">
+        <v>77701.10000000001</v>
+      </c>
+      <c r="T281" t="n">
+        <v>77386.3</v>
+      </c>
+      <c r="U281" t="n">
+        <v>77543.7</v>
+      </c>
+      <c r="V281" t="n">
+        <v>77541.8</v>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X281" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y281" t="n">
+        <v>77545.39999999999</v>
+      </c>
+      <c r="Z281" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="AA281" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB281" t="n">
+        <v>77671.2</v>
+      </c>
+      <c r="AC281" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD281" t="n">
+        <v>76871.2</v>
+      </c>
+      <c r="AE281" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF281" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>24200</v>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G282" t="n">
+        <v>24204.3</v>
+      </c>
+      <c r="H282" t="n">
+        <v>93</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K282" t="n">
+        <v>7</v>
+      </c>
+      <c r="L282" t="n">
+        <v>24231.9</v>
+      </c>
+      <c r="M282" t="n">
+        <v>24253.7</v>
+      </c>
+      <c r="N282" t="n">
+        <v>24207.3</v>
+      </c>
+      <c r="O282" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q282" t="n">
+        <v>24312.8</v>
+      </c>
+      <c r="R282" t="n">
+        <v>24276.8</v>
+      </c>
+      <c r="S282" t="n">
+        <v>24282</v>
+      </c>
+      <c r="T282" t="n">
+        <v>24206.9</v>
+      </c>
+      <c r="U282" t="n">
+        <v>24249.5</v>
+      </c>
+      <c r="V282" t="n">
+        <v>24244.5</v>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X282" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y282" t="n">
+        <v>24224.3</v>
+      </c>
+      <c r="Z282" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="AA282" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB282" t="n">
+        <v>24244.3</v>
+      </c>
+      <c r="AC282" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD282" t="n">
+        <v>24084.3</v>
+      </c>
+      <c r="AE282" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF282" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>57300</v>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G283" t="n">
+        <v>57345.6</v>
+      </c>
+      <c r="H283" t="n">
+        <v>90</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K283" t="n">
+        <v>6</v>
+      </c>
+      <c r="L283" t="n">
+        <v>57442.9</v>
+      </c>
+      <c r="M283" t="n">
+        <v>57546.5</v>
+      </c>
+      <c r="N283" t="n">
+        <v>57355.7</v>
+      </c>
+      <c r="O283" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q283" t="n">
+        <v>57873.8</v>
+      </c>
+      <c r="R283" t="n">
+        <v>57778.3</v>
+      </c>
+      <c r="S283" t="n">
+        <v>57772.2</v>
+      </c>
+      <c r="T283" t="n">
+        <v>57482.2</v>
+      </c>
+      <c r="U283" t="n">
+        <v>57717</v>
+      </c>
+      <c r="V283" t="n">
+        <v>57627.2</v>
+      </c>
+      <c r="W283" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X283" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y283" t="n">
+        <v>57459.5</v>
+      </c>
+      <c r="Z283" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="AA283" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB283" t="n">
+        <v>57465.6</v>
+      </c>
+      <c r="AC283" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD283" t="n">
+        <v>56985.6</v>
+      </c>
+      <c r="AE283" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF283" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="AG283" t="inlineStr"/>
+      <c r="AH283" t="inlineStr"/>
+      <c r="AI283" t="inlineStr"/>
+      <c r="AJ283" t="inlineStr"/>
+      <c r="AK283" t="inlineStr"/>
+      <c r="AL283" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-25
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL283"/>
+  <dimension ref="A1:AL289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34508,12 +34508,732 @@
       <c r="AF283" t="n">
         <v>11.57</v>
       </c>
-      <c r="AG283" t="inlineStr"/>
-      <c r="AH283" t="inlineStr"/>
-      <c r="AI283" t="inlineStr"/>
-      <c r="AJ283" t="inlineStr"/>
-      <c r="AK283" t="inlineStr"/>
-      <c r="AL283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G284" t="n">
+        <v>24138.1</v>
+      </c>
+      <c r="H284" t="n">
+        <v>81</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K284" t="n">
+        <v>6</v>
+      </c>
+      <c r="L284" t="n">
+        <v>24153</v>
+      </c>
+      <c r="M284" t="n">
+        <v>24165.8</v>
+      </c>
+      <c r="N284" t="n">
+        <v>24141.9</v>
+      </c>
+      <c r="O284" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q284" t="n">
+        <v>24198.1</v>
+      </c>
+      <c r="R284" t="n">
+        <v>24129.2</v>
+      </c>
+      <c r="S284" t="n">
+        <v>24312.8</v>
+      </c>
+      <c r="T284" t="n">
+        <v>24144.4</v>
+      </c>
+      <c r="U284" t="n">
+        <v>24228.6</v>
+      </c>
+      <c r="V284" t="n">
+        <v>24222.3</v>
+      </c>
+      <c r="W284" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X284" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y284" t="n">
+        <v>24145.4</v>
+      </c>
+      <c r="Z284" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA284" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB284" t="n">
+        <v>24178.1</v>
+      </c>
+      <c r="AC284" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD284" t="n">
+        <v>24018.1</v>
+      </c>
+      <c r="AE284" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF284" t="n">
+        <v>11.35</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>77200</v>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G285" t="n">
+        <v>77182</v>
+      </c>
+      <c r="H285" t="n">
+        <v>81</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K285" t="n">
+        <v>6</v>
+      </c>
+      <c r="L285" t="n">
+        <v>77274.3</v>
+      </c>
+      <c r="M285" t="n">
+        <v>77300.7</v>
+      </c>
+      <c r="N285" t="n">
+        <v>77202.39999999999</v>
+      </c>
+      <c r="O285" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q285" t="n">
+        <v>77378.39999999999</v>
+      </c>
+      <c r="R285" t="n">
+        <v>77152.2</v>
+      </c>
+      <c r="S285" t="n">
+        <v>77785.5</v>
+      </c>
+      <c r="T285" t="n">
+        <v>77201.7</v>
+      </c>
+      <c r="U285" t="n">
+        <v>77493.60000000001</v>
+      </c>
+      <c r="V285" t="n">
+        <v>77410.60000000001</v>
+      </c>
+      <c r="W285" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X285" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y285" t="n">
+        <v>77205.60000000001</v>
+      </c>
+      <c r="Z285" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="AA285" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB285" t="n">
+        <v>77382</v>
+      </c>
+      <c r="AC285" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD285" t="n">
+        <v>76582</v>
+      </c>
+      <c r="AE285" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF285" t="n">
+        <v>11.35</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G286" t="n">
+        <v>24128.4</v>
+      </c>
+      <c r="H286" t="n">
+        <v>78</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K286" t="n">
+        <v>6</v>
+      </c>
+      <c r="L286" t="n">
+        <v>24135.1</v>
+      </c>
+      <c r="M286" t="n">
+        <v>24149.9</v>
+      </c>
+      <c r="N286" t="n">
+        <v>24130.3</v>
+      </c>
+      <c r="O286" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q286" t="n">
+        <v>24198.1</v>
+      </c>
+      <c r="R286" t="n">
+        <v>24129.2</v>
+      </c>
+      <c r="S286" t="n">
+        <v>24312.8</v>
+      </c>
+      <c r="T286" t="n">
+        <v>24144.4</v>
+      </c>
+      <c r="U286" t="n">
+        <v>24228.6</v>
+      </c>
+      <c r="V286" t="n">
+        <v>24222.3</v>
+      </c>
+      <c r="W286" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X286" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y286" t="n">
+        <v>24135</v>
+      </c>
+      <c r="Z286" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AA286" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB286" t="n">
+        <v>24168.4</v>
+      </c>
+      <c r="AC286" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD286" t="n">
+        <v>24008.4</v>
+      </c>
+      <c r="AE286" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF286" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>77100</v>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G287" t="n">
+        <v>77148.3</v>
+      </c>
+      <c r="H287" t="n">
+        <v>78</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K287" t="n">
+        <v>6</v>
+      </c>
+      <c r="L287" t="n">
+        <v>77203.10000000001</v>
+      </c>
+      <c r="M287" t="n">
+        <v>77248.89999999999</v>
+      </c>
+      <c r="N287" t="n">
+        <v>77158.5</v>
+      </c>
+      <c r="O287" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q287" t="n">
+        <v>77378.39999999999</v>
+      </c>
+      <c r="R287" t="n">
+        <v>77152.2</v>
+      </c>
+      <c r="S287" t="n">
+        <v>77785.5</v>
+      </c>
+      <c r="T287" t="n">
+        <v>77201.7</v>
+      </c>
+      <c r="U287" t="n">
+        <v>77493.60000000001</v>
+      </c>
+      <c r="V287" t="n">
+        <v>77410.60000000001</v>
+      </c>
+      <c r="W287" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y287" t="n">
+        <v>77202.60000000001</v>
+      </c>
+      <c r="Z287" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="AA287" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB287" t="n">
+        <v>77348.3</v>
+      </c>
+      <c r="AC287" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD287" t="n">
+        <v>76548.3</v>
+      </c>
+      <c r="AE287" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF287" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>57600</v>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G288" t="n">
+        <v>57586.6</v>
+      </c>
+      <c r="H288" t="n">
+        <v>83</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K288" t="n">
+        <v>6</v>
+      </c>
+      <c r="L288" t="n">
+        <v>57488.4</v>
+      </c>
+      <c r="M288" t="n">
+        <v>57480.4</v>
+      </c>
+      <c r="N288" t="n">
+        <v>57559.5</v>
+      </c>
+      <c r="O288" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q288" t="n">
+        <v>57568.4</v>
+      </c>
+      <c r="R288" t="n">
+        <v>57231.6</v>
+      </c>
+      <c r="S288" t="n">
+        <v>57873.8</v>
+      </c>
+      <c r="T288" t="n">
+        <v>57248.9</v>
+      </c>
+      <c r="U288" t="n">
+        <v>57561.3</v>
+      </c>
+      <c r="V288" t="n">
+        <v>57537.7</v>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X288" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y288" t="n">
+        <v>57554.2</v>
+      </c>
+      <c r="Z288" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB288" t="n">
+        <v>57466.6</v>
+      </c>
+      <c r="AC288" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD288" t="n">
+        <v>57946.6</v>
+      </c>
+      <c r="AE288" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF288" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>77200</v>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G289" t="n">
+        <v>77181.5</v>
+      </c>
+      <c r="H289" t="n">
+        <v>76</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>6</v>
+      </c>
+      <c r="L289" t="n">
+        <v>77202.5</v>
+      </c>
+      <c r="M289" t="n">
+        <v>77220.3</v>
+      </c>
+      <c r="N289" t="n">
+        <v>77185.89999999999</v>
+      </c>
+      <c r="O289" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q289" t="n">
+        <v>77378.39999999999</v>
+      </c>
+      <c r="R289" t="n">
+        <v>77152.2</v>
+      </c>
+      <c r="S289" t="n">
+        <v>77785.5</v>
+      </c>
+      <c r="T289" t="n">
+        <v>77201.7</v>
+      </c>
+      <c r="U289" t="n">
+        <v>77493.60000000001</v>
+      </c>
+      <c r="V289" t="n">
+        <v>77410.60000000001</v>
+      </c>
+      <c r="W289" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X289" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y289" t="n">
+        <v>77185.89999999999</v>
+      </c>
+      <c r="Z289" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AA289" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB289" t="n">
+        <v>77381.5</v>
+      </c>
+      <c r="AC289" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD289" t="n">
+        <v>76581.5</v>
+      </c>
+      <c r="AE289" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF289" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="AG289" t="inlineStr"/>
+      <c r="AH289" t="inlineStr"/>
+      <c r="AI289" t="inlineStr"/>
+      <c r="AJ289" t="inlineStr"/>
+      <c r="AK289" t="inlineStr"/>
+      <c r="AL289" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-08-26
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL289"/>
+  <dimension ref="A1:AL295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35228,12 +35228,732 @@
       <c r="AF289" t="n">
         <v>11.45</v>
       </c>
-      <c r="AG289" t="inlineStr"/>
-      <c r="AH289" t="inlineStr"/>
-      <c r="AI289" t="inlineStr"/>
-      <c r="AJ289" t="inlineStr"/>
-      <c r="AK289" t="inlineStr"/>
-      <c r="AL289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>24300</v>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G290" t="n">
+        <v>24282.2</v>
+      </c>
+      <c r="H290" t="n">
+        <v>83</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K290" t="n">
+        <v>6</v>
+      </c>
+      <c r="L290" t="n">
+        <v>24284.7</v>
+      </c>
+      <c r="M290" t="n">
+        <v>24295.1</v>
+      </c>
+      <c r="N290" t="n">
+        <v>24282.3</v>
+      </c>
+      <c r="O290" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q290" t="n">
+        <v>24362.9</v>
+      </c>
+      <c r="R290" t="n">
+        <v>24309.9</v>
+      </c>
+      <c r="S290" t="n">
+        <v>24334.6</v>
+      </c>
+      <c r="T290" t="n">
+        <v>24115.6</v>
+      </c>
+      <c r="U290" t="n">
+        <v>24298.1</v>
+      </c>
+      <c r="V290" t="n">
+        <v>24225.1</v>
+      </c>
+      <c r="W290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X290" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y290" t="n">
+        <v>24289.4</v>
+      </c>
+      <c r="Z290" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA290" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB290" t="n">
+        <v>24322.2</v>
+      </c>
+      <c r="AC290" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD290" t="n">
+        <v>24162.2</v>
+      </c>
+      <c r="AE290" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF290" t="n">
+        <v>10.92</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D291" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>77700</v>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G291" t="n">
+        <v>77684.7</v>
+      </c>
+      <c r="H291" t="n">
+        <v>83</v>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K291" t="n">
+        <v>6</v>
+      </c>
+      <c r="L291" t="n">
+        <v>77689.89999999999</v>
+      </c>
+      <c r="M291" t="n">
+        <v>77726</v>
+      </c>
+      <c r="N291" t="n">
+        <v>77686.3</v>
+      </c>
+      <c r="O291" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q291" t="n">
+        <v>77948.3</v>
+      </c>
+      <c r="R291" t="n">
+        <v>77805.60000000001</v>
+      </c>
+      <c r="S291" t="n">
+        <v>77676.89999999999</v>
+      </c>
+      <c r="T291" t="n">
+        <v>77126.39999999999</v>
+      </c>
+      <c r="U291" t="n">
+        <v>77571.3</v>
+      </c>
+      <c r="V291" t="n">
+        <v>77401.7</v>
+      </c>
+      <c r="W291" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X291" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y291" t="n">
+        <v>77701.89999999999</v>
+      </c>
+      <c r="Z291" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AA291" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB291" t="n">
+        <v>77884.7</v>
+      </c>
+      <c r="AC291" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD291" t="n">
+        <v>77084.7</v>
+      </c>
+      <c r="AE291" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF291" t="n">
+        <v>10.92</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G292" t="n">
+        <v>57956.4</v>
+      </c>
+      <c r="H292" t="n">
+        <v>83</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K292" t="n">
+        <v>7</v>
+      </c>
+      <c r="L292" t="n">
+        <v>57944.6</v>
+      </c>
+      <c r="M292" t="n">
+        <v>57929.6</v>
+      </c>
+      <c r="N292" t="n">
+        <v>57952.5</v>
+      </c>
+      <c r="O292" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q292" t="n">
+        <v>57995.7</v>
+      </c>
+      <c r="R292" t="n">
+        <v>57636</v>
+      </c>
+      <c r="S292" t="n">
+        <v>57653.9</v>
+      </c>
+      <c r="T292" t="n">
+        <v>57231.6</v>
+      </c>
+      <c r="U292" t="n">
+        <v>57490.4</v>
+      </c>
+      <c r="V292" t="n">
+        <v>57442.8</v>
+      </c>
+      <c r="W292" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X292" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y292" t="n">
+        <v>57910.8</v>
+      </c>
+      <c r="Z292" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="AA292" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB292" t="n">
+        <v>57836.4</v>
+      </c>
+      <c r="AC292" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD292" t="n">
+        <v>58316.4</v>
+      </c>
+      <c r="AE292" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF292" t="n">
+        <v>10.92</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D293" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>24250</v>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G293" t="n">
+        <v>24269.3</v>
+      </c>
+      <c r="H293" t="n">
+        <v>83</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K293" t="n">
+        <v>6</v>
+      </c>
+      <c r="L293" t="n">
+        <v>24276.6</v>
+      </c>
+      <c r="M293" t="n">
+        <v>24285.4</v>
+      </c>
+      <c r="N293" t="n">
+        <v>24271</v>
+      </c>
+      <c r="O293" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q293" t="n">
+        <v>24362.9</v>
+      </c>
+      <c r="R293" t="n">
+        <v>24309.9</v>
+      </c>
+      <c r="S293" t="n">
+        <v>24334.6</v>
+      </c>
+      <c r="T293" t="n">
+        <v>24115.6</v>
+      </c>
+      <c r="U293" t="n">
+        <v>24298.1</v>
+      </c>
+      <c r="V293" t="n">
+        <v>24225.1</v>
+      </c>
+      <c r="W293" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X293" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y293" t="n">
+        <v>24289.4</v>
+      </c>
+      <c r="Z293" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="AA293" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB293" t="n">
+        <v>24309.3</v>
+      </c>
+      <c r="AC293" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD293" t="n">
+        <v>24149.3</v>
+      </c>
+      <c r="AE293" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF293" t="n">
+        <v>10.83</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>13:16</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>77700</v>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G294" t="n">
+        <v>77651.8</v>
+      </c>
+      <c r="H294" t="n">
+        <v>83</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K294" t="n">
+        <v>6</v>
+      </c>
+      <c r="L294" t="n">
+        <v>77669.39999999999</v>
+      </c>
+      <c r="M294" t="n">
+        <v>77695.3</v>
+      </c>
+      <c r="N294" t="n">
+        <v>77657.89999999999</v>
+      </c>
+      <c r="O294" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q294" t="n">
+        <v>77948.3</v>
+      </c>
+      <c r="R294" t="n">
+        <v>77805.60000000001</v>
+      </c>
+      <c r="S294" t="n">
+        <v>77676.89999999999</v>
+      </c>
+      <c r="T294" t="n">
+        <v>77126.39999999999</v>
+      </c>
+      <c r="U294" t="n">
+        <v>77571.3</v>
+      </c>
+      <c r="V294" t="n">
+        <v>77401.7</v>
+      </c>
+      <c r="W294" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X294" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y294" t="n">
+        <v>77701.89999999999</v>
+      </c>
+      <c r="Z294" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="AA294" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB294" t="n">
+        <v>77851.8</v>
+      </c>
+      <c r="AC294" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD294" t="n">
+        <v>77051.8</v>
+      </c>
+      <c r="AE294" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF294" t="n">
+        <v>10.83</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>77600</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G295" t="n">
+        <v>77591.60000000001</v>
+      </c>
+      <c r="H295" t="n">
+        <v>83</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K295" t="n">
+        <v>6</v>
+      </c>
+      <c r="L295" t="n">
+        <v>77617.7</v>
+      </c>
+      <c r="M295" t="n">
+        <v>77655</v>
+      </c>
+      <c r="N295" t="n">
+        <v>77593.39999999999</v>
+      </c>
+      <c r="O295" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q295" t="n">
+        <v>77948.3</v>
+      </c>
+      <c r="R295" t="n">
+        <v>77805.60000000001</v>
+      </c>
+      <c r="S295" t="n">
+        <v>77676.89999999999</v>
+      </c>
+      <c r="T295" t="n">
+        <v>77126.39999999999</v>
+      </c>
+      <c r="U295" t="n">
+        <v>77571.3</v>
+      </c>
+      <c r="V295" t="n">
+        <v>77401.7</v>
+      </c>
+      <c r="W295" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X295" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y295" t="n">
+        <v>77657.10000000001</v>
+      </c>
+      <c r="Z295" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AA295" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB295" t="n">
+        <v>77791.60000000001</v>
+      </c>
+      <c r="AC295" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD295" t="n">
+        <v>76991.60000000001</v>
+      </c>
+      <c r="AE295" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF295" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="AG295" t="inlineStr"/>
+      <c r="AH295" t="inlineStr"/>
+      <c r="AI295" t="inlineStr"/>
+      <c r="AJ295" t="inlineStr"/>
+      <c r="AK295" t="inlineStr"/>
+      <c r="AL295" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-01
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL295"/>
+  <dimension ref="A1:AL299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35948,12 +35948,492 @@
       <c r="AF295" t="n">
         <v>10.83</v>
       </c>
-      <c r="AG295" t="inlineStr"/>
-      <c r="AH295" t="inlineStr"/>
-      <c r="AI295" t="inlineStr"/>
-      <c r="AJ295" t="inlineStr"/>
-      <c r="AK295" t="inlineStr"/>
-      <c r="AL295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D296" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>23950</v>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G296" t="n">
+        <v>23962.6</v>
+      </c>
+      <c r="H296" t="n">
+        <v>93</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K296" t="n">
+        <v>7</v>
+      </c>
+      <c r="L296" t="n">
+        <v>23977.2</v>
+      </c>
+      <c r="M296" t="n">
+        <v>24006</v>
+      </c>
+      <c r="N296" t="n">
+        <v>23964.5</v>
+      </c>
+      <c r="O296" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q296" t="n">
+        <v>24077.1</v>
+      </c>
+      <c r="R296" t="n">
+        <v>24028</v>
+      </c>
+      <c r="S296" t="n">
+        <v>24126.6</v>
+      </c>
+      <c r="T296" t="n">
+        <v>23993.8</v>
+      </c>
+      <c r="U296" t="n">
+        <v>24073.7</v>
+      </c>
+      <c r="V296" t="n">
+        <v>24060.2</v>
+      </c>
+      <c r="W296" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X296" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y296" t="n">
+        <v>23982</v>
+      </c>
+      <c r="Z296" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="AA296" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB296" t="n">
+        <v>24002.6</v>
+      </c>
+      <c r="AC296" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD296" t="n">
+        <v>23842.6</v>
+      </c>
+      <c r="AE296" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF296" t="n">
+        <v>11.81</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D297" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G297" t="n">
+        <v>76675.8</v>
+      </c>
+      <c r="H297" t="n">
+        <v>93</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K297" t="n">
+        <v>7</v>
+      </c>
+      <c r="L297" t="n">
+        <v>76743.39999999999</v>
+      </c>
+      <c r="M297" t="n">
+        <v>76855.60000000001</v>
+      </c>
+      <c r="N297" t="n">
+        <v>76676.60000000001</v>
+      </c>
+      <c r="O297" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q297" t="n">
+        <v>77029.3</v>
+      </c>
+      <c r="R297" t="n">
+        <v>76837.60000000001</v>
+      </c>
+      <c r="S297" t="n">
+        <v>77147.5</v>
+      </c>
+      <c r="T297" t="n">
+        <v>76751.3</v>
+      </c>
+      <c r="U297" t="n">
+        <v>76954.60000000001</v>
+      </c>
+      <c r="V297" t="n">
+        <v>76949.39999999999</v>
+      </c>
+      <c r="W297" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X297" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y297" t="n">
+        <v>76744.39999999999</v>
+      </c>
+      <c r="Z297" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA297" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB297" t="n">
+        <v>76875.8</v>
+      </c>
+      <c r="AC297" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD297" t="n">
+        <v>76075.8</v>
+      </c>
+      <c r="AE297" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF297" t="n">
+        <v>11.81</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G298" t="n">
+        <v>23976.7</v>
+      </c>
+      <c r="H298" t="n">
+        <v>88</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K298" t="n">
+        <v>7</v>
+      </c>
+      <c r="L298" t="n">
+        <v>23975.8</v>
+      </c>
+      <c r="M298" t="n">
+        <v>23992.7</v>
+      </c>
+      <c r="N298" t="n">
+        <v>23971.8</v>
+      </c>
+      <c r="O298" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q298" t="n">
+        <v>24077.1</v>
+      </c>
+      <c r="R298" t="n">
+        <v>24028</v>
+      </c>
+      <c r="S298" t="n">
+        <v>24126.6</v>
+      </c>
+      <c r="T298" t="n">
+        <v>23993.8</v>
+      </c>
+      <c r="U298" t="n">
+        <v>24073.7</v>
+      </c>
+      <c r="V298" t="n">
+        <v>24060.2</v>
+      </c>
+      <c r="W298" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X298" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y298" t="n">
+        <v>23982</v>
+      </c>
+      <c r="Z298" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AA298" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB298" t="n">
+        <v>24016.7</v>
+      </c>
+      <c r="AC298" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD298" t="n">
+        <v>23856.7</v>
+      </c>
+      <c r="AE298" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF298" t="n">
+        <v>11.78</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>76700</v>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G299" t="n">
+        <v>76744</v>
+      </c>
+      <c r="H299" t="n">
+        <v>100</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K299" t="n">
+        <v>8</v>
+      </c>
+      <c r="L299" t="n">
+        <v>76734</v>
+      </c>
+      <c r="M299" t="n">
+        <v>76801.8</v>
+      </c>
+      <c r="N299" t="n">
+        <v>76753.8</v>
+      </c>
+      <c r="O299" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q299" t="n">
+        <v>77029.3</v>
+      </c>
+      <c r="R299" t="n">
+        <v>76837.60000000001</v>
+      </c>
+      <c r="S299" t="n">
+        <v>77147.5</v>
+      </c>
+      <c r="T299" t="n">
+        <v>76751.3</v>
+      </c>
+      <c r="U299" t="n">
+        <v>76954.60000000001</v>
+      </c>
+      <c r="V299" t="n">
+        <v>76949.39999999999</v>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y299" t="n">
+        <v>76744.39999999999</v>
+      </c>
+      <c r="Z299" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AA299" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB299" t="n">
+        <v>76944</v>
+      </c>
+      <c r="AC299" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD299" t="n">
+        <v>76144</v>
+      </c>
+      <c r="AE299" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF299" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="AG299" t="inlineStr"/>
+      <c r="AH299" t="inlineStr"/>
+      <c r="AI299" t="inlineStr"/>
+      <c r="AJ299" t="inlineStr"/>
+      <c r="AK299" t="inlineStr"/>
+      <c r="AL299" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-02
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL299"/>
+  <dimension ref="A1:AL306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36428,12 +36428,852 @@
       <c r="AF299" t="n">
         <v>11.78</v>
       </c>
-      <c r="AG299" t="inlineStr"/>
-      <c r="AH299" t="inlineStr"/>
-      <c r="AI299" t="inlineStr"/>
-      <c r="AJ299" t="inlineStr"/>
-      <c r="AK299" t="inlineStr"/>
-      <c r="AL299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>23850</v>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G300" t="n">
+        <v>23868.1</v>
+      </c>
+      <c r="H300" t="n">
+        <v>75</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K300" t="n">
+        <v>5</v>
+      </c>
+      <c r="L300" t="n">
+        <v>23867.3</v>
+      </c>
+      <c r="M300" t="n">
+        <v>23860.4</v>
+      </c>
+      <c r="N300" t="n">
+        <v>23867.9</v>
+      </c>
+      <c r="O300" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q300" t="n">
+        <v>23879.4</v>
+      </c>
+      <c r="R300" t="n">
+        <v>23788.1</v>
+      </c>
+      <c r="S300" t="n">
+        <v>24142.8</v>
+      </c>
+      <c r="T300" t="n">
+        <v>23952.6</v>
+      </c>
+      <c r="U300" t="n">
+        <v>24053.1</v>
+      </c>
+      <c r="V300" t="n">
+        <v>24047.7</v>
+      </c>
+      <c r="W300" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y300" t="n">
+        <v>23870.2</v>
+      </c>
+      <c r="Z300" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="AA300" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB300" t="n">
+        <v>23828.1</v>
+      </c>
+      <c r="AC300" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD300" t="n">
+        <v>23988.1</v>
+      </c>
+      <c r="AE300" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF300" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G301" t="n">
+        <v>57114.1</v>
+      </c>
+      <c r="H301" t="n">
+        <v>87</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K301" t="n">
+        <v>6</v>
+      </c>
+      <c r="L301" t="n">
+        <v>57070.9</v>
+      </c>
+      <c r="M301" t="n">
+        <v>57065.1</v>
+      </c>
+      <c r="N301" t="n">
+        <v>57107</v>
+      </c>
+      <c r="O301" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q301" t="n">
+        <v>57065.6</v>
+      </c>
+      <c r="R301" t="n">
+        <v>56824.8</v>
+      </c>
+      <c r="S301" t="n">
+        <v>57765.9</v>
+      </c>
+      <c r="T301" t="n">
+        <v>57150.7</v>
+      </c>
+      <c r="U301" t="n">
+        <v>57458.3</v>
+      </c>
+      <c r="V301" t="n">
+        <v>57425.8</v>
+      </c>
+      <c r="W301" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y301" t="n">
+        <v>57126.7</v>
+      </c>
+      <c r="Z301" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AA301" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB301" t="n">
+        <v>56994.1</v>
+      </c>
+      <c r="AC301" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD301" t="n">
+        <v>57474.1</v>
+      </c>
+      <c r="AE301" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF301" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G302" t="n">
+        <v>23894.1</v>
+      </c>
+      <c r="H302" t="n">
+        <v>87</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K302" t="n">
+        <v>6</v>
+      </c>
+      <c r="L302" t="n">
+        <v>23874.3</v>
+      </c>
+      <c r="M302" t="n">
+        <v>23864.9</v>
+      </c>
+      <c r="N302" t="n">
+        <v>23886.8</v>
+      </c>
+      <c r="O302" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q302" t="n">
+        <v>23879.4</v>
+      </c>
+      <c r="R302" t="n">
+        <v>23788.1</v>
+      </c>
+      <c r="S302" t="n">
+        <v>24142.8</v>
+      </c>
+      <c r="T302" t="n">
+        <v>23952.6</v>
+      </c>
+      <c r="U302" t="n">
+        <v>24053.1</v>
+      </c>
+      <c r="V302" t="n">
+        <v>24047.7</v>
+      </c>
+      <c r="W302" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X302" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y302" t="n">
+        <v>23870.2</v>
+      </c>
+      <c r="Z302" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AA302" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB302" t="n">
+        <v>23854.1</v>
+      </c>
+      <c r="AC302" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD302" t="n">
+        <v>24014.1</v>
+      </c>
+      <c r="AE302" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF302" t="n">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G303" t="n">
+        <v>76484.5</v>
+      </c>
+      <c r="H303" t="n">
+        <v>75</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K303" t="n">
+        <v>5</v>
+      </c>
+      <c r="L303" t="n">
+        <v>76438.8</v>
+      </c>
+      <c r="M303" t="n">
+        <v>76412</v>
+      </c>
+      <c r="N303" t="n">
+        <v>76470.3</v>
+      </c>
+      <c r="O303" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q303" t="n">
+        <v>76494.39999999999</v>
+      </c>
+      <c r="R303" t="n">
+        <v>76135.7</v>
+      </c>
+      <c r="S303" t="n">
+        <v>77231.89999999999</v>
+      </c>
+      <c r="T303" t="n">
+        <v>76656.39999999999</v>
+      </c>
+      <c r="U303" t="n">
+        <v>76944.2</v>
+      </c>
+      <c r="V303" t="n">
+        <v>76944.10000000001</v>
+      </c>
+      <c r="W303" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y303" t="n">
+        <v>76439.2</v>
+      </c>
+      <c r="Z303" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AA303" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB303" t="n">
+        <v>76284.5</v>
+      </c>
+      <c r="AC303" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD303" t="n">
+        <v>77084.5</v>
+      </c>
+      <c r="AE303" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF303" t="n">
+        <v>11.62</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G304" t="n">
+        <v>57113.4</v>
+      </c>
+      <c r="H304" t="n">
+        <v>87</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K304" t="n">
+        <v>6</v>
+      </c>
+      <c r="L304" t="n">
+        <v>57096.4</v>
+      </c>
+      <c r="M304" t="n">
+        <v>57083.4</v>
+      </c>
+      <c r="N304" t="n">
+        <v>57106.9</v>
+      </c>
+      <c r="O304" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q304" t="n">
+        <v>57065.6</v>
+      </c>
+      <c r="R304" t="n">
+        <v>56824.8</v>
+      </c>
+      <c r="S304" t="n">
+        <v>57765.9</v>
+      </c>
+      <c r="T304" t="n">
+        <v>57150.7</v>
+      </c>
+      <c r="U304" t="n">
+        <v>57458.3</v>
+      </c>
+      <c r="V304" t="n">
+        <v>57425.8</v>
+      </c>
+      <c r="W304" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X304" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y304" t="n">
+        <v>57126.7</v>
+      </c>
+      <c r="Z304" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA304" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB304" t="n">
+        <v>56993.4</v>
+      </c>
+      <c r="AC304" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD304" t="n">
+        <v>57473.4</v>
+      </c>
+      <c r="AE304" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF304" t="n">
+        <v>11.71</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G305" t="n">
+        <v>23898.8</v>
+      </c>
+      <c r="H305" t="n">
+        <v>87</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K305" t="n">
+        <v>6</v>
+      </c>
+      <c r="L305" t="n">
+        <v>23889.7</v>
+      </c>
+      <c r="M305" t="n">
+        <v>23878.9</v>
+      </c>
+      <c r="N305" t="n">
+        <v>23893.3</v>
+      </c>
+      <c r="O305" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q305" t="n">
+        <v>23879.4</v>
+      </c>
+      <c r="R305" t="n">
+        <v>23788.1</v>
+      </c>
+      <c r="S305" t="n">
+        <v>24142.8</v>
+      </c>
+      <c r="T305" t="n">
+        <v>23952.6</v>
+      </c>
+      <c r="U305" t="n">
+        <v>24053.1</v>
+      </c>
+      <c r="V305" t="n">
+        <v>24047.7</v>
+      </c>
+      <c r="W305" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X305" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y305" t="n">
+        <v>23881.6</v>
+      </c>
+      <c r="Z305" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB305" t="n">
+        <v>23858.8</v>
+      </c>
+      <c r="AC305" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD305" t="n">
+        <v>24018.8</v>
+      </c>
+      <c r="AE305" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF305" t="n">
+        <v>11.66</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G306" t="n">
+        <v>76521.5</v>
+      </c>
+      <c r="H306" t="n">
+        <v>87</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K306" t="n">
+        <v>6</v>
+      </c>
+      <c r="L306" t="n">
+        <v>76478.8</v>
+      </c>
+      <c r="M306" t="n">
+        <v>76446.60000000001</v>
+      </c>
+      <c r="N306" t="n">
+        <v>76511.8</v>
+      </c>
+      <c r="O306" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q306" t="n">
+        <v>76494.39999999999</v>
+      </c>
+      <c r="R306" t="n">
+        <v>76135.7</v>
+      </c>
+      <c r="S306" t="n">
+        <v>77231.89999999999</v>
+      </c>
+      <c r="T306" t="n">
+        <v>76656.39999999999</v>
+      </c>
+      <c r="U306" t="n">
+        <v>76944.2</v>
+      </c>
+      <c r="V306" t="n">
+        <v>76944.10000000001</v>
+      </c>
+      <c r="W306" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X306" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y306" t="n">
+        <v>76439.2</v>
+      </c>
+      <c r="Z306" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="AA306" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB306" t="n">
+        <v>76321.5</v>
+      </c>
+      <c r="AC306" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD306" t="n">
+        <v>77121.5</v>
+      </c>
+      <c r="AE306" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF306" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="AG306" t="inlineStr"/>
+      <c r="AH306" t="inlineStr"/>
+      <c r="AI306" t="inlineStr"/>
+      <c r="AJ306" t="inlineStr"/>
+      <c r="AK306" t="inlineStr"/>
+      <c r="AL306" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-03
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL306"/>
+  <dimension ref="A1:AL311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37268,12 +37268,612 @@
       <c r="AF306" t="n">
         <v>11.66</v>
       </c>
-      <c r="AG306" t="inlineStr"/>
-      <c r="AH306" t="inlineStr"/>
-      <c r="AI306" t="inlineStr"/>
-      <c r="AJ306" t="inlineStr"/>
-      <c r="AK306" t="inlineStr"/>
-      <c r="AL306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G307" t="n">
+        <v>23910.8</v>
+      </c>
+      <c r="H307" t="n">
+        <v>87</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K307" t="n">
+        <v>6</v>
+      </c>
+      <c r="L307" t="n">
+        <v>23913.4</v>
+      </c>
+      <c r="M307" t="n">
+        <v>23919.4</v>
+      </c>
+      <c r="N307" t="n">
+        <v>23913.2</v>
+      </c>
+      <c r="O307" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q307" t="n">
+        <v>24018.8</v>
+      </c>
+      <c r="R307" t="n">
+        <v>23955.4</v>
+      </c>
+      <c r="S307" t="n">
+        <v>23914.4</v>
+      </c>
+      <c r="T307" t="n">
+        <v>23788.1</v>
+      </c>
+      <c r="U307" t="n">
+        <v>23893.4</v>
+      </c>
+      <c r="V307" t="n">
+        <v>23851.2</v>
+      </c>
+      <c r="W307" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X307" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y307" t="n">
+        <v>23924</v>
+      </c>
+      <c r="Z307" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AA307" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB307" t="n">
+        <v>23950.8</v>
+      </c>
+      <c r="AC307" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD307" t="n">
+        <v>23790.8</v>
+      </c>
+      <c r="AE307" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF307" t="n">
+        <v>11.18</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D308" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>76600</v>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G308" t="n">
+        <v>76601.5</v>
+      </c>
+      <c r="H308" t="n">
+        <v>87</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K308" t="n">
+        <v>6</v>
+      </c>
+      <c r="L308" t="n">
+        <v>76611.39999999999</v>
+      </c>
+      <c r="M308" t="n">
+        <v>76629.39999999999</v>
+      </c>
+      <c r="N308" t="n">
+        <v>76610.2</v>
+      </c>
+      <c r="O308" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q308" t="n">
+        <v>76918.7</v>
+      </c>
+      <c r="R308" t="n">
+        <v>76706.7</v>
+      </c>
+      <c r="S308" t="n">
+        <v>76572.39999999999</v>
+      </c>
+      <c r="T308" t="n">
+        <v>76135.7</v>
+      </c>
+      <c r="U308" t="n">
+        <v>76498.3</v>
+      </c>
+      <c r="V308" t="n">
+        <v>76354.10000000001</v>
+      </c>
+      <c r="W308" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X308" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y308" t="n">
+        <v>76638.5</v>
+      </c>
+      <c r="Z308" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AA308" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB308" t="n">
+        <v>76801.5</v>
+      </c>
+      <c r="AC308" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD308" t="n">
+        <v>76001.5</v>
+      </c>
+      <c r="AE308" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF308" t="n">
+        <v>11.18</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>14:37</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>23900</v>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G309" t="n">
+        <v>23915.2</v>
+      </c>
+      <c r="H309" t="n">
+        <v>87</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K309" t="n">
+        <v>6</v>
+      </c>
+      <c r="L309" t="n">
+        <v>23915.9</v>
+      </c>
+      <c r="M309" t="n">
+        <v>23918.1</v>
+      </c>
+      <c r="N309" t="n">
+        <v>23916.3</v>
+      </c>
+      <c r="O309" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q309" t="n">
+        <v>24018.8</v>
+      </c>
+      <c r="R309" t="n">
+        <v>23955.4</v>
+      </c>
+      <c r="S309" t="n">
+        <v>23914.4</v>
+      </c>
+      <c r="T309" t="n">
+        <v>23788.1</v>
+      </c>
+      <c r="U309" t="n">
+        <v>23893.4</v>
+      </c>
+      <c r="V309" t="n">
+        <v>23851.2</v>
+      </c>
+      <c r="W309" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X309" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y309" t="n">
+        <v>23924</v>
+      </c>
+      <c r="Z309" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB309" t="n">
+        <v>23955.2</v>
+      </c>
+      <c r="AC309" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD309" t="n">
+        <v>23795.2</v>
+      </c>
+      <c r="AE309" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF309" t="n">
+        <v>11.18</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D310" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>76600</v>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G310" t="n">
+        <v>76597.89999999999</v>
+      </c>
+      <c r="H310" t="n">
+        <v>87</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K310" t="n">
+        <v>6</v>
+      </c>
+      <c r="L310" t="n">
+        <v>76611.39999999999</v>
+      </c>
+      <c r="M310" t="n">
+        <v>76619.89999999999</v>
+      </c>
+      <c r="N310" t="n">
+        <v>76606.5</v>
+      </c>
+      <c r="O310" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q310" t="n">
+        <v>76918.7</v>
+      </c>
+      <c r="R310" t="n">
+        <v>76706.7</v>
+      </c>
+      <c r="S310" t="n">
+        <v>76572.39999999999</v>
+      </c>
+      <c r="T310" t="n">
+        <v>76135.7</v>
+      </c>
+      <c r="U310" t="n">
+        <v>76498.3</v>
+      </c>
+      <c r="V310" t="n">
+        <v>76354.10000000001</v>
+      </c>
+      <c r="W310" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X310" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y310" t="n">
+        <v>76638.5</v>
+      </c>
+      <c r="Z310" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AA310" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB310" t="n">
+        <v>76797.89999999999</v>
+      </c>
+      <c r="AC310" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD310" t="n">
+        <v>75997.89999999999</v>
+      </c>
+      <c r="AE310" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF310" t="n">
+        <v>11.21</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G311" t="n">
+        <v>76508.7</v>
+      </c>
+      <c r="H311" t="n">
+        <v>87</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K311" t="n">
+        <v>6</v>
+      </c>
+      <c r="L311" t="n">
+        <v>76550.7</v>
+      </c>
+      <c r="M311" t="n">
+        <v>76583.10000000001</v>
+      </c>
+      <c r="N311" t="n">
+        <v>76519.5</v>
+      </c>
+      <c r="O311" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q311" t="n">
+        <v>76918.7</v>
+      </c>
+      <c r="R311" t="n">
+        <v>76706.7</v>
+      </c>
+      <c r="S311" t="n">
+        <v>76572.39999999999</v>
+      </c>
+      <c r="T311" t="n">
+        <v>76135.7</v>
+      </c>
+      <c r="U311" t="n">
+        <v>76498.3</v>
+      </c>
+      <c r="V311" t="n">
+        <v>76354.10000000001</v>
+      </c>
+      <c r="W311" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X311" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y311" t="n">
+        <v>76571.2</v>
+      </c>
+      <c r="Z311" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB311" t="n">
+        <v>76708.7</v>
+      </c>
+      <c r="AC311" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD311" t="n">
+        <v>75908.7</v>
+      </c>
+      <c r="AE311" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF311" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="AG311" t="inlineStr"/>
+      <c r="AH311" t="inlineStr"/>
+      <c r="AI311" t="inlineStr"/>
+      <c r="AJ311" t="inlineStr"/>
+      <c r="AK311" t="inlineStr"/>
+      <c r="AL311" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-07
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL311"/>
+  <dimension ref="A1:AL315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37868,12 +37868,492 @@
       <c r="AF311" t="n">
         <v>11.27</v>
       </c>
-      <c r="AG311" t="inlineStr"/>
-      <c r="AH311" t="inlineStr"/>
-      <c r="AI311" t="inlineStr"/>
-      <c r="AJ311" t="inlineStr"/>
-      <c r="AK311" t="inlineStr"/>
-      <c r="AL311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>23750</v>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G312" t="n">
+        <v>23753</v>
+      </c>
+      <c r="H312" t="n">
+        <v>88</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K312" t="n">
+        <v>7</v>
+      </c>
+      <c r="L312" t="n">
+        <v>23761.6</v>
+      </c>
+      <c r="M312" t="n">
+        <v>23764.8</v>
+      </c>
+      <c r="N312" t="n">
+        <v>23753</v>
+      </c>
+      <c r="O312" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q312" t="n">
+        <v>23888.8</v>
+      </c>
+      <c r="R312" t="n">
+        <v>23819.2</v>
+      </c>
+      <c r="S312" t="n">
+        <v>24004.8</v>
+      </c>
+      <c r="T312" t="n">
+        <v>23896</v>
+      </c>
+      <c r="U312" t="n">
+        <v>23950.4</v>
+      </c>
+      <c r="V312" t="n">
+        <v>23915.3</v>
+      </c>
+      <c r="W312" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X312" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y312" t="n">
+        <v>23774.6</v>
+      </c>
+      <c r="Z312" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB312" t="n">
+        <v>23793</v>
+      </c>
+      <c r="AC312" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD312" t="n">
+        <v>23633</v>
+      </c>
+      <c r="AE312" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF312" t="n">
+        <v>11.04</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D313" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>76000</v>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G313" t="n">
+        <v>76023.7</v>
+      </c>
+      <c r="H313" t="n">
+        <v>88</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K313" t="n">
+        <v>7</v>
+      </c>
+      <c r="L313" t="n">
+        <v>76069.5</v>
+      </c>
+      <c r="M313" t="n">
+        <v>76072.7</v>
+      </c>
+      <c r="N313" t="n">
+        <v>76023.7</v>
+      </c>
+      <c r="O313" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="P313" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q313" t="n">
+        <v>76456.5</v>
+      </c>
+      <c r="R313" t="n">
+        <v>76252.7</v>
+      </c>
+      <c r="S313" t="n">
+        <v>76882.10000000001</v>
+      </c>
+      <c r="T313" t="n">
+        <v>76489.39999999999</v>
+      </c>
+      <c r="U313" t="n">
+        <v>76685.7</v>
+      </c>
+      <c r="V313" t="n">
+        <v>76572.2</v>
+      </c>
+      <c r="W313" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X313" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y313" t="n">
+        <v>76093</v>
+      </c>
+      <c r="Z313" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB313" t="n">
+        <v>76223.7</v>
+      </c>
+      <c r="AC313" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD313" t="n">
+        <v>75423.7</v>
+      </c>
+      <c r="AE313" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF313" t="n">
+        <v>11.04</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>23750</v>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G314" t="n">
+        <v>23760.3</v>
+      </c>
+      <c r="H314" t="n">
+        <v>88</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K314" t="n">
+        <v>7</v>
+      </c>
+      <c r="L314" t="n">
+        <v>23758.1</v>
+      </c>
+      <c r="M314" t="n">
+        <v>23760.8</v>
+      </c>
+      <c r="N314" t="n">
+        <v>23760.3</v>
+      </c>
+      <c r="O314" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P314" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q314" t="n">
+        <v>23888.8</v>
+      </c>
+      <c r="R314" t="n">
+        <v>23819.2</v>
+      </c>
+      <c r="S314" t="n">
+        <v>24004.8</v>
+      </c>
+      <c r="T314" t="n">
+        <v>23896</v>
+      </c>
+      <c r="U314" t="n">
+        <v>23950.4</v>
+      </c>
+      <c r="V314" t="n">
+        <v>23915.3</v>
+      </c>
+      <c r="W314" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X314" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y314" t="n">
+        <v>23773.6</v>
+      </c>
+      <c r="Z314" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="AA314" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB314" t="n">
+        <v>23800.3</v>
+      </c>
+      <c r="AC314" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD314" t="n">
+        <v>23640.3</v>
+      </c>
+      <c r="AE314" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF314" t="n">
+        <v>11.04</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>76000</v>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G315" t="n">
+        <v>76042.2</v>
+      </c>
+      <c r="H315" t="n">
+        <v>88</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K315" t="n">
+        <v>7</v>
+      </c>
+      <c r="L315" t="n">
+        <v>76030</v>
+      </c>
+      <c r="M315" t="n">
+        <v>76048.60000000001</v>
+      </c>
+      <c r="N315" t="n">
+        <v>76023.89999999999</v>
+      </c>
+      <c r="O315" t="n">
+        <v>47</v>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q315" t="n">
+        <v>76456.5</v>
+      </c>
+      <c r="R315" t="n">
+        <v>76252.7</v>
+      </c>
+      <c r="S315" t="n">
+        <v>76882.10000000001</v>
+      </c>
+      <c r="T315" t="n">
+        <v>76489.39999999999</v>
+      </c>
+      <c r="U315" t="n">
+        <v>76685.7</v>
+      </c>
+      <c r="V315" t="n">
+        <v>76572.2</v>
+      </c>
+      <c r="W315" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X315" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y315" t="n">
+        <v>76085.8</v>
+      </c>
+      <c r="Z315" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB315" t="n">
+        <v>76242.2</v>
+      </c>
+      <c r="AC315" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD315" t="n">
+        <v>75442.2</v>
+      </c>
+      <c r="AE315" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF315" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="AG315" t="inlineStr"/>
+      <c r="AH315" t="inlineStr"/>
+      <c r="AI315" t="inlineStr"/>
+      <c r="AJ315" t="inlineStr"/>
+      <c r="AK315" t="inlineStr"/>
+      <c r="AL315" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-08
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL315"/>
+  <dimension ref="A1:AL321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38348,12 +38348,732 @@
       <c r="AF315" t="n">
         <v>11.16</v>
       </c>
-      <c r="AG315" t="inlineStr"/>
-      <c r="AH315" t="inlineStr"/>
-      <c r="AI315" t="inlineStr"/>
-      <c r="AJ315" t="inlineStr"/>
-      <c r="AK315" t="inlineStr"/>
-      <c r="AL315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>14:09</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>23650</v>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G316" t="n">
+        <v>23648.4</v>
+      </c>
+      <c r="H316" t="n">
+        <v>88</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K316" t="n">
+        <v>7</v>
+      </c>
+      <c r="L316" t="n">
+        <v>23643.5</v>
+      </c>
+      <c r="M316" t="n">
+        <v>23649</v>
+      </c>
+      <c r="N316" t="n">
+        <v>23649.6</v>
+      </c>
+      <c r="O316" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q316" t="n">
+        <v>23755.6</v>
+      </c>
+      <c r="R316" t="n">
+        <v>23669.7</v>
+      </c>
+      <c r="S316" t="n">
+        <v>23888.8</v>
+      </c>
+      <c r="T316" t="n">
+        <v>23738.1</v>
+      </c>
+      <c r="U316" t="n">
+        <v>23813.4</v>
+      </c>
+      <c r="V316" t="n">
+        <v>23790.6</v>
+      </c>
+      <c r="W316" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X316" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y316" t="n">
+        <v>23654.5</v>
+      </c>
+      <c r="Z316" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AA316" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB316" t="n">
+        <v>23688.4</v>
+      </c>
+      <c r="AC316" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD316" t="n">
+        <v>23528.4</v>
+      </c>
+      <c r="AE316" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF316" t="n">
+        <v>11.24</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>14:09</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D317" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>56800</v>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G317" t="n">
+        <v>56770.4</v>
+      </c>
+      <c r="H317" t="n">
+        <v>100</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K317" t="n">
+        <v>8</v>
+      </c>
+      <c r="L317" t="n">
+        <v>56766.8</v>
+      </c>
+      <c r="M317" t="n">
+        <v>56783.3</v>
+      </c>
+      <c r="N317" t="n">
+        <v>56787.7</v>
+      </c>
+      <c r="O317" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q317" t="n">
+        <v>57041.4</v>
+      </c>
+      <c r="R317" t="n">
+        <v>56857.8</v>
+      </c>
+      <c r="S317" t="n">
+        <v>57426.2</v>
+      </c>
+      <c r="T317" t="n">
+        <v>57002.9</v>
+      </c>
+      <c r="U317" t="n">
+        <v>57214.6</v>
+      </c>
+      <c r="V317" t="n">
+        <v>57130.4</v>
+      </c>
+      <c r="W317" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X317" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y317" t="n">
+        <v>56796.7</v>
+      </c>
+      <c r="Z317" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="AA317" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB317" t="n">
+        <v>56890.4</v>
+      </c>
+      <c r="AC317" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD317" t="n">
+        <v>56410.4</v>
+      </c>
+      <c r="AE317" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF317" t="n">
+        <v>11.24</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>14:09</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>75600</v>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G318" t="n">
+        <v>75572.89999999999</v>
+      </c>
+      <c r="H318" t="n">
+        <v>93</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K318" t="n">
+        <v>7</v>
+      </c>
+      <c r="L318" t="n">
+        <v>75610.5</v>
+      </c>
+      <c r="M318" t="n">
+        <v>75636</v>
+      </c>
+      <c r="N318" t="n">
+        <v>75578</v>
+      </c>
+      <c r="O318" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q318" t="n">
+        <v>75988.2</v>
+      </c>
+      <c r="R318" t="n">
+        <v>75722.2</v>
+      </c>
+      <c r="S318" t="n">
+        <v>76456.5</v>
+      </c>
+      <c r="T318" t="n">
+        <v>75971.3</v>
+      </c>
+      <c r="U318" t="n">
+        <v>76213.89999999999</v>
+      </c>
+      <c r="V318" t="n">
+        <v>76159.8</v>
+      </c>
+      <c r="W318" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X318" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y318" t="n">
+        <v>75656.3</v>
+      </c>
+      <c r="Z318" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AA318" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB318" t="n">
+        <v>75772.89999999999</v>
+      </c>
+      <c r="AC318" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD318" t="n">
+        <v>74972.89999999999</v>
+      </c>
+      <c r="AE318" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF318" t="n">
+        <v>11.24</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>23650</v>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G319" t="n">
+        <v>23648.4</v>
+      </c>
+      <c r="H319" t="n">
+        <v>88</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K319" t="n">
+        <v>7</v>
+      </c>
+      <c r="L319" t="n">
+        <v>23649.8</v>
+      </c>
+      <c r="M319" t="n">
+        <v>23650.3</v>
+      </c>
+      <c r="N319" t="n">
+        <v>23651</v>
+      </c>
+      <c r="O319" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q319" t="n">
+        <v>23755.6</v>
+      </c>
+      <c r="R319" t="n">
+        <v>23669.7</v>
+      </c>
+      <c r="S319" t="n">
+        <v>23888.8</v>
+      </c>
+      <c r="T319" t="n">
+        <v>23738.1</v>
+      </c>
+      <c r="U319" t="n">
+        <v>23813.4</v>
+      </c>
+      <c r="V319" t="n">
+        <v>23790.6</v>
+      </c>
+      <c r="W319" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X319" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y319" t="n">
+        <v>23654.5</v>
+      </c>
+      <c r="Z319" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AA319" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB319" t="n">
+        <v>23688.4</v>
+      </c>
+      <c r="AC319" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD319" t="n">
+        <v>23528.4</v>
+      </c>
+      <c r="AE319" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF319" t="n">
+        <v>11.21</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D320" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>56800</v>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G320" t="n">
+        <v>56797.9</v>
+      </c>
+      <c r="H320" t="n">
+        <v>88</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K320" t="n">
+        <v>7</v>
+      </c>
+      <c r="L320" t="n">
+        <v>56796.8</v>
+      </c>
+      <c r="M320" t="n">
+        <v>56794</v>
+      </c>
+      <c r="N320" t="n">
+        <v>56804.7</v>
+      </c>
+      <c r="O320" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q320" t="n">
+        <v>57041.4</v>
+      </c>
+      <c r="R320" t="n">
+        <v>56857.8</v>
+      </c>
+      <c r="S320" t="n">
+        <v>57426.2</v>
+      </c>
+      <c r="T320" t="n">
+        <v>57002.9</v>
+      </c>
+      <c r="U320" t="n">
+        <v>57214.6</v>
+      </c>
+      <c r="V320" t="n">
+        <v>57130.4</v>
+      </c>
+      <c r="W320" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X320" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y320" t="n">
+        <v>56796.7</v>
+      </c>
+      <c r="Z320" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AA320" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB320" t="n">
+        <v>56917.9</v>
+      </c>
+      <c r="AC320" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD320" t="n">
+        <v>56437.9</v>
+      </c>
+      <c r="AE320" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF320" t="n">
+        <v>11.21</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D321" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>75600</v>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G321" t="n">
+        <v>75629.8</v>
+      </c>
+      <c r="H321" t="n">
+        <v>100</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K321" t="n">
+        <v>8</v>
+      </c>
+      <c r="L321" t="n">
+        <v>75625.10000000001</v>
+      </c>
+      <c r="M321" t="n">
+        <v>75632.5</v>
+      </c>
+      <c r="N321" t="n">
+        <v>75637.89999999999</v>
+      </c>
+      <c r="O321" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q321" t="n">
+        <v>75988.2</v>
+      </c>
+      <c r="R321" t="n">
+        <v>75722.2</v>
+      </c>
+      <c r="S321" t="n">
+        <v>76456.5</v>
+      </c>
+      <c r="T321" t="n">
+        <v>75971.3</v>
+      </c>
+      <c r="U321" t="n">
+        <v>76213.89999999999</v>
+      </c>
+      <c r="V321" t="n">
+        <v>76159.8</v>
+      </c>
+      <c r="W321" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X321" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y321" t="n">
+        <v>75656.3</v>
+      </c>
+      <c r="Z321" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AA321" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB321" t="n">
+        <v>75829.8</v>
+      </c>
+      <c r="AC321" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD321" t="n">
+        <v>75029.8</v>
+      </c>
+      <c r="AE321" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF321" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="AG321" t="inlineStr"/>
+      <c r="AH321" t="inlineStr"/>
+      <c r="AI321" t="inlineStr"/>
+      <c r="AJ321" t="inlineStr"/>
+      <c r="AK321" t="inlineStr"/>
+      <c r="AL321" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-09
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL321"/>
+  <dimension ref="A1:AL327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39068,12 +39068,732 @@
       <c r="AF321" t="n">
         <v>11.21</v>
       </c>
-      <c r="AG321" t="inlineStr"/>
-      <c r="AH321" t="inlineStr"/>
-      <c r="AI321" t="inlineStr"/>
-      <c r="AJ321" t="inlineStr"/>
-      <c r="AK321" t="inlineStr"/>
-      <c r="AL321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>23550</v>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G322" t="n">
+        <v>23554.8</v>
+      </c>
+      <c r="H322" t="n">
+        <v>87</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K322" t="n">
+        <v>6</v>
+      </c>
+      <c r="L322" t="n">
+        <v>23552.3</v>
+      </c>
+      <c r="M322" t="n">
+        <v>23545.6</v>
+      </c>
+      <c r="N322" t="n">
+        <v>23553.1</v>
+      </c>
+      <c r="O322" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q322" t="n">
+        <v>23531.8</v>
+      </c>
+      <c r="R322" t="n">
+        <v>23478.9</v>
+      </c>
+      <c r="S322" t="n">
+        <v>23755.6</v>
+      </c>
+      <c r="T322" t="n">
+        <v>23623.2</v>
+      </c>
+      <c r="U322" t="n">
+        <v>23689.4</v>
+      </c>
+      <c r="V322" t="n">
+        <v>23653.2</v>
+      </c>
+      <c r="W322" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X322" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y322" t="n">
+        <v>23549.5</v>
+      </c>
+      <c r="Z322" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA322" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB322" t="n">
+        <v>23514.8</v>
+      </c>
+      <c r="AC322" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD322" t="n">
+        <v>23674.8</v>
+      </c>
+      <c r="AE322" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF322" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>56700</v>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G323" t="n">
+        <v>56650.6</v>
+      </c>
+      <c r="H323" t="n">
+        <v>87</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K323" t="n">
+        <v>6</v>
+      </c>
+      <c r="L323" t="n">
+        <v>56665.7</v>
+      </c>
+      <c r="M323" t="n">
+        <v>56647.3</v>
+      </c>
+      <c r="N323" t="n">
+        <v>56649.6</v>
+      </c>
+      <c r="O323" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q323" t="n">
+        <v>56615.5</v>
+      </c>
+      <c r="R323" t="n">
+        <v>56416.9</v>
+      </c>
+      <c r="S323" t="n">
+        <v>57041.4</v>
+      </c>
+      <c r="T323" t="n">
+        <v>56721.1</v>
+      </c>
+      <c r="U323" t="n">
+        <v>56881.2</v>
+      </c>
+      <c r="V323" t="n">
+        <v>56812.1</v>
+      </c>
+      <c r="W323" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X323" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y323" t="n">
+        <v>56665.9</v>
+      </c>
+      <c r="Z323" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AA323" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB323" t="n">
+        <v>56530.6</v>
+      </c>
+      <c r="AC323" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD323" t="n">
+        <v>57010.6</v>
+      </c>
+      <c r="AE323" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF323" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>75200</v>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G324" t="n">
+        <v>75200.7</v>
+      </c>
+      <c r="H324" t="n">
+        <v>87</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K324" t="n">
+        <v>6</v>
+      </c>
+      <c r="L324" t="n">
+        <v>75171.2</v>
+      </c>
+      <c r="M324" t="n">
+        <v>75146.8</v>
+      </c>
+      <c r="N324" t="n">
+        <v>75190</v>
+      </c>
+      <c r="O324" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="P324" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q324" t="n">
+        <v>75179.39999999999</v>
+      </c>
+      <c r="R324" t="n">
+        <v>74970.60000000001</v>
+      </c>
+      <c r="S324" t="n">
+        <v>75988.2</v>
+      </c>
+      <c r="T324" t="n">
+        <v>75540.8</v>
+      </c>
+      <c r="U324" t="n">
+        <v>75764.5</v>
+      </c>
+      <c r="V324" t="n">
+        <v>75639.89999999999</v>
+      </c>
+      <c r="W324" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X324" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y324" t="n">
+        <v>75183.5</v>
+      </c>
+      <c r="Z324" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AA324" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB324" t="n">
+        <v>75000.7</v>
+      </c>
+      <c r="AC324" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD324" t="n">
+        <v>75800.7</v>
+      </c>
+      <c r="AE324" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF324" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D325" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>56600</v>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G325" t="n">
+        <v>56551.6</v>
+      </c>
+      <c r="H325" t="n">
+        <v>92</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K325" t="n">
+        <v>7</v>
+      </c>
+      <c r="L325" t="n">
+        <v>56625.7</v>
+      </c>
+      <c r="M325" t="n">
+        <v>56633.7</v>
+      </c>
+      <c r="N325" t="n">
+        <v>56559.2</v>
+      </c>
+      <c r="O325" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="P325" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q325" t="n">
+        <v>56615.5</v>
+      </c>
+      <c r="R325" t="n">
+        <v>56416.9</v>
+      </c>
+      <c r="S325" t="n">
+        <v>57041.4</v>
+      </c>
+      <c r="T325" t="n">
+        <v>56721.1</v>
+      </c>
+      <c r="U325" t="n">
+        <v>56881.2</v>
+      </c>
+      <c r="V325" t="n">
+        <v>56812.1</v>
+      </c>
+      <c r="W325" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X325" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="Y325" t="n">
+        <v>56539.6</v>
+      </c>
+      <c r="Z325" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AA325" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB325" t="n">
+        <v>56671.6</v>
+      </c>
+      <c r="AC325" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD325" t="n">
+        <v>56191.6</v>
+      </c>
+      <c r="AE325" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF325" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D326" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G326" t="n">
+        <v>74957.60000000001</v>
+      </c>
+      <c r="H326" t="n">
+        <v>93</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K326" t="n">
+        <v>7</v>
+      </c>
+      <c r="L326" t="n">
+        <v>75063.8</v>
+      </c>
+      <c r="M326" t="n">
+        <v>75102.2</v>
+      </c>
+      <c r="N326" t="n">
+        <v>74963.2</v>
+      </c>
+      <c r="O326" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="P326" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q326" t="n">
+        <v>75179.39999999999</v>
+      </c>
+      <c r="R326" t="n">
+        <v>74970.60000000001</v>
+      </c>
+      <c r="S326" t="n">
+        <v>75988.2</v>
+      </c>
+      <c r="T326" t="n">
+        <v>75540.8</v>
+      </c>
+      <c r="U326" t="n">
+        <v>75764.5</v>
+      </c>
+      <c r="V326" t="n">
+        <v>75639.89999999999</v>
+      </c>
+      <c r="W326" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X326" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y326" t="n">
+        <v>74977.7</v>
+      </c>
+      <c r="Z326" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AA326" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB326" t="n">
+        <v>75157.60000000001</v>
+      </c>
+      <c r="AC326" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD326" t="n">
+        <v>74357.60000000001</v>
+      </c>
+      <c r="AE326" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF326" t="n">
+        <v>11.71</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D327" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>23450</v>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G327" t="n">
+        <v>23474.2</v>
+      </c>
+      <c r="H327" t="n">
+        <v>93</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K327" t="n">
+        <v>7</v>
+      </c>
+      <c r="L327" t="n">
+        <v>23498.4</v>
+      </c>
+      <c r="M327" t="n">
+        <v>23516.6</v>
+      </c>
+      <c r="N327" t="n">
+        <v>23478.7</v>
+      </c>
+      <c r="O327" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="P327" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q327" t="n">
+        <v>23531.8</v>
+      </c>
+      <c r="R327" t="n">
+        <v>23478.9</v>
+      </c>
+      <c r="S327" t="n">
+        <v>23755.6</v>
+      </c>
+      <c r="T327" t="n">
+        <v>23623.2</v>
+      </c>
+      <c r="U327" t="n">
+        <v>23689.4</v>
+      </c>
+      <c r="V327" t="n">
+        <v>23653.2</v>
+      </c>
+      <c r="W327" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X327" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y327" t="n">
+        <v>23482.4</v>
+      </c>
+      <c r="Z327" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AA327" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB327" t="n">
+        <v>23514.2</v>
+      </c>
+      <c r="AC327" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD327" t="n">
+        <v>23354.2</v>
+      </c>
+      <c r="AE327" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF327" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="AG327" t="inlineStr"/>
+      <c r="AH327" t="inlineStr"/>
+      <c r="AI327" t="inlineStr"/>
+      <c r="AJ327" t="inlineStr"/>
+      <c r="AK327" t="inlineStr"/>
+      <c r="AL327" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-10
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL327"/>
+  <dimension ref="A1:AL333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39788,12 +39788,732 @@
       <c r="AF327" t="n">
         <v>11.71</v>
       </c>
-      <c r="AG327" t="inlineStr"/>
-      <c r="AH327" t="inlineStr"/>
-      <c r="AI327" t="inlineStr"/>
-      <c r="AJ327" t="inlineStr"/>
-      <c r="AK327" t="inlineStr"/>
-      <c r="AL327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D328" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>23400</v>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G328" t="n">
+        <v>23416.9</v>
+      </c>
+      <c r="H328" t="n">
+        <v>76</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K328" t="n">
+        <v>6</v>
+      </c>
+      <c r="L328" t="n">
+        <v>23426</v>
+      </c>
+      <c r="M328" t="n">
+        <v>23432.5</v>
+      </c>
+      <c r="N328" t="n">
+        <v>23418</v>
+      </c>
+      <c r="O328" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="P328" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q328" t="n">
+        <v>23489.7</v>
+      </c>
+      <c r="R328" t="n">
+        <v>23414.4</v>
+      </c>
+      <c r="S328" t="n">
+        <v>23571.3</v>
+      </c>
+      <c r="T328" t="n">
+        <v>23431.5</v>
+      </c>
+      <c r="U328" t="n">
+        <v>23501.4</v>
+      </c>
+      <c r="V328" t="n">
+        <v>23454.8</v>
+      </c>
+      <c r="W328" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X328" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y328" t="n">
+        <v>23423.6</v>
+      </c>
+      <c r="Z328" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AA328" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB328" t="n">
+        <v>23456.9</v>
+      </c>
+      <c r="AC328" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD328" t="n">
+        <v>23296.9</v>
+      </c>
+      <c r="AE328" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF328" t="n">
+        <v>11.86</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D329" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>23400</v>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G329" t="n">
+        <v>23415</v>
+      </c>
+      <c r="H329" t="n">
+        <v>91</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K329" t="n">
+        <v>7</v>
+      </c>
+      <c r="L329" t="n">
+        <v>23423.9</v>
+      </c>
+      <c r="M329" t="n">
+        <v>23431</v>
+      </c>
+      <c r="N329" t="n">
+        <v>23415.7</v>
+      </c>
+      <c r="O329" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="P329" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q329" t="n">
+        <v>23489.7</v>
+      </c>
+      <c r="R329" t="n">
+        <v>23414.4</v>
+      </c>
+      <c r="S329" t="n">
+        <v>23571.3</v>
+      </c>
+      <c r="T329" t="n">
+        <v>23431.5</v>
+      </c>
+      <c r="U329" t="n">
+        <v>23501.4</v>
+      </c>
+      <c r="V329" t="n">
+        <v>23454.8</v>
+      </c>
+      <c r="W329" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X329" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y329" t="n">
+        <v>23423.6</v>
+      </c>
+      <c r="Z329" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="AA329" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB329" t="n">
+        <v>23455</v>
+      </c>
+      <c r="AC329" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD329" t="n">
+        <v>23295</v>
+      </c>
+      <c r="AE329" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF329" t="n">
+        <v>11.86</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D330" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>74700</v>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G330" t="n">
+        <v>74718.10000000001</v>
+      </c>
+      <c r="H330" t="n">
+        <v>81</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K330" t="n">
+        <v>6</v>
+      </c>
+      <c r="L330" t="n">
+        <v>74751.2</v>
+      </c>
+      <c r="M330" t="n">
+        <v>74773.3</v>
+      </c>
+      <c r="N330" t="n">
+        <v>74722</v>
+      </c>
+      <c r="O330" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q330" t="n">
+        <v>74909.7</v>
+      </c>
+      <c r="R330" t="n">
+        <v>74711.2</v>
+      </c>
+      <c r="S330" t="n">
+        <v>75249.3</v>
+      </c>
+      <c r="T330" t="n">
+        <v>74745.3</v>
+      </c>
+      <c r="U330" t="n">
+        <v>74997.3</v>
+      </c>
+      <c r="V330" t="n">
+        <v>74841.89999999999</v>
+      </c>
+      <c r="W330" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X330" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y330" t="n">
+        <v>74723.60000000001</v>
+      </c>
+      <c r="Z330" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AA330" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB330" t="n">
+        <v>74918.10000000001</v>
+      </c>
+      <c r="AC330" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD330" t="n">
+        <v>74118.10000000001</v>
+      </c>
+      <c r="AE330" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF330" t="n">
+        <v>11.86</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D331" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>74700</v>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G331" t="n">
+        <v>74691.89999999999</v>
+      </c>
+      <c r="H331" t="n">
+        <v>93</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K331" t="n">
+        <v>7</v>
+      </c>
+      <c r="L331" t="n">
+        <v>74725.8</v>
+      </c>
+      <c r="M331" t="n">
+        <v>74751.39999999999</v>
+      </c>
+      <c r="N331" t="n">
+        <v>74695</v>
+      </c>
+      <c r="O331" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="P331" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q331" t="n">
+        <v>74909.7</v>
+      </c>
+      <c r="R331" t="n">
+        <v>74711.2</v>
+      </c>
+      <c r="S331" t="n">
+        <v>75249.3</v>
+      </c>
+      <c r="T331" t="n">
+        <v>74745.3</v>
+      </c>
+      <c r="U331" t="n">
+        <v>74997.3</v>
+      </c>
+      <c r="V331" t="n">
+        <v>74841.89999999999</v>
+      </c>
+      <c r="W331" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X331" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y331" t="n">
+        <v>74723.60000000001</v>
+      </c>
+      <c r="Z331" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AA331" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB331" t="n">
+        <v>74891.89999999999</v>
+      </c>
+      <c r="AC331" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD331" t="n">
+        <v>74091.89999999999</v>
+      </c>
+      <c r="AE331" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF331" t="n">
+        <v>11.89</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D332" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>23400</v>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G332" t="n">
+        <v>23395.3</v>
+      </c>
+      <c r="H332" t="n">
+        <v>93</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K332" t="n">
+        <v>7</v>
+      </c>
+      <c r="L332" t="n">
+        <v>23413.9</v>
+      </c>
+      <c r="M332" t="n">
+        <v>23421.1</v>
+      </c>
+      <c r="N332" t="n">
+        <v>23396.5</v>
+      </c>
+      <c r="O332" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="P332" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q332" t="n">
+        <v>23489.7</v>
+      </c>
+      <c r="R332" t="n">
+        <v>23414.4</v>
+      </c>
+      <c r="S332" t="n">
+        <v>23571.3</v>
+      </c>
+      <c r="T332" t="n">
+        <v>23431.5</v>
+      </c>
+      <c r="U332" t="n">
+        <v>23501.4</v>
+      </c>
+      <c r="V332" t="n">
+        <v>23454.8</v>
+      </c>
+      <c r="W332" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X332" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y332" t="n">
+        <v>23407.4</v>
+      </c>
+      <c r="Z332" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="AA332" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB332" t="n">
+        <v>23435.3</v>
+      </c>
+      <c r="AC332" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD332" t="n">
+        <v>23275.3</v>
+      </c>
+      <c r="AE332" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF332" t="n">
+        <v>11.89</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D333" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>56200</v>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G333" t="n">
+        <v>56247.7</v>
+      </c>
+      <c r="H333" t="n">
+        <v>93</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K333" t="n">
+        <v>7</v>
+      </c>
+      <c r="L333" t="n">
+        <v>56308.7</v>
+      </c>
+      <c r="M333" t="n">
+        <v>56342</v>
+      </c>
+      <c r="N333" t="n">
+        <v>56248.9</v>
+      </c>
+      <c r="O333" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q333" t="n">
+        <v>56573.4</v>
+      </c>
+      <c r="R333" t="n">
+        <v>56255.4</v>
+      </c>
+      <c r="S333" t="n">
+        <v>56742.9</v>
+      </c>
+      <c r="T333" t="n">
+        <v>56295.6</v>
+      </c>
+      <c r="U333" t="n">
+        <v>56519.2</v>
+      </c>
+      <c r="V333" t="n">
+        <v>56370.1</v>
+      </c>
+      <c r="W333" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y333" t="n">
+        <v>56312.9</v>
+      </c>
+      <c r="Z333" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="AA333" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB333" t="n">
+        <v>56367.7</v>
+      </c>
+      <c r="AC333" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD333" t="n">
+        <v>55887.7</v>
+      </c>
+      <c r="AE333" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF333" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="AG333" t="inlineStr"/>
+      <c r="AH333" t="inlineStr"/>
+      <c r="AI333" t="inlineStr"/>
+      <c r="AJ333" t="inlineStr"/>
+      <c r="AK333" t="inlineStr"/>
+      <c r="AL333" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-11
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL333"/>
+  <dimension ref="A1:AL336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40508,12 +40508,372 @@
       <c r="AF333" t="n">
         <v>11.89</v>
       </c>
-      <c r="AG333" t="inlineStr"/>
-      <c r="AH333" t="inlineStr"/>
-      <c r="AI333" t="inlineStr"/>
-      <c r="AJ333" t="inlineStr"/>
-      <c r="AK333" t="inlineStr"/>
-      <c r="AL333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>56500</v>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G334" t="n">
+        <v>56498.6</v>
+      </c>
+      <c r="H334" t="n">
+        <v>75</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K334" t="n">
+        <v>5</v>
+      </c>
+      <c r="L334" t="n">
+        <v>56459.5</v>
+      </c>
+      <c r="M334" t="n">
+        <v>56368.2</v>
+      </c>
+      <c r="N334" t="n">
+        <v>56491.9</v>
+      </c>
+      <c r="O334" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q334" t="n">
+        <v>55970.1</v>
+      </c>
+      <c r="R334" t="n">
+        <v>55702.6</v>
+      </c>
+      <c r="S334" t="n">
+        <v>56573.4</v>
+      </c>
+      <c r="T334" t="n">
+        <v>56232.4</v>
+      </c>
+      <c r="U334" t="n">
+        <v>56448.9</v>
+      </c>
+      <c r="V334" t="n">
+        <v>56402.9</v>
+      </c>
+      <c r="W334" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X334" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y334" t="n">
+        <v>56407.8</v>
+      </c>
+      <c r="Z334" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="AA334" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB334" t="n">
+        <v>56378.6</v>
+      </c>
+      <c r="AC334" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD334" t="n">
+        <v>56858.6</v>
+      </c>
+      <c r="AE334" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF334" t="n">
+        <v>12.31</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>56600</v>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G335" t="n">
+        <v>56591.5</v>
+      </c>
+      <c r="H335" t="n">
+        <v>85</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K335" t="n">
+        <v>6</v>
+      </c>
+      <c r="L335" t="n">
+        <v>56528.2</v>
+      </c>
+      <c r="M335" t="n">
+        <v>56433.6</v>
+      </c>
+      <c r="N335" t="n">
+        <v>56588.4</v>
+      </c>
+      <c r="O335" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="P335" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q335" t="n">
+        <v>55970.1</v>
+      </c>
+      <c r="R335" t="n">
+        <v>55702.6</v>
+      </c>
+      <c r="S335" t="n">
+        <v>56573.4</v>
+      </c>
+      <c r="T335" t="n">
+        <v>56232.4</v>
+      </c>
+      <c r="U335" t="n">
+        <v>56448.9</v>
+      </c>
+      <c r="V335" t="n">
+        <v>56402.9</v>
+      </c>
+      <c r="W335" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X335" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y335" t="n">
+        <v>56412.8</v>
+      </c>
+      <c r="Z335" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="AA335" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB335" t="n">
+        <v>56471.5</v>
+      </c>
+      <c r="AC335" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD335" t="n">
+        <v>56951.5</v>
+      </c>
+      <c r="AE335" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF335" t="n">
+        <v>12.27</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>56600</v>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G336" t="n">
+        <v>56586.6</v>
+      </c>
+      <c r="H336" t="n">
+        <v>95</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K336" t="n">
+        <v>7</v>
+      </c>
+      <c r="L336" t="n">
+        <v>56562</v>
+      </c>
+      <c r="M336" t="n">
+        <v>56489.6</v>
+      </c>
+      <c r="N336" t="n">
+        <v>56559</v>
+      </c>
+      <c r="O336" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="P336" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q336" t="n">
+        <v>55970.1</v>
+      </c>
+      <c r="R336" t="n">
+        <v>55702.6</v>
+      </c>
+      <c r="S336" t="n">
+        <v>56573.4</v>
+      </c>
+      <c r="T336" t="n">
+        <v>56232.4</v>
+      </c>
+      <c r="U336" t="n">
+        <v>56448.9</v>
+      </c>
+      <c r="V336" t="n">
+        <v>56402.9</v>
+      </c>
+      <c r="W336" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X336" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y336" t="n">
+        <v>56418.4</v>
+      </c>
+      <c r="Z336" t="n">
+        <v>0.297</v>
+      </c>
+      <c r="AA336" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB336" t="n">
+        <v>56466.6</v>
+      </c>
+      <c r="AC336" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD336" t="n">
+        <v>56946.6</v>
+      </c>
+      <c r="AE336" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF336" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="AG336" t="inlineStr"/>
+      <c r="AH336" t="inlineStr"/>
+      <c r="AI336" t="inlineStr"/>
+      <c r="AJ336" t="inlineStr"/>
+      <c r="AK336" t="inlineStr"/>
+      <c r="AL336" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>